<commit_message>
feat: Product/Offer schema on deal listings; strengthen page-build pipeline
- Add lib/dealSchema.ts: Product/Offer JSON-LD matching Google's product
  rich-result guidance, applied to /deals, both branches of
  /postcode/[area], and /providers/[slug]. Prices mirror what each page
  already displays; no fabricated aggregateRating since the data model
  has no real review-count field
- Update scripts/build_keyword_mapping.py's page-build prompt and
  docs/page-build-pipeline-brief.md to require, for every future build:
  live keyword/SERP research before writing (not just the static curated
  dataset), matching content depth to what's actually ranking for that
  keyword rather than a fixed word count, and explicit GEO/AI-citation
  practices (standalone quotable excerpts and FAQ answers)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -653,7 +653,7 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="50" customWidth="1" min="12" max="12"/>
@@ -758,12 +758,16 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Committed 0536abb, pushed to origin/main 2026-08-21. Production and git are back in sync.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -802,22 +806,14 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Sahil</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr"/>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Started scoping the schema fields</t>
+          <t>Shipped 2026-08-21: Product/Offer JSON-LD (lib/dealSchema.ts) added to /deals, /postcode/[area] (both branches) and /providers/[slug]. Prices mirror visible content; no fabricated aggregateRating (no real review-count field in the data model).</t>
         </is>
       </c>
     </row>
@@ -1782,14 +1778,14 @@
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Built locally — not deployed</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr"/>
       <c r="K25" s="3" t="inlineStr"/>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>Component + page built and validated (npm run build, local render check) 2026-08-21. Not committed/pushed/deployed — held back pending the git/Vercel reconciliation (see rank #1).</t>
+          <t>Live at /tools/broadband-cost-calculator, committed and deployed 2026-08-21.</t>
         </is>
       </c>
     </row>
@@ -2697,9 +2693,9 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="31" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="50" customWidth="1" min="12" max="12"/>
@@ -2794,10 +2790,14 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Done</t>
@@ -2844,10 +2844,14 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Done</t>
@@ -2894,10 +2898,14 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Done</t>
@@ -2944,10 +2952,14 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Done</t>
@@ -2994,10 +3006,14 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3044,10 +3060,14 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3094,10 +3114,14 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3144,10 +3168,14 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3194,10 +3222,14 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3244,10 +3276,14 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3294,10 +3330,14 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3344,10 +3384,14 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3394,10 +3438,14 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3444,10 +3492,14 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3494,10 +3546,14 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3544,10 +3600,14 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3594,10 +3654,14 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3644,10 +3708,14 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3694,10 +3762,14 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -3744,13 +3816,13 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
+          <t>Planned — not live</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr"/>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Built locally — not deployed</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -3794,7 +3866,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
+          <t>Planned — not live</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -3844,7 +3916,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
+          <t>Planned — not live</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr"/>
@@ -3894,7 +3966,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
+          <t>Planned — not live</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -3944,7 +4016,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
+          <t>Planned — not live</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr"/>
@@ -3994,7 +4066,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
+          <t>Planned — not live</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -4044,7 +4116,7 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
+          <t>Planned — not live</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr"/>
@@ -4094,7 +4166,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
+          <t>Planned — not live</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -4144,10 +4216,14 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Live but not committed to git</t>
+        </is>
+      </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
           <t>Done</t>
@@ -4194,7 +4270,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
+          <t>Planned — not live</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -4244,7 +4320,7 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
+          <t>Planned — not live</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr"/>
@@ -4294,7 +4370,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
+          <t>Planned — not live</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -4344,7 +4420,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
+          <t>Planned — not live</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr"/>
@@ -4394,7 +4470,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
+          <t>Planned — not live</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -4558,7 +4634,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -4614,7 +4690,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
@@ -5169,7 +5245,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>44 total (33 page builds, 11 feature/strategy builds); 19 already marked Done.</t>
+          <t>44 total (33 page builds, 11 feature/strategy builds); 22 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add Instagram link to footer
Added @broadbandpicker Instagram as a second social pill button next to
X, same hover-interactive treatment.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -2727,7 +2727,11 @@
       </c>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr"/>
-      <c r="L46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Follow-up 2026-08-23: added Instagram (@broadbandpicker) as a second social pill button next to X, same hover treatment.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
@@ -2930,7 +2934,7 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="31" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
@@ -3031,7 +3035,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -3085,7 +3089,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -3139,7 +3143,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -3193,7 +3197,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -3247,7 +3251,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -3301,7 +3305,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -3355,7 +3359,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -3409,7 +3413,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -3463,7 +3467,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -3517,7 +3521,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -3571,7 +3575,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -3625,7 +3629,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -3679,7 +3683,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -3733,7 +3737,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -3787,7 +3791,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -3841,7 +3845,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -3895,7 +3899,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -3949,7 +3953,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -4003,7 +4007,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -4057,7 +4061,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -4111,7 +4115,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -4165,7 +4169,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -4219,7 +4223,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -4273,7 +4277,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -4327,7 +4331,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -4381,7 +4385,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -4435,7 +4439,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -4489,7 +4493,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -4543,7 +4547,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -4597,7 +4601,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -4651,7 +4655,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: reconcile keyword-mapping workbook against live sitemap
Re-ran scripts/build_keyword_mapping.py against production after
deploying the new TalkTalk/Zzoomm/Highland Broadband content and
comparison pages, so the Content Gap Roadmap reflects them as shipped.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$65</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PendingBuildPriorityTable" displayName="PendingBuildPriorityTable" ref="A1:N48" headerRowCount="1">
-  <autoFilter ref="A1:N48"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PendingBuildPriorityTable" displayName="PendingBuildPriorityTable" ref="A1:N15" headerRowCount="1">
+  <autoFilter ref="A1:N15"/>
   <tableColumns count="14">
     <tableColumn id="1" name="Pending Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr"/>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr"/>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr"/>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr"/>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr"/>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr"/>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr"/>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr"/>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr"/>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr"/>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr"/>
@@ -1819,7 +1819,7 @@
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr"/>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr"/>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr"/>
@@ -2179,7 +2179,7 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr"/>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr"/>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr"/>
@@ -2487,7 +2487,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr"/>
@@ -2619,7 +2619,7 @@
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr"/>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr"/>
@@ -2843,7 +2843,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
@@ -3617,23 +3617,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N48"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="50" customWidth="1" min="10" max="10"/>
     <col width="50" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -3714,46 +3714,50 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>page-providers/compare/hyperoptic-vs-youfibre</t>
+          <t>growth-awin-advertiser-outreach</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Partnerships</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Monetisation</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Hyperoptic vs YouFibre broadband: which is better in 2026?</t>
+          <t>Continue selective Awin advertiser outreach</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>67.90000000000001</v>
+        <v>60</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>37</v>
+        <v>70</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Very easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/compare/hyperoptic-vs-youfibre</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr"/>
+          <t>Awin publisher 2942019 and partner application log</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Current audience evidence and compliant commercial pages</t>
+        </is>
+      </c>
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr"/>
@@ -3764,33 +3768,33 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>page-postcode/sheffield</t>
+          <t>feat-review-aggregation-module</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Broadband providers in Sheffield: coverage and best deals</t>
+          <t>Real review-aggregation trust module</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>66.8</v>
+        <v>59</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Very easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -3800,10 +3804,14 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/postcode/sheffield</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr"/>
+          <t>New shared component, used on provider + comparison pages</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>research/uk-broadband-customer-satisfaction methodology</t>
+        </is>
+      </c>
       <c r="L3" s="3" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="3" t="inlineStr"/>
@@ -3814,46 +3822,50 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>page-guides/static-ip-business-broadband-explained</t>
+          <t>ops-adsense-site-review</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Monetisation</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Static IP business broadband: when you need one and how much it costs</t>
+          <t>Complete AdSense site review and authorisation monitoring</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>66.3</v>
+        <v>58</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>46.1</v>
+        <v>55</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/guides/static-ip-business-broadband-explained</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr"/>
+          <t>AdSense status and /ads.txt</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Google site-review processing</t>
+        </is>
+      </c>
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr"/>
@@ -3864,12 +3876,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>page-guides/student-broadband-by-university-city</t>
+          <t>audit-city-hub-thinness</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Content audit</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -3879,18 +3891,18 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Student broadband by university city: short-term and rolling deals</t>
+          <t>Verify each new city hub has a genuinely local fact</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>65.90000000000001</v>
+        <v>56</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>36.2</v>
+        <v>50</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Very easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -3900,10 +3912,14 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/guides/student-broadband-by-university-city</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr"/>
+          <t>data/priority-pages.ts city entries</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="L5" s="3" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="3" t="inlineStr"/>
@@ -3914,46 +3930,50 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>page-postcode/edinburgh</t>
+          <t>feat-contact-form-email-delivery</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Broadband providers in Edinburgh: coverage and best deals</t>
+          <t>Working contact form delivering to a real inbox, no third-party service</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>65.8</v>
+        <v>55</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/postcode/edinburgh</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr"/>
+          <t>app/api/contact/route.ts, components/ContactForm.tsx, app/contact/page.tsx</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>CONTACT_SMTP_USER / CONTACT_SMTP_PASS Gmail App Password set in Vercel env vars</t>
+        </is>
+      </c>
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr"/>
@@ -3964,12 +3984,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>page-guides/small-office-broadband-setup-uk</t>
+          <t>growth-original-research-outreach</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -3979,31 +3999,35 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Small office broadband setup: routers, backup and support checklist</t>
+          <t>Run original-research outreach and digital PR</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>65.8</v>
+        <v>54</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>41.9</v>
+        <v>68</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/guides/small-office-broadband-setup-uk</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr"/>
+          <t>/research/uk-broadband-customer-satisfaction</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Research page and source methodology are live</t>
+        </is>
+      </c>
       <c r="L7" s="3" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="3" t="inlineStr"/>
@@ -4014,33 +4038,33 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>page-providers/compare/bt-vs-plusnet</t>
+          <t>growth-quarterly-data-reprioritisation</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>BT vs Plusnet broadband: which is better in 2026?</t>
+          <t>Reprioritise quarter two using GSC, engagement and affiliate evidence</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>65.5</v>
+        <v>53</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>36.4</v>
+        <v>63</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Very easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -4050,10 +4074,14 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/compare/bt-vs-plusnet</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr"/>
+          <t>Next-quarter decision log</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>ops-conversion-reporting-loop and sufficient observation period</t>
+        </is>
+      </c>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="inlineStr"/>
@@ -4064,33 +4092,33 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>page-postcode/glasgow</t>
+          <t>feat-price-drop-alerts</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Broadband providers in Glasgow: coverage and best deals</t>
+          <t>Price-drop alerts</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>65.5</v>
+        <v>49</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>40.2</v>
+        <v>55</v>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -4100,10 +4128,14 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/postcode/glasgow</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr"/>
+          <t>New subscription flow + data/provider-live-deals.json</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Email delivery provider</t>
+        </is>
+      </c>
       <c r="L9" s="3" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="3" t="inlineStr"/>
@@ -4114,33 +4146,33 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>page-postcode/liverpool</t>
+          <t>audit-core-web-vitals-reporting</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Broadband providers in Liverpool: coverage and best deals</t>
+          <t>Establish monthly Core Web Vitals reporting by template</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>65.5</v>
+        <v>47</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>40.1</v>
+        <v>50</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -4150,10 +4182,14 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/postcode/liverpool</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr"/>
+          <t>Sitewide template performance report</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Field data or representative lab baselines</t>
+        </is>
+      </c>
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr"/>
@@ -4164,33 +4200,33 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>page-guides/broadband-for-landlords-and-hmos-uk</t>
+          <t>audit-mobile-checkout-flow</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>UX audit</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Broadband for landlords and HMOs: what to set up and who pays</t>
+          <t>Mobile checkout-flow audit</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>65.09999999999999</v>
+        <v>45</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>36.6</v>
+        <v>58</v>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Very easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -4200,10 +4236,14 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/guides/broadband-for-landlords-and-hmos-uk</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr"/>
+          <t>Sitewide mobile layout</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Mobile analytics/drop-off data</t>
+        </is>
+      </c>
       <c r="L11" s="3" t="inlineStr"/>
       <c r="M11" s="3" t="inlineStr"/>
       <c r="N11" s="3" t="inlineStr"/>
@@ -4214,33 +4254,33 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>page-postcode/leeds</t>
+          <t>audit-broken-links-redirects</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Crawlability</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Broadband providers in Leeds: coverage and best deals</t>
+          <t>Add routine broken-link and redirect reporting</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>65.09999999999999</v>
+        <v>44</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>40.3</v>
+        <v>48</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -4250,10 +4290,14 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/postcode/leeds</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr"/>
+          <t>Sitewide crawl and redirect report</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr"/>
@@ -4264,12 +4308,12 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>page-providers/compare/ee-vs-talktalk</t>
+          <t>bet-annual-research-report</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -4279,18 +4323,18 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>EE vs TalkTalk broadband: which is better in 2026?</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="F13" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="G13" s="3" t="n">
         <v>65</v>
       </c>
-      <c r="G13" s="3" t="n">
-        <v>36.4</v>
-      </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Very easy</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -4300,10 +4344,14 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/compare/ee-vs-talktalk</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr"/>
+          <t>New annual research page + methodology extension</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>research/uk-broadband-customer-satisfaction methodology</t>
+        </is>
+      </c>
       <c r="L13" s="3" t="inlineStr"/>
       <c r="M13" s="3" t="inlineStr"/>
       <c r="N13" s="3" t="inlineStr"/>
@@ -4314,33 +4362,33 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>page-postcode/bristol</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Broadband providers in Bristol: coverage and best deals</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>64.90000000000001</v>
+        <v>38</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>40.8</v>
+        <v>45</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -4350,10 +4398,14 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/postcode/bristol</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr"/>
+          <t>components/</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+        </is>
+      </c>
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr"/>
@@ -4364,12 +4416,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>page-postcode/birmingham</t>
+          <t>bet-decouple-content-from-code</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -4379,18 +4431,18 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Broadband providers in Birmingham: coverage and best deals</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="F15" s="3" t="n">
-        <v>64.5</v>
+        <v>35</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>41.1</v>
+        <v>48</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -4400,1726 +4452,20 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/postcode/birmingham</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr"/>
+          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>None, but easier before the guide count grows further</t>
+        </is>
+      </c>
       <c r="L15" s="3" t="inlineStr"/>
       <c r="M15" s="3" t="inlineStr"/>
       <c r="N15" s="3" t="inlineStr"/>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>page-postcode/manchester</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Broadband providers in Manchester: coverage and best deals</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>64.2</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>41.2</v>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/postcode/manchester</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>page-guides/leased-line-cost-uk-explained</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Leased line cost UK: what small businesses actually pay</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="n">
-        <v>63.3</v>
-      </c>
-      <c r="G17" s="3" t="n">
-        <v>58.6</v>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/leased-line-cost-uk-explained</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr"/>
-      <c r="L17" s="3" t="inlineStr"/>
-      <c r="M17" s="3" t="inlineStr"/>
-      <c r="N17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>page-guides/starlink-vs-fibre-broadband-uk</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Starlink vs fibre broadband: when satellite makes sense in the UK</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>62.9</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/starlink-vs-fibre-broadband-uk</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>page-providers/compare/virgin-media-vs-sky</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>Virgin Media vs Sky broadband: which is better in 2026?</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="n">
-        <v>62.8</v>
-      </c>
-      <c r="G19" s="3" t="n">
-        <v>36.2</v>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/providers/compare/virgin-media-vs-sky</t>
-        </is>
-      </c>
-      <c r="K19" s="3" t="inlineStr"/>
-      <c r="L19" s="3" t="inlineStr"/>
-      <c r="M19" s="3" t="inlineStr"/>
-      <c r="N19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>page-guides/january-broadband-deals-uk</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>January broadband deals UK: new-year switching guide</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="n">
-        <v>61.7</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>36.9</v>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/january-broadband-deals-uk</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>growth-awin-advertiser-outreach</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Partnerships</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Monetisation</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>Continue selective Awin advertiser outreach</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="n">
-        <v>60</v>
-      </c>
-      <c r="G21" s="3" t="n">
-        <v>70</v>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>Awin publisher 2942019 and partner application log</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="inlineStr">
-        <is>
-          <t>Current audience evidence and compliant commercial pages</t>
-        </is>
-      </c>
-      <c r="L21" s="3" t="inlineStr"/>
-      <c r="M21" s="3" t="inlineStr"/>
-      <c r="N21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>page-tools/broadband-cost-calculator</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Functionality</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Broadband cost calculator: true monthly and contract-length cost</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="n">
-        <v>59.9</v>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>27.6</v>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>Very easy</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/tools/broadband-cost-calculator</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>Live at /tools/broadband-cost-calculator, committed and deployed 2026-08-21.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>page-providers/onestream</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>Onestream — plans, coverage and Awin-tracked deals</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="n">
-        <v>59.4</v>
-      </c>
-      <c r="G23" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Very easy</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/providers/onestream</t>
-        </is>
-      </c>
-      <c r="K23" s="3" t="inlineStr"/>
-      <c r="L23" s="3" t="inlineStr"/>
-      <c r="M23" s="3" t="inlineStr"/>
-      <c r="N23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>page-guides/no-credit-check-broadband-uk</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>No credit check broadband in the UK: options and what to expect</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>34.8</v>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/no-credit-check-broadband-uk</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>feat-review-aggregation-module</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>Functionality</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>Real review-aggregation trust module</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="n">
-        <v>59</v>
-      </c>
-      <c r="G25" s="3" t="n">
-        <v>62</v>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
-          <t>New shared component, used on provider + comparison pages</t>
-        </is>
-      </c>
-      <c r="K25" s="3" t="inlineStr">
-        <is>
-          <t>research/uk-broadband-customer-satisfaction methodology</t>
-        </is>
-      </c>
-      <c r="L25" s="3" t="inlineStr"/>
-      <c r="M25" s="3" t="inlineStr"/>
-      <c r="N25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>page-providers/brsk</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Brsk — plans, coverage and Awin-tracked deals</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>Very easy</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/providers/brsk</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>page-guides/fttp-vs-fttc-explained</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>FTTP vs FTTC: what the difference means for your speed</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="n">
-        <v>58.4</v>
-      </c>
-      <c r="G27" s="3" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>Very easy</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/fttp-vs-fttc-explained</t>
-        </is>
-      </c>
-      <c r="K27" s="3" t="inlineStr"/>
-      <c r="L27" s="3" t="inlineStr"/>
-      <c r="M27" s="3" t="inlineStr"/>
-      <c r="N27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>page-guides/best-mesh-wifi-for-your-broadband-router</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Best mesh Wi-Fi systems to pair with your broadband router</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="n">
-        <v>58.4</v>
-      </c>
-      <c r="G28" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/best-mesh-wifi-for-your-broadband-router</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>page-guides/broadband-help-if-you-claim-benefits-uk</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>Cheaper broadband if you claim benefits: social tariffs explained</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="n">
-        <v>58.2</v>
-      </c>
-      <c r="G29" s="3" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>Very easy</t>
-        </is>
-      </c>
-      <c r="I29" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J29" s="3" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/broadband-help-if-you-claim-benefits-uk</t>
-        </is>
-      </c>
-      <c r="K29" s="3" t="inlineStr"/>
-      <c r="L29" s="3" t="inlineStr"/>
-      <c r="M29" s="3" t="inlineStr"/>
-      <c r="N29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>ops-adsense-site-review</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Monetisation</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Infrastructure</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Complete AdSense site review and authorisation monitoring</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="G30" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>AdSense status and /ads.txt</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>Google site-review processing</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>page-providers/gigaclear</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>Gigaclear — plans, coverage and Awin-tracked deals</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="n">
-        <v>56.9</v>
-      </c>
-      <c r="G31" s="3" t="n">
-        <v>27.9</v>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/providers/gigaclear</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr"/>
-      <c r="L31" s="3" t="inlineStr"/>
-      <c r="M31" s="3" t="inlineStr"/>
-      <c r="N31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>page-providers/youfibre</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>YouFibre — plans, coverage and Awin-tracked deals</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="n">
-        <v>56.6</v>
-      </c>
-      <c r="G32" s="2" t="n">
-        <v>28.7</v>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/providers/youfibre</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr"/>
-      <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>page-providers/cuckoo</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>Cuckoo Broadband — plans, coverage and Awin-tracked deals</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="n">
-        <v>56.5</v>
-      </c>
-      <c r="G33" s="3" t="n">
-        <v>27.9</v>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="I33" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J33" s="3" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/providers/cuckoo</t>
-        </is>
-      </c>
-      <c r="K33" s="3" t="inlineStr"/>
-      <c r="L33" s="3" t="inlineStr"/>
-      <c r="M33" s="3" t="inlineStr"/>
-      <c r="N33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>audit-city-hub-thinness</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Content audit</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Verify each new city hub has a genuinely local fact</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="n">
-        <v>56</v>
-      </c>
-      <c r="G34" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>data/priority-pages.ts city entries</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr"/>
-      <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>page-guides/black-friday-broadband-deals-uk</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>Black Friday broadband deals UK: what to expect and how to compare</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="n">
-        <v>55.8</v>
-      </c>
-      <c r="G35" s="3" t="n">
-        <v>37</v>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>Competitive</t>
-        </is>
-      </c>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J35" s="3" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/black-friday-broadband-deals-uk</t>
-        </is>
-      </c>
-      <c r="K35" s="3" t="inlineStr"/>
-      <c r="L35" s="3" t="inlineStr"/>
-      <c r="M35" s="3" t="inlineStr"/>
-      <c r="N35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>page-providers/shell-energy</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Shell Energy Broadband — plans, coverage and Awin-tracked deals</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="n">
-        <v>55.7</v>
-      </c>
-      <c r="G36" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/providers/shell-energy</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr"/>
-      <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>page-research/broadband-customer-service-rankings-uk</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>Broadband customer service rankings: Ofcom-evidenced comparison</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="n">
-        <v>55.1</v>
-      </c>
-      <c r="G37" s="3" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="I37" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J37" s="3" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/research/broadband-customer-service-rankings-uk</t>
-        </is>
-      </c>
-      <c r="K37" s="3" t="inlineStr"/>
-      <c r="L37" s="3" t="inlineStr"/>
-      <c r="M37" s="3" t="inlineStr"/>
-      <c r="N37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>feat-contact-form-email-delivery</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>Infrastructure</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Working contact form delivering to a real inbox, no third-party service</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G38" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>app/api/contact/route.ts, components/ContactForm.tsx, app/contact/page.tsx</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>CONTACT_SMTP_USER / CONTACT_SMTP_PASS Gmail App Password set in Vercel env vars</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr"/>
-      <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>page-guides/broadband-complaints-and-ombudsman-uk</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Broadband complaints and the ombudsman: your UK rights</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="n">
-        <v>54.7</v>
-      </c>
-      <c r="G39" s="3" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="I39" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J39" s="3" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/broadband-complaints-and-ombudsman-uk</t>
-        </is>
-      </c>
-      <c r="K39" s="3" t="inlineStr"/>
-      <c r="L39" s="3" t="inlineStr"/>
-      <c r="M39" s="3" t="inlineStr"/>
-      <c r="N39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>growth-original-research-outreach</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Run original-research outreach and digital PR</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="G40" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>/research/uk-broadband-customer-satisfaction</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>Research page and source methodology are live</t>
-        </is>
-      </c>
-      <c r="L40" s="2" t="inlineStr"/>
-      <c r="M40" s="2" t="inlineStr"/>
-      <c r="N40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>growth-quarterly-data-reprioritisation</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>Strategy</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>Reprioritise quarter two using GSC, engagement and affiliate evidence</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="n">
-        <v>53</v>
-      </c>
-      <c r="G41" s="3" t="n">
-        <v>63</v>
-      </c>
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I41" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J41" s="3" t="inlineStr">
-        <is>
-          <t>Next-quarter decision log</t>
-        </is>
-      </c>
-      <c r="K41" s="3" t="inlineStr">
-        <is>
-          <t>ops-conversion-reporting-loop and sufficient observation period</t>
-        </is>
-      </c>
-      <c r="L41" s="3" t="inlineStr"/>
-      <c r="M41" s="3" t="inlineStr"/>
-      <c r="N41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>feat-price-drop-alerts</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Functionality</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Price-drop alerts</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="G42" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>New subscription flow + data/provider-live-deals.json</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>Email delivery provider</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr"/>
-      <c r="M42" s="2" t="inlineStr"/>
-      <c r="N42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>audit-core-web-vitals-reporting</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>Technical SEO</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>Performance</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>Establish monthly Core Web Vitals reporting by template</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="n">
-        <v>47</v>
-      </c>
-      <c r="G43" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J43" s="3" t="inlineStr">
-        <is>
-          <t>Sitewide template performance report</t>
-        </is>
-      </c>
-      <c r="K43" s="3" t="inlineStr">
-        <is>
-          <t>Field data or representative lab baselines</t>
-        </is>
-      </c>
-      <c r="L43" s="3" t="inlineStr"/>
-      <c r="M43" s="3" t="inlineStr"/>
-      <c r="N43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>audit-mobile-checkout-flow</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>UX audit</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>UX</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Mobile checkout-flow audit</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="G44" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>Sitewide mobile layout</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="inlineStr">
-        <is>
-          <t>Mobile analytics/drop-off data</t>
-        </is>
-      </c>
-      <c r="L44" s="2" t="inlineStr"/>
-      <c r="M44" s="2" t="inlineStr"/>
-      <c r="N44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>audit-broken-links-redirects</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>Technical SEO</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>Crawlability</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>Add routine broken-link and redirect reporting</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="n">
-        <v>44</v>
-      </c>
-      <c r="G45" s="3" t="n">
-        <v>48</v>
-      </c>
-      <c r="H45" s="3" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="I45" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J45" s="3" t="inlineStr">
-        <is>
-          <t>Sitewide crawl and redirect report</t>
-        </is>
-      </c>
-      <c r="K45" s="3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L45" s="3" t="inlineStr"/>
-      <c r="M45" s="3" t="inlineStr"/>
-      <c r="N45" s="3" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>bet-annual-research-report</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Bigger bet</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Annual 'State of UK Broadband' research report</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="G46" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>New annual research page + methodology extension</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>research/uk-broadband-customer-satisfaction methodology</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr"/>
-      <c r="M46" s="2" t="inlineStr"/>
-      <c r="N46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>bet-componentise-interactive-layer</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>Bigger bet</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>Functionality</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="n">
-        <v>38</v>
-      </c>
-      <c r="G47" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="H47" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I47" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J47" s="3" t="inlineStr">
-        <is>
-          <t>components/</t>
-        </is>
-      </c>
-      <c r="K47" s="3" t="inlineStr">
-        <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
-        </is>
-      </c>
-      <c r="L47" s="3" t="inlineStr"/>
-      <c r="M47" s="3" t="inlineStr"/>
-      <c r="N47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>bet-decouple-content-from-code</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Bigger bet</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Decouple guide content from code deploys</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="G48" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>None, but easier before the guide count grows further</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr"/>
-      <c r="M48" s="2" t="inlineStr"/>
-      <c r="N48" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N48"/>
+  <autoFilter ref="A1:N15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6142,9 +4488,9 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="50" customWidth="1" min="12" max="12"/>
@@ -6239,13 +4585,17 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -6289,13 +4639,17 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -6339,13 +4693,17 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -6389,13 +4747,17 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -6439,13 +4801,17 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -6489,13 +4855,17 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -6539,13 +4909,17 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -6589,13 +4963,17 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -6639,13 +5017,17 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -6689,13 +5071,17 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
@@ -6739,13 +5125,17 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -6789,13 +5179,17 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
@@ -6839,13 +5233,17 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -6889,13 +5287,17 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
@@ -6939,13 +5341,17 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -6989,13 +5395,17 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
@@ -7039,13 +5449,17 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -7089,13 +5503,17 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
@@ -7139,13 +5557,17 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -7189,13 +5611,17 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -7239,13 +5665,17 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -7289,13 +5719,17 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
@@ -7339,13 +5773,17 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -7389,13 +5827,17 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
@@ -7439,13 +5881,17 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -7489,13 +5935,17 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
@@ -7539,13 +5989,17 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -7589,13 +6043,17 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
@@ -7639,13 +6097,17 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -7689,13 +6151,17 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
@@ -7739,13 +6205,17 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -7789,13 +6259,17 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
@@ -7839,13 +6313,17 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Planned — live check unavailable</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr"/>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -9734,7 +8212,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>64 total (33 page builds, 31 feature/strategy builds); 17 already marked Done.</t>
+          <t>64 total (33 page builds, 31 feature/strategy builds); 50 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: reconcile keyword-mapping workbook after TV deals guide refresh
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -4621,7 +4621,7 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="31" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -4776,7 +4776,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -4830,7 +4830,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -4992,7 +4992,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -5046,7 +5046,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -5100,7 +5100,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -5262,7 +5262,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -5370,7 +5370,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -5424,7 +5424,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -5478,7 +5478,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -5532,7 +5532,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -5586,7 +5586,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -5640,7 +5640,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -5694,7 +5694,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -5748,7 +5748,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -5802,7 +5802,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -5856,7 +5856,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -5910,7 +5910,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -6018,7 +6018,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -6072,7 +6072,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -6234,7 +6234,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -6396,7 +6396,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -6450,7 +6450,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">

</xml_diff>

<commit_message>
content: deep rewrite of best-phone-and-broadband-deals guide
Fifth target from scripts/analyze_content_priority.py's ranked list
(457 words, no dates or stats, one stray em dash). Rewrote with the
real PSTN switch-off timeline: full shutdown locked in for 31 January
2027 (moved from Dec 2025 after Openreach confirmed the technical
barriers were resolved), PSTN customer numbers falling from 5.2
million (July 2024) to 3.2 million (July 2025), Ofcom's one-hour
battery backup requirement during power cuts, and the industry PSTN
Charter's telecare/vulnerable-user protections. Added a real call-plan
cost example (TalkTalk Anytime Calls, GBP12/mo). FAQs expanded 3->5,
em dash fixed, updated date set to 2026-08-24.

Also bundles the concurrently-running content pipeline's
scripts/manage_ga4_key_events.py, already present in the working tree
and validated by the build above.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$74</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L73" headerRowCount="1">
-  <autoFilter ref="A1:L73"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L74" headerRowCount="1">
+  <autoFilter ref="A1:L74"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L40" headerRowCount="1">
-  <autoFilter ref="A1:L40"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L41" headerRowCount="1">
+  <autoFilter ref="A1:L41"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3784,38 +3784,38 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>audit-broken-links-redirects</t>
+          <t>content-refresh-best-phone-and-broadband-deals-guide</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Crawlability</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Add routine broken-link and redirect reporting</t>
+          <t>Deep rewrite: Best Phone and Broadband Deals guide (5th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G70" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="G70" s="2" t="n">
-        <v>48</v>
-      </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr"/>
@@ -3828,33 +3828,33 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>bet-annual-research-report</t>
+          <t>audit-broken-links-redirects</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Crawlability</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Add routine broken-link and redirect reporting</t>
         </is>
       </c>
       <c r="F71" s="3" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="G71" s="3" t="n">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
@@ -3872,7 +3872,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>bet-componentise-interactive-layer</t>
+          <t>bet-annual-research-report</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -3882,19 +3882,19 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
@@ -3916,7 +3916,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -3926,19 +3926,19 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F73" s="3" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G73" s="3" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
@@ -3954,8 +3954,52 @@
       <c r="K73" s="3" t="inlineStr"/>
       <c r="L73" s="3" t="inlineStr"/>
     </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>bet-decouple-content-from-code</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Decouple guide content from code deploys</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L73"/>
+  <autoFilter ref="A1:L74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6707,7 +6751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8752,53 +8796,53 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Crawlability</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Add routine broken-link and redirect reporting</t>
+          <t>Deep rewrite: Best Phone and Broadband Deals guide (5th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Monitor broken inbound and internal URLs and maintain relevant one-hop redirects.</t>
+          <t>Fifth target from scripts/analyze_content_priority.py's ranked list: the old copy was generic Digital Voice/line-rental advice with no dates, no stats and one pre-existing em dash, at 457 words. Rewritten with the real PSTN switch-off timeline: full shutdown now locked in for 31 January 2027 (moved from the original December 2025 target after Openreach confirmed the technical barriers were resolved), with PSTN customer numbers falling from 5.2 million (July 2024) to 3.2 million (July 2025). Added Ofcom's minimum one-hour battery backup requirement for emergency-services access during a power cut, and the industry PSTN Charter's commitment not to migrate telecare/vulnerable users without confirmed-compatible equipment. Added a real, specific call-plan cost example (TalkTalk's Anytime Calls add-on at GBP12/mo on top of base broadband) to replace the previous fully generic 'compare the whole contract' advice. FAQs expanded from 3 to 5. Fixed the pre-existing em dash in the dek field.</t>
         </is>
       </c>
       <c r="F37" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="G37" s="3" t="n">
         <v>44</v>
       </c>
-      <c r="G37" s="3" t="n">
-        <v>48</v>
-      </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>Sitewide crawl and redirect report</t>
+          <t>data/priority-pages.ts (phone)</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t>BroadbandPicker SEO &amp; Content Plan — Live: Technical SEO</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -8808,43 +8852,43 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Crawlability</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Add routine broken-link and redirect reporting</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
+          <t>Monitor broken inbound and internal URLs and maintain relevant one-hop redirects.</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>New annual research page + methodology extension</t>
+          <t>Sitewide crawl and redirect report</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>research/uk-broadband-customer-satisfaction methodology</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -8854,7 +8898,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>BroadbandPicker SEO &amp; Content Plan — Live: Technical SEO</t>
         </is>
       </c>
     </row>
@@ -8869,24 +8913,24 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
         </is>
       </c>
       <c r="F39" s="3" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
@@ -8895,12 +8939,12 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>components/</t>
+          <t>New annual research page + methodology extension</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+          <t>research/uk-broadband-customer-satisfaction methodology</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
@@ -8910,7 +8954,7 @@
       </c>
       <c r="L39" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -8925,53 +8969,109 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
+          <t>Functionality</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Componentise the interactive layer on accessible primitives</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>components/</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Growth playbook — Functionality pillar</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>Decouple guide content from code deploys</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
-      <c r="F40" s="2" t="n">
+      <c r="F41" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="G40" s="2" t="n">
+      <c r="G41" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="I41" s="3" t="inlineStr">
         <is>
           <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="J41" s="3" t="inlineStr">
         <is>
           <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
-      <c r="K40" s="2" t="inlineStr">
+      <c r="K41" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="L40" s="2" t="inlineStr">
+      <c r="L41" s="3" t="inlineStr">
         <is>
           <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L40"/>
+  <autoFilter ref="A1:L41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9012,7 +9112,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>72 total (33 page builds, 39 feature/strategy builds); 58 already marked Done.</t>
+          <t>73 total (33 page builds, 40 feature/strategy builds); 59 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of NOW Broadband provider page
Seventh target from scripts/analyze_content_priority.py's ranked list:
/providers/now-broadband was 386 words with no excerpt or contentSections,
and its top-level fields were stale on two counts -- contractLengths was
still [12] (NOW dropped its flexible 12-month contracts; every current
package is now a standard 24-month term) and monthlyPriceFrom was a
stale GBP17.99 against a real current cheapest tier of GBP23.

Rewritten to ~1,450 words with 5 sections. The distinctive finding here:
NOW is a genuine exception to the usual Trustpilot-vs-Ofcom divergence
pattern used elsewhere on this site -- it scores poorly on BOTH
Trustpilot (1.2/5, corrected from a stale 3.2) AND Ofcom's Q4 2025
complaints data (11 per 100k vs the 8 industry average), noticeably
worse than sister brand Sky on the same underlying Openreach network.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L75" headerRowCount="1">
-  <autoFilter ref="A1:L75"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L76" headerRowCount="1">
+  <autoFilter ref="A1:L76"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L42" headerRowCount="1">
-  <autoFilter ref="A1:L42"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L43" headerRowCount="1">
+  <autoFilter ref="A1:L43"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3916,12 +3916,12 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>bet-annual-research-report</t>
+          <t>content-refresh-now-broadband-provider-page</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -3931,23 +3931,23 @@
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F73" s="3" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="G73" s="3" t="n">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr"/>
@@ -3960,7 +3960,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>bet-componentise-interactive-layer</t>
+          <t>bet-annual-research-report</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -3970,19 +3970,19 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
@@ -4004,7 +4004,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -4014,19 +4014,19 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F75" s="3" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G75" s="3" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
@@ -4042,8 +4042,52 @@
       <c r="K75" s="3" t="inlineStr"/>
       <c r="L75" s="3" t="inlineStr"/>
     </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>bet-decouple-content-from-code</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>Decouple guide content from code deploys</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr"/>
+      <c r="L76" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L75"/>
+  <autoFilter ref="A1:L76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6795,7 +6839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9008,7 +9052,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -9018,43 +9062,43 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
+          <t>Seventh target from scripts/analyze_content_priority.py's ranked list: /providers/now-broadband was 386 words with no excerpt or contentSections, and its top-level fields were stale on two counts that research corrected -- contractLengths was still [12] (NOW dropped its flexible 12-month contracts; every current package is now a standard 24-month term, per thinkbroadband's dedicated news item on the change) and monthlyPriceFrom was a stale GBP17.99 against a real current cheapest tier of GBP23 (Full Fibre 100). Rewritten to ~1,450 words with 5 contentSections. The genuinely distinctive finding here, different from every other Trustpilot-vs-Ofcom section written this session: NOW is a real exception to the usual pattern, scoring poorly on BOTH Trustpilot (1.2/5, corrected from a stale 3.2) AND Ofcom's Q4 2025 complaints data (11 per 100k vs the 8 industry average), noticeably worse than sister brand Sky on the same underlying Openreach network -- written up as a genuine data point about support quality diverging from infrastructure quality within the same corporate group, not just review-platform noise. Also corrected trustpilotScore 3.2 -&gt; 1.2.</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>New annual research page + methodology extension</t>
+          <t>data/providers.ts (now-broadband)</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>research/uk-broadband-customer-satisfaction methodology</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9069,24 +9113,24 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
         </is>
       </c>
       <c r="F41" s="3" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
@@ -9095,12 +9139,12 @@
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>components/</t>
+          <t>New annual research page + methodology extension</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+          <t>research/uk-broadband-customer-satisfaction methodology</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
@@ -9110,7 +9154,7 @@
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -9125,53 +9169,109 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
+          <t>Functionality</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Componentise the interactive layer on accessible primitives</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>components/</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Growth playbook — Functionality pillar</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>Decouple guide content from code deploys</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
-      <c r="F42" s="2" t="n">
+      <c r="F43" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="G42" s="2" t="n">
+      <c r="G43" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="I43" s="3" t="inlineStr">
         <is>
           <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="J43" s="3" t="inlineStr">
         <is>
           <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
-      <c r="K42" s="2" t="inlineStr">
+      <c r="K43" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr">
+      <c r="L43" s="3" t="inlineStr">
         <is>
           <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L42"/>
+  <autoFilter ref="A1:L43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9212,7 +9312,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>74 total (33 page builds, 41 feature/strategy builds); 60 already marked Done.</t>
+          <t>75 total (33 page builds, 42 feature/strategy builds); 61 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of YouFibre provider page
Eighth target from scripts/analyze_content_priority.py's ranked list:
/providers/youfibre was 397 words with no excerpt or contentSections.

The standout finding, verified against a primary Virgin Media O2 press
release: YouFibre's parent company, Substantial Group (Netomnia), is
being acquired for GBP2bn by nexfibre (InfraVia/Liberty Global/
Telefonica), which then plans to resell the YouFibre/Brsk retail
brands to Virgin Media O2 for GBP150m. Announced Feb 2026, referred to
the CMA for a Phase 2 investigation on 1 July 2026, not yet completed.

Also wrote up the real, documented fallout from the March 2026
Brsk-to-YouFibre migration (billing errors, login failures, reported
speed drops, overwhelmed support), sourced from ISPreview. Updated the
speeds array to the real current symmetrical tiers (200/1000/2000/8000
Mbps) and contractLengths to match current pricing research.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$77</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L76" headerRowCount="1">
-  <autoFilter ref="A1:L76"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L77" headerRowCount="1">
+  <autoFilter ref="A1:L77"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L43" headerRowCount="1">
-  <autoFilter ref="A1:L43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L44" headerRowCount="1">
+  <autoFilter ref="A1:L44"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3960,12 +3960,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>bet-annual-research-report</t>
+          <t>content-refresh-youfibre-provider-page</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -3975,23 +3975,23 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr"/>
@@ -4004,7 +4004,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>bet-componentise-interactive-layer</t>
+          <t>bet-annual-research-report</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -4014,19 +4014,19 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="F75" s="3" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G75" s="3" t="n">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -4058,19 +4058,19 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
@@ -4086,8 +4086,52 @@
       <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr"/>
     </row>
+    <row r="77">
+      <c r="A77" s="3" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>bet-decouple-content-from-code</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>Decouple guide content from code deploys</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="G77" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr"/>
+      <c r="K77" s="3" t="inlineStr"/>
+      <c r="L77" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L76"/>
+  <autoFilter ref="A1:L77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6839,7 +6883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9108,7 +9152,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -9118,43 +9162,43 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
+          <t>Eighth target from scripts/analyze_content_priority.py's ranked list: /providers/youfibre was 397 words with no excerpt or contentSections. Rewritten to ~1,575 words with 6 contentSections. The standout finding, verified against a primary Virgin Media O2 press release after a first-pass WebSearch AI summary over-stated it as a done deal: YouFibre's parent company, Substantial Group (Netomnia), is being acquired for GBP2bn by nexfibre (a joint venture of InfraVia, Liberty Global and Telefonica), which then plans to resell the YouFibre/Brsk retail brands to Virgin Media O2 for GBP150m -- announced Feb 2026, referred to the CMA for a Phase 2 investigation on 1 July 2026, and NOT yet completed (expected ~Q3 2026 at the earliest). Also wrote up the real, documented fallout from the March 2026 Brsk-to-YouFibre customer migration (billing errors, login/password-reset failures, reported speed drops, overwhelmed support chat), sourced from ISPreview rather than the vague pre-existing 'Trustpilot sentiment has been mixed' line. Updated the speeds array to the real current tiers (200/1000/2000/8000 Mbps symmetrical, replacing stale 200/900/1800) and contractLengths from [1,12,24] to [1,24] to match the two options confirmed by current pricing research.</t>
         </is>
       </c>
       <c r="F41" s="3" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>New annual research page + methodology extension</t>
+          <t>data/providers.ts (youfibre)</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>research/uk-broadband-customer-satisfaction methodology</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9169,24 +9213,24 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -9195,12 +9239,12 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>components/</t>
+          <t>New annual research page + methodology extension</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+          <t>research/uk-broadband-customer-satisfaction methodology</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -9210,7 +9254,7 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -9225,53 +9269,109 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
+          <t>Functionality</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Componentise the interactive layer on accessible primitives</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>components/</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>Growth playbook — Functionality pillar</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>Decouple guide content from code deploys</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
-      <c r="F43" s="3" t="n">
+      <c r="F44" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="G43" s="3" t="n">
+      <c r="G44" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="H43" s="3" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I43" s="3" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
-      <c r="J43" s="3" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
         <is>
           <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
-      <c r="K43" s="3" t="inlineStr">
+      <c r="K44" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="L43" s="3" t="inlineStr">
+      <c r="L44" s="2" t="inlineStr">
         <is>
           <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L43"/>
+  <autoFilter ref="A1:L44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9312,7 +9412,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>75 total (33 page builds, 42 feature/strategy builds); 61 already marked Done.</t>
+          <t>76 total (33 page builds, 43 feature/strategy builds); 62 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Broadband Without a Phone Line guide
Tenth target from scripts/analyze_content_priority.py's ranked list:
770 words, a stale pricing table, and a wrong PSTN switch-off date
("by the end of 2027" -- the real, now-locked-in date is 31 January
2027). Reused the PSTN research from the earlier phone-and-broadband
guide refresh (5.2m -> 3.2m migration stat, Ofcom's 1-hour power-cut
battery backup minimum, PSTN Charter telecare protections) and added
a genuinely missing section on what actually happens to a Digital
Voice phone during a power cut, since the old version only covered
whether a line is needed at all.

Refreshed all 8 provider prices against this site's own current
provider-page data and added Ofcom's Spring 2026 Connected Nations
coverage split (89% gigabit-capable, 82% full fibre, 93% urban vs
66% rural).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L78" headerRowCount="1">
-  <autoFilter ref="A1:L78"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L79" headerRowCount="1">
+  <autoFilter ref="A1:L79"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L45" headerRowCount="1">
-  <autoFilter ref="A1:L45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L46" headerRowCount="1">
+  <autoFilter ref="A1:L46"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L78"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4092,38 +4092,38 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>bet-componentise-interactive-layer</t>
+          <t>content-refresh-broadband-without-phone-line-guide</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F77" s="3" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr"/>
@@ -4136,7 +4136,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -4146,19 +4146,19 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -4174,8 +4174,52 @@
       <c r="K78" s="2" t="inlineStr"/>
       <c r="L78" s="2" t="inlineStr"/>
     </row>
+    <row r="79">
+      <c r="A79" s="3" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>bet-decouple-content-from-code</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Decouple guide content from code deploys</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="G79" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J79" s="3" t="inlineStr"/>
+      <c r="K79" s="3" t="inlineStr"/>
+      <c r="L79" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L78"/>
+  <autoFilter ref="A1:L79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6927,7 +6971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9364,53 +9408,53 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+          <t>Tenth target from scripts/analyze_content_priority.py's ranked list: 770 words, stale pricing table (every one of 8 providers priced against months-old figures already corrected on this site's own provider pages), and a wrong PSTN switch-off date ('by the end of 2027' -- the real, now-locked-in date is 31 January 2027). Rewrote using the same PSTN research gathered for the best-phone-and-broadband-deals refresh earlier this session (5.2m -&gt; 3.2m migration stat, Ofcom's 1-hour power-cut battery backup minimum, the PSTN Charter's telecare protections), added a genuinely missing section -- 'What happens to a home phone during a power cut?' -- since the old version covered whether a line is needed at all but never addressed the actual practical question once Digital Voice is the default. Refreshed all 8 provider prices against data/providers.ts's own current fields, updated Virgin Media coverage 52% (was 53%) and added Ofcom's Spring 2026 Connected Nations split (89% gigabit-capable, 82% full fibre, 93% urban vs 66% rural). Word count 770 -&gt; 1,196; left just under the self-imposed 1,200-word floor rather than pad.</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>components/</t>
+          <t>app/guides/[slug]/page.tsx (broadband-without-phone-line), data/guides.ts</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9425,53 +9469,109 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
+          <t>Componentise the interactive layer on accessible primitives</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>components/</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>Growth playbook — Functionality pillar</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
           <t>Decouple guide content from code deploys</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
-      <c r="F45" s="3" t="n">
+      <c r="F46" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="G45" s="3" t="n">
+      <c r="G46" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="H45" s="3" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I45" s="3" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
-      <c r="J45" s="3" t="inlineStr">
+      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
-      <c r="K45" s="3" t="inlineStr">
+      <c r="K46" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="L45" s="3" t="inlineStr">
+      <c r="L46" s="2" t="inlineStr">
         <is>
           <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L45"/>
+  <autoFilter ref="A1:L46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9512,7 +9612,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>77 total (33 page builds, 44 feature/strategy builds); 63 already marked Done.</t>
+          <t>78 total (33 page builds, 45 feature/strategy builds); 64 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Broadband When Moving House checklist guide
Eleventh target from scripts/analyze_content_priority.py's ranked list:
948 words, structurally sound but missing a genuinely newsworthy
development -- Ofcom closed its One Touch Switch enforcement case on
11 June 2026 after finding more than 2 million customers had already
used the process successfully, making it the industry's permanent
standard rather than a monitored pilot.

Added this, plus a section on what a house move means for a home
phone line given the 31 January 2027 PSTN switch-off, Ofcom's Spring
2026 coverage split, and corrected the ETC explanation to reflect
Ofcom's actual cap rule. Re-verified the existing GBP183.60/year
switching-saving stat against fresh 2026 sources.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L79" headerRowCount="1">
-  <autoFilter ref="A1:L79"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L80" headerRowCount="1">
+  <autoFilter ref="A1:L80"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L46" headerRowCount="1">
-  <autoFilter ref="A1:L46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L47" headerRowCount="1">
+  <autoFilter ref="A1:L47"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4136,38 +4136,38 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>bet-componentise-interactive-layer</t>
+          <t>content-refresh-broadband-moving-house-guide</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr"/>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -4190,19 +4190,19 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F79" s="3" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
@@ -4218,8 +4218,52 @@
       <c r="K79" s="3" t="inlineStr"/>
       <c r="L79" s="3" t="inlineStr"/>
     </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>bet-decouple-content-from-code</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Decouple guide content from code deploys</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G80" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr"/>
+      <c r="L80" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L79"/>
+  <autoFilter ref="A1:L80"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6971,7 +7015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9464,53 +9508,53 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+          <t>Eleventh target from scripts/analyze_content_priority.py's ranked list: 948 words, structurally sound (evergreen checklist format) but missing a genuinely newsworthy development -- Ofcom closed its One Touch Switch enforcement case on 11 June 2026 after finding more than 2 million customers had already used the process successfully, meaning it is now the industry's permanent standard rather than a monitored pilot, which the old copy still implied. Added this, plus a genuinely missing section on what a house move means for a home phone line given the 31 January 2027 PSTN switch-off (reusing research from the phone-and-broadband and broadband-without-phone-line refreshes earlier this session), Ofcom's Spring 2026 coverage split for the 'check availability' step, and corrected the ETC explanation to reflect Ofcom's actual cap rule (remaining payments, ex-VAT) rather than a flat multiplication. Re-verified the pre-existing GBP183.60/year switching-saving stat against fresh 2026 sources (found independently corroborated) and added the 4.2m/GBP100-240 social tariff stat already used elsewhere on this site. Word count 948 -&gt; 1,446.</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>components/</t>
+          <t>app/guides/[slug]/page.tsx (broadband-moving-house), data/guides.ts</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9525,53 +9569,109 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
+          <t>Componentise the interactive layer on accessible primitives</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>components/</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Growth playbook — Functionality pillar</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
           <t>Decouple guide content from code deploys</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
-      <c r="F46" s="2" t="n">
+      <c r="F47" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="G46" s="2" t="n">
+      <c r="G47" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="I47" s="3" t="inlineStr">
         <is>
           <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="J47" s="3" t="inlineStr">
         <is>
           <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
-      <c r="K46" s="2" t="inlineStr">
+      <c r="K47" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="L46" s="2" t="inlineStr">
+      <c r="L47" s="3" t="inlineStr">
         <is>
           <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L46"/>
+  <autoFilter ref="A1:L47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9612,7 +9712,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>78 total (33 page builds, 45 feature/strategy builds); 64 already marked Done.</t>
+          <t>79 total (33 page builds, 46 feature/strategy builds); 65 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Satellite Broadband UK guide
Twelfth target from scripts/analyze_content_priority.py's ranked list.
The old copy was generic to the point of naming no real prices at all.
Rewritten with real, current Starlink UK pricing (Residential
100/200/Max at GBP40/60/80/mo, Roam at GBP55-100, Standard Kit GBP449
commonly discounted to ~GBP299 or free on Max), and a genuinely
current news item: Starlink's Global Roam plan stopped taking new
customers 15 July 2026 and was withdrawn entirely for existing
customers on 17 August 2026, one week before this rewrite.

Named 2 real smaller alternatives (SkyDSL, Bigblu Broadband) and
clarified that Eutelsat/OneWeb sells no UK consumer home-broadband
plans at all, despite frequent mention alongside Starlink.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$81</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L80" headerRowCount="1">
-  <autoFilter ref="A1:L80"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L81" headerRowCount="1">
+  <autoFilter ref="A1:L81"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L47" headerRowCount="1">
-  <autoFilter ref="A1:L47"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L48" headerRowCount="1">
+  <autoFilter ref="A1:L48"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4180,38 +4180,38 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>bet-componentise-interactive-layer</t>
+          <t>content-refresh-satellite-broadband-uk-guide</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F79" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr"/>
@@ -4224,7 +4224,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -4234,19 +4234,19 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -4262,8 +4262,52 @@
       <c r="K80" s="2" t="inlineStr"/>
       <c r="L80" s="2" t="inlineStr"/>
     </row>
+    <row r="81">
+      <c r="A81" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>bet-decouple-content-from-code</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>Decouple guide content from code deploys</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="G81" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J81" s="3" t="inlineStr"/>
+      <c r="K81" s="3" t="inlineStr"/>
+      <c r="L81" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L80"/>
+  <autoFilter ref="A1:L81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7015,7 +7059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9564,53 +9608,53 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+          <t>Twelfth target from scripts/analyze_content_priority.py's ranked list, and the page whose DATE_RE regex bug was found and fixed earlier this session (58.2 -&gt; 53.2) without ever getting a content rewrite. The old copy was generic to the point of naming no real prices at all -- 'Starlink is the most visible option' with zero named plans, figures or alternatives. Rewritten with real, current Starlink UK pricing (Residential 100/200/Max at GBP40/60/80 per month, Roam at GBP55-100, Standard Kit GBP449 commonly discounted to ~GBP299 or free on Max), and a genuinely current news item: Starlink's Global Roam plan stopped taking new customers 15 July 2026 and was withdrawn entirely for existing customers on 17 August 2026, one week before this rewrite. Named 2 real smaller alternatives (SkyDSL, Bigblu Broadband) and clarified that Eutelsat/OneWeb, despite frequent mention alongside Starlink, sells no UK consumer home-broadband plans at all. Word count 437 -&gt; 1,038.</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>components/</t>
+          <t>data/priority-pages.ts (satellite)</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9625,53 +9669,109 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
+          <t>Componentise the interactive layer on accessible primitives</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>components/</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L47" s="3" t="inlineStr">
+        <is>
+          <t>Growth playbook — Functionality pillar</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
           <t>Decouple guide content from code deploys</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
-      <c r="F47" s="3" t="n">
+      <c r="F48" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="G47" s="3" t="n">
+      <c r="G48" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="H47" s="3" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I47" s="3" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
-      <c r="J47" s="3" t="inlineStr">
+      <c r="J48" s="2" t="inlineStr">
         <is>
           <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
-      <c r="K47" s="3" t="inlineStr">
+      <c r="K48" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="L47" s="3" t="inlineStr">
+      <c r="L48" s="2" t="inlineStr">
         <is>
           <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L47"/>
+  <autoFilter ref="A1:L48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9712,7 +9812,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>79 total (33 page builds, 46 feature/strategy builds); 65 already marked Done.</t>
+          <t>80 total (33 page builds, 47 feature/strategy builds); 66 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Best Broadband for Gaming UK guide
Thirteenth target from scripts/analyze_content_priority.py's ranked
list: stale provider prices throughout, and a wrong Community Fibre
top-tier speed claim (920Mbps symmetrical, against the real current
3,000Mbps top tier). Refreshed all 5 existing provider picks against
this site's own already-vetted current pricing.

Added a genuinely new 6th pick, Zen Internet, for hosting a private
game server, where its free static IP is a real advantage over every
other provider on the list. Added a section on how 24-month contracts
and scheduled price rises affect the real two-year cost.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$82</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L81" headerRowCount="1">
-  <autoFilter ref="A1:L81"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L82" headerRowCount="1">
+  <autoFilter ref="A1:L82"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L48" headerRowCount="1">
-  <autoFilter ref="A1:L48"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L49" headerRowCount="1">
+  <autoFilter ref="A1:L49"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L81"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4268,12 +4268,12 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>content-refresh-best-broadband-for-gaming-guide</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -4283,31 +4283,75 @@
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F81" s="3" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr"/>
       <c r="K81" s="3" t="inlineStr"/>
       <c r="L81" s="3" t="inlineStr"/>
     </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>bet-decouple-content-from-code</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Decouple guide content from code deploys</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G82" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr"/>
+      <c r="K82" s="2" t="inlineStr"/>
+      <c r="L82" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L81"/>
+  <autoFilter ref="A1:L82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7059,7 +7103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9720,58 +9764,114 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Thirteenth target from scripts/analyze_content_priority.py's ranked list: 836 words with stale provider prices (EE GBP26.99, Community Fibre GBP21.99, Hyperoptic GBP22, BT GBP30.99, all already corrected on this site's own provider pages) and a wrong Community Fibre top-tier speed claim (920Mbps symmetrical, against the real current 3,000Mbps top tier confirmed in data/providers.ts). Refreshed all 5 existing provider picks against already-vetted current pricing, and added a genuinely new 6th pick, Zen Internet, for a use case the old page didn't cover at all: hosting a private game server, where Zen's free static IP (already documented on its own provider page) is a real, specific advantage over every other provider on the list. Added a short section on how 24-month contracts and scheduled price rises affect the real two-year cost of a gaming-suitable package. Word count 836 -&gt; 1,184; left just under the self-imposed 1,200-word floor rather than pad.</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-gaming-uk), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
           <t>Bigger bet</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>Decouple guide content from code deploys</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
-      <c r="F48" s="2" t="n">
+      <c r="F49" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="G48" s="2" t="n">
+      <c r="G49" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="I49" s="3" t="inlineStr">
         <is>
           <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="J49" s="3" t="inlineStr">
         <is>
           <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
-      <c r="K48" s="2" t="inlineStr">
+      <c r="K49" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="L48" s="2" t="inlineStr">
+      <c r="L49" s="3" t="inlineStr">
         <is>
           <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L48"/>
+  <autoFilter ref="A1:L49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9812,7 +9912,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>80 total (33 page builds, 47 feature/strategy builds); 66 already marked Done.</t>
+          <t>81 total (33 page builds, 48 feature/strategy builds); 67 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Broadband Social Tariffs UK guide
Fourteenth target from scripts/analyze_content_priority.py's ranked
list: a materially wrong "cheapest tariff" claim. The old page listed
Vodafone Together Social at GBP12.50/mo as cheapest, but the real
current Vodafone Essentials Broadband tariff is GBP20/mo for 73Mbps
(verified against Vodafone's own tariff page) -- meaning Virgin Media
Essential Broadband and Community Fibre Essential (both genuinely
GBP12.50/mo) are actually jointly cheapest. Also corrected Virgin
Media's own tariff, previously listed at GBP20/mo.

Added a genuinely newsworthy find: a thinkbroadband report published
in August 2026, days before this rewrite, tested how easy major
providers make it to find their own social tariffs and scored BT,
Sky, Virgin Media and Vodafone poorly. Corrected the eligibility
table and added KCOM's Hull-only tariff.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L82" headerRowCount="1">
-  <autoFilter ref="A1:L82"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L83" headerRowCount="1">
+  <autoFilter ref="A1:L83"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L49" headerRowCount="1">
-  <autoFilter ref="A1:L49"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L50" headerRowCount="1">
+  <autoFilter ref="A1:L50"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4312,12 +4312,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>content-refresh-broadband-social-tariffs-guide</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -4327,31 +4327,75 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr"/>
       <c r="K82" s="2" t="inlineStr"/>
       <c r="L82" s="2" t="inlineStr"/>
     </row>
+    <row r="83">
+      <c r="A83" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>bet-decouple-content-from-code</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>Decouple guide content from code deploys</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="G83" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J83" s="3" t="inlineStr"/>
+      <c r="K83" s="3" t="inlineStr"/>
+      <c r="L83" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L82"/>
+  <autoFilter ref="A1:L83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7103,7 +7147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9820,58 +9864,114 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Fourteenth target from scripts/analyze_content_priority.py's ranked list: 777 words with a materially wrong 'cheapest tariff' claim -- Vodafone Together Social was listed at GBP12.50/mo for 38Mbps and named the cheapest option, but the real current Vodafone Essentials Broadband tariff is GBP20/mo for 73Mbps (verified directly against Vodafone's own tariff page), meaning Virgin Media Essential Broadband and Community Fibre Essential (both genuinely GBP12.50/mo) are actually jointly cheapest. Also corrected Virgin Media's own tariff, which the old page listed at GBP20/mo. Added a genuinely newsworthy find: a thinkbroadband report published in August 2026 (days before this rewrite) tested how easy major providers make it to find their own social tariffs and scored BT, Sky, Virgin Media and Vodafone poorly, with a pointed BT quote, against smaller altnets scoring better. Corrected the eligibility table (Sky accepts UC/PC only, existing customers only, a real restriction the old page omitted) and added KCOM's Hull-only tariff. Refreshed the awareness stat with the newer, more specific thinkbroadband figures (34% aware, 8.6% UC take-up). Word count 777 -&gt; 1,161.</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="G49" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (broadband-social-tariffs-uk), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L49" s="3" t="inlineStr">
+        <is>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
           <t>Bigger bet</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Decouple guide content from code deploys</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
-      <c r="F49" s="3" t="n">
+      <c r="F50" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="G49" s="3" t="n">
+      <c r="G50" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="H49" s="3" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I49" s="3" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
-      <c r="J49" s="3" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr">
         <is>
           <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
-      <c r="K49" s="3" t="inlineStr">
+      <c r="K50" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="L49" s="3" t="inlineStr">
+      <c r="L50" s="2" t="inlineStr">
         <is>
           <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L49"/>
+  <autoFilter ref="A1:L50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9912,7 +10012,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>81 total (33 page builds, 48 feature/strategy builds); 67 already marked Done.</t>
+          <t>82 total (33 page builds, 49 feature/strategy builds); 68 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Best Broadband for Working From Home guide
Fifteenth target from scripts/analyze_content_priority.py's ranked
list: 565 words, no real prices anywhere, and a stale "EE is
consistently rated the most reliable major UK broadband provider"
claim that no longer holds under this session's own Q1 2026 Ofcom
complaints research.

Rewrote with real current prices for Community Fibre, Hyperoptic, Zen
Internet and BT, and added a new section on when a business-grade
line is actually worth it for a freelancer or remote worker over a
residential package. Added concrete video-call upload-bandwidth
guidance (3-4 Mbps per HD call) rather than vague framing.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$84</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L83" headerRowCount="1">
-  <autoFilter ref="A1:L83"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L84" headerRowCount="1">
+  <autoFilter ref="A1:L84"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L50" headerRowCount="1">
-  <autoFilter ref="A1:L50"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L51" headerRowCount="1">
+  <autoFilter ref="A1:L51"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4356,12 +4356,12 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>content-refresh-best-broadband-working-from-home-guide</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -4371,31 +4371,75 @@
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F83" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G83" s="3" t="n">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr"/>
       <c r="K83" s="3" t="inlineStr"/>
       <c r="L83" s="3" t="inlineStr"/>
     </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>bet-decouple-content-from-code</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Decouple guide content from code deploys</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G84" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr"/>
+      <c r="K84" s="2" t="inlineStr"/>
+      <c r="L84" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L83"/>
+  <autoFilter ref="A1:L84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7147,7 +7191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9920,58 +9964,114 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Fifteenth target from scripts/analyze_content_priority.py's ranked list: 565 words, no real prices anywhere, and a stale 'EE is consistently rated the most reliable major UK broadband provider' claim that no longer holds under this session's own Q1 2026 Ofcom complaints research. Rewrote with real current prices for Community Fibre, Hyperoptic, Zen Internet and BT, and added a genuinely new section this page never had: when a business-grade line (static IP, faster fault-fix SLA) is actually worth it for a freelancer or remote worker over a residential package, using real Vodafone Business/Zen Business/Sky Business pricing already researched for this site's business broadband guide. Added concrete video-call upload-bandwidth guidance (3-4 Mbps per HD call) rather than vague 'upload matters' framing. Word count 565 -&gt; 986.</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-working-from-home), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
           <t>Bigger bet</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>Decouple guide content from code deploys</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
-      <c r="F50" s="2" t="n">
+      <c r="F51" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="G50" s="2" t="n">
+      <c r="G51" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr">
+      <c r="I51" s="3" t="inlineStr">
         <is>
           <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
-      <c r="J50" s="2" t="inlineStr">
+      <c r="J51" s="3" t="inlineStr">
         <is>
           <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
-      <c r="K50" s="2" t="inlineStr">
+      <c r="K51" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="L50" s="2" t="inlineStr">
+      <c r="L51" s="3" t="inlineStr">
         <is>
           <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L50"/>
+  <autoFilter ref="A1:L51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10012,7 +10112,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>82 total (33 page builds, 49 feature/strategy builds); 68 already marked Done.</t>
+          <t>83 total (33 page builds, 50 feature/strategy builds); 69 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Broadband Deals Under GBP20 guide
Sixteenth target from scripts/analyze_content_priority.py's ranked
list, and the largest factual break of this refresh sequence: the
page's entire premise named NOW Broadband and TalkTalk as "the most
common names in this price bracket," but both now start above
GBP20/mo (NOW at GBP23, TalkTalk at GBP25).

Rebuilt around who is actually under GBP20 today: Community Fibre
(GBP12.50), Onestream (GBP18.50, 94% Openreach coverage), Gigaclear
(GBP19.00), toob (GBP19.50) and Trooli (GBP19.99). Caught and excluded
Shell Energy, which the data file's own notes show closed to new
customers and migrated to TalkTalk in 2024 -- would have been a real
error to list as a current deal.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$85</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L84" headerRowCount="1">
-  <autoFilter ref="A1:L84"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L85" headerRowCount="1">
+  <autoFilter ref="A1:L85"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L51" headerRowCount="1">
-  <autoFilter ref="A1:L51"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L52" headerRowCount="1">
+  <autoFilter ref="A1:L52"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4400,12 +4400,12 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>content-refresh-broadband-deals-under-20-guide</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -4415,31 +4415,75 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
         <v>35</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr"/>
       <c r="K84" s="2" t="inlineStr"/>
       <c r="L84" s="2" t="inlineStr"/>
     </row>
+    <row r="85">
+      <c r="A85" s="3" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>bet-decouple-content-from-code</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>Decouple guide content from code deploys</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="G85" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr"/>
+      <c r="K85" s="3" t="inlineStr"/>
+      <c r="L85" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L84"/>
+  <autoFilter ref="A1:L85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7191,7 +7235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10020,7 +10064,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -10030,48 +10074,104 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
+          <t>Sixteenth target from scripts/analyze_content_priority.py's ranked list, and the one with the largest factual break of this whole refresh sequence: the page's entire premise named NOW Broadband and TalkTalk as 'the most common names in this price bracket,' but both now start above GBP20/mo (NOW at GBP23, TalkTalk at GBP25, both already corrected on their own provider pages this session). Rebuilt the page around who is actually under GBP20 today by querying data/providers.ts directly for every provider with monthlyPriceFrom &lt; 20: Community Fibre (GBP12.50), Onestream (GBP18.50, 94% Openreach coverage -- the most realistic pick for most addresses), Gigaclear (GBP19.00, rural symmetrical), toob (GBP19.50) and Trooli (GBP19.99). Also caught and excluded Shell Energy (GBP19.99 in the data file) after finding its own provider-page highlights note it closed to new customers and migrated to TalkTalk in 2024 -- an old, non-orderable plan that would have been a real error to list as a current deal. Word count 608 -&gt; 890.</t>
         </is>
       </c>
       <c r="F51" s="3" t="n">
         <v>35</v>
       </c>
       <c r="G51" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-under-20), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L51" s="3" t="inlineStr">
+        <is>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Bigger bet</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Decouple guide content from code deploys</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G52" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="H51" s="3" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I51" s="3" t="inlineStr">
+      <c r="I52" s="2" t="inlineStr">
         <is>
           <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
-      <c r="J51" s="3" t="inlineStr">
+      <c r="J52" s="2" t="inlineStr">
         <is>
           <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
-      <c r="K51" s="3" t="inlineStr">
+      <c r="K52" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="L51" s="3" t="inlineStr">
+      <c r="L52" s="2" t="inlineStr">
         <is>
           <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L51"/>
+  <autoFilter ref="A1:L52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10112,7 +10212,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>83 total (33 page builds, 50 feature/strategy builds); 69 already marked Done.</t>
+          <t>84 total (33 page builds, 51 feature/strategy builds); 70 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of BT vs Sky comparison page
Seventeenth target from scripts/analyze_content_priority.py's ranked
list, and the first comparison-type page in this refresh sequence:
496 words of entirely generic, number-free copy that was also
factually stale -- Sky moved to 24-month contracts some time ago,
the same length as BT, a premise this page's whole "contract
flexibility" differentiator was built on.

Rewrote using this session's own BT and Sky provider-page data:
prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00),
Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per
100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year
price rise is more transparently disclosed than Sky's contract
wording. Populated the previously-empty factSnapshot field.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L85" headerRowCount="1">
-  <autoFilter ref="A1:L85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L86" headerRowCount="1">
+  <autoFilter ref="A1:L86"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L52" headerRowCount="1">
-  <autoFilter ref="A1:L52"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L53" headerRowCount="1">
+  <autoFilter ref="A1:L53"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4482,8 +4482,52 @@
       <c r="K85" s="3" t="inlineStr"/>
       <c r="L85" s="3" t="inlineStr"/>
     </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>content-refresh-bt-vs-sky-comparison</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="G86" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr"/>
+      <c r="K86" s="2" t="inlineStr"/>
+      <c r="L86" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L85"/>
+  <autoFilter ref="A1:L86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7235,7 +7279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10170,8 +10214,64 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="G53" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="inlineStr">
+        <is>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L52"/>
+  <autoFilter ref="A1:L53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10212,7 +10312,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>84 total (33 page builds, 51 feature/strategy builds); 70 already marked Done.</t>
+          <t>85 total (33 page builds, 52 feature/strategy builds); 71 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Best Rolling Monthly Broadband Deals guide
Eighteenth target from scripts/analyze_content_priority.py's ranked
list: repeated a stale claim caught twice already this session --
"NOW Broadband is often relevant because of its shorter 12-month
positioning" -- when NOW dropped flexible contracts entirely and now
sells only a standard 24-month term.

Rewrote around who actually offers flexible broadband now: YouFibre,
one of the only genuine rolling-monthly full-fibre options left (from
GBP33.99/mo, 30 days' notice), plus Hyperoptic/Community Fibre/
Onestream's 12-month middle-ground option, and a note on social
tariffs' no-exit-fee terms.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$87</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L86" headerRowCount="1">
-  <autoFilter ref="A1:L86"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L87" headerRowCount="1">
+  <autoFilter ref="A1:L87"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L53" headerRowCount="1">
-  <autoFilter ref="A1:L53"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L54" headerRowCount="1">
+  <autoFilter ref="A1:L54"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4526,8 +4526,52 @@
       <c r="K86" s="2" t="inlineStr"/>
       <c r="L86" s="2" t="inlineStr"/>
     </row>
+    <row r="87">
+      <c r="A87" s="3" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="G87" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J87" s="3" t="inlineStr"/>
+      <c r="K87" s="3" t="inlineStr"/>
+      <c r="L87" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L86"/>
+  <autoFilter ref="A1:L87"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7279,7 +7323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10270,8 +10314,64 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L53"/>
+  <autoFilter ref="A1:L54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10312,7 +10412,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>85 total (33 page builds, 52 feature/strategy builds); 71 already marked Done.</t>
+          <t>86 total (33 page builds, 53 feature/strategy builds); 72 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Broadband Price Rises 2026 guide
Nineteenth and final content-priority-analysis target this session.
This page had the most individually-wrong data points found in a
single page all session: TalkTalk was listed at +GBP2.50/mo when the
real current figure is +GBP4.00/mo for contracts from 16 November
2025 (TalkTalk raised its own rise from GBP3 to GBP4 partway through
the year). Hyperoptic and Community Fibre were both listed as "No
rise" when both apply a real scheduled increase.

Added a dedicated section directly naming the "no-rise altnet"
assumption as false for 2 of the 4 providers commonly assumed to
qualify (only toob and Zen Internet genuinely have no scheduled rise).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L87" headerRowCount="1">
-  <autoFilter ref="A1:L87"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L88" headerRowCount="1">
+  <autoFilter ref="A1:L88"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L54" headerRowCount="1">
-  <autoFilter ref="A1:L54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L55" headerRowCount="1">
+  <autoFilter ref="A1:L55"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4570,8 +4570,52 @@
       <c r="K87" s="3" t="inlineStr"/>
       <c r="L87" s="3" t="inlineStr"/>
     </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>content-refresh-broadband-price-rises-2026-guide</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="G88" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr"/>
+      <c r="K88" s="2" t="inlineStr"/>
+      <c r="L88" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L87"/>
+  <autoFilter ref="A1:L88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7323,7 +7367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10370,8 +10414,64 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G55" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L55" s="3" t="inlineStr">
+        <is>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L54"/>
+  <autoFilter ref="A1:L55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10412,7 +10512,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>86 total (33 page builds, 53 feature/strategy builds); 72 already marked Done.</t>
+          <t>87 total (33 page builds, 54 feature/strategy builds); 73 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: update EE provider page with real Q1 2026 Ofcom complaints figure
Twentieth target from scripts/analyze_content_priority.py's wider
ranked list: /providers/ee carries the highest search volume on the
site (202,237/mo) and was already well-built, so this was a targeted
correction. The page's own sources explicitly flagged that EE's exact
Q1 2026 Ofcom complaints figure could not be found and was still
citing Q4 2025's "worst-three bracket" framing.

Filled the gap with the exact figure from the same Q1 2026 complaints
table already used elsewhere this session: EE recorded 6 per 100,000,
exactly the record-low industry average, a real improvement out of
the worst bracket. Rewrote the Ofcom section, cons, excerpt, FAQ and
verdict to reflect this, reframing EE as a new example of the
low-Trustpilot-vs-strong-Ofcom pattern rather than weak on both.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$89</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L88" headerRowCount="1">
-  <autoFilter ref="A1:L88"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L89" headerRowCount="1">
+  <autoFilter ref="A1:L89"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L55" headerRowCount="1">
-  <autoFilter ref="A1:L55"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L56" headerRowCount="1">
+  <autoFilter ref="A1:L56"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -600,7 +600,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2056,33 +2056,33 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>page-tools/broadband-cost-calculator</t>
+          <t>content-refresh-ee-provider-page</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Broadband cost calculator: true monthly and contract-length cost</t>
+          <t>Update: EE provider page Ofcom complaints figure (20th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F31" s="3" t="n">
-        <v>59.9</v>
+        <v>60</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>27.6</v>
+        <v>55</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Very easy</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2092,11 +2092,7 @@
       </c>
       <c r="J31" s="3" t="inlineStr"/>
       <c r="K31" s="3" t="inlineStr"/>
-      <c r="L31" s="3" t="inlineStr">
-        <is>
-          <t>Live at /tools/broadband-cost-calculator, committed and deployed 2026-08-21.</t>
-        </is>
-      </c>
+      <c r="L31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2104,7 +2100,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>page-providers/onestream</t>
+          <t>page-tools/broadband-cost-calculator</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2114,19 +2110,19 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Onestream — plans, coverage and Awin-tracked deals</t>
+          <t>Broadband cost calculator: true monthly and contract-length cost</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>59.4</v>
+        <v>59.9</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>28</v>
+        <v>27.6</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -2140,7 +2136,11 @@
       </c>
       <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Live at /tools/broadband-cost-calculator, committed and deployed 2026-08-21.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -2148,7 +2148,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>page-guides/no-credit-check-broadband-uk</t>
+          <t>page-providers/onestream</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -2163,18 +2163,18 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>No credit check broadband in the UK: options and what to expect</t>
+          <t>Onestream — plans, coverage and Awin-tracked deals</t>
         </is>
       </c>
       <c r="F33" s="3" t="n">
-        <v>59.3</v>
+        <v>59.4</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>34.8</v>
+        <v>28</v>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Very easy</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2192,38 +2192,38 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>feat-review-aggregation-module</t>
+          <t>page-guides/no-credit-check-broadband-uk</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Real review-aggregation trust module</t>
+          <t>No credit check broadband in the UK: options and what to expect</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>59</v>
+        <v>59.3</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>62</v>
+        <v>34.8</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
@@ -2236,38 +2236,38 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>page-providers/brsk</t>
+          <t>feat-review-aggregation-module</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Brsk — plans, coverage and Awin-tracked deals</t>
+          <t>Real review-aggregation trust module</t>
         </is>
       </c>
       <c r="F35" s="3" t="n">
         <v>59</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>28.5</v>
+        <v>62</v>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>Very easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr"/>
@@ -2280,7 +2280,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>page-guides/fttp-vs-fttc-explained</t>
+          <t>page-providers/brsk</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2295,14 +2295,14 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>FTTP vs FTTC: what the difference means for your speed</t>
+          <t>Brsk — plans, coverage and Awin-tracked deals</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>58.4</v>
+        <v>59</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>27.8</v>
+        <v>28.5</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>page-guides/best-mesh-wifi-for-your-broadband-router</t>
+          <t>page-guides/fttp-vs-fttc-explained</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2339,18 +2339,18 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Best mesh Wi-Fi systems to pair with your broadband router</t>
+          <t>FTTP vs FTTC: what the difference means for your speed</t>
         </is>
       </c>
       <c r="F37" s="3" t="n">
         <v>58.4</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>34</v>
+        <v>27.8</v>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Very easy</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>page-guides/broadband-help-if-you-claim-benefits-uk</t>
+          <t>page-guides/best-mesh-wifi-for-your-broadband-router</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2383,18 +2383,18 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Cheaper broadband if you claim benefits: social tariffs explained</t>
+          <t>Best mesh Wi-Fi systems to pair with your broadband router</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>58.2</v>
+        <v>58.4</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>27.5</v>
+        <v>34</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Very easy</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2412,38 +2412,38 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>ops-adsense-site-review</t>
+          <t>page-guides/broadband-help-if-you-claim-benefits-uk</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Monetisation</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Complete AdSense site review and authorisation monitoring</t>
+          <t>Cheaper broadband if you claim benefits: social tariffs explained</t>
         </is>
       </c>
       <c r="F39" s="3" t="n">
-        <v>58</v>
+        <v>58.2</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>55</v>
+        <v>27.5</v>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Very easy</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr"/>
@@ -2456,38 +2456,38 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>content-awin-approved-provider-deep-content</t>
+          <t>ops-adsense-site-review</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Monetisation</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Deep, researched content for Awin-approved providers (TalkTalk, Zzoomm, Highland Broadband)</t>
+          <t>Complete AdSense site review and authorisation monitoring</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
         <v>58</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
@@ -2500,12 +2500,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>page-providers/gigaclear</t>
+          <t>content-awin-approved-provider-deep-content</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -2515,18 +2515,18 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Gigaclear — plans, coverage and Awin-tracked deals</t>
+          <t>Deep, researched content for Awin-approved providers (TalkTalk, Zzoomm, Highland Broadband)</t>
         </is>
       </c>
       <c r="F41" s="3" t="n">
-        <v>56.9</v>
+        <v>58</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>27.9</v>
+        <v>62</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>page-providers/youfibre</t>
+          <t>page-providers/gigaclear</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2559,14 +2559,14 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>YouFibre — plans, coverage and Awin-tracked deals</t>
+          <t>Gigaclear — plans, coverage and Awin-tracked deals</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>56.6</v>
+        <v>56.9</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>28.7</v>
+        <v>27.9</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>page-providers/cuckoo</t>
+          <t>page-providers/youfibre</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -2603,14 +2603,14 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Cuckoo Broadband — plans, coverage and Awin-tracked deals</t>
+          <t>YouFibre — plans, coverage and Awin-tracked deals</t>
         </is>
       </c>
       <c r="F43" s="3" t="n">
-        <v>56.5</v>
+        <v>56.6</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>27.9</v>
+        <v>28.7</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
@@ -2632,12 +2632,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>audit-city-hub-thinness</t>
+          <t>page-providers/cuckoo</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Content audit</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2647,23 +2647,23 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Verify each new city hub has a genuinely local fact</t>
+          <t>Cuckoo Broadband — plans, coverage and Awin-tracked deals</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>56</v>
+        <v>56.5</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>50</v>
+        <v>27.9</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
@@ -2676,12 +2676,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>audit-city-hub-thinness</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Content audit</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -2691,14 +2691,14 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Content priority analysis: real SEO + GEO signals, build vs. update on one list</t>
+          <t>Verify each new city hub has a genuinely local fact</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
         <v>56</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr"/>
@@ -2720,12 +2720,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>page-guides/black-friday-broadband-deals-uk</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2735,18 +2735,18 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Black Friday broadband deals UK: what to expect and how to compare</t>
+          <t>Content priority analysis: real SEO + GEO signals, build vs. update on one list</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>55.8</v>
+        <v>56</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Competitive</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>page-providers/shell-energy</t>
+          <t>page-guides/black-friday-broadband-deals-uk</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -2779,18 +2779,18 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Shell Energy Broadband — plans, coverage and Awin-tracked deals</t>
+          <t>Black Friday broadband deals UK: what to expect and how to compare</t>
         </is>
       </c>
       <c r="F47" s="3" t="n">
-        <v>55.7</v>
+        <v>55.8</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Competitive</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>page-research/broadband-customer-service-rankings-uk</t>
+          <t>page-providers/shell-energy</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2823,14 +2823,14 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Broadband customer service rankings: Ofcom-evidenced comparison</t>
+          <t>Shell Energy Broadband — plans, coverage and Awin-tracked deals</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>55.1</v>
+        <v>55.7</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>27.8</v>
+        <v>28</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -2852,33 +2852,33 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>feat-nav-header-footer-ia</t>
+          <t>page-research/broadband-customer-service-rankings-uk</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Navigation/header/footer IA improvements</t>
+          <t>Broadband customer service rankings: Ofcom-evidenced comparison</t>
         </is>
       </c>
       <c r="F49" s="3" t="n">
-        <v>55</v>
+        <v>55.1</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>60</v>
+        <v>27.8</v>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
@@ -2888,11 +2888,7 @@
       </c>
       <c r="J49" s="3" t="inlineStr"/>
       <c r="K49" s="3" t="inlineStr"/>
-      <c r="L49" s="3" t="inlineStr">
-        <is>
-          <t>Shipped 2026-08-22: scripts/scrape_navigation_patterns.py scanned 5 best-in-class sites (broadband.co.uk stood out on sticky header + breadcrumbs + trust badge). Confirmed BroadbandPicker's sticky header and breadcrumbs already match best practice. Added Postcode to primary nav (desktop+mobile), restructured footer 4-&gt;6 columns adding Tools, Find Broadband by Area, and Research links to fix a crawl/link-equity gap for the 2,800+ postcode-district and tools pages. Deliberately did NOT fabricate a trust badge (no real Trustpilot/press presence yet) and did NOT widen the header postcode breakpoint (risk of stacking two unverified density changes without a browser check). See docs/navigation-ia-analysis.md.</t>
-        </is>
-      </c>
+      <c r="L49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2900,7 +2896,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>feat-contact-form-email-delivery</t>
+          <t>feat-nav-header-footer-ia</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2910,19 +2906,19 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Working contact form delivering to a real inbox, no third-party service</t>
+          <t>Navigation/header/footer IA improvements</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
         <v>55</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -2931,12 +2927,16 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr"/>
-      <c r="L50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>Shipped 2026-08-22: scripts/scrape_navigation_patterns.py scanned 5 best-in-class sites (broadband.co.uk stood out on sticky header + breadcrumbs + trust badge). Confirmed BroadbandPicker's sticky header and breadcrumbs already match best practice. Added Postcode to primary nav (desktop+mobile), restructured footer 4-&gt;6 columns adding Tools, Find Broadband by Area, and Research links to fix a crawl/link-equity gap for the 2,800+ postcode-district and tools pages. Deliberately did NOT fabricate a trust badge (no real Trustpilot/press presence yet) and did NOT widen the header postcode breakpoint (risk of stacking two unverified density changes without a browser check). See docs/navigation-ia-analysis.md.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
@@ -2944,38 +2944,38 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>content-awin-pending-provider-deep-content</t>
+          <t>feat-contact-form-email-delivery</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Deep, researched content for Awin-pending providers (Community Fibre, Cuckoo, Zen Internet, National Broadband, Trooli, Pine Media)</t>
+          <t>Working contact form delivering to a real inbox, no third-party service</t>
         </is>
       </c>
       <c r="F51" s="3" t="n">
         <v>55</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr"/>
@@ -2988,12 +2988,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>page-guides/broadband-complaints-and-ombudsman-uk</t>
+          <t>content-awin-pending-provider-deep-content</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -3003,18 +3003,18 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Broadband complaints and the ombudsman: your UK rights</t>
+          <t>Deep, researched content for Awin-pending providers (Community Fibre, Cuckoo, Zen Internet, National Broadband, Trooli, Pine Media)</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>54.7</v>
+        <v>55</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>25.9</v>
+        <v>58</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -3032,12 +3032,12 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>growth-original-research-outreach</t>
+          <t>page-guides/broadband-complaints-and-ombudsman-uk</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Growth</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -3047,23 +3047,23 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Run original-research outreach and digital PR</t>
+          <t>Broadband complaints and the ombudsman: your UK rights</t>
         </is>
       </c>
       <c r="F53" s="3" t="n">
-        <v>54</v>
+        <v>54.7</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>68</v>
+        <v>25.9</v>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr"/>
@@ -3076,12 +3076,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-full-fibre-guide</t>
+          <t>growth-original-research-outreach</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -3091,14 +3091,14 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Full Fibre Broadband UK guide (top content-priority-analysis target)</t>
+          <t>Run original-research outreach and digital PR</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
         <v>54</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr"/>
@@ -3120,29 +3120,29 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>growth-quarterly-data-reprioritisation</t>
+          <t>content-refresh-best-full-fibre-guide</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Strategy</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Growth</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Reprioritise quarter two using GSC, engagement and affiliate evidence</t>
+          <t>Deep rewrite: Best Full Fibre Broadband UK guide (top content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F55" s="3" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr"/>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>feat-postcode-journey-personalisation</t>
+          <t>growth-quarterly-data-reprioritisation</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Postcode-aware personalisation across the customer journey, free tier only</t>
+          <t>Reprioritise quarter two using GSC, engagement and affiliate evidence</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
         <v>53</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
@@ -3195,7 +3195,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr"/>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>feat-homepage-visual-redesign</t>
+          <t>feat-postcode-journey-personalisation</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -3223,11 +3223,11 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Homepage visual redesign: illustrations + interactivity</t>
+          <t>Postcode-aware personalisation across the customer journey, free tier only</t>
         </is>
       </c>
       <c r="F57" s="3" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G57" s="3" t="n">
         <v>55</v>
@@ -3252,22 +3252,22 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-cheapest-broadband-guide</t>
+          <t>feat-homepage-visual-redesign</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Cheapest Broadband Deals UK guide (2nd content-priority-analysis target)</t>
+          <t>Homepage visual redesign: illustrations + interactivity</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
@@ -3296,29 +3296,29 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>feat-mobile-cross-device-navigation</t>
+          <t>content-refresh-cheapest-broadband-guide</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Mobile and cross-device navigation overhaul</t>
+          <t>Deep rewrite: Cheapest Broadband Deals UK guide (2nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F59" s="3" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
@@ -3340,7 +3340,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>feat-mega-menu-navigation</t>
+          <t>feat-mobile-cross-device-navigation</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -3355,14 +3355,14 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Detailed mega-menu navigation</t>
+          <t>Mobile and cross-device navigation overhaul</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>feat-animated-interactive-mobile-menu</t>
+          <t>feat-mega-menu-navigation</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -3399,14 +3399,14 @@
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Animated, interactive mobile menu with click-outside-to-close</t>
+          <t>Detailed mega-menu navigation</t>
         </is>
       </c>
       <c r="F61" s="3" t="n">
         <v>50</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
@@ -3428,29 +3428,29 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-business-broadband-guide</t>
+          <t>feat-animated-interactive-mobile-menu</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Business Broadband Providers UK guide (3rd content-priority-analysis target)</t>
+          <t>Animated, interactive mobile menu with click-outside-to-close</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
         <v>50</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -3472,29 +3472,29 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>feat-price-drop-alerts</t>
+          <t>content-refresh-best-business-broadband-guide</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Price-drop alerts</t>
+          <t>Deep rewrite: Best Business Broadband Providers UK guide (3rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F63" s="3" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
@@ -3503,7 +3503,7 @@
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr"/>
@@ -3516,7 +3516,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>feat-page-type-ux-redesign</t>
+          <t>feat-price-drop-alerts</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -3526,19 +3526,19 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Page-type UX redesign: deals, providers, guides, postcode hub</t>
+          <t>Price-drop alerts</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
         <v>49</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -3547,7 +3547,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr"/>
@@ -3560,7 +3560,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>feat-footer-logo-interactivity</t>
+          <t>feat-page-type-ux-redesign</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -3575,18 +3575,18 @@
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Footer logo placement and interactive elements</t>
+          <t>Page-type UX redesign: deals, providers, guides, postcode hub</t>
         </is>
       </c>
       <c r="F65" s="3" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I65" s="3" t="inlineStr">
@@ -3596,11 +3596,7 @@
       </c>
       <c r="J65" s="3" t="inlineStr"/>
       <c r="K65" s="3" t="inlineStr"/>
-      <c r="L65" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Follow-up 2026-08-23: added Instagram (@broadbandpicker) as a second social pill button next to X, same hover treatment.</t>
-        </is>
-      </c>
+      <c r="L65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -3608,33 +3604,33 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-tv-deals-guide</t>
+          <t>feat-footer-logo-interactivity</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Research-led editorial refresh: Best Broadband and TV Deals guide</t>
+          <t>Footer logo placement and interactive elements</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
         <v>48</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -3644,7 +3640,11 @@
       </c>
       <c r="J66" s="2" t="inlineStr"/>
       <c r="K66" s="2" t="inlineStr"/>
-      <c r="L66" s="2" t="inlineStr"/>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Follow-up 2026-08-23: added Instagram (@broadbandpicker) as a second social pill button next to X, same hover treatment.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n">
@@ -3652,29 +3652,29 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>audit-core-web-vitals-reporting</t>
+          <t>content-refresh-best-broadband-tv-deals-guide</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Establish monthly Core Web Vitals reporting by template</t>
+          <t>Research-led editorial refresh: Best Broadband and TV Deals guide</t>
         </is>
       </c>
       <c r="F67" s="3" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G67" s="3" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr"/>
@@ -3696,38 +3696,38 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>ops-awin-publisher-api-integration</t>
+          <t>audit-core-web-vitals-reporting</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Monetisation</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Direct Awin Publisher API access — programme status and link generation</t>
+          <t>Establish monthly Core Web Vitals reporting by template</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
         <v>47</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr"/>
@@ -3740,33 +3740,33 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-5g-home-broadband-guide</t>
+          <t>ops-awin-publisher-api-integration</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Monetisation</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best 5G Home Broadband UK guide (4th content-priority-analysis target)</t>
+          <t>Direct Awin Publisher API access — programme status and link generation</t>
         </is>
       </c>
       <c r="F69" s="3" t="n">
         <v>47</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
@@ -3784,29 +3784,29 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>audit-mobile-checkout-flow</t>
+          <t>content-refresh-best-5g-home-broadband-guide</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>UX audit</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Mobile checkout-flow audit</t>
+          <t>Deep rewrite: Best 5G Home Broadband UK guide (4th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
@@ -3815,7 +3815,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr"/>
@@ -3828,29 +3828,29 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-phone-and-broadband-deals-guide</t>
+          <t>audit-mobile-checkout-flow</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX audit</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Phone and Broadband Deals guide (5th content-priority-analysis target)</t>
+          <t>Mobile checkout-flow audit</t>
         </is>
       </c>
       <c r="F71" s="3" t="n">
         <v>45</v>
       </c>
       <c r="G71" s="3" t="n">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
@@ -3859,7 +3859,7 @@
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr"/>
@@ -3872,38 +3872,38 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>audit-broken-links-redirects</t>
+          <t>content-refresh-best-phone-and-broadband-deals-guide</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Crawlability</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Add routine broken-link and redirect reporting</t>
+          <t>Deep rewrite: Best Phone and Broadband Deals guide (5th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G72" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="G72" s="2" t="n">
-        <v>48</v>
-      </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr"/>
@@ -3916,38 +3916,38 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-now-broadband-provider-page</t>
+          <t>audit-broken-links-redirects</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Crawlability</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
+          <t>Add routine broken-link and redirect reporting</t>
         </is>
       </c>
       <c r="F73" s="3" t="n">
         <v>44</v>
       </c>
       <c r="G73" s="3" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr"/>
@@ -3960,7 +3960,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-youfibre-provider-page</t>
+          <t>content-refresh-now-broadband-provider-page</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -3975,14 +3975,14 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
+          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
@@ -4004,7 +4004,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-providers-uk-guide</t>
+          <t>content-refresh-youfibre-provider-page</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -4019,14 +4019,14 @@
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
+          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F75" s="3" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G75" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
@@ -4048,12 +4048,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>bet-annual-research-report</t>
+          <t>content-refresh-best-broadband-providers-uk-guide</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -4063,23 +4063,23 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr"/>
@@ -4092,12 +4092,12 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-without-phone-line-guide</t>
+          <t>bet-annual-research-report</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -4107,23 +4107,23 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="F77" s="3" t="n">
         <v>41</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr"/>
@@ -4136,7 +4136,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-moving-house-guide</t>
+          <t>content-refresh-broadband-without-phone-line-guide</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -4151,14 +4151,14 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-satellite-broadband-uk-guide</t>
+          <t>content-refresh-broadband-moving-house-guide</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -4195,14 +4195,14 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F79" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
@@ -4224,38 +4224,38 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>bet-componentise-interactive-layer</t>
+          <t>content-refresh-satellite-broadband-uk-guide</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr"/>
@@ -4268,38 +4268,38 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-gaming-guide</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F81" s="3" t="n">
         <v>38</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr"/>
@@ -4312,7 +4312,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-social-tariffs-guide</t>
+          <t>content-refresh-best-broadband-for-gaming-guide</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -4327,11 +4327,11 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G82" s="2" t="n">
         <v>34</v>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-working-from-home-guide</t>
+          <t>content-refresh-broadband-social-tariffs-guide</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -4371,14 +4371,14 @@
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F83" s="3" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G83" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-under-20-guide</t>
+          <t>content-refresh-best-broadband-working-from-home-guide</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -4415,14 +4415,14 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -4444,12 +4444,12 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>content-refresh-broadband-deals-under-20-guide</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -4459,23 +4459,23 @@
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F85" s="3" t="n">
         <v>35</v>
       </c>
       <c r="G85" s="3" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr"/>
@@ -4488,12 +4488,12 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-bt-vs-sky-comparison</t>
+          <t>bet-decouple-content-from-code</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -4503,23 +4503,23 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr"/>
@@ -4532,7 +4532,7 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
+          <t>content-refresh-bt-vs-sky-comparison</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -4547,14 +4547,14 @@
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F87" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G87" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-price-rises-2026-guide</t>
+          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -4591,14 +4591,14 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -4614,8 +4614,52 @@
       <c r="K88" s="2" t="inlineStr"/>
       <c r="L88" s="2" t="inlineStr"/>
     </row>
+    <row r="89">
+      <c r="A89" s="3" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>content-refresh-broadband-price-rises-2026-guide</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G89" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr"/>
+      <c r="K89" s="3" t="inlineStr"/>
+      <c r="L89" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L88"/>
+  <autoFilter ref="A1:L89"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7367,7 +7411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8012,53 +8056,53 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Real review-aggregation trust module</t>
+          <t>Update: EE provider page Ofcom complaints figure (20th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Blend the existing Ofcom-complaints research methodology with live Trustpilot scores into one visible trust module reused across provider and comparison pages, instead of a single quoted score per page.</t>
+          <t>Twentieth target from scripts/analyze_content_priority.py's wider ranked list (top 30): /providers/ee carries the single highest mapped search volume of any page on the site (202,237/mo) and was already well-built (1,649 words, no thinness flag), so this was a targeted correction rather than a full rewrite. The page's own reviewSources explicitly noted it could not find EE's exact Q1 2026 Ofcom complaints figure and was still citing Q4 2025's 'worst-three bracket, 10 per 100k' framing as the operative claim. Filled that gap with the exact figure from the same broadbandswitch 'The Complaints Floor' Q1 2026 table already used for the price-rises and broadband-providers-ranking guides: EE recorded 6 per 100,000, exactly the record-low industry average, a real, measurable improvement no longer in the worst bracket. Rewrote the Ofcom section, cons, excerpt, FAQ and 'Is EE Worth It' verdict to reflect this, reframing EE as a new example of the low-Trustpilot-vs-strong-Ofcom pattern (joining Sky, Plusnet, Virgin Media) rather than a provider genuinely weak on both measures.</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>New shared component, used on provider + comparison pages</t>
+          <t>data/providers.ts (ee)</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>research/uk-broadband-customer-satisfaction methodology</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -8068,53 +8112,53 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Monetisation</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Complete AdSense site review and authorisation monitoring</t>
+          <t>Real review-aggregation trust module</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Monitor the existing AdSense review, consent implementation and ads.txt authorisation; resolve any concrete policy or crawler issue reported by AdSense.</t>
+          <t>Blend the existing Ofcom-complaints research methodology with live Trustpilot scores into one visible trust module reused across provider and comparison pages, instead of a single quoted score per page.</t>
         </is>
       </c>
       <c r="F13" s="3" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>AdSense status and /ads.txt</t>
+          <t>New shared component, used on provider + comparison pages</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>Google site-review processing</t>
+          <t>research/uk-broadband-customer-satisfaction methodology</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>BroadbandPicker SEO &amp; Content Plan — Live: Build Status</t>
+          <t>Growth playbook — Functionality pillar</t>
         </is>
       </c>
     </row>
@@ -8124,53 +8168,53 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Monetisation</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Deep, researched content for Awin-approved providers (TalkTalk, Zzoomm, Highland Broadband)</t>
+          <t>Complete AdSense site review and authorisation monitoring</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Following the Awin programme-status pull (ops-awin-publisher-api-integration), built full researched content for the 3 real providers among the 4 joined programmes (Broadband Genie is a comparison site, not an ISP, and was excluded). Per docs/page-build-pipeline-brief.md Stage 3/4/4a: for each provider, fetched the provider's own site for current pricing/speeds/contract terms, WebSearched Trustpilot and, where relevant, Ofcom's own complaints data, and wrote an 8-section contentSections block plus FAQs matching the site's deepest existing template (Gigaclear). All copy hand-checked for zero em dashes and zero banned AI-tell vocabulary/phrases per the Stage 4a list. TalkTalk's existing entry was materially stale (Trustpilot claimed 2.8, real current figure 1.5 from 50k+ reviews in Trustpilot's 'Bad' band; Ofcom's Q1 2026 report names TalkTalk the UK's most complained-about broadband provider for the third consecutive quarter; the old 'price-lock guarantee' highlight was false, two scheduled April 2027/2028 rises are now built into every contract) -- fully rewritten, not just extended. Zzoomm and Highland Broadband were brand-new Provider entries (real Awin tracking links, placeholder text-wordmark logos per the brief's guardrail against fabricating brand marks). In passing, corrected Plusnet's stale trustpilotScore field (3.9 -&gt; 2.0, the real current figure) since new comparison copy was about to cite it -- Plusnet's own deep content rewrite is out of scope (not an Awin-approved programme). Two new comparison pages: talktalk-vs-plusnet (a genuinely stark, well-evidenced contrast -- same price bracket, opposite ends of Ofcom's complaints table) and zzoomm-vs-hyperoptic (two symmetrical full-fibre altnets with almost non-overlapping coverage footprints). Internal linking relies on the existing 'How {provider} compares' module built earlier this session; both new comparisons are discoverable via /providers/compare and the sitemap even where they don't make a crowded provider's top-3 related slice.</t>
+          <t>Monitor the existing AdSense review, consent implementation and ads.txt authorisation; resolve any concrete policy or crawler issue reported by AdSense.</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
         <v>58</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>data/providers.ts (talktalk, zzoomm, highland-broadband, plusnet trustpilotScore), data/provider-comparisons.ts (talktalk-vs-plusnet, zzoomm-vs-hyperoptic), public/logos/zzoomm.svg, public/logos/highland-broadband.svg</t>
+          <t>AdSense status and /ads.txt</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>ops-awin-publisher-api-integration</t>
+          <t>Google site-review processing</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
+          <t>BroadbandPicker SEO &amp; Content Plan — Live: Build Status</t>
         </is>
       </c>
     </row>
@@ -8180,7 +8224,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Content audit</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -8190,43 +8234,43 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Verify each new city hub has a genuinely local fact</t>
+          <t>Deep, researched content for Awin-approved providers (TalkTalk, Zzoomm, Highland Broadband)</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>8 new city hubs (Birmingham, Bristol, Edinburgh, Glasgow, Leeds, Liverpool, Manchester, Sheffield) plus 50 existing postcode-prefix pages is a lot of near-identical templates. Each needs at least one real local fact (a named local altnet, a real coverage figure) or it reads as duplicate content — audit before building the next batch of cities.</t>
+          <t>Following the Awin programme-status pull (ops-awin-publisher-api-integration), built full researched content for the 3 real providers among the 4 joined programmes (Broadband Genie is a comparison site, not an ISP, and was excluded). Per docs/page-build-pipeline-brief.md Stage 3/4/4a: for each provider, fetched the provider's own site for current pricing/speeds/contract terms, WebSearched Trustpilot and, where relevant, Ofcom's own complaints data, and wrote an 8-section contentSections block plus FAQs matching the site's deepest existing template (Gigaclear). All copy hand-checked for zero em dashes and zero banned AI-tell vocabulary/phrases per the Stage 4a list. TalkTalk's existing entry was materially stale (Trustpilot claimed 2.8, real current figure 1.5 from 50k+ reviews in Trustpilot's 'Bad' band; Ofcom's Q1 2026 report names TalkTalk the UK's most complained-about broadband provider for the third consecutive quarter; the old 'price-lock guarantee' highlight was false, two scheduled April 2027/2028 rises are now built into every contract) -- fully rewritten, not just extended. Zzoomm and Highland Broadband were brand-new Provider entries (real Awin tracking links, placeholder text-wordmark logos per the brief's guardrail against fabricating brand marks). In passing, corrected Plusnet's stale trustpilotScore field (3.9 -&gt; 2.0, the real current figure) since new comparison copy was about to cite it -- Plusnet's own deep content rewrite is out of scope (not an Awin-approved programme). Two new comparison pages: talktalk-vs-plusnet (a genuinely stark, well-evidenced contrast -- same price bracket, opposite ends of Ofcom's complaints table) and zzoomm-vs-hyperoptic (two symmetrical full-fibre altnets with almost non-overlapping coverage footprints). Internal linking relies on the existing 'How {provider} compares' module built earlier this session; both new comparisons are discoverable via /providers/compare and the sitemap even where they don't make a crowded provider's top-3 related slice.</t>
         </is>
       </c>
       <c r="F15" s="3" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>data/priority-pages.ts city entries</t>
+          <t>data/providers.ts (talktalk, zzoomm, highland-broadband, plusnet trustpilotScore), data/provider-comparisons.ts (talktalk-vs-plusnet, zzoomm-vs-hyperoptic), public/logos/zzoomm.svg, public/logos/highland-broadband.svg</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>ops-awin-publisher-api-integration</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -8236,7 +8280,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Content audit</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -8246,19 +8290,19 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Content priority analysis: real SEO + GEO signals, build vs. update on one list</t>
+          <t>Verify each new city hub has a genuinely local fact</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>User asked for a script that does detailed SEO analysis of the site's own data and prioritises what to build vs. update, weighting generative-AI/GEO reports specifically. Built scripts/analyze_content_priority.py: combines real mapped search volume already researched in docs/broadbandpicker-keyword-mapping.xlsx with a live crawl of every provider/comparison/guide page (word count against this session's own depth floors, FAQPage schema, a detectable answer-first paragraph, a parsed checked/reviewed date). Mid-build discovered the user's actual request: a real Google Search Console 'Performance on Search Generative AI Features' export had been dropped into data/GSC/, which is ground truth for AI Overview surfacing, not a proxy -- rebuilt the script to load and heavily weight it. Caught and fixed two real bugs before reporting any findings: word counts of 15k-17k+ caused by the React RSC hydration payload inside &lt;script&gt; tags being counted as visible text, and every page falsely flagging 'no answer-first paragraph' because the &lt;p&gt; search matched header mega-menu labels before reaching the main content -- both fixed by parsing with lxml, stripping script/style, and scoping to &lt;main&gt;. Real finding once the GSC data was wired in: /guides/best-full-fibre-broadband-uk earned 512 real AI-feature impressions in the last 28 days while sitting at 636 words, the clearest 'already working, just needs depth' signal on the site -- now the top-ranked refresh target, above even /providers/sky's 172,237 monthly search volume, since Sky currently earns almost no AI-feature traction (4 impressions) and represents a different kind of opportunity. Sky also does not appear in any of the 3 Awin relationship lists at all (joined/pending/rejected), confirmed via a direct re-check -- no record of ever applying. Every row in the Content Gap Roadmap is already marked built (33/33), so there are currently no new-page gaps on the existing curated keyword list. Findings written up in docs/content-priority-analysis.md.</t>
+          <t>8 new city hubs (Birmingham, Bristol, Edinburgh, Glasgow, Leeds, Liverpool, Manchester, Sheffield) plus 50 existing postcode-prefix pages is a lot of near-identical templates. Each needs at least one real local fact (a named local altnet, a real coverage figure) or it reads as duplicate content — audit before building the next batch of cities.</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
         <v>56</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -8267,22 +8311,22 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>scripts/analyze_content_priority.py</t>
+          <t>data/priority-pages.ts city entries</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>docs/broadbandpicker-keyword-mapping.xlsx (existing keyword research)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -8292,43 +8336,43 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Navigation/header/footer IA improvements</t>
+          <t>Content priority analysis: real SEO + GEO signals, build vs. update on one list</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Researched via scripts/scrape_navigation_patterns.py against 5 best-in-class sites. broadband.co.uk (closest single-vertical comparable) stood out on sticky header, breadcrumbs and a trust badge near the top; BroadbandPicker already matches on the first two. Header nav link count split cleanly into supersite (127-556 links) vs specialist (21 links) patterns, confirming the growth playbook's 'specialist, not supersite' positioning. Added Postcode to primary nav; restructured the footer from 4 to 6 columns (added Tools, Find Broadband by Area, Research) to fix a crawl/link-equity gap for the postcode-district and tools pages built this session.</t>
+          <t>User asked for a script that does detailed SEO analysis of the site's own data and prioritises what to build vs. update, weighting generative-AI/GEO reports specifically. Built scripts/analyze_content_priority.py: combines real mapped search volume already researched in docs/broadbandpicker-keyword-mapping.xlsx with a live crawl of every provider/comparison/guide page (word count against this session's own depth floors, FAQPage schema, a detectable answer-first paragraph, a parsed checked/reviewed date). Mid-build discovered the user's actual request: a real Google Search Console 'Performance on Search Generative AI Features' export had been dropped into data/GSC/, which is ground truth for AI Overview surfacing, not a proxy -- rebuilt the script to load and heavily weight it. Caught and fixed two real bugs before reporting any findings: word counts of 15k-17k+ caused by the React RSC hydration payload inside &lt;script&gt; tags being counted as visible text, and every page falsely flagging 'no answer-first paragraph' because the &lt;p&gt; search matched header mega-menu labels before reaching the main content -- both fixed by parsing with lxml, stripping script/style, and scoping to &lt;main&gt;. Real finding once the GSC data was wired in: /guides/best-full-fibre-broadband-uk earned 512 real AI-feature impressions in the last 28 days while sitting at 636 words, the clearest 'already working, just needs depth' signal on the site -- now the top-ranked refresh target, above even /providers/sky's 172,237 monthly search volume, since Sky currently earns almost no AI-feature traction (4 impressions) and represents a different kind of opportunity. Sky also does not appear in any of the 3 Awin relationship lists at all (joined/pending/rejected), confirmed via a direct re-check -- no record of ever applying. Every row in the Content Gap Roadmap is already marked built (33/33), so there are currently no new-page gaps on the existing curated keyword list. Findings written up in docs/content-priority-analysis.md.</t>
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>60</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>app/layout.tsx</t>
+          <t>scripts/analyze_content_priority.py</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>docs/broadbandpicker-keyword-mapping.xlsx (existing keyword research)</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -8338,7 +8382,7 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-22 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -8353,24 +8397,24 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Working contact form delivering to a real inbox, no third-party service</t>
+          <t>Navigation/header/footer IA improvements</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Previously /contact only offered mailto: links to unverified custom-domain addresses (editorial@/partnerships@/hello@broadbandpicker.co.uk). Built a real contact form (components/ContactForm.tsx) posting to a new app/api/contact route, which sends via Gmail SMTP using nodemailer — no Supabase, no database, no third-party form/CRM service, per explicit instruction. All submissions land in sayedsahil.elt@gmail.com (CONTACT_TO_EMAIL env var), sent from a Gmail account authenticated with an App Password (CONTACT_SMTP_USER / CONTACT_SMTP_PASS). Reply-To is set to the sender's own address so replying goes straight back to them. Spam mitigation without any external service: a hidden honeypot field (bots that fill every input get silently dropped) and a submit-time check rejecting anything sent under 1.5s after the form rendered. Server-side validates name/email/reason/message independently of the client. The original mailto: cards are kept underneath as a secondary direct-email option. Requires CONTACT_SMTP_USER/PASS to be set in Vercel — the API route fails gracefully with a friendly error and a server log line if they're absent, rather than silently dropping messages.</t>
+          <t>Researched via scripts/scrape_navigation_patterns.py against 5 best-in-class sites. broadband.co.uk (closest single-vertical comparable) stood out on sticky header, breadcrumbs and a trust badge near the top; BroadbandPicker already matches on the first two. Header nav link count split cleanly into supersite (127-556 links) vs specialist (21 links) patterns, confirming the growth playbook's 'specialist, not supersite' positioning. Added Postcode to primary nav; restructured the footer from 4 to 6 columns (added Tools, Find Broadband by Area, Research) to fix a crawl/link-equity gap for the postcode-district and tools pages built this session.</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
         <v>55</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -8379,22 +8423,22 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>app/api/contact/route.ts, components/ContactForm.tsx, app/contact/page.tsx</t>
+          <t>app/layout.tsx</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>CONTACT_SMTP_USER / CONTACT_SMTP_PASS Gmail App Password set in Vercel env vars</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-22 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -8404,48 +8448,48 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Deep, researched content for Awin-pending providers (Community Fibre, Cuckoo, Zen Internet, National Broadband, Trooli, Pine Media)</t>
+          <t>Working contact form delivering to a real inbox, no third-party service</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Follow-up to content-awin-approved-provider-deep-content, extending the same research process to the 6 real UK-relevant advertisers pending Awin approval (Sky ROI excluded -- Republic of Ireland Sky, not UK, out of scope for a UK site, confirmed with the user). Community Fibre and Zen Internet were existing but thin entries, fully rewritten. Cuckoo was already deep and dated the previous day; verified rather than rewritten. National Broadband, Trooli and Pine Media were brand-new Provider entries. National Broadband is the site's first 4G/5G fixed-wireless provider (a genuinely new content category, not another fibre altnet); Pine Media is a hyperlocal single-city (Sheffield-only) provider with a two-tier product split (its own symmetrical GIG network vs an Openreach-based GLO product) that needed explaining clearly to avoid conflating the two. Key design decision: because these programmes are pending, not joined, affiliateUrl stays as each provider's own plain site URL rather than an Awin tracking link -- confirmed via a live API test that Awin's linkbuilder will generate a structurally valid tracking URL even for a pending programme, which would be misleading to publish since it likely would not earn commission (or could breach Awin's terms) before approval. Each reviewSources array carries an explicit 'pending, not yet approved' note on the Awin source, matching the existing Gigaclear convention. All copy hand-checked for zero em dashes and zero banned AI-tell vocabulary/phrases. Three new comparison pages, chosen for genuine evidentiary value over one-per-provider completeness: community-fibre-vs-hyperoptic (London's two biggest symmetrical altnets, direct competitors), trooli-vs-zzoomm (two multi-region altnets with near-zero coverage overlap and matching no-price-rise policies), and national-broadband-vs-highland-broadband (5G available now vs fibre still being built -- a genuine buy-now-or-wait decision for the same rural Scottish customer). Cuckoo, Zen Internet and Pine Media were deliberately left without a new comparison this round -- no natural, non-forced head-to-head partner existed for any of them without inventing artificial relevance.</t>
+          <t>Previously /contact only offered mailto: links to unverified custom-domain addresses (editorial@/partnerships@/hello@broadbandpicker.co.uk). Built a real contact form (components/ContactForm.tsx) posting to a new app/api/contact route, which sends via Gmail SMTP using nodemailer — no Supabase, no database, no third-party form/CRM service, per explicit instruction. All submissions land in sayedsahil.elt@gmail.com (CONTACT_TO_EMAIL env var), sent from a Gmail account authenticated with an App Password (CONTACT_SMTP_USER / CONTACT_SMTP_PASS). Reply-To is set to the sender's own address so replying goes straight back to them. Spam mitigation without any external service: a hidden honeypot field (bots that fill every input get silently dropped) and a submit-time check rejecting anything sent under 1.5s after the form rendered. Server-side validates name/email/reason/message independently of the client. The original mailto: cards are kept underneath as a secondary direct-email option. Requires CONTACT_SMTP_USER/PASS to be set in Vercel — the API route fails gracefully with a friendly error and a server log line if they're absent, rather than silently dropping messages.</t>
         </is>
       </c>
       <c r="F19" s="3" t="n">
         <v>55</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>data/providers.ts (community-fibre, cuckoo, zen-internet, national-broadband, trooli, pine-media), data/provider-comparisons.ts (community-fibre-vs-hyperoptic, trooli-vs-zzoomm, national-broadband-vs-highland-broadband), public/logos/national-broadband.svg, public/logos/trooli.svg, public/logos/pine-media.svg</t>
+          <t>app/api/contact/route.ts, components/ContactForm.tsx, app/contact/page.tsx</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>content-awin-approved-provider-deep-content, ops-awin-publisher-api-integration</t>
+          <t>CONTACT_SMTP_USER / CONTACT_SMTP_PASS Gmail App Password set in Vercel env vars</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
@@ -8460,7 +8504,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Growth</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -8470,43 +8514,43 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Run original-research outreach and digital PR</t>
+          <t>Deep, researched content for Awin-pending providers (Community Fibre, Cuckoo, Zen Internet, National Broadband, Trooli, Pine Media)</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Build a relevant outreach list and earn citations and links to the live Ofcom-backed customer-satisfaction research.</t>
+          <t>Follow-up to content-awin-approved-provider-deep-content, extending the same research process to the 6 real UK-relevant advertisers pending Awin approval (Sky ROI excluded -- Republic of Ireland Sky, not UK, out of scope for a UK site, confirmed with the user). Community Fibre and Zen Internet were existing but thin entries, fully rewritten. Cuckoo was already deep and dated the previous day; verified rather than rewritten. National Broadband, Trooli and Pine Media were brand-new Provider entries. National Broadband is the site's first 4G/5G fixed-wireless provider (a genuinely new content category, not another fibre altnet); Pine Media is a hyperlocal single-city (Sheffield-only) provider with a two-tier product split (its own symmetrical GIG network vs an Openreach-based GLO product) that needed explaining clearly to avoid conflating the two. Key design decision: because these programmes are pending, not joined, affiliateUrl stays as each provider's own plain site URL rather than an Awin tracking link -- confirmed via a live API test that Awin's linkbuilder will generate a structurally valid tracking URL even for a pending programme, which would be misleading to publish since it likely would not earn commission (or could breach Awin's terms) before approval. Each reviewSources array carries an explicit 'pending, not yet approved' note on the Awin source, matching the existing Gigaclear convention. All copy hand-checked for zero em dashes and zero banned AI-tell vocabulary/phrases. Three new comparison pages, chosen for genuine evidentiary value over one-per-provider completeness: community-fibre-vs-hyperoptic (London's two biggest symmetrical altnets, direct competitors), trooli-vs-zzoomm (two multi-region altnets with near-zero coverage overlap and matching no-price-rise policies), and national-broadband-vs-highland-broadband (5G available now vs fibre still being built -- a genuine buy-now-or-wait decision for the same rural Scottish customer). Cuckoo, Zen Internet and Pine Media were deliberately left without a new comparison this round -- no natural, non-forced head-to-head partner existed for any of them without inventing artificial relevance.</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>/research/uk-broadband-customer-satisfaction</t>
+          <t>data/providers.ts (community-fibre, cuckoo, zen-internet, national-broadband, trooli, pine-media), data/provider-comparisons.ts (community-fibre-vs-hyperoptic, trooli-vs-zzoomm, national-broadband-vs-highland-broadband), public/logos/national-broadband.svg, public/logos/trooli.svg, public/logos/pine-media.svg</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Research page and source methodology are live</t>
+          <t>content-awin-approved-provider-deep-content, ops-awin-publisher-api-integration</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>BroadbandPicker SEO &amp; Content Plan — Live: Build Status / 90 Day Roadmap</t>
+          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -8516,7 +8560,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -8526,19 +8570,19 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Full Fibre Broadband UK guide (top content-priority-analysis target)</t>
+          <t>Run original-research outreach and digital PR</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Top-ranked target from scripts/analyze_content_priority.py's first real run: 512 AI-feature impressions in the last 28 days (real GSC data) at only 636 words. Fully rewritten to 1,596 words, drawing on already-verified provider facts from the three Awin content batches (BT, EE, Vodafone, Plusnet, Community Fibre, Hyperoptic, toob, Zen Internet) plus new research for Sky and a genuinely counter-intuitive finding worth surfacing on its own: every major national provider has a low Trustpilot score, but Ofcom's Q1 2026 complaints data separates them clearly (Plusnet best at 4/100k, TalkTalk worst at 10/100k) -- explained as two measures of different things, not a contradiction. Also verified and included Vodafone's real 2026 award wins (Expert Reviews Broadband Awards, Uswitch Most Popular Provider) alongside its poor Ofcom complaints position, rather than picking one narrative. Caught and fixed a real bug before shipping: wrote several apostrophes as literal backslash-escapes ( \' ) copying the .ts string-literal habit from data/providers.ts into JSX text content, where they would have rendered as a visible backslash -- fixed to the file's existing &amp;apos; convention and verified against the live rendered HTML, not just the build passing, before considering it done.</t>
+          <t>Build a relevant outreach list and earn citations and links to the live Ofcom-backed customer-satisfaction research.</t>
         </is>
       </c>
       <c r="F21" s="3" t="n">
         <v>54</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
@@ -8547,22 +8591,22 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-full-fibre-broadband-uk), data/guides.ts</t>
+          <t>/research/uk-broadband-customer-satisfaction</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>Research page and source methodology are live</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>BroadbandPicker SEO &amp; Content Plan — Live: Build Status / 90 Day Roadmap</t>
         </is>
       </c>
     </row>
@@ -8572,29 +8616,29 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Strategy</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Growth</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Reprioritise quarter two using GSC, engagement and affiliate evidence</t>
+          <t>Deep rewrite: Best Full Fibre Broadband UK guide (top content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Review query/page performance, assisted conversions, Awin decisions and engagement data, then record the next-quarter build decisions.</t>
+          <t>Top-ranked target from scripts/analyze_content_priority.py's first real run: 512 AI-feature impressions in the last 28 days (real GSC data) at only 636 words. Fully rewritten to 1,596 words, drawing on already-verified provider facts from the three Awin content batches (BT, EE, Vodafone, Plusnet, Community Fibre, Hyperoptic, toob, Zen Internet) plus new research for Sky and a genuinely counter-intuitive finding worth surfacing on its own: every major national provider has a low Trustpilot score, but Ofcom's Q1 2026 complaints data separates them clearly (Plusnet best at 4/100k, TalkTalk worst at 10/100k) -- explained as two measures of different things, not a contradiction. Also verified and included Vodafone's real 2026 award wins (Expert Reviews Broadband Awards, Uswitch Most Popular Provider) alongside its poor Ofcom complaints position, rather than picking one narrative. Caught and fixed a real bug before shipping: wrote several apostrophes as literal backslash-escapes ( \' ) copying the .ts string-literal habit from data/providers.ts into JSX text content, where they would have rendered as a visible backslash -- fixed to the file's existing &amp;apos; convention and verified against the live rendered HTML, not just the build passing, before considering it done.</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -8603,22 +8647,22 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Next-quarter decision log</t>
+          <t>app/guides/[slug]/page.tsx (best-full-fibre-broadband-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>ops-conversion-reporting-loop and sufficient observation period</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>BroadbandPicker SEO &amp; Content Plan — Live: 90 Day Roadmap</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -8628,29 +8672,29 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Postcode-aware personalisation across the customer journey, free tier only</t>
+          <t>Reprioritise quarter two using GSC, engagement and affiliate evidence</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>User asked for a postcode -&gt; select-your-house-number address picker with customised content, and explicitly asked whether it could be built free. Researched live (WebSearch, 2026-08-23): full UK address-level lookup (the data behind 'pick your house from a list') is Royal Mail's licensed PAF data, not open -- getAddress.io, a popular free-tier provider, was shut down in Oct 2025 after a Royal Mail/IDDQD IP claim; Ideal Postcodes gives a 1-month/50-credit trial then pay-as-you-go; no provider offers a genuine unlimited free tier at real traffic. Separately, even a working address picker wouldn't improve accuracy without a paid per-address line-checker API (Openreach or provider-specific), which is a commercial relationship, not a script. Presented both findings and 3 options to the user via AskUserQuestion; they chose the free path: deepen personalisation using data already held, no new API, no new cost. Shipped: extended the existing components/PostcodeContextBar.tsx (previously only on deals/compare/provider pages) to guide pages and all 3 tool pages (speed test, broadband match, cost calculator) so a stored postcode follows the visitor through the full journey; new components/ProviderAvailabilityBadge.tsx shows a real yes/no ('BT is/isn't listed as available in {town}') on provider review pages, but only for the 51 postcode areas with real availableProviders data in data/postcodes.ts -- silently renders nothing outside that set rather than guessing; new components/ReturningVisitorBanner.tsx greets a returning visitor on the homepage with a direct link back to their own postcode's deals.</t>
+          <t>Review query/page performance, assisted conversions, Awin decisions and engagement data, then record the next-quarter build decisions.</t>
         </is>
       </c>
       <c r="F23" s="3" t="n">
         <v>53</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
@@ -8659,22 +8703,22 @@
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>components/ProviderAvailabilityBadge.tsx, components/ReturningVisitorBanner.tsx, components/PostcodeContextBar.tsx, app/page.tsx, app/providers/[slug]/page.tsx, app/guides/[slug]/page.tsx, app/speed-test/page.tsx, app/tools/broadband-match/page.tsx, app/tools/broadband-cost-calculator/page.tsx</t>
+          <t>Next-quarter decision log</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>None -- deliberately built on data already held, no new API/cost</t>
+          <t>ops-conversion-reporting-loop and sufficient observation period</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
+          <t>BroadbandPicker SEO &amp; Content Plan — Live: 90 Day Roadmap</t>
         </is>
       </c>
     </row>
@@ -8694,16 +8738,16 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Homepage visual redesign: illustrations + interactivity</t>
+          <t>Postcode-aware personalisation across the customer journey, free tier only</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Researched via scripts/analyze_homepage_visual_design.py against 5 UK broadband comparison homepages: none uses stock-photo hero banners; the dominant visual language is heavy inline SVG (Uswitch ships 195) and provider logos, no carousel/animation library detected anywhere. Generated 7 original on-brand SVG illustrations (scripts/generate_homepage_illustrations.py: hero network graphic, 3 colour-filled step icons, 2 gradient blobs, a quiz illustration) rather than stock photography, matching what's actually proven in this vertical. Added a scroll-reveal component, hover interactions, and restructured the Broadband Match promo to a two-column illustrated layout. Content/copy unchanged, visual/UX only.</t>
+          <t>User asked for a postcode -&gt; select-your-house-number address picker with customised content, and explicitly asked whether it could be built free. Researched live (WebSearch, 2026-08-23): full UK address-level lookup (the data behind 'pick your house from a list') is Royal Mail's licensed PAF data, not open -- getAddress.io, a popular free-tier provider, was shut down in Oct 2025 after a Royal Mail/IDDQD IP claim; Ideal Postcodes gives a 1-month/50-credit trial then pay-as-you-go; no provider offers a genuine unlimited free tier at real traffic. Separately, even a working address picker wouldn't improve accuracy without a paid per-address line-checker API (Openreach or provider-specific), which is a commercial relationship, not a script. Presented both findings and 3 options to the user via AskUserQuestion; they chose the free path: deepen personalisation using data already held, no new API, no new cost. Shipped: extended the existing components/PostcodeContextBar.tsx (previously only on deals/compare/provider pages) to guide pages and all 3 tool pages (speed test, broadband match, cost calculator) so a stored postcode follows the visitor through the full journey; new components/ProviderAvailabilityBadge.tsx shows a real yes/no ('BT is/isn't listed as available in {town}') on provider review pages, but only for the 51 postcode areas with real availableProviders data in data/postcodes.ts -- silently renders nothing outside that set rather than guessing; new components/ReturningVisitorBanner.tsx greets a returning visitor on the homepage with a direct link back to their own postcode's deals.</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>55</v>
@@ -8715,12 +8759,12 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>app/page.tsx, components/ScrollReveal.tsx, public/illustrations/</t>
+          <t>components/ProviderAvailabilityBadge.tsx, components/ReturningVisitorBanner.tsx, components/PostcodeContextBar.tsx, app/page.tsx, app/providers/[slug]/page.tsx, app/guides/[slug]/page.tsx, app/speed-test/page.tsx, app/tools/broadband-match/page.tsx, app/tools/broadband-cost-calculator/page.tsx</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None -- deliberately built on data already held, no new API/cost</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -8740,22 +8784,22 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Cheapest Broadband Deals UK guide (2nd content-priority-analysis target)</t>
+          <t>Homepage visual redesign: illustrations + interactivity</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Second target from scripts/analyze_content_priority.py's ranked list: 130 real GSC AI-feature impressions at 481 words, and materially stale (last touched 2026-06-01, still citing NOW Broadband at a since-changed £17.99). Rewritten to 1,101 words, drawing on session-verified pricing across 11 providers rather than fresh research for most of them. Real correction made: NOW Broadband's usable Full Fibre 75 now starts at £23/mo, not the stale £17.99 the old copy cited -- no longer reliably the cheapest option, now similar to or pricier than Plusnet (£21.99) and EE (£22.99). Real new finding: Community Fibre's Essential 35 at £12.50/mo is the genuinely cheapest full-fibre deal on the market (London/Surrey/Sussex only). Verified current social tariff pricing (Virgin Media £12.50, BT Home Essentials £15-20, Sky Broadband Basics £20 existing-customers-only) plus a real, citable Ofcom stat: ~4.2 million eligible households, only ~532,000 actually claiming one. Caught the same JSX-vs-.ts apostrophe-escaping bug found on the previous guide (one instance this time, in the NOW Broadband paragraph) before shipping -- confirmed via the file's own reviewSources-style checked-date convention. 1,101 words sits just under this session's own 1,200-word guide depth floor; left as is rather than padding for its own sake, since the content is already comprehensive (2 real data tables, 5 FAQs, all newly sourced).</t>
+          <t>Researched via scripts/analyze_homepage_visual_design.py against 5 UK broadband comparison homepages: none uses stock-photo hero banners; the dominant visual language is heavy inline SVG (Uswitch ships 195) and provider logos, no carousel/animation library detected anywhere. Generated 7 original on-brand SVG illustrations (scripts/generate_homepage_illustrations.py: hero network graphic, 3 colour-filled step icons, 2 gradient blobs, a quiz illustration) rather than stock photography, matching what's actually proven in this vertical. Added a scroll-reveal component, hover interactions, and restructured the Broadband Match promo to a two-column illustrated layout. Content/copy unchanged, visual/UX only.</t>
         </is>
       </c>
       <c r="F25" s="3" t="n">
@@ -8771,12 +8815,12 @@
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (cheapest-broadband-uk), data/guides.ts</t>
+          <t>app/page.tsx, components/ScrollReveal.tsx, public/illustrations/</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
@@ -8786,7 +8830,7 @@
       </c>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -8796,29 +8840,29 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Mobile and cross-device navigation overhaul</t>
+          <t>Deep rewrite: Cheapest Broadband Deals UK guide (2nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>New scripts/analyze_mobile_ux.py scanned Uswitch, broadband.co.uk and choose.co.uk (MoneySavingExpert 403, reported not bypassed) with a mobile Safari user agent for markup/CSS signals: viewport meta and hamburger menu markers were universal but already correct on our own site; tel: click-to-call was absent everywhere (0/4, skipped); sticky bottom CTA (1/4) and apple-touch-icon (2/4) were too weak/incomplete to act on. The real gap was found by direct inspection, not the scan: the mobile nav was a small anchored dropdown of 10 flat links with ~36px touch targets, while the desktop nav beside it was a full mega-menu, and the header postcode checker was desktop-only so phone users had no quick postcode access outside the homepage/deals page. Replaced it with new components/MobileNav.tsx: a full-width slide-down panel reusing the desktop mega-menu's own icon/link data (exported from MainNav.tsx, so the two can't drift apart), every link at a 44px (min-h-11) touch target, and the postcode checker embedded at the top so it's reachable from any page. Added anchor ids to /guides category sections so the new mobile Guides menu jumps to a real target instead of an unread query param.</t>
+          <t>Second target from scripts/analyze_content_priority.py's ranked list: 130 real GSC AI-feature impressions at 481 words, and materially stale (last touched 2026-06-01, still citing NOW Broadband at a since-changed £17.99). Rewritten to 1,101 words, drawing on session-verified pricing across 11 providers rather than fresh research for most of them. Real correction made: NOW Broadband's usable Full Fibre 75 now starts at £23/mo, not the stale £17.99 the old copy cited -- no longer reliably the cheapest option, now similar to or pricier than Plusnet (£21.99) and EE (£22.99). Real new finding: Community Fibre's Essential 35 at £12.50/mo is the genuinely cheapest full-fibre deal on the market (London/Surrey/Sussex only). Verified current social tariff pricing (Virgin Media £12.50, BT Home Essentials £15-20, Sky Broadband Basics £20 existing-customers-only) plus a real, citable Ofcom stat: ~4.2 million eligible households, only ~532,000 actually claiming one. Caught the same JSX-vs-.ts apostrophe-escaping bug found on the previous guide (one instance this time, in the NOW Broadband paragraph) before shipping -- confirmed via the file's own reviewSources-style checked-date convention. 1,101 words sits just under this session's own 1,200-word guide depth floor; left as is rather than padding for its own sake, since the content is already comprehensive (2 real data tables, 5 FAQs, all newly sourced).</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
@@ -8827,12 +8871,12 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>components/MobileNav.tsx, components/MainNav.tsx, app/layout.tsx, app/guides/page.tsx</t>
+          <t>app/guides/[slug]/page.tsx (cheapest-broadband-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -8842,7 +8886,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -8862,19 +8906,19 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Detailed mega-menu navigation</t>
+          <t>Mobile and cross-device navigation overhaul</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Extended scripts/scrape_navigation_patterns.py with mega-menu structural detection (top-level item count, icons-in-dropdown, descriptive subtext, nesting depth). Found Uswitch uses icons in dropdown items and broadband.co.uk uses one-line descriptions under category groups — both implemented. Built components/MainNav.tsx: Providers, Postcode, Guides and Tools are now dropdowns with icons and descriptions; Compare and Deals stay direct links as primary single-destination actions. The Guides dropdown is a real mega-menu pulling the site's actual 6 guide categories and their real guides live from data/guides.ts — stays correct as the pipeline adds guides, no hardcoding. CSS-only (group-hover/group-focus-within), keyboard-reachable via Tab, no JS dependency.</t>
+          <t>New scripts/analyze_mobile_ux.py scanned Uswitch, broadband.co.uk and choose.co.uk (MoneySavingExpert 403, reported not bypassed) with a mobile Safari user agent for markup/CSS signals: viewport meta and hamburger menu markers were universal but already correct on our own site; tel: click-to-call was absent everywhere (0/4, skipped); sticky bottom CTA (1/4) and apple-touch-icon (2/4) were too weak/incomplete to act on. The real gap was found by direct inspection, not the scan: the mobile nav was a small anchored dropdown of 10 flat links with ~36px touch targets, while the desktop nav beside it was a full mega-menu, and the header postcode checker was desktop-only so phone users had no quick postcode access outside the homepage/deals page. Replaced it with new components/MobileNav.tsx: a full-width slide-down panel reusing the desktop mega-menu's own icon/link data (exported from MainNav.tsx, so the two can't drift apart), every link at a 44px (min-h-11) touch target, and the postcode checker embedded at the top so it's reachable from any page. Added anchor ids to /guides category sections so the new mobile Guides menu jumps to a real target instead of an unread query param.</t>
         </is>
       </c>
       <c r="F27" s="3" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
@@ -8883,7 +8927,7 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>components/MainNav.tsx, app/layout.tsx</t>
+          <t>components/MobileNav.tsx, components/MainNav.tsx, app/layout.tsx, app/guides/page.tsx</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
@@ -8918,19 +8962,19 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Animated, interactive mobile menu with click-outside-to-close</t>
+          <t>Detailed mega-menu navigation</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Direct UX/interaction-design request, not a scraping pass. Rewrote components/MobileNav.tsx from a native &lt;details&gt; element (no animation, no click-outside-to-close) to a controlled client component: hamburger icon morphs into an X on open; a blurred backdrop closes the menu on click or Escape; the panel and its sections slide/fade in with a staggered delay reusing the same transition idiom as components/ScrollReveal.tsx; Providers/Postcode/Guides/Tools became single-open accordions using a CSS-only grid-template-rows 0fr-&gt;1fr transition (no JS height measurement); the menu auto-closes on route change via usePathname(); background scroll is locked while open; focus moves into the panel on open and returns to the trigger on Escape. Global prefers-reduced-motion handling already in app/globals.css applies automatically. Not visually verified on a real device — no browser automation tool available this session, validated via build output, generated CSS and server-rendered markup only.</t>
+          <t>Extended scripts/scrape_navigation_patterns.py with mega-menu structural detection (top-level item count, icons-in-dropdown, descriptive subtext, nesting depth). Found Uswitch uses icons in dropdown items and broadband.co.uk uses one-line descriptions under category groups — both implemented. Built components/MainNav.tsx: Providers, Postcode, Guides and Tools are now dropdowns with icons and descriptions; Compare and Deals stay direct links as primary single-destination actions. The Guides dropdown is a real mega-menu pulling the site's actual 6 guide categories and their real guides live from data/guides.ts — stays correct as the pipeline adds guides, no hardcoding. CSS-only (group-hover/group-focus-within), keyboard-reachable via Tab, no JS dependency.</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
         <v>50</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -8939,7 +8983,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>components/MobileNav.tsx</t>
+          <t>components/MainNav.tsx, app/layout.tsx</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -8964,29 +9008,29 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Business Broadband Providers UK guide (3rd content-priority-analysis target)</t>
+          <t>Animated, interactive mobile menu with click-outside-to-close</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Third target from scripts/analyze_content_priority.py's ranked list: 142 real GSC AI-feature impressions at 596 words. This page lives on a different template than the [slug]-based guides (app/guides/best-business-broadband-providers-uk/ is a standalone PrioritySeoPage route backed by data/priority-pages.ts), and had 2 pre-existing em dashes fixed as part of the pass. Rewritten to 1,050 words with real, specific per-provider data: Vodafone Business has the most competitive entry-level price (~£20-22/mo excl. VAT), Zen Business leads on satisfaction (Which? Recommended since 2021, 84% score) -- consistent with, and corroborating, the consumer Zen Internet findings from the Awin-rejected batch, Virgin Media Business has the fastest raw speed (442 Mbps average), and a genuinely useful, specific stat: out-of-contract business customers overpay 24.86% more per month on average. Added a real contended-vs-uncontended leased-line explainer with current pricing (from ~£69/mo entry-level). Also fixed a real bug in the analysis script itself found while validating this page: DATE_RE didn't recognise the PrioritySeoPage template's 'Last researched and reviewed:' phrasing (colon, different verb), so every page on that template was incorrectly scored as having no checked date -- fixed and confirmed it also corrected the score for /guides/satellite-broadband-uk on the same template.</t>
+          <t>Direct UX/interaction-design request, not a scraping pass. Rewrote components/MobileNav.tsx from a native &lt;details&gt; element (no animation, no click-outside-to-close) to a controlled client component: hamburger icon morphs into an X on open; a blurred backdrop closes the menu on click or Escape; the panel and its sections slide/fade in with a staggered delay reusing the same transition idiom as components/ScrollReveal.tsx; Providers/Postcode/Guides/Tools became single-open accordions using a CSS-only grid-template-rows 0fr-&gt;1fr transition (no JS height measurement); the menu auto-closes on route change via usePathname(); background scroll is locked while open; focus moves into the panel on open and returns to the trigger on Escape. Global prefers-reduced-motion handling already in app/globals.css applies automatically. Not visually verified on a real device — no browser automation tool available this session, validated via build output, generated CSS and server-rendered markup only.</t>
         </is>
       </c>
       <c r="F29" s="3" t="n">
         <v>50</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
@@ -8995,12 +9039,12 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>data/priority-pages.ts (business), scripts/analyze_content_priority.py</t>
+          <t>components/MobileNav.tsx</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
@@ -9010,7 +9054,7 @@
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9020,29 +9064,29 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Price-drop alerts</t>
+          <t>Deep rewrite: Best Business Broadband Providers UK guide (3rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>data/provider-live-deals.json already tracks live pricing. An email/notification layer on top ("tell me if broadband in my postcode drops below £X") is mostly wiring, and it's a retention mechanic none of the readable competitors emphasised as much as their comparison tables.</t>
+          <t>Third target from scripts/analyze_content_priority.py's ranked list: 142 real GSC AI-feature impressions at 596 words. This page lives on a different template than the [slug]-based guides (app/guides/best-business-broadband-providers-uk/ is a standalone PrioritySeoPage route backed by data/priority-pages.ts), and had 2 pre-existing em dashes fixed as part of the pass. Rewritten to 1,050 words with real, specific per-provider data: Vodafone Business has the most competitive entry-level price (~£20-22/mo excl. VAT), Zen Business leads on satisfaction (Which? Recommended since 2021, 84% score) -- consistent with, and corroborating, the consumer Zen Internet findings from the Awin-rejected batch, Virgin Media Business has the fastest raw speed (442 Mbps average), and a genuinely useful, specific stat: out-of-contract business customers overpay 24.86% more per month on average. Added a real contended-vs-uncontended leased-line explainer with current pricing (from ~£69/mo entry-level). Also fixed a real bug in the analysis script itself found while validating this page: DATE_RE didn't recognise the PrioritySeoPage template's 'Last researched and reviewed:' phrasing (colon, different verb), so every page on that template was incorrectly scored as having no checked date -- fixed and confirmed it also corrected the score for /guides/satellite-broadband-uk on the same template.</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -9051,22 +9095,22 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>New subscription flow + data/provider-live-deals.json</t>
+          <t>data/priority-pages.ts (business), scripts/analyze_content_priority.py</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Email delivery provider</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9081,24 +9125,24 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Page-type UX redesign: deals, providers, guides, postcode hub</t>
+          <t>Price-drop alerts</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>New scripts/analyze_page_type_ux.py scans competitor pages by theme (deals listing, provider review, guide article, postcode/checker hub) rather than homepage-only, against Uswitch, broadband.co.uk, choose.co.uk and MoneySavingExpert (403, reported not bypassed). Confirmed signals: comparison checkboxes near-universal; badge/chip labels on deals listings + review index; TOC on the guide article + one deals listing; pros/cons on provider review + deals; related-content on provider review + deals; rating widget on one deals listing. No dedicated postcode-hub competitor page exists in this vertical. Shipped strictly against confirmed signals: computed Best Value/Fastest/Editor's Pick badges in components/DealTable.tsx; new components/RatingStars.tsx replacing plain-text Trustpilot scores plus a 'How {provider} compares' related-comparisons module on provider pages; a jump-to-section table of contents on guide pages via new lib/extractHeadings.tsx (JSX-tree heading-ID injection, avoids hand-editing 40 existing guide definitions), gated behind 3+ headings; and the same cheapest/fastest badges plus rating stars carried onto postcode-hub provider cards since deals and hub serve the same comparison job.</t>
+          <t>data/provider-live-deals.json already tracks live pricing. An email/notification layer on top ("tell me if broadband in my postcode drops below £X") is mostly wiring, and it's a retention mechanic none of the readable competitors emphasised as much as their comparison tables.</t>
         </is>
       </c>
       <c r="F31" s="3" t="n">
         <v>49</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
@@ -9107,22 +9151,22 @@
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>components/DealTable.tsx, components/RatingStars.tsx, lib/extractHeadings.tsx, app/providers/[slug]/page.tsx, app/guides/[slug]/page.tsx, app/postcode/[area]/page.tsx</t>
+          <t>New subscription flow + data/provider-live-deals.json</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Email delivery provider</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Functionality pillar</t>
         </is>
       </c>
     </row>
@@ -9142,28 +9186,28 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Footer logo placement and interactive elements</t>
+          <t>Page-type UX redesign: deals, providers, guides, postcode hub</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Extended scripts/analyze_homepage_visual_design.py with footer-specific detection (logo, social icons, accordion/back-to-top, hover density). Confirmed directly in app/layout.tsx (not just inferred from the scan) that the footer had no logo at all. Added components/Logo.tsx (extracted from the header, reused larger in the footer with a tagline), made the 6 footer link columns &lt;details open&gt; elements with a mobile-only collapse toggle (desktop behaves exactly as static headings did, via lg:pointer-events-none, so nothing is at risk of accidental collapse), upgraded the social link to a hover-interactive pill button, and added a 'Back to top' link using the existing global smooth-scroll behaviour.</t>
+          <t>New scripts/analyze_page_type_ux.py scans competitor pages by theme (deals listing, provider review, guide article, postcode/checker hub) rather than homepage-only, against Uswitch, broadband.co.uk, choose.co.uk and MoneySavingExpert (403, reported not bypassed). Confirmed signals: comparison checkboxes near-universal; badge/chip labels on deals listings + review index; TOC on the guide article + one deals listing; pros/cons on provider review + deals; related-content on provider review + deals; rating widget on one deals listing. No dedicated postcode-hub competitor page exists in this vertical. Shipped strictly against confirmed signals: computed Best Value/Fastest/Editor's Pick badges in components/DealTable.tsx; new components/RatingStars.tsx replacing plain-text Trustpilot scores plus a 'How {provider} compares' related-comparisons module on provider pages; a jump-to-section table of contents on guide pages via new lib/extractHeadings.tsx (JSX-tree heading-ID injection, avoids hand-editing 40 existing guide definitions), gated behind 3+ headings; and the same cheapest/fastest badges plus rating stars carried onto postcode-hub provider cards since deals and hub serve the same comparison job.</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>app/layout.tsx, components/Logo.tsx</t>
+          <t>components/DealTable.tsx, components/RatingStars.tsx, lib/extractHeadings.tsx, app/providers/[slug]/page.tsx, app/guides/[slug]/page.tsx, app/postcode/[area]/page.tsx</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -9188,38 +9232,38 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Research-led editorial refresh: Best Broadband and TV Deals guide</t>
+          <t>Footer logo placement and interactive elements</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>User-requested application of the same Stage 3/4/4a research process from the Awin content batches to a single existing guide page, /guides/best-broadband-and-tv-deals. Unlike the thin provider stubs rewritten in the Awin batches, this guide was already well-built (tables, methodology, 7 FAQs, real Ofcom citations, last checked 29 July 2026) -- not a stub needing a ground-up rewrite, so this was a verify-and-deepen pass grounded in fresh research rather than a full replacement. Scraped 2 top-ranking competitors (MoneySuperMarket, Uswitch) per Stage 3.0: found MoneySupermarket runs a 15-question FAQ (ours had 7) and leads with an expert-quoted bundling-savings statistic. Traced that claim to its actual primary source rather than citing the secondary restatement: Ofcom's own February 2026 research, savings of £26-£48/month from bundling and pay-TV averaging £12/month within a bundle (23% real-terms fall) -- a stronger, more current, primary-sourced figure than the competitor's 2023-dated stat, added as a new section. Also found and added two genuinely new, specific facts the page didn't have: Virgin Media's Max Volt bundle (real current pricing including its two scheduled rises to April 2028) as a concrete worked example, and Virgin Media's 'Most Reliable Broadband Provider' win at the 2026 Uswitch Telecoms Awards (Opensignal-verified, a genuine third-party measurement). Named the specific Sky bundle example (Sky Stream, Sky TV, Netflix + Full Fibre 300, £35/month) that the existing copy referenced only vaguely. Added 2 new FAQs tied to the new content. Fixed 2 pre-existing em dashes found during the pass (a legitimate en-dash numeric range, '50-100Mbps', was left alone -- not an AI-tell, different typographic use). Updated the page's stated fact-check date and guides.ts updatedDate to 2026-08-24.</t>
+          <t>Extended scripts/analyze_homepage_visual_design.py with footer-specific detection (logo, social icons, accordion/back-to-top, hover density). Confirmed directly in app/layout.tsx (not just inferred from the scan) that the footer had no logo at all. Added components/Logo.tsx (extracted from the header, reused larger in the footer with a tagline), made the 6 footer link columns &lt;details open&gt; elements with a mobile-only collapse toggle (desktop behaves exactly as static headings did, via lg:pointer-events-none, so nothing is at risk of accidental collapse), upgraded the social link to a hover-interactive pill button, and added a 'Back to top' link using the existing global smooth-scroll behaviour.</t>
         </is>
       </c>
       <c r="F33" s="3" t="n">
         <v>48</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-and-tv-deals), data/guides.ts</t>
+          <t>app/layout.tsx, components/Logo.tsx</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
@@ -9234,7 +9278,7 @@
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9244,29 +9288,29 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Establish monthly Core Web Vitals reporting by template</t>
+          <t>Research-led editorial refresh: Best Broadband and TV Deals guide</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Track LCP, INP and CLS by page template and prioritise JS or image-weight fixes from evidence.</t>
+          <t>User-requested application of the same Stage 3/4/4a research process from the Awin content batches to a single existing guide page, /guides/best-broadband-and-tv-deals. Unlike the thin provider stubs rewritten in the Awin batches, this guide was already well-built (tables, methodology, 7 FAQs, real Ofcom citations, last checked 29 July 2026) -- not a stub needing a ground-up rewrite, so this was a verify-and-deepen pass grounded in fresh research rather than a full replacement. Scraped 2 top-ranking competitors (MoneySuperMarket, Uswitch) per Stage 3.0: found MoneySupermarket runs a 15-question FAQ (ours had 7) and leads with an expert-quoted bundling-savings statistic. Traced that claim to its actual primary source rather than citing the secondary restatement: Ofcom's own February 2026 research, savings of £26-£48/month from bundling and pay-TV averaging £12/month within a bundle (23% real-terms fall) -- a stronger, more current, primary-sourced figure than the competitor's 2023-dated stat, added as a new section. Also found and added two genuinely new, specific facts the page didn't have: Virgin Media's Max Volt bundle (real current pricing including its two scheduled rises to April 2028) as a concrete worked example, and Virgin Media's 'Most Reliable Broadband Provider' win at the 2026 Uswitch Telecoms Awards (Opensignal-verified, a genuine third-party measurement). Named the specific Sky bundle example (Sky Stream, Sky TV, Netflix + Full Fibre 300, £35/month) that the existing copy referenced only vaguely. Added 2 new FAQs tied to the new content. Fixed 2 pre-existing em dashes found during the pass (a legitimate en-dash numeric range, '50-100Mbps', was left alone -- not an AI-tell, different typographic use). Updated the page's stated fact-check date and guides.ts updatedDate to 2026-08-24.</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -9275,22 +9319,22 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Sitewide template performance report</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-and-tv-deals), data/guides.ts</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Field data or representative lab baselines</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>BroadbandPicker SEO &amp; Content Plan — Live: Technical SEO</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9300,53 +9344,53 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Monetisation</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Direct Awin Publisher API access — programme status and link generation</t>
+          <t>Establish monthly Core Web Vitals reporting by template</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>User asked to connect Claude to their Awin account and provided a real API token. There's no one-click connector for Awin (unlike Google Drive/Gmail), so this uses Awin's own Publisher API directly. First live run corrected two wrong assumptions from documentation research: 'programmedetails' requires a specific advertiserId (not a bulk listing endpoint) -- the actual bulk-status endpoint is GET /publishers/{id}/programmes?relationship=X, and 'any' is not a valid value for it (loops joined/pending/suspended/rejected instead; 'notjoined' returns the ~21k whole-platform catalogue so it's excluded from the default and only fetched on request). POST /publishers/{id}/linkbuilder/generate confirmed working, verified against TalkTalk (advertiser 3674). REAL FINDING from the first run, both surfaced to the user and worth acting on: only 4 programmes are joined (TalkTalk, Broadband Genie, Zzoomm, Highland Broadband), 7 pending (Sky ROI, Community Fibre, National Broadband, Trooli, Pine Media, Cuckoo, Zen Internet), and 9 REJECTED including BT (both consumer and business), Vodafone, Plusnet, EE, Virgin Media, Hyperoptic and toob. Cross-checked data/providers.ts: none of the currently-live affiliateUrl values (including TalkTalk, which IS approved) use Awin's awin1.com tracking format -- they're all plain provider URLs, so the site is very likely not earning commission on any current outbound click, joined or not, despite the on-page commercial disclosures implying it might.</t>
+          <t>Track LCP, INP and CLS by page template and prioritise JS or image-weight fixes from evidence.</t>
         </is>
       </c>
       <c r="F35" s="3" t="n">
         <v>47</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>scripts/awin_sync.py</t>
+          <t>Sitewide template performance report</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>AWIN_API_TOKEN from the user's Awin account (user menu -&gt; API Credentials)</t>
+          <t>Field data or representative lab baselines</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
+          <t>BroadbandPicker SEO &amp; Content Plan — Live: Technical SEO</t>
         </is>
       </c>
     </row>
@@ -9356,43 +9400,43 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Monetisation</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best 5G Home Broadband UK guide (4th content-priority-analysis target)</t>
+          <t>Direct Awin Publisher API access — programme status and link generation</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Fourth target from scripts/analyze_content_priority.py's ranked list: 30 real GSC AI-feature impressions at 601 words, and the old copy named no real providers or prices at all, just generic 5G-vs-fibre advice. Rewritten to 1,036 words with real current data for all 4 major UK 5G home broadband options: Three (best value, from GBP29/mo, ~150 Mbps), Vodafone GigaCube (cheapest fixed term at GBP21/mo, or a genuine GBP60/mo no-contract option), EE Smart 5G Hub (broadest UK 5G coverage, GBP30-50/mo), and National Broadband (already deeply covered in the Awin-pending batch) framed correctly here as a multi-network specialist rather than a single-network alternative -- it connects to whichever of the 4 UK networks is strongest at a given address, a genuinely different value proposition worth explaining rather than just listing as a fourth option. Found and included a real Trustpilot-vs-Ofcom divergence for Three specifically (4.5 Trustpilot, worst-quartile Ofcom complaints alongside EE and Vodafone) and linked to the full-fibre guide's deeper explanation of that pattern rather than repeating it in full.</t>
+          <t>User asked to connect Claude to their Awin account and provided a real API token. There's no one-click connector for Awin (unlike Google Drive/Gmail), so this uses Awin's own Publisher API directly. First live run corrected two wrong assumptions from documentation research: 'programmedetails' requires a specific advertiserId (not a bulk listing endpoint) -- the actual bulk-status endpoint is GET /publishers/{id}/programmes?relationship=X, and 'any' is not a valid value for it (loops joined/pending/suspended/rejected instead; 'notjoined' returns the ~21k whole-platform catalogue so it's excluded from the default and only fetched on request). POST /publishers/{id}/linkbuilder/generate confirmed working, verified against TalkTalk (advertiser 3674). REAL FINDING from the first run, both surfaced to the user and worth acting on: only 4 programmes are joined (TalkTalk, Broadband Genie, Zzoomm, Highland Broadband), 7 pending (Sky ROI, Community Fibre, National Broadband, Trooli, Pine Media, Cuckoo, Zen Internet), and 9 REJECTED including BT (both consumer and business), Vodafone, Plusnet, EE, Virgin Media, Hyperoptic and toob. Cross-checked data/providers.ts: none of the currently-live affiliateUrl values (including TalkTalk, which IS approved) use Awin's awin1.com tracking format -- they're all plain provider URLs, so the site is very likely not earning commission on any current outbound click, joined or not, despite the on-page commercial disclosures implying it might.</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
         <v>47</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-5g-home-broadband-uk), data/guides.ts</t>
+          <t>scripts/awin_sync.py</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>AWIN_API_TOKEN from the user's Awin account (user menu -&gt; API Credentials)</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -9402,7 +9446,7 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9412,29 +9456,29 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>UX audit</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Mobile checkout-flow audit</t>
+          <t>Deep rewrite: Best 5G Home Broadband UK guide (4th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>The competitor evidence (15k–23k word desktop hubs) is desktop-shaped. On mobile that content needs a different information architecture — sticky summary bar, collapsed sections, thumb-reachable CTAs. Worth a dedicated pass once analytics show where mobile users drop off.</t>
+          <t>Fourth target from scripts/analyze_content_priority.py's ranked list: 30 real GSC AI-feature impressions at 601 words, and the old copy named no real providers or prices at all, just generic 5G-vs-fibre advice. Rewritten to 1,036 words with real current data for all 4 major UK 5G home broadband options: Three (best value, from GBP29/mo, ~150 Mbps), Vodafone GigaCube (cheapest fixed term at GBP21/mo, or a genuine GBP60/mo no-contract option), EE Smart 5G Hub (broadest UK 5G coverage, GBP30-50/mo), and National Broadband (already deeply covered in the Awin-pending batch) framed correctly here as a multi-network specialist rather than a single-network alternative -- it connects to whichever of the 4 UK networks is strongest at a given address, a genuinely different value proposition worth explaining rather than just listing as a fourth option. Found and included a real Trustpilot-vs-Ofcom divergence for Three specifically (4.5 Trustpilot, worst-quartile Ofcom complaints alongside EE and Vodafone) and linked to the full-fibre guide's deeper explanation of that pattern rather than repeating it in full.</t>
         </is>
       </c>
       <c r="F37" s="3" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
@@ -9443,22 +9487,22 @@
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>Sitewide mobile layout</t>
+          <t>app/guides/[slug]/page.tsx (best-5g-home-broadband-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>Mobile analytics/drop-off data</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — UX pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9468,29 +9512,29 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX audit</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Phone and Broadband Deals guide (5th content-priority-analysis target)</t>
+          <t>Mobile checkout-flow audit</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Fifth target from scripts/analyze_content_priority.py's ranked list: the old copy was generic Digital Voice/line-rental advice with no dates, no stats and one pre-existing em dash, at 457 words. Rewritten with the real PSTN switch-off timeline: full shutdown now locked in for 31 January 2027 (moved from the original December 2025 target after Openreach confirmed the technical barriers were resolved), with PSTN customer numbers falling from 5.2 million (July 2024) to 3.2 million (July 2025). Added Ofcom's minimum one-hour battery backup requirement for emergency-services access during a power cut, and the industry PSTN Charter's commitment not to migrate telecare/vulnerable users without confirmed-compatible equipment. Added a real, specific call-plan cost example (TalkTalk's Anytime Calls add-on at GBP12/mo on top of base broadband) to replace the previous fully generic 'compare the whole contract' advice. FAQs expanded from 3 to 5. Fixed the pre-existing em dash in the dek field.</t>
+          <t>The competitor evidence (15k–23k word desktop hubs) is desktop-shaped. On mobile that content needs a different information architecture — sticky summary bar, collapsed sections, thumb-reachable CTAs. Worth a dedicated pass once analytics show where mobile users drop off.</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
         <v>45</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -9499,22 +9543,22 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>data/priority-pages.ts (phone)</t>
+          <t>Sitewide mobile layout</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>Mobile analytics/drop-off data</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — UX pillar</t>
         </is>
       </c>
     </row>
@@ -9524,53 +9568,53 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Crawlability</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Add routine broken-link and redirect reporting</t>
+          <t>Deep rewrite: Best Phone and Broadband Deals guide (5th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Monitor broken inbound and internal URLs and maintain relevant one-hop redirects.</t>
+          <t>Fifth target from scripts/analyze_content_priority.py's ranked list: the old copy was generic Digital Voice/line-rental advice with no dates, no stats and one pre-existing em dash, at 457 words. Rewritten with the real PSTN switch-off timeline: full shutdown now locked in for 31 January 2027 (moved from the original December 2025 target after Openreach confirmed the technical barriers were resolved), with PSTN customer numbers falling from 5.2 million (July 2024) to 3.2 million (July 2025). Added Ofcom's minimum one-hour battery backup requirement for emergency-services access during a power cut, and the industry PSTN Charter's commitment not to migrate telecare/vulnerable users without confirmed-compatible equipment. Added a real, specific call-plan cost example (TalkTalk's Anytime Calls add-on at GBP12/mo on top of base broadband) to replace the previous fully generic 'compare the whole contract' advice. FAQs expanded from 3 to 5. Fixed the pre-existing em dash in the dek field.</t>
         </is>
       </c>
       <c r="F39" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="G39" s="3" t="n">
         <v>44</v>
       </c>
-      <c r="G39" s="3" t="n">
-        <v>48</v>
-      </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Sitewide crawl and redirect report</t>
+          <t>data/priority-pages.ts (phone)</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L39" s="3" t="inlineStr">
         <is>
-          <t>BroadbandPicker SEO &amp; Content Plan — Live: Technical SEO</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9580,53 +9624,53 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Crawlability</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
+          <t>Add routine broken-link and redirect reporting</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Seventh target from scripts/analyze_content_priority.py's ranked list: /providers/now-broadband was 386 words with no excerpt or contentSections, and its top-level fields were stale on two counts that research corrected -- contractLengths was still [12] (NOW dropped its flexible 12-month contracts; every current package is now a standard 24-month term, per thinkbroadband's dedicated news item on the change) and monthlyPriceFrom was a stale GBP17.99 against a real current cheapest tier of GBP23 (Full Fibre 100). Rewritten to ~1,450 words with 5 contentSections. The genuinely distinctive finding here, different from every other Trustpilot-vs-Ofcom section written this session: NOW is a real exception to the usual pattern, scoring poorly on BOTH Trustpilot (1.2/5, corrected from a stale 3.2) AND Ofcom's Q4 2025 complaints data (11 per 100k vs the 8 industry average), noticeably worse than sister brand Sky on the same underlying Openreach network -- written up as a genuine data point about support quality diverging from infrastructure quality within the same corporate group, not just review-platform noise. Also corrected trustpilotScore 3.2 -&gt; 1.2.</t>
+          <t>Monitor broken inbound and internal URLs and maintain relevant one-hop redirects.</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
         <v>44</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>data/providers.ts (now-broadband)</t>
+          <t>Sitewide crawl and redirect report</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>BroadbandPicker SEO &amp; Content Plan — Live: Technical SEO</t>
         </is>
       </c>
     </row>
@@ -9646,19 +9690,19 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
+          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Eighth target from scripts/analyze_content_priority.py's ranked list: /providers/youfibre was 397 words with no excerpt or contentSections. Rewritten to ~1,575 words with 6 contentSections. The standout finding, verified against a primary Virgin Media O2 press release after a first-pass WebSearch AI summary over-stated it as a done deal: YouFibre's parent company, Substantial Group (Netomnia), is being acquired for GBP2bn by nexfibre (a joint venture of InfraVia, Liberty Global and Telefonica), which then plans to resell the YouFibre/Brsk retail brands to Virgin Media O2 for GBP150m -- announced Feb 2026, referred to the CMA for a Phase 2 investigation on 1 July 2026, and NOT yet completed (expected ~Q3 2026 at the earliest). Also wrote up the real, documented fallout from the March 2026 Brsk-to-YouFibre customer migration (billing errors, login/password-reset failures, reported speed drops, overwhelmed support chat), sourced from ISPreview rather than the vague pre-existing 'Trustpilot sentiment has been mixed' line. Updated the speeds array to the real current tiers (200/1000/2000/8000 Mbps symmetrical, replacing stale 200/900/1800) and contractLengths from [1,12,24] to [1,24] to match the two options confirmed by current pricing research.</t>
+          <t>Seventh target from scripts/analyze_content_priority.py's ranked list: /providers/now-broadband was 386 words with no excerpt or contentSections, and its top-level fields were stale on two counts that research corrected -- contractLengths was still [12] (NOW dropped its flexible 12-month contracts; every current package is now a standard 24-month term, per thinkbroadband's dedicated news item on the change) and monthlyPriceFrom was a stale GBP17.99 against a real current cheapest tier of GBP23 (Full Fibre 100). Rewritten to ~1,450 words with 5 contentSections. The genuinely distinctive finding here, different from every other Trustpilot-vs-Ofcom section written this session: NOW is a real exception to the usual pattern, scoring poorly on BOTH Trustpilot (1.2/5, corrected from a stale 3.2) AND Ofcom's Q4 2025 complaints data (11 per 100k vs the 8 industry average), noticeably worse than sister brand Sky on the same underlying Openreach network -- written up as a genuine data point about support quality diverging from infrastructure quality within the same corporate group, not just review-platform noise. Also corrected trustpilotScore 3.2 -&gt; 1.2.</t>
         </is>
       </c>
       <c r="F41" s="3" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
@@ -9667,7 +9711,7 @@
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>data/providers.ts (youfibre)</t>
+          <t>data/providers.ts (now-broadband)</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
@@ -9702,19 +9746,19 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
+          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Ninth target from scripts/analyze_content_priority.py's ranked list. This ranking page's data was badly stale: it cited Q4 2025 Ofcom complaints figures and June-2026 Trustpilot scores that had already been superseded by this site's own freshly-researched provider pages (Sky, NOW Broadband, BT, Virgin Media, EE, Plusnet, Vodafone, TalkTalk from earlier this session). Rather than re-researching each provider from scratch, cross-referenced this page's ranking table against data/providers.ts's own already-vetted current fields (price, Trustpilot, reviewedDate) and fetched a fresh single-source Ofcom Q1 2026 complaints table (published 23 July 2026, record-low industry average of 6 per 100k) to replace the mixed-quarter data. Corrected several materially wrong claims: TalkTalk was still framed as 'budget only' at GBP19.99 when it is now GBP25 and no longer the cheapest big-name option; Community Fibre was described as 'London-only' when coverage has expanded into Surrey and Sussex; EE's 'best for reliability' halo no longer holds under Q1 2026 data (6 per 100k, tied with Virgin Media, not uniquely best). Added a new section contrasting sister brands Sky (5 per 100k) and NOW Broadband (11 per 100k, different quarter, footnoted) on the identical Openreach network, a genuine support-quality data point. Word count 872 -&gt; 1,333.</t>
+          <t>Eighth target from scripts/analyze_content_priority.py's ranked list: /providers/youfibre was 397 words with no excerpt or contentSections. Rewritten to ~1,575 words with 6 contentSections. The standout finding, verified against a primary Virgin Media O2 press release after a first-pass WebSearch AI summary over-stated it as a done deal: YouFibre's parent company, Substantial Group (Netomnia), is being acquired for GBP2bn by nexfibre (a joint venture of InfraVia, Liberty Global and Telefonica), which then plans to resell the YouFibre/Brsk retail brands to Virgin Media O2 for GBP150m -- announced Feb 2026, referred to the CMA for a Phase 2 investigation on 1 July 2026, and NOT yet completed (expected ~Q3 2026 at the earliest). Also wrote up the real, documented fallout from the March 2026 Brsk-to-YouFibre customer migration (billing errors, login/password-reset failures, reported speed drops, overwhelmed support chat), sourced from ISPreview rather than the vague pre-existing 'Trustpilot sentiment has been mixed' line. Updated the speeds array to the real current tiers (200/1000/2000/8000 Mbps symmetrical, replacing stale 200/900/1800) and contractLengths from [1,12,24] to [1,24] to match the two options confirmed by current pricing research.</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -9723,7 +9767,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-providers-uk), data/guides.ts</t>
+          <t>data/providers.ts (youfibre)</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -9748,7 +9792,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -9758,43 +9802,43 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
+          <t>Ninth target from scripts/analyze_content_priority.py's ranked list. This ranking page's data was badly stale: it cited Q4 2025 Ofcom complaints figures and June-2026 Trustpilot scores that had already been superseded by this site's own freshly-researched provider pages (Sky, NOW Broadband, BT, Virgin Media, EE, Plusnet, Vodafone, TalkTalk from earlier this session). Rather than re-researching each provider from scratch, cross-referenced this page's ranking table against data/providers.ts's own already-vetted current fields (price, Trustpilot, reviewedDate) and fetched a fresh single-source Ofcom Q1 2026 complaints table (published 23 July 2026, record-low industry average of 6 per 100k) to replace the mixed-quarter data. Corrected several materially wrong claims: TalkTalk was still framed as 'budget only' at GBP19.99 when it is now GBP25 and no longer the cheapest big-name option; Community Fibre was described as 'London-only' when coverage has expanded into Surrey and Sussex; EE's 'best for reliability' halo no longer holds under Q1 2026 data (6 per 100k, tied with Virgin Media, not uniquely best). Added a new section contrasting sister brands Sky (5 per 100k) and NOW Broadband (11 per 100k, different quarter, footnoted) on the identical Openreach network, a genuine support-quality data point. Word count 872 -&gt; 1,333.</t>
         </is>
       </c>
       <c r="F43" s="3" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>New annual research page + methodology extension</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-providers-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>research/uk-broadband-customer-satisfaction methodology</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9804,7 +9848,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -9814,43 +9858,43 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Tenth target from scripts/analyze_content_priority.py's ranked list: 770 words, stale pricing table (every one of 8 providers priced against months-old figures already corrected on this site's own provider pages), and a wrong PSTN switch-off date ('by the end of 2027' -- the real, now-locked-in date is 31 January 2027). Rewrote using the same PSTN research gathered for the best-phone-and-broadband-deals refresh earlier this session (5.2m -&gt; 3.2m migration stat, Ofcom's 1-hour power-cut battery backup minimum, the PSTN Charter's telecare protections), added a genuinely missing section -- 'What happens to a home phone during a power cut?' -- since the old version covered whether a line is needed at all but never addressed the actual practical question once Digital Voice is the default. Refreshed all 8 provider prices against data/providers.ts's own current fields, updated Virgin Media coverage 52% (was 53%) and added Ofcom's Spring 2026 Connected Nations split (89% gigabit-capable, 82% full fibre, 93% urban vs 66% rural). Word count 770 -&gt; 1,196; left just under the self-imposed 1,200-word floor rather than pad.</t>
+          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
         <v>41</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-without-phone-line), data/guides.ts</t>
+          <t>New annual research page + methodology extension</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>research/uk-broadband-customer-satisfaction methodology</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -9870,19 +9914,19 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Eleventh target from scripts/analyze_content_priority.py's ranked list: 948 words, structurally sound (evergreen checklist format) but missing a genuinely newsworthy development -- Ofcom closed its One Touch Switch enforcement case on 11 June 2026 after finding more than 2 million customers had already used the process successfully, meaning it is now the industry's permanent standard rather than a monitored pilot, which the old copy still implied. Added this, plus a genuinely missing section on what a house move means for a home phone line given the 31 January 2027 PSTN switch-off (reusing research from the phone-and-broadband and broadband-without-phone-line refreshes earlier this session), Ofcom's Spring 2026 coverage split for the 'check availability' step, and corrected the ETC explanation to reflect Ofcom's actual cap rule (remaining payments, ex-VAT) rather than a flat multiplication. Re-verified the pre-existing GBP183.60/year switching-saving stat against fresh 2026 sources (found independently corroborated) and added the 4.2m/GBP100-240 social tariff stat already used elsewhere on this site. Word count 948 -&gt; 1,446.</t>
+          <t>Tenth target from scripts/analyze_content_priority.py's ranked list: 770 words, stale pricing table (every one of 8 providers priced against months-old figures already corrected on this site's own provider pages), and a wrong PSTN switch-off date ('by the end of 2027' -- the real, now-locked-in date is 31 January 2027). Rewrote using the same PSTN research gathered for the best-phone-and-broadband-deals refresh earlier this session (5.2m -&gt; 3.2m migration stat, Ofcom's 1-hour power-cut battery backup minimum, the PSTN Charter's telecare protections), added a genuinely missing section -- 'What happens to a home phone during a power cut?' -- since the old version covered whether a line is needed at all but never addressed the actual practical question once Digital Voice is the default. Refreshed all 8 provider prices against data/providers.ts's own current fields, updated Virgin Media coverage 52% (was 53%) and added Ofcom's Spring 2026 Connected Nations split (89% gigabit-capable, 82% full fibre, 93% urban vs 66% rural). Word count 770 -&gt; 1,196; left just under the self-imposed 1,200-word floor rather than pad.</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
@@ -9891,7 +9935,7 @@
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-moving-house), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-without-phone-line), data/guides.ts</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
@@ -9926,19 +9970,19 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Twelfth target from scripts/analyze_content_priority.py's ranked list, and the page whose DATE_RE regex bug was found and fixed earlier this session (58.2 -&gt; 53.2) without ever getting a content rewrite. The old copy was generic to the point of naming no real prices at all -- 'Starlink is the most visible option' with zero named plans, figures or alternatives. Rewritten with real, current Starlink UK pricing (Residential 100/200/Max at GBP40/60/80 per month, Roam at GBP55-100, Standard Kit GBP449 commonly discounted to ~GBP299 or free on Max), and a genuinely current news item: Starlink's Global Roam plan stopped taking new customers 15 July 2026 and was withdrawn entirely for existing customers on 17 August 2026, one week before this rewrite. Named 2 real smaller alternatives (SkyDSL, Bigblu Broadband) and clarified that Eutelsat/OneWeb, despite frequent mention alongside Starlink, sells no UK consumer home-broadband plans at all. Word count 437 -&gt; 1,038.</t>
+          <t>Eleventh target from scripts/analyze_content_priority.py's ranked list: 948 words, structurally sound (evergreen checklist format) but missing a genuinely newsworthy development -- Ofcom closed its One Touch Switch enforcement case on 11 June 2026 after finding more than 2 million customers had already used the process successfully, meaning it is now the industry's permanent standard rather than a monitored pilot, which the old copy still implied. Added this, plus a genuinely missing section on what a house move means for a home phone line given the 31 January 2027 PSTN switch-off (reusing research from the phone-and-broadband and broadband-without-phone-line refreshes earlier this session), Ofcom's Spring 2026 coverage split for the 'check availability' step, and corrected the ETC explanation to reflect Ofcom's actual cap rule (remaining payments, ex-VAT) rather than a flat multiplication. Re-verified the pre-existing GBP183.60/year switching-saving stat against fresh 2026 sources (found independently corroborated) and added the 4.2m/GBP100-240 social tariff stat already used elsewhere on this site. Word count 948 -&gt; 1,446.</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -9947,7 +9991,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>data/priority-pages.ts (satellite)</t>
+          <t>app/guides/[slug]/page.tsx (broadband-moving-house), data/guides.ts</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -9972,53 +10016,53 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+          <t>Twelfth target from scripts/analyze_content_priority.py's ranked list, and the page whose DATE_RE regex bug was found and fixed earlier this session (58.2 -&gt; 53.2) without ever getting a content rewrite. The old copy was generic to the point of naming no real prices at all -- 'Starlink is the most visible option' with zero named plans, figures or alternatives. Rewritten with real, current Starlink UK pricing (Residential 100/200/Max at GBP40/60/80 per month, Roam at GBP55-100, Standard Kit GBP449 commonly discounted to ~GBP299 or free on Max), and a genuinely current news item: Starlink's Global Roam plan stopped taking new customers 15 July 2026 and was withdrawn entirely for existing customers on 17 August 2026, one week before this rewrite. Named 2 real smaller alternatives (SkyDSL, Bigblu Broadband) and clarified that Eutelsat/OneWeb, despite frequent mention alongside Starlink, sells no UK consumer home-broadband plans at all. Word count 437 -&gt; 1,038.</t>
         </is>
       </c>
       <c r="F47" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>components/</t>
+          <t>data/priority-pages.ts (satellite)</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10028,53 +10072,53 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Thirteenth target from scripts/analyze_content_priority.py's ranked list: 836 words with stale provider prices (EE GBP26.99, Community Fibre GBP21.99, Hyperoptic GBP22, BT GBP30.99, all already corrected on this site's own provider pages) and a wrong Community Fibre top-tier speed claim (920Mbps symmetrical, against the real current 3,000Mbps top tier confirmed in data/providers.ts). Refreshed all 5 existing provider picks against already-vetted current pricing, and added a genuinely new 6th pick, Zen Internet, for a use case the old page didn't cover at all: hosting a private game server, where Zen's free static IP (already documented on its own provider page) is a real, specific advantage over every other provider on the list. Added a short section on how 24-month contracts and scheduled price rises affect the real two-year cost of a gaming-suitable package. Word count 836 -&gt; 1,184; left just under the self-imposed 1,200-word floor rather than pad.</t>
+          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
         <v>38</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-gaming-uk), data/guides.ts</t>
+          <t>components/</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Functionality pillar</t>
         </is>
       </c>
     </row>
@@ -10094,16 +10138,16 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Fourteenth target from scripts/analyze_content_priority.py's ranked list: 777 words with a materially wrong 'cheapest tariff' claim -- Vodafone Together Social was listed at GBP12.50/mo for 38Mbps and named the cheapest option, but the real current Vodafone Essentials Broadband tariff is GBP20/mo for 73Mbps (verified directly against Vodafone's own tariff page), meaning Virgin Media Essential Broadband and Community Fibre Essential (both genuinely GBP12.50/mo) are actually jointly cheapest. Also corrected Virgin Media's own tariff, which the old page listed at GBP20/mo. Added a genuinely newsworthy find: a thinkbroadband report published in August 2026 (days before this rewrite) tested how easy major providers make it to find their own social tariffs and scored BT, Sky, Virgin Media and Vodafone poorly, with a pointed BT quote, against smaller altnets scoring better. Corrected the eligibility table (Sky accepts UC/PC only, existing customers only, a real restriction the old page omitted) and added KCOM's Hull-only tariff. Refreshed the awareness stat with the newer, more specific thinkbroadband figures (34% aware, 8.6% UC take-up). Word count 777 -&gt; 1,161.</t>
+          <t>Thirteenth target from scripts/analyze_content_priority.py's ranked list: 836 words with stale provider prices (EE GBP26.99, Community Fibre GBP21.99, Hyperoptic GBP22, BT GBP30.99, all already corrected on this site's own provider pages) and a wrong Community Fibre top-tier speed claim (920Mbps symmetrical, against the real current 3,000Mbps top tier confirmed in data/providers.ts). Refreshed all 5 existing provider picks against already-vetted current pricing, and added a genuinely new 6th pick, Zen Internet, for a use case the old page didn't cover at all: hosting a private game server, where Zen's free static IP (already documented on its own provider page) is a real, specific advantage over every other provider on the list. Added a short section on how 24-month contracts and scheduled price rises affect the real two-year cost of a gaming-suitable package. Word count 836 -&gt; 1,184; left just under the self-imposed 1,200-word floor rather than pad.</t>
         </is>
       </c>
       <c r="F49" s="3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G49" s="3" t="n">
         <v>34</v>
@@ -10115,7 +10159,7 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-social-tariffs-uk), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-gaming-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
@@ -10150,19 +10194,19 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Fifteenth target from scripts/analyze_content_priority.py's ranked list: 565 words, no real prices anywhere, and a stale 'EE is consistently rated the most reliable major UK broadband provider' claim that no longer holds under this session's own Q1 2026 Ofcom complaints research. Rewrote with real current prices for Community Fibre, Hyperoptic, Zen Internet and BT, and added a genuinely new section this page never had: when a business-grade line (static IP, faster fault-fix SLA) is actually worth it for a freelancer or remote worker over a residential package, using real Vodafone Business/Zen Business/Sky Business pricing already researched for this site's business broadband guide. Added concrete video-call upload-bandwidth guidance (3-4 Mbps per HD call) rather than vague 'upload matters' framing. Word count 565 -&gt; 986.</t>
+          <t>Fourteenth target from scripts/analyze_content_priority.py's ranked list: 777 words with a materially wrong 'cheapest tariff' claim -- Vodafone Together Social was listed at GBP12.50/mo for 38Mbps and named the cheapest option, but the real current Vodafone Essentials Broadband tariff is GBP20/mo for 73Mbps (verified directly against Vodafone's own tariff page), meaning Virgin Media Essential Broadband and Community Fibre Essential (both genuinely GBP12.50/mo) are actually jointly cheapest. Also corrected Virgin Media's own tariff, which the old page listed at GBP20/mo. Added a genuinely newsworthy find: a thinkbroadband report published in August 2026 (days before this rewrite) tested how easy major providers make it to find their own social tariffs and scored BT, Sky, Virgin Media and Vodafone poorly, with a pointed BT quote, against smaller altnets scoring better. Corrected the eligibility table (Sky accepts UC/PC only, existing customers only, a real restriction the old page omitted) and added KCOM's Hull-only tariff. Refreshed the awareness stat with the newer, more specific thinkbroadband figures (34% aware, 8.6% UC take-up). Word count 777 -&gt; 1,161.</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -10171,7 +10215,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-working-from-home), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-social-tariffs-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -10206,19 +10250,19 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Sixteenth target from scripts/analyze_content_priority.py's ranked list, and the one with the largest factual break of this whole refresh sequence: the page's entire premise named NOW Broadband and TalkTalk as 'the most common names in this price bracket,' but both now start above GBP20/mo (NOW at GBP23, TalkTalk at GBP25, both already corrected on their own provider pages this session). Rebuilt the page around who is actually under GBP20 today by querying data/providers.ts directly for every provider with monthlyPriceFrom &lt; 20: Community Fibre (GBP12.50), Onestream (GBP18.50, 94% Openreach coverage -- the most realistic pick for most addresses), Gigaclear (GBP19.00, rural symmetrical), toob (GBP19.50) and Trooli (GBP19.99). Also caught and excluded Shell Energy (GBP19.99 in the data file) after finding its own provider-page highlights note it closed to new customers and migrated to TalkTalk in 2024 -- an old, non-orderable plan that would have been a real error to list as a current deal. Word count 608 -&gt; 890.</t>
+          <t>Fifteenth target from scripts/analyze_content_priority.py's ranked list: 565 words, no real prices anywhere, and a stale 'EE is consistently rated the most reliable major UK broadband provider' claim that no longer holds under this session's own Q1 2026 Ofcom complaints research. Rewrote with real current prices for Community Fibre, Hyperoptic, Zen Internet and BT, and added a genuinely new section this page never had: when a business-grade line (static IP, faster fault-fix SLA) is actually worth it for a freelancer or remote worker over a residential package, using real Vodafone Business/Zen Business/Sky Business pricing already researched for this site's business broadband guide. Added concrete video-call upload-bandwidth guidance (3-4 Mbps per HD call) rather than vague 'upload matters' framing. Word count 565 -&gt; 986.</t>
         </is>
       </c>
       <c r="F51" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
@@ -10227,7 +10271,7 @@
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-deals-under-20), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-working-from-home), data/guides.ts</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
@@ -10252,7 +10296,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -10262,43 +10306,43 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
+          <t>Sixteenth target from scripts/analyze_content_priority.py's ranked list, and the one with the largest factual break of this whole refresh sequence: the page's entire premise named NOW Broadband and TalkTalk as 'the most common names in this price bracket,' but both now start above GBP20/mo (NOW at GBP23, TalkTalk at GBP25, both already corrected on their own provider pages this session). Rebuilt the page around who is actually under GBP20 today by querying data/providers.ts directly for every provider with monthlyPriceFrom &lt; 20: Community Fibre (GBP12.50), Onestream (GBP18.50, 94% Openreach coverage -- the most realistic pick for most addresses), Gigaclear (GBP19.00, rural symmetrical), toob (GBP19.50) and Trooli (GBP19.99). Also caught and excluded Shell Energy (GBP19.99 in the data file) after finding its own provider-page highlights note it closed to new customers and migrated to TalkTalk in 2024 -- an old, non-orderable plan that would have been a real error to list as a current deal. Word count 608 -&gt; 890.</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
         <v>35</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-under-20), data/guides.ts</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>None, but easier before the guide count grows further</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10308,7 +10352,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -10318,43 +10362,43 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
+          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
       <c r="F53" s="3" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
+          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L53" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -10374,19 +10418,19 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
+          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
@@ -10395,7 +10439,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
+          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -10430,48 +10474,104 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="G55" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L55" s="3" t="inlineStr">
+        <is>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
           <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
         </is>
       </c>
-      <c r="F55" s="3" t="n">
+      <c r="F56" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="G55" s="3" t="n">
+      <c r="G56" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="H55" s="3" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I55" s="3" t="inlineStr">
+      <c r="I56" s="2" t="inlineStr">
         <is>
           <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
         </is>
       </c>
-      <c r="J55" s="3" t="inlineStr">
+      <c r="J56" s="2" t="inlineStr">
         <is>
           <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
-      <c r="K55" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L55" s="3" t="inlineStr">
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
         <is>
           <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L55"/>
+  <autoFilter ref="A1:L56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10512,7 +10612,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>87 total (33 page builds, 54 feature/strategy builds); 73 already marked Done.</t>
+          <t>88 total (33 page builds, 55 feature/strategy builds); 74 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of BT vs Virgin Media comparison page
Twenty-first target from the wider content-priority-analysis list:
526 words of entirely generic, number-free copy, including a wrong
claim that BT has no setup fee (it does, GBP30). Rewrote using this
session's own BT and Virgin Media provider-page data: BT from
GBP23.99/mo (98% coverage) vs Virgin Media from GBP33.00/mo (52%
coverage, 1,130Mbps fastest widely available speed, and a genuinely
better Q1 2026 Ofcom complaints record than BT despite a much lower
Trustpilot score).

Added the practical point this page never covered: switching to
Virgin Media never qualifies for One Touch Switch since it runs on a
separate network from Openreach. Populated the factSnapshot field.

Also bundles the concurrently-running content pipeline's Search
Console connection check script, already present in the working tree
and validated by the build above.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$90</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L89" headerRowCount="1">
-  <autoFilter ref="A1:L89"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L90" headerRowCount="1">
+  <autoFilter ref="A1:L90"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L56" headerRowCount="1">
-  <autoFilter ref="A1:L56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L57" headerRowCount="1">
+  <autoFilter ref="A1:L57"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L89"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-moving-house-guide</t>
+          <t>content-refresh-bt-vs-virgin-media-comparison</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -4195,14 +4195,14 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F79" s="3" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
@@ -4224,7 +4224,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-satellite-broadband-uk-guide</t>
+          <t>content-refresh-broadband-moving-house-guide</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -4239,14 +4239,14 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -4268,38 +4268,38 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>bet-componentise-interactive-layer</t>
+          <t>content-refresh-satellite-broadband-uk-guide</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F81" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr"/>
@@ -4312,38 +4312,38 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-gaming-guide</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
         <v>38</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr"/>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-social-tariffs-guide</t>
+          <t>content-refresh-best-broadband-for-gaming-guide</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -4371,11 +4371,11 @@
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F83" s="3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G83" s="3" t="n">
         <v>34</v>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-working-from-home-guide</t>
+          <t>content-refresh-broadband-social-tariffs-guide</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -4415,14 +4415,14 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-under-20-guide</t>
+          <t>content-refresh-best-broadband-working-from-home-guide</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -4459,14 +4459,14 @@
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F85" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G85" s="3" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
@@ -4488,12 +4488,12 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>content-refresh-broadband-deals-under-20-guide</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -4503,23 +4503,23 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F86" s="2" t="n">
         <v>35</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr"/>
@@ -4532,12 +4532,12 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-bt-vs-sky-comparison</t>
+          <t>bet-decouple-content-from-code</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -4547,23 +4547,23 @@
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="F87" s="3" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G87" s="3" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr"/>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
+          <t>content-refresh-bt-vs-sky-comparison</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -4591,14 +4591,14 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-price-rises-2026-guide</t>
+          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -4635,14 +4635,14 @@
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F89" s="3" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G89" s="3" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
@@ -4658,8 +4658,52 @@
       <c r="K89" s="3" t="inlineStr"/>
       <c r="L89" s="3" t="inlineStr"/>
     </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>content-refresh-broadband-price-rises-2026-guide</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="G90" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr"/>
+      <c r="K90" s="2" t="inlineStr"/>
+      <c r="L90" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L89"/>
+  <autoFilter ref="A1:L90"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7411,7 +7455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9970,19 +10014,19 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Eleventh target from scripts/analyze_content_priority.py's ranked list: 948 words, structurally sound (evergreen checklist format) but missing a genuinely newsworthy development -- Ofcom closed its One Touch Switch enforcement case on 11 June 2026 after finding more than 2 million customers had already used the process successfully, meaning it is now the industry's permanent standard rather than a monitored pilot, which the old copy still implied. Added this, plus a genuinely missing section on what a house move means for a home phone line given the 31 January 2027 PSTN switch-off (reusing research from the phone-and-broadband and broadband-without-phone-line refreshes earlier this session), Ofcom's Spring 2026 coverage split for the 'check availability' step, and corrected the ETC explanation to reflect Ofcom's actual cap rule (remaining payments, ex-VAT) rather than a flat multiplication. Re-verified the pre-existing GBP183.60/year switching-saving stat against fresh 2026 sources (found independently corroborated) and added the 4.2m/GBP100-240 social tariff stat already used elsewhere on this site. Word count 948 -&gt; 1,446.</t>
+          <t>Twenty-first target from the wider top-30 content-priority-analysis list: 526 words of entirely generic, number-free copy ('BT has no setup fee in the current dataset' -- itself wrong, BT's setup fee is GBP30). Rewrote using already-vetted current data from this session's own BT and Virgin Media provider-page work: BT from GBP23.99/mo (24-month, 98% coverage, Trustpilot 4.0/1.5 two-page split) vs Virgin Media from GBP33.00/mo (18-month, 52% coverage, 1,130Mbps fastest widely available speed, Trustpilot 1.4 but a genuinely better Q1 2026 Ofcom complaints record than BT, 6 vs 7 per 100k). Added the genuinely important practical point this page never covered: switching to Virgin Media never qualifies for One Touch Switch since it runs on a separate network from Openreach. Populated the previously-empty factSnapshot field. Word count 526 -&gt; 718.</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -9991,7 +10035,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-moving-house), data/guides.ts</t>
+          <t>data/provider-comparisons.ts (bt-vs-virgin-media)</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -10006,7 +10050,7 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10026,19 +10070,19 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Twelfth target from scripts/analyze_content_priority.py's ranked list, and the page whose DATE_RE regex bug was found and fixed earlier this session (58.2 -&gt; 53.2) without ever getting a content rewrite. The old copy was generic to the point of naming no real prices at all -- 'Starlink is the most visible option' with zero named plans, figures or alternatives. Rewritten with real, current Starlink UK pricing (Residential 100/200/Max at GBP40/60/80 per month, Roam at GBP55-100, Standard Kit GBP449 commonly discounted to ~GBP299 or free on Max), and a genuinely current news item: Starlink's Global Roam plan stopped taking new customers 15 July 2026 and was withdrawn entirely for existing customers on 17 August 2026, one week before this rewrite. Named 2 real smaller alternatives (SkyDSL, Bigblu Broadband) and clarified that Eutelsat/OneWeb, despite frequent mention alongside Starlink, sells no UK consumer home-broadband plans at all. Word count 437 -&gt; 1,038.</t>
+          <t>Eleventh target from scripts/analyze_content_priority.py's ranked list: 948 words, structurally sound (evergreen checklist format) but missing a genuinely newsworthy development -- Ofcom closed its One Touch Switch enforcement case on 11 June 2026 after finding more than 2 million customers had already used the process successfully, meaning it is now the industry's permanent standard rather than a monitored pilot, which the old copy still implied. Added this, plus a genuinely missing section on what a house move means for a home phone line given the 31 January 2027 PSTN switch-off (reusing research from the phone-and-broadband and broadband-without-phone-line refreshes earlier this session), Ofcom's Spring 2026 coverage split for the 'check availability' step, and corrected the ETC explanation to reflect Ofcom's actual cap rule (remaining payments, ex-VAT) rather than a flat multiplication. Re-verified the pre-existing GBP183.60/year switching-saving stat against fresh 2026 sources (found independently corroborated) and added the 4.2m/GBP100-240 social tariff stat already used elsewhere on this site. Word count 948 -&gt; 1,446.</t>
         </is>
       </c>
       <c r="F47" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
@@ -10047,7 +10091,7 @@
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>data/priority-pages.ts (satellite)</t>
+          <t>app/guides/[slug]/page.tsx (broadband-moving-house), data/guides.ts</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
@@ -10072,53 +10116,53 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+          <t>Twelfth target from scripts/analyze_content_priority.py's ranked list, and the page whose DATE_RE regex bug was found and fixed earlier this session (58.2 -&gt; 53.2) without ever getting a content rewrite. The old copy was generic to the point of naming no real prices at all -- 'Starlink is the most visible option' with zero named plans, figures or alternatives. Rewritten with real, current Starlink UK pricing (Residential 100/200/Max at GBP40/60/80 per month, Roam at GBP55-100, Standard Kit GBP449 commonly discounted to ~GBP299 or free on Max), and a genuinely current news item: Starlink's Global Roam plan stopped taking new customers 15 July 2026 and was withdrawn entirely for existing customers on 17 August 2026, one week before this rewrite. Named 2 real smaller alternatives (SkyDSL, Bigblu Broadband) and clarified that Eutelsat/OneWeb, despite frequent mention alongside Starlink, sells no UK consumer home-broadband plans at all. Word count 437 -&gt; 1,038.</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>components/</t>
+          <t>data/priority-pages.ts (satellite)</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10128,53 +10172,53 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Thirteenth target from scripts/analyze_content_priority.py's ranked list: 836 words with stale provider prices (EE GBP26.99, Community Fibre GBP21.99, Hyperoptic GBP22, BT GBP30.99, all already corrected on this site's own provider pages) and a wrong Community Fibre top-tier speed claim (920Mbps symmetrical, against the real current 3,000Mbps top tier confirmed in data/providers.ts). Refreshed all 5 existing provider picks against already-vetted current pricing, and added a genuinely new 6th pick, Zen Internet, for a use case the old page didn't cover at all: hosting a private game server, where Zen's free static IP (already documented on its own provider page) is a real, specific advantage over every other provider on the list. Added a short section on how 24-month contracts and scheduled price rises affect the real two-year cost of a gaming-suitable package. Word count 836 -&gt; 1,184; left just under the self-imposed 1,200-word floor rather than pad.</t>
+          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
         </is>
       </c>
       <c r="F49" s="3" t="n">
         <v>38</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-gaming-uk), data/guides.ts</t>
+          <t>components/</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Functionality pillar</t>
         </is>
       </c>
     </row>
@@ -10194,16 +10238,16 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Fourteenth target from scripts/analyze_content_priority.py's ranked list: 777 words with a materially wrong 'cheapest tariff' claim -- Vodafone Together Social was listed at GBP12.50/mo for 38Mbps and named the cheapest option, but the real current Vodafone Essentials Broadband tariff is GBP20/mo for 73Mbps (verified directly against Vodafone's own tariff page), meaning Virgin Media Essential Broadband and Community Fibre Essential (both genuinely GBP12.50/mo) are actually jointly cheapest. Also corrected Virgin Media's own tariff, which the old page listed at GBP20/mo. Added a genuinely newsworthy find: a thinkbroadband report published in August 2026 (days before this rewrite) tested how easy major providers make it to find their own social tariffs and scored BT, Sky, Virgin Media and Vodafone poorly, with a pointed BT quote, against smaller altnets scoring better. Corrected the eligibility table (Sky accepts UC/PC only, existing customers only, a real restriction the old page omitted) and added KCOM's Hull-only tariff. Refreshed the awareness stat with the newer, more specific thinkbroadband figures (34% aware, 8.6% UC take-up). Word count 777 -&gt; 1,161.</t>
+          <t>Thirteenth target from scripts/analyze_content_priority.py's ranked list: 836 words with stale provider prices (EE GBP26.99, Community Fibre GBP21.99, Hyperoptic GBP22, BT GBP30.99, all already corrected on this site's own provider pages) and a wrong Community Fibre top-tier speed claim (920Mbps symmetrical, against the real current 3,000Mbps top tier confirmed in data/providers.ts). Refreshed all 5 existing provider picks against already-vetted current pricing, and added a genuinely new 6th pick, Zen Internet, for a use case the old page didn't cover at all: hosting a private game server, where Zen's free static IP (already documented on its own provider page) is a real, specific advantage over every other provider on the list. Added a short section on how 24-month contracts and scheduled price rises affect the real two-year cost of a gaming-suitable package. Word count 836 -&gt; 1,184; left just under the self-imposed 1,200-word floor rather than pad.</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G50" s="2" t="n">
         <v>34</v>
@@ -10215,7 +10259,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-social-tariffs-uk), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-gaming-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -10250,19 +10294,19 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Fifteenth target from scripts/analyze_content_priority.py's ranked list: 565 words, no real prices anywhere, and a stale 'EE is consistently rated the most reliable major UK broadband provider' claim that no longer holds under this session's own Q1 2026 Ofcom complaints research. Rewrote with real current prices for Community Fibre, Hyperoptic, Zen Internet and BT, and added a genuinely new section this page never had: when a business-grade line (static IP, faster fault-fix SLA) is actually worth it for a freelancer or remote worker over a residential package, using real Vodafone Business/Zen Business/Sky Business pricing already researched for this site's business broadband guide. Added concrete video-call upload-bandwidth guidance (3-4 Mbps per HD call) rather than vague 'upload matters' framing. Word count 565 -&gt; 986.</t>
+          <t>Fourteenth target from scripts/analyze_content_priority.py's ranked list: 777 words with a materially wrong 'cheapest tariff' claim -- Vodafone Together Social was listed at GBP12.50/mo for 38Mbps and named the cheapest option, but the real current Vodafone Essentials Broadband tariff is GBP20/mo for 73Mbps (verified directly against Vodafone's own tariff page), meaning Virgin Media Essential Broadband and Community Fibre Essential (both genuinely GBP12.50/mo) are actually jointly cheapest. Also corrected Virgin Media's own tariff, which the old page listed at GBP20/mo. Added a genuinely newsworthy find: a thinkbroadband report published in August 2026 (days before this rewrite) tested how easy major providers make it to find their own social tariffs and scored BT, Sky, Virgin Media and Vodafone poorly, with a pointed BT quote, against smaller altnets scoring better. Corrected the eligibility table (Sky accepts UC/PC only, existing customers only, a real restriction the old page omitted) and added KCOM's Hull-only tariff. Refreshed the awareness stat with the newer, more specific thinkbroadband figures (34% aware, 8.6% UC take-up). Word count 777 -&gt; 1,161.</t>
         </is>
       </c>
       <c r="F51" s="3" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
@@ -10271,7 +10315,7 @@
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-working-from-home), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-social-tariffs-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
@@ -10306,19 +10350,19 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Sixteenth target from scripts/analyze_content_priority.py's ranked list, and the one with the largest factual break of this whole refresh sequence: the page's entire premise named NOW Broadband and TalkTalk as 'the most common names in this price bracket,' but both now start above GBP20/mo (NOW at GBP23, TalkTalk at GBP25, both already corrected on their own provider pages this session). Rebuilt the page around who is actually under GBP20 today by querying data/providers.ts directly for every provider with monthlyPriceFrom &lt; 20: Community Fibre (GBP12.50), Onestream (GBP18.50, 94% Openreach coverage -- the most realistic pick for most addresses), Gigaclear (GBP19.00, rural symmetrical), toob (GBP19.50) and Trooli (GBP19.99). Also caught and excluded Shell Energy (GBP19.99 in the data file) after finding its own provider-page highlights note it closed to new customers and migrated to TalkTalk in 2024 -- an old, non-orderable plan that would have been a real error to list as a current deal. Word count 608 -&gt; 890.</t>
+          <t>Fifteenth target from scripts/analyze_content_priority.py's ranked list: 565 words, no real prices anywhere, and a stale 'EE is consistently rated the most reliable major UK broadband provider' claim that no longer holds under this session's own Q1 2026 Ofcom complaints research. Rewrote with real current prices for Community Fibre, Hyperoptic, Zen Internet and BT, and added a genuinely new section this page never had: when a business-grade line (static IP, faster fault-fix SLA) is actually worth it for a freelancer or remote worker over a residential package, using real Vodafone Business/Zen Business/Sky Business pricing already researched for this site's business broadband guide. Added concrete video-call upload-bandwidth guidance (3-4 Mbps per HD call) rather than vague 'upload matters' framing. Word count 565 -&gt; 986.</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
@@ -10327,7 +10371,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-deals-under-20), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-working-from-home), data/guides.ts</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -10352,7 +10396,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -10362,43 +10406,43 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
+          <t>Sixteenth target from scripts/analyze_content_priority.py's ranked list, and the one with the largest factual break of this whole refresh sequence: the page's entire premise named NOW Broadband and TalkTalk as 'the most common names in this price bracket,' but both now start above GBP20/mo (NOW at GBP23, TalkTalk at GBP25, both already corrected on their own provider pages this session). Rebuilt the page around who is actually under GBP20 today by querying data/providers.ts directly for every provider with monthlyPriceFrom &lt; 20: Community Fibre (GBP12.50), Onestream (GBP18.50, 94% Openreach coverage -- the most realistic pick for most addresses), Gigaclear (GBP19.00, rural symmetrical), toob (GBP19.50) and Trooli (GBP19.99). Also caught and excluded Shell Energy (GBP19.99 in the data file) after finding its own provider-page highlights note it closed to new customers and migrated to TalkTalk in 2024 -- an old, non-orderable plan that would have been a real error to list as a current deal. Word count 608 -&gt; 890.</t>
         </is>
       </c>
       <c r="F53" s="3" t="n">
         <v>35</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-under-20), data/guides.ts</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>None, but easier before the guide count grows further</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L53" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10408,7 +10452,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -10418,43 +10462,43 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
+          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
+          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -10474,19 +10518,19 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
+          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
         </is>
       </c>
       <c r="F55" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
@@ -10495,7 +10539,7 @@
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
+          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
@@ -10530,48 +10574,104 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
           <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
         </is>
       </c>
-      <c r="F56" s="2" t="n">
+      <c r="F57" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="G56" s="2" t="n">
+      <c r="G57" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="H57" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr">
+      <c r="I57" s="3" t="inlineStr">
         <is>
           <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
         </is>
       </c>
-      <c r="J56" s="2" t="inlineStr">
+      <c r="J57" s="3" t="inlineStr">
         <is>
           <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
-      <c r="K56" s="2" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L56" s="2" t="inlineStr">
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="inlineStr">
         <is>
           <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L56"/>
+  <autoFilter ref="A1:L57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10612,7 +10712,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>88 total (33 page builds, 55 feature/strategy builds); 74 already marked Done.</t>
+          <t>89 total (33 page builds, 56 feature/strategy builds); 75 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Full Fibre Broadband Explained guide
Twenty-second target from the wider content-priority-analysis list:
538 words with a stale "speeds of up to 1,000 Mbps (1 Gbps)" ceiling
claim and a vague "Openreach targeting 25 million premises by 2026"
coverage stat with no real current figure.

Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82%
full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural) and
updated the speed ceiling to reflect real current top tiers already
verified on this site's own provider pages -- Community Fibre up to
3,000 Mbps and YouFibre up to 8,000 Mbps, both symmetrical. Added a
section connecting full fibre to the 31 January 2027 PSTN switch-off.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L90" headerRowCount="1">
-  <autoFilter ref="A1:L90"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L91" headerRowCount="1">
+  <autoFilter ref="A1:L91"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L57" headerRowCount="1">
-  <autoFilter ref="A1:L57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L58" headerRowCount="1">
+  <autoFilter ref="A1:L58"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L90"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4702,8 +4702,52 @@
       <c r="K90" s="2" t="inlineStr"/>
       <c r="L90" s="2" t="inlineStr"/>
     </row>
+    <row r="91">
+      <c r="A91" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>content-refresh-full-fibre-broadband-explained-guide</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="G91" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="H91" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J91" s="3" t="inlineStr"/>
+      <c r="K91" s="3" t="inlineStr"/>
+      <c r="L91" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L90"/>
+  <autoFilter ref="A1:L91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7455,7 +7499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10670,8 +10714,64 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L57"/>
+  <autoFilter ref="A1:L58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10712,7 +10812,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>89 total (33 page builds, 56 feature/strategy builds); 75 already marked Done.</t>
+          <t>90 total (33 page builds, 57 feature/strategy builds); 76 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Best Broadband for Students guide
Twenty-third target from the wider content-priority-analysis list,
and the third page this session found repeating the exact same stale
claim about NOW Broadband's "shorter-term positioning" (also caught
and fixed on best-rolling-monthly-broadband-deals and
broadband-deals-under-20 earlier this session). Also corrected
"TalkTalk can work well for low-cost shared houses," no longer true
now that TalkTalk starts at GBP25/mo.

Replaced both with real current options: YouFibre's genuine rolling
monthly contract for uncertain tenancies, and Onestream (GBP18.50/mo,
94% Openreach coverage) as the realistic default for most student
addresses, alongside Hyperoptic/Community Fibre's 12-month option.

Also bundles the concurrently-running content pipeline's weekly SEO
intelligence report generator, already present in the working tree
and validated by the build above.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L91" headerRowCount="1">
-  <autoFilter ref="A1:L91"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L92" headerRowCount="1">
+  <autoFilter ref="A1:L92"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L58" headerRowCount="1">
-  <autoFilter ref="A1:L58"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L59" headerRowCount="1">
+  <autoFilter ref="A1:L59"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4746,8 +4746,52 @@
       <c r="K91" s="3" t="inlineStr"/>
       <c r="L91" s="3" t="inlineStr"/>
     </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>content-refresh-best-broadband-for-students-guide</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G92" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr"/>
+      <c r="K92" s="2" t="inlineStr"/>
+      <c r="L92" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L91"/>
+  <autoFilter ref="A1:L92"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7499,7 +7543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10770,8 +10814,64 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="3" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G59" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L58"/>
+  <autoFilter ref="A1:L59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10812,7 +10912,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>90 total (33 page builds, 57 feature/strategy builds); 76 already marked Done.</t>
+          <t>91 total (33 page builds, 58 feature/strategy builds); 77 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: update Virgin Media provider page with real Q1 2026 Ofcom figure
Twenty-fourth target, found via the same spot-check pattern that
caught EE's stale figure: /providers/virgin-media was still citing
its Q4 2025 Ofcom complaints figure (7 per 100k) with vague framing
about the more recent report.

Replaced with the exact Q1 2026 figure from the same source used for
EE and the price-rises guide: Virgin Media recorded 6 per 100,000,
exactly the industry average, a further improvement on its already-
decent Q4 2025 position.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -13,14 +13,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Page Builds" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature &amp; Strategy Builds" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly SEO Actions" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -176,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L92" headerRowCount="1">
-  <autoFilter ref="A1:L92"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L93" headerRowCount="1">
+  <autoFilter ref="A1:L93"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -241,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L59" headerRowCount="1">
-  <autoFilter ref="A1:L59"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L60" headerRowCount="1">
+  <autoFilter ref="A1:L60"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -267,6 +269,31 @@
   <tableColumns count="2">
     <tableColumn id="1" name="Aspect"/>
     <tableColumn id="2" name="Detail"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="WeeklySEOActionsTable" displayName="WeeklySEOActionsTable" ref="A1:P31" headerRowCount="1">
+  <autoFilter ref="A1:P31"/>
+  <tableColumns count="16">
+    <tableColumn id="1" name="Rank"/>
+    <tableColumn id="2" name="Page"/>
+    <tableColumn id="3" name="Opportunity"/>
+    <tableColumn id="4" name="Score"/>
+    <tableColumn id="5" name="Clicks"/>
+    <tableColumn id="6" name="Impressions"/>
+    <tableColumn id="7" name="CTR"/>
+    <tableColumn id="8" name="Position"/>
+    <tableColumn id="9" name="Impression Change"/>
+    <tableColumn id="10" name="GA4 Sessions"/>
+    <tableColumn id="11" name="Engagement Rate"/>
+    <tableColumn id="12" name="Affiliate Clicks"/>
+    <tableColumn id="13" name="AI Referral Visits"/>
+    <tableColumn id="14" name="Top Queries"/>
+    <tableColumn id="15" name="Recommended Action"/>
+    <tableColumn id="16" name="Generated"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -667,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3916,29 +3943,29 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>audit-broken-links-redirects</t>
+          <t>content-refresh-virgin-media-provider-page</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Crawlability</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Add routine broken-link and redirect reporting</t>
+          <t>Update: Virgin Media provider page Ofcom complaints figure (24th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F73" s="3" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G73" s="3" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
@@ -3947,7 +3974,7 @@
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr"/>
@@ -3960,38 +3987,38 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-now-broadband-provider-page</t>
+          <t>audit-broken-links-redirects</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Crawlability</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
+          <t>Add routine broken-link and redirect reporting</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
         <v>44</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr"/>
@@ -4004,7 +4031,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-youfibre-provider-page</t>
+          <t>content-refresh-now-broadband-provider-page</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -4019,14 +4046,14 @@
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
+          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F75" s="3" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G75" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
@@ -4048,7 +4075,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-providers-uk-guide</t>
+          <t>content-refresh-youfibre-provider-page</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -4063,14 +4090,14 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
+          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
@@ -4092,12 +4119,12 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>bet-annual-research-report</t>
+          <t>content-refresh-best-broadband-providers-uk-guide</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -4107,23 +4134,23 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F77" s="3" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr"/>
@@ -4136,12 +4163,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-without-phone-line-guide</t>
+          <t>bet-annual-research-report</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -4151,23 +4178,23 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
         <v>41</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr"/>
@@ -4180,7 +4207,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-bt-vs-virgin-media-comparison</t>
+          <t>content-refresh-broadband-without-phone-line-guide</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -4195,14 +4222,14 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F79" s="3" t="n">
         <v>41</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
@@ -4224,7 +4251,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-moving-house-guide</t>
+          <t>content-refresh-bt-vs-virgin-media-comparison</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -4239,14 +4266,14 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -4268,7 +4295,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-satellite-broadband-uk-guide</t>
+          <t>content-refresh-broadband-moving-house-guide</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -4283,14 +4310,14 @@
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F81" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
@@ -4312,38 +4339,38 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>bet-componentise-interactive-layer</t>
+          <t>content-refresh-satellite-broadband-uk-guide</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr"/>
@@ -4356,38 +4383,38 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-gaming-guide</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F83" s="3" t="n">
         <v>38</v>
       </c>
       <c r="G83" s="3" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr"/>
@@ -4400,7 +4427,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-social-tariffs-guide</t>
+          <t>content-refresh-best-broadband-for-gaming-guide</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -4415,11 +4442,11 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G84" s="2" t="n">
         <v>34</v>
@@ -4444,7 +4471,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-working-from-home-guide</t>
+          <t>content-refresh-broadband-social-tariffs-guide</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -4459,14 +4486,14 @@
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F85" s="3" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G85" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
@@ -4488,7 +4515,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-under-20-guide</t>
+          <t>content-refresh-best-broadband-working-from-home-guide</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -4503,14 +4530,14 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
@@ -4532,12 +4559,12 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>content-refresh-broadband-deals-under-20-guide</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -4547,23 +4574,23 @@
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F87" s="3" t="n">
         <v>35</v>
       </c>
       <c r="G87" s="3" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr"/>
@@ -4576,12 +4603,12 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-bt-vs-sky-comparison</t>
+          <t>bet-decouple-content-from-code</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -4591,23 +4618,23 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr"/>
@@ -4620,7 +4647,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
+          <t>content-refresh-bt-vs-sky-comparison</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -4635,14 +4662,14 @@
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F89" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G89" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
@@ -4664,7 +4691,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-price-rises-2026-guide</t>
+          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -4679,14 +4706,14 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
@@ -4708,7 +4735,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-full-fibre-broadband-explained-guide</t>
+          <t>content-refresh-broadband-price-rises-2026-guide</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -4723,14 +4750,14 @@
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="F91" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G91" s="3" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
@@ -4752,7 +4779,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-students-guide</t>
+          <t>content-refresh-full-fibre-broadband-explained-guide</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -4767,14 +4794,14 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
@@ -4790,8 +4817,52 @@
       <c r="K92" s="2" t="inlineStr"/>
       <c r="L92" s="2" t="inlineStr"/>
     </row>
+    <row r="93">
+      <c r="A93" s="3" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>content-refresh-best-broadband-for-students-guide</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G93" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="H93" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J93" s="3" t="inlineStr"/>
+      <c r="K93" s="3" t="inlineStr"/>
+      <c r="L93" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L92"/>
+  <autoFilter ref="A1:L93"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7543,7 +7614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9756,29 +9827,29 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Crawlability</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Add routine broken-link and redirect reporting</t>
+          <t>Update: Virgin Media provider page Ofcom complaints figure (24th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Monitor broken inbound and internal URLs and maintain relevant one-hop redirects.</t>
+          <t>Twenty-fourth target, found via the same spot-check pattern that caught EE's stale figure: /providers/virgin-media (63,112/mo volume, already well-built at 1,798 words) was still citing its Q4 2025 Ofcom complaints figure (7 per 100k) with vague framing ('has not appeared among the top complained-about providers in Q1 2026 either'). Replaced with the exact Q1 2026 figure from the same broadbandswitch table used for EE and the price-rises guide: Virgin Media recorded 6 per 100,000, exactly the industry average, a further improvement on its already-decent Q4 2025 position. Added a dedicated source citation and updated reviewedDate.</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
@@ -9787,22 +9858,22 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Sitewide crawl and redirect report</t>
+          <t>data/providers.ts (virgin-media)</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>BroadbandPicker SEO &amp; Content Plan — Live: Technical SEO</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9812,53 +9883,53 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Crawlability</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
+          <t>Add routine broken-link and redirect reporting</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Seventh target from scripts/analyze_content_priority.py's ranked list: /providers/now-broadband was 386 words with no excerpt or contentSections, and its top-level fields were stale on two counts that research corrected -- contractLengths was still [12] (NOW dropped its flexible 12-month contracts; every current package is now a standard 24-month term, per thinkbroadband's dedicated news item on the change) and monthlyPriceFrom was a stale GBP17.99 against a real current cheapest tier of GBP23 (Full Fibre 100). Rewritten to ~1,450 words with 5 contentSections. The genuinely distinctive finding here, different from every other Trustpilot-vs-Ofcom section written this session: NOW is a real exception to the usual pattern, scoring poorly on BOTH Trustpilot (1.2/5, corrected from a stale 3.2) AND Ofcom's Q4 2025 complaints data (11 per 100k vs the 8 industry average), noticeably worse than sister brand Sky on the same underlying Openreach network -- written up as a genuine data point about support quality diverging from infrastructure quality within the same corporate group, not just review-platform noise. Also corrected trustpilotScore 3.2 -&gt; 1.2.</t>
+          <t>Monitor broken inbound and internal URLs and maintain relevant one-hop redirects.</t>
         </is>
       </c>
       <c r="F41" s="3" t="n">
         <v>44</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>data/providers.ts (now-broadband)</t>
+          <t>Sitewide crawl and redirect report</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>BroadbandPicker SEO &amp; Content Plan — Live: Technical SEO</t>
         </is>
       </c>
     </row>
@@ -9878,19 +9949,19 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
+          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Eighth target from scripts/analyze_content_priority.py's ranked list: /providers/youfibre was 397 words with no excerpt or contentSections. Rewritten to ~1,575 words with 6 contentSections. The standout finding, verified against a primary Virgin Media O2 press release after a first-pass WebSearch AI summary over-stated it as a done deal: YouFibre's parent company, Substantial Group (Netomnia), is being acquired for GBP2bn by nexfibre (a joint venture of InfraVia, Liberty Global and Telefonica), which then plans to resell the YouFibre/Brsk retail brands to Virgin Media O2 for GBP150m -- announced Feb 2026, referred to the CMA for a Phase 2 investigation on 1 July 2026, and NOT yet completed (expected ~Q3 2026 at the earliest). Also wrote up the real, documented fallout from the March 2026 Brsk-to-YouFibre customer migration (billing errors, login/password-reset failures, reported speed drops, overwhelmed support chat), sourced from ISPreview rather than the vague pre-existing 'Trustpilot sentiment has been mixed' line. Updated the speeds array to the real current tiers (200/1000/2000/8000 Mbps symmetrical, replacing stale 200/900/1800) and contractLengths from [1,12,24] to [1,24] to match the two options confirmed by current pricing research.</t>
+          <t>Seventh target from scripts/analyze_content_priority.py's ranked list: /providers/now-broadband was 386 words with no excerpt or contentSections, and its top-level fields were stale on two counts that research corrected -- contractLengths was still [12] (NOW dropped its flexible 12-month contracts; every current package is now a standard 24-month term, per thinkbroadband's dedicated news item on the change) and monthlyPriceFrom was a stale GBP17.99 against a real current cheapest tier of GBP23 (Full Fibre 100). Rewritten to ~1,450 words with 5 contentSections. The genuinely distinctive finding here, different from every other Trustpilot-vs-Ofcom section written this session: NOW is a real exception to the usual pattern, scoring poorly on BOTH Trustpilot (1.2/5, corrected from a stale 3.2) AND Ofcom's Q4 2025 complaints data (11 per 100k vs the 8 industry average), noticeably worse than sister brand Sky on the same underlying Openreach network -- written up as a genuine data point about support quality diverging from infrastructure quality within the same corporate group, not just review-platform noise. Also corrected trustpilotScore 3.2 -&gt; 1.2.</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -9899,7 +9970,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>data/providers.ts (youfibre)</t>
+          <t>data/providers.ts (now-broadband)</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -9934,19 +10005,19 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
+          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Ninth target from scripts/analyze_content_priority.py's ranked list. This ranking page's data was badly stale: it cited Q4 2025 Ofcom complaints figures and June-2026 Trustpilot scores that had already been superseded by this site's own freshly-researched provider pages (Sky, NOW Broadband, BT, Virgin Media, EE, Plusnet, Vodafone, TalkTalk from earlier this session). Rather than re-researching each provider from scratch, cross-referenced this page's ranking table against data/providers.ts's own already-vetted current fields (price, Trustpilot, reviewedDate) and fetched a fresh single-source Ofcom Q1 2026 complaints table (published 23 July 2026, record-low industry average of 6 per 100k) to replace the mixed-quarter data. Corrected several materially wrong claims: TalkTalk was still framed as 'budget only' at GBP19.99 when it is now GBP25 and no longer the cheapest big-name option; Community Fibre was described as 'London-only' when coverage has expanded into Surrey and Sussex; EE's 'best for reliability' halo no longer holds under Q1 2026 data (6 per 100k, tied with Virgin Media, not uniquely best). Added a new section contrasting sister brands Sky (5 per 100k) and NOW Broadband (11 per 100k, different quarter, footnoted) on the identical Openreach network, a genuine support-quality data point. Word count 872 -&gt; 1,333.</t>
+          <t>Eighth target from scripts/analyze_content_priority.py's ranked list: /providers/youfibre was 397 words with no excerpt or contentSections. Rewritten to ~1,575 words with 6 contentSections. The standout finding, verified against a primary Virgin Media O2 press release after a first-pass WebSearch AI summary over-stated it as a done deal: YouFibre's parent company, Substantial Group (Netomnia), is being acquired for GBP2bn by nexfibre (a joint venture of InfraVia, Liberty Global and Telefonica), which then plans to resell the YouFibre/Brsk retail brands to Virgin Media O2 for GBP150m -- announced Feb 2026, referred to the CMA for a Phase 2 investigation on 1 July 2026, and NOT yet completed (expected ~Q3 2026 at the earliest). Also wrote up the real, documented fallout from the March 2026 Brsk-to-YouFibre customer migration (billing errors, login/password-reset failures, reported speed drops, overwhelmed support chat), sourced from ISPreview rather than the vague pre-existing 'Trustpilot sentiment has been mixed' line. Updated the speeds array to the real current tiers (200/1000/2000/8000 Mbps symmetrical, replacing stale 200/900/1800) and contractLengths from [1,12,24] to [1,24] to match the two options confirmed by current pricing research.</t>
         </is>
       </c>
       <c r="F43" s="3" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
@@ -9955,7 +10026,7 @@
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-providers-uk), data/guides.ts</t>
+          <t>data/providers.ts (youfibre)</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
@@ -9980,7 +10051,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -9990,43 +10061,43 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
+          <t>Ninth target from scripts/analyze_content_priority.py's ranked list. This ranking page's data was badly stale: it cited Q4 2025 Ofcom complaints figures and June-2026 Trustpilot scores that had already been superseded by this site's own freshly-researched provider pages (Sky, NOW Broadband, BT, Virgin Media, EE, Plusnet, Vodafone, TalkTalk from earlier this session). Rather than re-researching each provider from scratch, cross-referenced this page's ranking table against data/providers.ts's own already-vetted current fields (price, Trustpilot, reviewedDate) and fetched a fresh single-source Ofcom Q1 2026 complaints table (published 23 July 2026, record-low industry average of 6 per 100k) to replace the mixed-quarter data. Corrected several materially wrong claims: TalkTalk was still framed as 'budget only' at GBP19.99 when it is now GBP25 and no longer the cheapest big-name option; Community Fibre was described as 'London-only' when coverage has expanded into Surrey and Sussex; EE's 'best for reliability' halo no longer holds under Q1 2026 data (6 per 100k, tied with Virgin Media, not uniquely best). Added a new section contrasting sister brands Sky (5 per 100k) and NOW Broadband (11 per 100k, different quarter, footnoted) on the identical Openreach network, a genuine support-quality data point. Word count 872 -&gt; 1,333.</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>New annual research page + methodology extension</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-providers-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>research/uk-broadband-customer-satisfaction methodology</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10036,7 +10107,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -10046,43 +10117,43 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Tenth target from scripts/analyze_content_priority.py's ranked list: 770 words, stale pricing table (every one of 8 providers priced against months-old figures already corrected on this site's own provider pages), and a wrong PSTN switch-off date ('by the end of 2027' -- the real, now-locked-in date is 31 January 2027). Rewrote using the same PSTN research gathered for the best-phone-and-broadband-deals refresh earlier this session (5.2m -&gt; 3.2m migration stat, Ofcom's 1-hour power-cut battery backup minimum, the PSTN Charter's telecare protections), added a genuinely missing section -- 'What happens to a home phone during a power cut?' -- since the old version covered whether a line is needed at all but never addressed the actual practical question once Digital Voice is the default. Refreshed all 8 provider prices against data/providers.ts's own current fields, updated Virgin Media coverage 52% (was 53%) and added Ofcom's Spring 2026 Connected Nations split (89% gigabit-capable, 82% full fibre, 93% urban vs 66% rural). Word count 770 -&gt; 1,196; left just under the self-imposed 1,200-word floor rather than pad.</t>
+          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
         <v>41</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-without-phone-line), data/guides.ts</t>
+          <t>New annual research page + methodology extension</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>research/uk-broadband-customer-satisfaction methodology</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -10102,19 +10173,19 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Twenty-first target from the wider top-30 content-priority-analysis list: 526 words of entirely generic, number-free copy ('BT has no setup fee in the current dataset' -- itself wrong, BT's setup fee is GBP30). Rewrote using already-vetted current data from this session's own BT and Virgin Media provider-page work: BT from GBP23.99/mo (24-month, 98% coverage, Trustpilot 4.0/1.5 two-page split) vs Virgin Media from GBP33.00/mo (18-month, 52% coverage, 1,130Mbps fastest widely available speed, Trustpilot 1.4 but a genuinely better Q1 2026 Ofcom complaints record than BT, 6 vs 7 per 100k). Added the genuinely important practical point this page never covered: switching to Virgin Media never qualifies for One Touch Switch since it runs on a separate network from Openreach. Populated the previously-empty factSnapshot field. Word count 526 -&gt; 718.</t>
+          <t>Tenth target from scripts/analyze_content_priority.py's ranked list: 770 words, stale pricing table (every one of 8 providers priced against months-old figures already corrected on this site's own provider pages), and a wrong PSTN switch-off date ('by the end of 2027' -- the real, now-locked-in date is 31 January 2027). Rewrote using the same PSTN research gathered for the best-phone-and-broadband-deals refresh earlier this session (5.2m -&gt; 3.2m migration stat, Ofcom's 1-hour power-cut battery backup minimum, the PSTN Charter's telecare protections), added a genuinely missing section -- 'What happens to a home phone during a power cut?' -- since the old version covered whether a line is needed at all but never addressed the actual practical question once Digital Voice is the default. Refreshed all 8 provider prices against data/providers.ts's own current fields, updated Virgin Media coverage 52% (was 53%) and added Ofcom's Spring 2026 Connected Nations split (89% gigabit-capable, 82% full fibre, 93% urban vs 66% rural). Word count 770 -&gt; 1,196; left just under the self-imposed 1,200-word floor rather than pad.</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
         <v>41</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -10123,7 +10194,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>data/provider-comparisons.ts (bt-vs-virgin-media)</t>
+          <t>app/guides/[slug]/page.tsx (broadband-without-phone-line), data/guides.ts</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -10138,7 +10209,7 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10158,19 +10229,19 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Eleventh target from scripts/analyze_content_priority.py's ranked list: 948 words, structurally sound (evergreen checklist format) but missing a genuinely newsworthy development -- Ofcom closed its One Touch Switch enforcement case on 11 June 2026 after finding more than 2 million customers had already used the process successfully, meaning it is now the industry's permanent standard rather than a monitored pilot, which the old copy still implied. Added this, plus a genuinely missing section on what a house move means for a home phone line given the 31 January 2027 PSTN switch-off (reusing research from the phone-and-broadband and broadband-without-phone-line refreshes earlier this session), Ofcom's Spring 2026 coverage split for the 'check availability' step, and corrected the ETC explanation to reflect Ofcom's actual cap rule (remaining payments, ex-VAT) rather than a flat multiplication. Re-verified the pre-existing GBP183.60/year switching-saving stat against fresh 2026 sources (found independently corroborated) and added the 4.2m/GBP100-240 social tariff stat already used elsewhere on this site. Word count 948 -&gt; 1,446.</t>
+          <t>Twenty-first target from the wider top-30 content-priority-analysis list: 526 words of entirely generic, number-free copy ('BT has no setup fee in the current dataset' -- itself wrong, BT's setup fee is GBP30). Rewrote using already-vetted current data from this session's own BT and Virgin Media provider-page work: BT from GBP23.99/mo (24-month, 98% coverage, Trustpilot 4.0/1.5 two-page split) vs Virgin Media from GBP33.00/mo (18-month, 52% coverage, 1,130Mbps fastest widely available speed, Trustpilot 1.4 but a genuinely better Q1 2026 Ofcom complaints record than BT, 6 vs 7 per 100k). Added the genuinely important practical point this page never covered: switching to Virgin Media never qualifies for One Touch Switch since it runs on a separate network from Openreach. Populated the previously-empty factSnapshot field. Word count 526 -&gt; 718.</t>
         </is>
       </c>
       <c r="F47" s="3" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
@@ -10179,7 +10250,7 @@
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-moving-house), data/guides.ts</t>
+          <t>data/provider-comparisons.ts (bt-vs-virgin-media)</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
@@ -10194,7 +10265,7 @@
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10214,19 +10285,19 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Twelfth target from scripts/analyze_content_priority.py's ranked list, and the page whose DATE_RE regex bug was found and fixed earlier this session (58.2 -&gt; 53.2) without ever getting a content rewrite. The old copy was generic to the point of naming no real prices at all -- 'Starlink is the most visible option' with zero named plans, figures or alternatives. Rewritten with real, current Starlink UK pricing (Residential 100/200/Max at GBP40/60/80 per month, Roam at GBP55-100, Standard Kit GBP449 commonly discounted to ~GBP299 or free on Max), and a genuinely current news item: Starlink's Global Roam plan stopped taking new customers 15 July 2026 and was withdrawn entirely for existing customers on 17 August 2026, one week before this rewrite. Named 2 real smaller alternatives (SkyDSL, Bigblu Broadband) and clarified that Eutelsat/OneWeb, despite frequent mention alongside Starlink, sells no UK consumer home-broadband plans at all. Word count 437 -&gt; 1,038.</t>
+          <t>Eleventh target from scripts/analyze_content_priority.py's ranked list: 948 words, structurally sound (evergreen checklist format) but missing a genuinely newsworthy development -- Ofcom closed its One Touch Switch enforcement case on 11 June 2026 after finding more than 2 million customers had already used the process successfully, meaning it is now the industry's permanent standard rather than a monitored pilot, which the old copy still implied. Added this, plus a genuinely missing section on what a house move means for a home phone line given the 31 January 2027 PSTN switch-off (reusing research from the phone-and-broadband and broadband-without-phone-line refreshes earlier this session), Ofcom's Spring 2026 coverage split for the 'check availability' step, and corrected the ETC explanation to reflect Ofcom's actual cap rule (remaining payments, ex-VAT) rather than a flat multiplication. Re-verified the pre-existing GBP183.60/year switching-saving stat against fresh 2026 sources (found independently corroborated) and added the 4.2m/GBP100-240 social tariff stat already used elsewhere on this site. Word count 948 -&gt; 1,446.</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -10235,7 +10306,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>data/priority-pages.ts (satellite)</t>
+          <t>app/guides/[slug]/page.tsx (broadband-moving-house), data/guides.ts</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -10260,53 +10331,53 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+          <t>Twelfth target from scripts/analyze_content_priority.py's ranked list, and the page whose DATE_RE regex bug was found and fixed earlier this session (58.2 -&gt; 53.2) without ever getting a content rewrite. The old copy was generic to the point of naming no real prices at all -- 'Starlink is the most visible option' with zero named plans, figures or alternatives. Rewritten with real, current Starlink UK pricing (Residential 100/200/Max at GBP40/60/80 per month, Roam at GBP55-100, Standard Kit GBP449 commonly discounted to ~GBP299 or free on Max), and a genuinely current news item: Starlink's Global Roam plan stopped taking new customers 15 July 2026 and was withdrawn entirely for existing customers on 17 August 2026, one week before this rewrite. Named 2 real smaller alternatives (SkyDSL, Bigblu Broadband) and clarified that Eutelsat/OneWeb, despite frequent mention alongside Starlink, sells no UK consumer home-broadband plans at all. Word count 437 -&gt; 1,038.</t>
         </is>
       </c>
       <c r="F49" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>components/</t>
+          <t>data/priority-pages.ts (satellite)</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10316,53 +10387,53 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Thirteenth target from scripts/analyze_content_priority.py's ranked list: 836 words with stale provider prices (EE GBP26.99, Community Fibre GBP21.99, Hyperoptic GBP22, BT GBP30.99, all already corrected on this site's own provider pages) and a wrong Community Fibre top-tier speed claim (920Mbps symmetrical, against the real current 3,000Mbps top tier confirmed in data/providers.ts). Refreshed all 5 existing provider picks against already-vetted current pricing, and added a genuinely new 6th pick, Zen Internet, for a use case the old page didn't cover at all: hosting a private game server, where Zen's free static IP (already documented on its own provider page) is a real, specific advantage over every other provider on the list. Added a short section on how 24-month contracts and scheduled price rises affect the real two-year cost of a gaming-suitable package. Word count 836 -&gt; 1,184; left just under the self-imposed 1,200-word floor rather than pad.</t>
+          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
         <v>38</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-gaming-uk), data/guides.ts</t>
+          <t>components/</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Functionality pillar</t>
         </is>
       </c>
     </row>
@@ -10382,16 +10453,16 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Fourteenth target from scripts/analyze_content_priority.py's ranked list: 777 words with a materially wrong 'cheapest tariff' claim -- Vodafone Together Social was listed at GBP12.50/mo for 38Mbps and named the cheapest option, but the real current Vodafone Essentials Broadband tariff is GBP20/mo for 73Mbps (verified directly against Vodafone's own tariff page), meaning Virgin Media Essential Broadband and Community Fibre Essential (both genuinely GBP12.50/mo) are actually jointly cheapest. Also corrected Virgin Media's own tariff, which the old page listed at GBP20/mo. Added a genuinely newsworthy find: a thinkbroadband report published in August 2026 (days before this rewrite) tested how easy major providers make it to find their own social tariffs and scored BT, Sky, Virgin Media and Vodafone poorly, with a pointed BT quote, against smaller altnets scoring better. Corrected the eligibility table (Sky accepts UC/PC only, existing customers only, a real restriction the old page omitted) and added KCOM's Hull-only tariff. Refreshed the awareness stat with the newer, more specific thinkbroadband figures (34% aware, 8.6% UC take-up). Word count 777 -&gt; 1,161.</t>
+          <t>Thirteenth target from scripts/analyze_content_priority.py's ranked list: 836 words with stale provider prices (EE GBP26.99, Community Fibre GBP21.99, Hyperoptic GBP22, BT GBP30.99, all already corrected on this site's own provider pages) and a wrong Community Fibre top-tier speed claim (920Mbps symmetrical, against the real current 3,000Mbps top tier confirmed in data/providers.ts). Refreshed all 5 existing provider picks against already-vetted current pricing, and added a genuinely new 6th pick, Zen Internet, for a use case the old page didn't cover at all: hosting a private game server, where Zen's free static IP (already documented on its own provider page) is a real, specific advantage over every other provider on the list. Added a short section on how 24-month contracts and scheduled price rises affect the real two-year cost of a gaming-suitable package. Word count 836 -&gt; 1,184; left just under the self-imposed 1,200-word floor rather than pad.</t>
         </is>
       </c>
       <c r="F51" s="3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G51" s="3" t="n">
         <v>34</v>
@@ -10403,7 +10474,7 @@
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-social-tariffs-uk), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-gaming-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
@@ -10438,19 +10509,19 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Fifteenth target from scripts/analyze_content_priority.py's ranked list: 565 words, no real prices anywhere, and a stale 'EE is consistently rated the most reliable major UK broadband provider' claim that no longer holds under this session's own Q1 2026 Ofcom complaints research. Rewrote with real current prices for Community Fibre, Hyperoptic, Zen Internet and BT, and added a genuinely new section this page never had: when a business-grade line (static IP, faster fault-fix SLA) is actually worth it for a freelancer or remote worker over a residential package, using real Vodafone Business/Zen Business/Sky Business pricing already researched for this site's business broadband guide. Added concrete video-call upload-bandwidth guidance (3-4 Mbps per HD call) rather than vague 'upload matters' framing. Word count 565 -&gt; 986.</t>
+          <t>Fourteenth target from scripts/analyze_content_priority.py's ranked list: 777 words with a materially wrong 'cheapest tariff' claim -- Vodafone Together Social was listed at GBP12.50/mo for 38Mbps and named the cheapest option, but the real current Vodafone Essentials Broadband tariff is GBP20/mo for 73Mbps (verified directly against Vodafone's own tariff page), meaning Virgin Media Essential Broadband and Community Fibre Essential (both genuinely GBP12.50/mo) are actually jointly cheapest. Also corrected Virgin Media's own tariff, which the old page listed at GBP20/mo. Added a genuinely newsworthy find: a thinkbroadband report published in August 2026 (days before this rewrite) tested how easy major providers make it to find their own social tariffs and scored BT, Sky, Virgin Media and Vodafone poorly, with a pointed BT quote, against smaller altnets scoring better. Corrected the eligibility table (Sky accepts UC/PC only, existing customers only, a real restriction the old page omitted) and added KCOM's Hull-only tariff. Refreshed the awareness stat with the newer, more specific thinkbroadband figures (34% aware, 8.6% UC take-up). Word count 777 -&gt; 1,161.</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
@@ -10459,7 +10530,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-working-from-home), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-social-tariffs-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -10494,19 +10565,19 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Sixteenth target from scripts/analyze_content_priority.py's ranked list, and the one with the largest factual break of this whole refresh sequence: the page's entire premise named NOW Broadband and TalkTalk as 'the most common names in this price bracket,' but both now start above GBP20/mo (NOW at GBP23, TalkTalk at GBP25, both already corrected on their own provider pages this session). Rebuilt the page around who is actually under GBP20 today by querying data/providers.ts directly for every provider with monthlyPriceFrom &lt; 20: Community Fibre (GBP12.50), Onestream (GBP18.50, 94% Openreach coverage -- the most realistic pick for most addresses), Gigaclear (GBP19.00, rural symmetrical), toob (GBP19.50) and Trooli (GBP19.99). Also caught and excluded Shell Energy (GBP19.99 in the data file) after finding its own provider-page highlights note it closed to new customers and migrated to TalkTalk in 2024 -- an old, non-orderable plan that would have been a real error to list as a current deal. Word count 608 -&gt; 890.</t>
+          <t>Fifteenth target from scripts/analyze_content_priority.py's ranked list: 565 words, no real prices anywhere, and a stale 'EE is consistently rated the most reliable major UK broadband provider' claim that no longer holds under this session's own Q1 2026 Ofcom complaints research. Rewrote with real current prices for Community Fibre, Hyperoptic, Zen Internet and BT, and added a genuinely new section this page never had: when a business-grade line (static IP, faster fault-fix SLA) is actually worth it for a freelancer or remote worker over a residential package, using real Vodafone Business/Zen Business/Sky Business pricing already researched for this site's business broadband guide. Added concrete video-call upload-bandwidth guidance (3-4 Mbps per HD call) rather than vague 'upload matters' framing. Word count 565 -&gt; 986.</t>
         </is>
       </c>
       <c r="F53" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
@@ -10515,7 +10586,7 @@
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-deals-under-20), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-working-from-home), data/guides.ts</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
@@ -10540,7 +10611,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -10550,43 +10621,43 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
+          <t>Sixteenth target from scripts/analyze_content_priority.py's ranked list, and the one with the largest factual break of this whole refresh sequence: the page's entire premise named NOW Broadband and TalkTalk as 'the most common names in this price bracket,' but both now start above GBP20/mo (NOW at GBP23, TalkTalk at GBP25, both already corrected on their own provider pages this session). Rebuilt the page around who is actually under GBP20 today by querying data/providers.ts directly for every provider with monthlyPriceFrom &lt; 20: Community Fibre (GBP12.50), Onestream (GBP18.50, 94% Openreach coverage -- the most realistic pick for most addresses), Gigaclear (GBP19.00, rural symmetrical), toob (GBP19.50) and Trooli (GBP19.99). Also caught and excluded Shell Energy (GBP19.99 in the data file) after finding its own provider-page highlights note it closed to new customers and migrated to TalkTalk in 2024 -- an old, non-orderable plan that would have been a real error to list as a current deal. Word count 608 -&gt; 890.</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
         <v>35</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-under-20), data/guides.ts</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>None, but easier before the guide count grows further</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10596,7 +10667,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -10606,43 +10677,43 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
+          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
       <c r="F55" s="3" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
+          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L55" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -10662,19 +10733,19 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
+          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
@@ -10683,7 +10754,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
+          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -10718,19 +10789,19 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
+          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
         </is>
       </c>
       <c r="F57" s="3" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
@@ -10739,7 +10810,7 @@
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
+          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
@@ -10774,19 +10845,19 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
+          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -10795,7 +10866,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -10810,7 +10881,7 @@
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10830,48 +10901,104 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="G59" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
           <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
-      <c r="E59" s="3" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
         </is>
       </c>
-      <c r="F59" s="3" t="n">
+      <c r="F60" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="G59" s="3" t="n">
+      <c r="G60" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="H59" s="3" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I59" s="3" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr">
         <is>
           <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
         </is>
       </c>
-      <c r="J59" s="3" t="inlineStr">
+      <c r="J60" s="2" t="inlineStr">
         <is>
           <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
-      <c r="K59" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L59" s="3" t="inlineStr">
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
         <is>
           <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L59"/>
+  <autoFilter ref="A1:L60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10912,7 +11039,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>91 total (33 page builds, 58 feature/strategy builds); 77 already marked Done.</t>
+          <t>92 total (33 page builds, 59 feature/strategy builds); 78 already marked Done.</t>
         </is>
       </c>
     </row>
@@ -10983,4 +11110,1854 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Opportunity</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Clicks</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>CTR</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Impression Change</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>GA4 Sessions</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Engagement Rate</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Affiliate Clicks</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>AI Referral Visits</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Top Queries</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Recommended Action</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/da1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>913</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0.001095290251916758</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>9.460021905805039</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>213.7</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>broadband deals in dartford</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/m1</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>12.875</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>-17.6</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>m1 broadband; cheap broadband deals manchester; m1 wifi broadband; m1 internet plan; m1 internet broadband</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/ng1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>132</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>13.64393939393939</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>broadband deals nottingham; broadband deals in nottingham; broadband deals nottinghamshire; internet deals nottingham; cheapest broadband nottingham</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/rg1</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>126</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>14.90476190476191</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>broadband deals in reading; broadband in reading; broadband deals reading; broadband reading; cheapest</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/ct1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>9.866666666666667</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>broadband deals in canterbury</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>/providers/compare/ee-vs-talktalk</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>107</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0.01869158878504673</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>8.317757009345794</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>is ee broadband better than talktalk; are talktalk and ee the same; who is dido harding; talktalk.co.uk/homesafe; talktalk uswitch</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/rm1</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>9.574468085106384</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>broadband deals in romford; broadband deals romford; internet deals romford; best internet provider romford; whats the best broadband in my area</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>/guides/broadband-deals-with-cashback</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>91</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>14.54945054945055</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>compare broadband providers with cashback; broadband price rises with cashback; compare internet providers with cashback; broadband switching deals with cashback; where should i look for broadband deals that offer extra perks?</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/bs1</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Page-two opportunity</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0.009523809523809525</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>21.93333333333333</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>-29.5</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>broadband deals bristol; broadband deals in bristol; best broadband deals bristol; best broadband deals in bristol</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/e1</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>0.01298701298701299</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>4.870129870129871</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>yes please; ee whitechapel; e1</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/ne1</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Page-two opportunity</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>23.11340206185567</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>-31.7</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>broadband deals newcastle; broadband deals in newcastle; broadband newcastle; broadband deals north tyneside; best broadband deals newcastle</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/bn1</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>73</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>0.0136986301369863</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>11.49315068493151</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>broadband deals in brighton; broadband deals brighton</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/gu1</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>0.01538461538461539</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>11.64615384615385</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>broadband deals in guildford</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/ha1</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>8.533333333333333</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>broadband deals in harrow; ha1 4bh; ha1; broadband</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>/guides/broadband-deals-with-no-setup-fee</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Page-two opportunity</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>548</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>26.25547445255474</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>broadband deals no upfront cost; broadband no upfront cost; broadband and tv deals no upfront cost; broadband no upfront costs; broadband no setup fee</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/w5</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>6.732142857142857</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="3" t="n"/>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/se1</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>6.037735849056604</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>find the best broadband deals in southwark under £30 a month.; find the best broadband deals in southwark under £25 a month.; fibre broadband in southwark</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>3283</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>0.0009137983551629607</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>31.69966494060311</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>-51.5</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="3" t="n"/>
+      <c r="L19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>internet comparison; compare broadband deals; broadband deals compare; compare broadband packages; broadband price comparison</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>Monitor until the page accumulates enough demand or behavioural evidence for a confident intervention.</t>
+        </is>
+      </c>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/en1</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>14.13953488372093</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>broadband deals in enfield</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/nw1</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="3" t="n"/>
+      <c r="L21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="3" t="n"/>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P21" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/ub1</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>8.025</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>broadband deals in southall; yes; and cheapest</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>/guides/best-broadband-and-tv-deals</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>18477</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>0.0005953347404881745</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>61.46468582562104</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="3" t="n"/>
+      <c r="L23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="3" t="inlineStr">
+        <is>
+          <t>best broadband and tv deals; compare broadband and tv; broadband and tv deals; tv package deals; tv and broadband deals</t>
+        </is>
+      </c>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>Monitor until the page accumulates enough demand or behavioural evidence for a confident intervention.</t>
+        </is>
+      </c>
+      <c r="P23" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>/guides/best-phone-and-broadband-deals</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>14411</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>50.85365345916314</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>unlimited phone calls and broadband packages; home phone and broadband; broadband and line rental deals; best phone and broadband; compare broadband and phone</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Monitor until the page accumulates enough demand or behavioural evidence for a confident intervention.</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>/guides/cheapest-broadband-uk</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>907</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>0.002205071664829107</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>37.60529217199559</v>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>-59.6</v>
+      </c>
+      <c r="J25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="3" t="n"/>
+      <c r="L25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="3" t="inlineStr">
+        <is>
+          <t>cheap broadband deals uk; cheapest broadband uk; cheapest broadband; cheap broadband uk; cheapest uk broadband</t>
+        </is>
+      </c>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>Monitor until the page accumulates enough demand or behavioural evidence for a confident intervention.</t>
+        </is>
+      </c>
+      <c r="P25" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/lu1</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Page-two opportunity</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>15.546875</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="2" t="n"/>
+      <c r="L26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>broadband deals in luton; broadband deals luton; broadband luton; internet providers luton; broadband deals near me</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>/guides/best-full-fibre-broadband-uk</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>6039</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>0.0003311806590495115</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>50.10250041397583</v>
+      </c>
+      <c r="I27" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="3" t="n"/>
+      <c r="L27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="3" t="inlineStr">
+        <is>
+          <t>fibre broadband; fibre optic broadband; best fibre broadband; full fibre broadband; best fibre broadband deals</t>
+        </is>
+      </c>
+      <c r="O27" s="3" t="inlineStr">
+        <is>
+          <t>Monitor until the page accumulates enough demand or behavioural evidence for a confident intervention.</t>
+        </is>
+      </c>
+      <c r="P27" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/so14</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Page-two opportunity</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>104</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>0.009615384615384616</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>26.42307692307692</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="2" t="n"/>
+      <c r="L28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>broadband deals in southampton; broadband deals southampton; broadband company southampton; internet providers southampton; fibre broadband southampton</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/l1</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Page-two opportunity</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>26.25974025974026</v>
+      </c>
+      <c r="I29" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="3" t="n"/>
+      <c r="L29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
+          <t>broadband deals liverpool; broadband comparison liverpool; internet deals liverpool; broadband deals in liverpool; best broadband deals liverpool</t>
+        </is>
+      </c>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+        </is>
+      </c>
+      <c r="P29" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>/providers/virgin-media/deals</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>2404</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>0.000415973377703827</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>60.52953410981697</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="J30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="2" t="n"/>
+      <c r="L30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>virgin media deals; virgin media offers; virgin broadband deals; virgin media packages; virgin media broadband deals</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>Monitor until the page accumulates enough demand or behavioural evidence for a confident intervention.</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>/guides/broadband-speeds-explained</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>326</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>57.91104294478528</v>
+      </c>
+      <c r="I31" s="3" t="n">
+        <v>-47.9</v>
+      </c>
+      <c r="J31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="3" t="n"/>
+      <c r="L31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="3" t="inlineStr">
+        <is>
+          <t>broadband speeds explained; what is broadband speed; broadband speeds; broadband speed explained; what is a good broadband speed mbps</t>
+        </is>
+      </c>
+      <c r="O31" s="3" t="inlineStr">
+        <is>
+          <t>Monitor until the page accumulates enough demand or behavioural evidence for a confident intervention.</t>
+        </is>
+      </c>
+      <c r="P31" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:44:19.638288+00:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:P31"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
content: enhance How to Switch Broadband Provider guide with One Touch Switch closure news
Twenty-fifth target from the content-priority-analysis list: the guide
was already excellent (dated citations, real compensation figures,
no thinness flags), so this was a targeted enhancement rather than a
rewrite. Added the one genuinely relevant, on-topic development it
was missing: Ofcom closed its dedicated One Touch Switch enforcement
programme on 11 June 2026 after finding more than 2 million customers
had already used it successfully, confirming it as the industry's
permanent standard.

Also bundles the concurrently-running content pipeline's new
Dartford (DA1) postcode page enhancement and em-dash style cleanup,
already present in the working tree and validated by the build above.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L93" headerRowCount="1">
-  <autoFilter ref="A1:L93"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L94" headerRowCount="1">
+  <autoFilter ref="A1:L94"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L60" headerRowCount="1">
-  <autoFilter ref="A1:L60"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L61" headerRowCount="1">
+  <autoFilter ref="A1:L61"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4075,7 +4075,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-youfibre-provider-page</t>
+          <t>content-refresh-how-to-switch-broadband-guide</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -4090,18 +4090,18 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
+          <t>Update: How to Switch Broadband Provider guide (25th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -4119,7 +4119,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-providers-uk-guide</t>
+          <t>content-refresh-youfibre-provider-page</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -4134,14 +4134,14 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
+          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F77" s="3" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
@@ -4163,12 +4163,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>bet-annual-research-report</t>
+          <t>content-refresh-best-broadband-providers-uk-guide</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -4178,23 +4178,23 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr"/>
@@ -4207,12 +4207,12 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-without-phone-line-guide</t>
+          <t>bet-annual-research-report</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -4222,23 +4222,23 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="F79" s="3" t="n">
         <v>41</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr"/>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-bt-vs-virgin-media-comparison</t>
+          <t>content-refresh-broadband-without-phone-line-guide</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -4266,14 +4266,14 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
         <v>41</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -4295,7 +4295,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-moving-house-guide</t>
+          <t>content-refresh-bt-vs-virgin-media-comparison</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -4310,14 +4310,14 @@
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F81" s="3" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-satellite-broadband-uk-guide</t>
+          <t>content-refresh-broadband-moving-house-guide</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -4354,14 +4354,14 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -4383,38 +4383,38 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>bet-componentise-interactive-layer</t>
+          <t>content-refresh-satellite-broadband-uk-guide</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F83" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G83" s="3" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr"/>
@@ -4427,38 +4427,38 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-gaming-guide</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
         <v>38</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr"/>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-social-tariffs-guide</t>
+          <t>content-refresh-best-broadband-for-gaming-guide</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -4486,11 +4486,11 @@
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F85" s="3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G85" s="3" t="n">
         <v>34</v>
@@ -4515,7 +4515,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-working-from-home-guide</t>
+          <t>content-refresh-broadband-social-tariffs-guide</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -4530,14 +4530,14 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-under-20-guide</t>
+          <t>content-refresh-best-broadband-working-from-home-guide</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -4574,14 +4574,14 @@
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F87" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G87" s="3" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
@@ -4603,12 +4603,12 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>content-refresh-broadband-deals-under-20-guide</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -4618,23 +4618,23 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
         <v>35</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr"/>
@@ -4647,12 +4647,12 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-bt-vs-sky-comparison</t>
+          <t>bet-decouple-content-from-code</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
@@ -4662,23 +4662,23 @@
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="F89" s="3" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G89" s="3" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr"/>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
+          <t>content-refresh-bt-vs-sky-comparison</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -4706,14 +4706,14 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
@@ -4735,7 +4735,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-price-rises-2026-guide</t>
+          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -4750,14 +4750,14 @@
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F91" s="3" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G91" s="3" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
@@ -4779,7 +4779,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-full-fibre-broadband-explained-guide</t>
+          <t>content-refresh-broadband-price-rises-2026-guide</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -4794,14 +4794,14 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-students-guide</t>
+          <t>content-refresh-full-fibre-broadband-explained-guide</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -4838,14 +4838,14 @@
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F93" s="3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G93" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
@@ -4861,8 +4861,52 @@
       <c r="K93" s="3" t="inlineStr"/>
       <c r="L93" s="3" t="inlineStr"/>
     </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>content-refresh-best-broadband-for-students-guide</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G94" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr"/>
+      <c r="K94" s="2" t="inlineStr"/>
+      <c r="L94" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L93"/>
+  <autoFilter ref="A1:L94"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7614,7 +7658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10005,28 +10049,28 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
+          <t>Update: How to Switch Broadband Provider guide (25th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Eighth target from scripts/analyze_content_priority.py's ranked list: /providers/youfibre was 397 words with no excerpt or contentSections. Rewritten to ~1,575 words with 6 contentSections. The standout finding, verified against a primary Virgin Media O2 press release after a first-pass WebSearch AI summary over-stated it as a done deal: YouFibre's parent company, Substantial Group (Netomnia), is being acquired for GBP2bn by nexfibre (a joint venture of InfraVia, Liberty Global and Telefonica), which then plans to resell the YouFibre/Brsk retail brands to Virgin Media O2 for GBP150m -- announced Feb 2026, referred to the CMA for a Phase 2 investigation on 1 July 2026, and NOT yet completed (expected ~Q3 2026 at the earliest). Also wrote up the real, documented fallout from the March 2026 Brsk-to-YouFibre customer migration (billing errors, login/password-reset failures, reported speed drops, overwhelmed support chat), sourced from ISPreview rather than the vague pre-existing 'Trustpilot sentiment has been mixed' line. Updated the speeds array to the real current tiers (200/1000/2000/8000 Mbps symmetrical, replacing stale 200/900/1800) and contractLengths from [1,12,24] to [1,24] to match the two options confirmed by current pricing research.</t>
+          <t>Twenty-fifth target: /guides/how-to-switch-broadband-uk (6,000/mo volume) was already excellent -- 1,913 words, dated citations, real Automatic Compensation Scheme figures (GBP6.46/day, GBP32.31 per missed appointment), no thinness or staleness flags. This was a targeted enhancement rather than a rewrite: added the one genuinely relevant, on-topic development the page was missing -- Ofcom closed its dedicated One Touch Switch enforcement programme on 11 June 2026 after finding more than 2 million customers had already used it successfully, confirming it as the industry's permanent standard rather than a still-bedding-in process. Added this to the intro, a new FAQ, and the guide's keyTakeaways/sources. Word count 1,913 -&gt; 2,043.</t>
         </is>
       </c>
       <c r="F43" s="3" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>data/providers.ts (youfibre)</t>
+          <t>app/guides/[slug]/page.tsx (how-to-switch-broadband-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
@@ -10041,7 +10085,7 @@
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10061,19 +10105,19 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
+          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Ninth target from scripts/analyze_content_priority.py's ranked list. This ranking page's data was badly stale: it cited Q4 2025 Ofcom complaints figures and June-2026 Trustpilot scores that had already been superseded by this site's own freshly-researched provider pages (Sky, NOW Broadband, BT, Virgin Media, EE, Plusnet, Vodafone, TalkTalk from earlier this session). Rather than re-researching each provider from scratch, cross-referenced this page's ranking table against data/providers.ts's own already-vetted current fields (price, Trustpilot, reviewedDate) and fetched a fresh single-source Ofcom Q1 2026 complaints table (published 23 July 2026, record-low industry average of 6 per 100k) to replace the mixed-quarter data. Corrected several materially wrong claims: TalkTalk was still framed as 'budget only' at GBP19.99 when it is now GBP25 and no longer the cheapest big-name option; Community Fibre was described as 'London-only' when coverage has expanded into Surrey and Sussex; EE's 'best for reliability' halo no longer holds under Q1 2026 data (6 per 100k, tied with Virgin Media, not uniquely best). Added a new section contrasting sister brands Sky (5 per 100k) and NOW Broadband (11 per 100k, different quarter, footnoted) on the identical Openreach network, a genuine support-quality data point. Word count 872 -&gt; 1,333.</t>
+          <t>Eighth target from scripts/analyze_content_priority.py's ranked list: /providers/youfibre was 397 words with no excerpt or contentSections. Rewritten to ~1,575 words with 6 contentSections. The standout finding, verified against a primary Virgin Media O2 press release after a first-pass WebSearch AI summary over-stated it as a done deal: YouFibre's parent company, Substantial Group (Netomnia), is being acquired for GBP2bn by nexfibre (a joint venture of InfraVia, Liberty Global and Telefonica), which then plans to resell the YouFibre/Brsk retail brands to Virgin Media O2 for GBP150m -- announced Feb 2026, referred to the CMA for a Phase 2 investigation on 1 July 2026, and NOT yet completed (expected ~Q3 2026 at the earliest). Also wrote up the real, documented fallout from the March 2026 Brsk-to-YouFibre customer migration (billing errors, login/password-reset failures, reported speed drops, overwhelmed support chat), sourced from ISPreview rather than the vague pre-existing 'Trustpilot sentiment has been mixed' line. Updated the speeds array to the real current tiers (200/1000/2000/8000 Mbps symmetrical, replacing stale 200/900/1800) and contractLengths from [1,12,24] to [1,24] to match the two options confirmed by current pricing research.</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -10082,7 +10126,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-providers-uk), data/guides.ts</t>
+          <t>data/providers.ts (youfibre)</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -10107,7 +10151,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -10117,43 +10161,43 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
+          <t>Ninth target from scripts/analyze_content_priority.py's ranked list. This ranking page's data was badly stale: it cited Q4 2025 Ofcom complaints figures and June-2026 Trustpilot scores that had already been superseded by this site's own freshly-researched provider pages (Sky, NOW Broadband, BT, Virgin Media, EE, Plusnet, Vodafone, TalkTalk from earlier this session). Rather than re-researching each provider from scratch, cross-referenced this page's ranking table against data/providers.ts's own already-vetted current fields (price, Trustpilot, reviewedDate) and fetched a fresh single-source Ofcom Q1 2026 complaints table (published 23 July 2026, record-low industry average of 6 per 100k) to replace the mixed-quarter data. Corrected several materially wrong claims: TalkTalk was still framed as 'budget only' at GBP19.99 when it is now GBP25 and no longer the cheapest big-name option; Community Fibre was described as 'London-only' when coverage has expanded into Surrey and Sussex; EE's 'best for reliability' halo no longer holds under Q1 2026 data (6 per 100k, tied with Virgin Media, not uniquely best). Added a new section contrasting sister brands Sky (5 per 100k) and NOW Broadband (11 per 100k, different quarter, footnoted) on the identical Openreach network, a genuine support-quality data point. Word count 872 -&gt; 1,333.</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>New annual research page + methodology extension</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-providers-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>research/uk-broadband-customer-satisfaction methodology</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10163,7 +10207,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -10173,43 +10217,43 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Tenth target from scripts/analyze_content_priority.py's ranked list: 770 words, stale pricing table (every one of 8 providers priced against months-old figures already corrected on this site's own provider pages), and a wrong PSTN switch-off date ('by the end of 2027' -- the real, now-locked-in date is 31 January 2027). Rewrote using the same PSTN research gathered for the best-phone-and-broadband-deals refresh earlier this session (5.2m -&gt; 3.2m migration stat, Ofcom's 1-hour power-cut battery backup minimum, the PSTN Charter's telecare protections), added a genuinely missing section -- 'What happens to a home phone during a power cut?' -- since the old version covered whether a line is needed at all but never addressed the actual practical question once Digital Voice is the default. Refreshed all 8 provider prices against data/providers.ts's own current fields, updated Virgin Media coverage 52% (was 53%) and added Ofcom's Spring 2026 Connected Nations split (89% gigabit-capable, 82% full fibre, 93% urban vs 66% rural). Word count 770 -&gt; 1,196; left just under the self-imposed 1,200-word floor rather than pad.</t>
+          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
         <v>41</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-without-phone-line), data/guides.ts</t>
+          <t>New annual research page + methodology extension</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>research/uk-broadband-customer-satisfaction methodology</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -10229,19 +10273,19 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Twenty-first target from the wider top-30 content-priority-analysis list: 526 words of entirely generic, number-free copy ('BT has no setup fee in the current dataset' -- itself wrong, BT's setup fee is GBP30). Rewrote using already-vetted current data from this session's own BT and Virgin Media provider-page work: BT from GBP23.99/mo (24-month, 98% coverage, Trustpilot 4.0/1.5 two-page split) vs Virgin Media from GBP33.00/mo (18-month, 52% coverage, 1,130Mbps fastest widely available speed, Trustpilot 1.4 but a genuinely better Q1 2026 Ofcom complaints record than BT, 6 vs 7 per 100k). Added the genuinely important practical point this page never covered: switching to Virgin Media never qualifies for One Touch Switch since it runs on a separate network from Openreach. Populated the previously-empty factSnapshot field. Word count 526 -&gt; 718.</t>
+          <t>Tenth target from scripts/analyze_content_priority.py's ranked list: 770 words, stale pricing table (every one of 8 providers priced against months-old figures already corrected on this site's own provider pages), and a wrong PSTN switch-off date ('by the end of 2027' -- the real, now-locked-in date is 31 January 2027). Rewrote using the same PSTN research gathered for the best-phone-and-broadband-deals refresh earlier this session (5.2m -&gt; 3.2m migration stat, Ofcom's 1-hour power-cut battery backup minimum, the PSTN Charter's telecare protections), added a genuinely missing section -- 'What happens to a home phone during a power cut?' -- since the old version covered whether a line is needed at all but never addressed the actual practical question once Digital Voice is the default. Refreshed all 8 provider prices against data/providers.ts's own current fields, updated Virgin Media coverage 52% (was 53%) and added Ofcom's Spring 2026 Connected Nations split (89% gigabit-capable, 82% full fibre, 93% urban vs 66% rural). Word count 770 -&gt; 1,196; left just under the self-imposed 1,200-word floor rather than pad.</t>
         </is>
       </c>
       <c r="F47" s="3" t="n">
         <v>41</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
@@ -10250,7 +10294,7 @@
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>data/provider-comparisons.ts (bt-vs-virgin-media)</t>
+          <t>app/guides/[slug]/page.tsx (broadband-without-phone-line), data/guides.ts</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
@@ -10265,7 +10309,7 @@
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10285,19 +10329,19 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Eleventh target from scripts/analyze_content_priority.py's ranked list: 948 words, structurally sound (evergreen checklist format) but missing a genuinely newsworthy development -- Ofcom closed its One Touch Switch enforcement case on 11 June 2026 after finding more than 2 million customers had already used the process successfully, meaning it is now the industry's permanent standard rather than a monitored pilot, which the old copy still implied. Added this, plus a genuinely missing section on what a house move means for a home phone line given the 31 January 2027 PSTN switch-off (reusing research from the phone-and-broadband and broadband-without-phone-line refreshes earlier this session), Ofcom's Spring 2026 coverage split for the 'check availability' step, and corrected the ETC explanation to reflect Ofcom's actual cap rule (remaining payments, ex-VAT) rather than a flat multiplication. Re-verified the pre-existing GBP183.60/year switching-saving stat against fresh 2026 sources (found independently corroborated) and added the 4.2m/GBP100-240 social tariff stat already used elsewhere on this site. Word count 948 -&gt; 1,446.</t>
+          <t>Twenty-first target from the wider top-30 content-priority-analysis list: 526 words of entirely generic, number-free copy ('BT has no setup fee in the current dataset' -- itself wrong, BT's setup fee is GBP30). Rewrote using already-vetted current data from this session's own BT and Virgin Media provider-page work: BT from GBP23.99/mo (24-month, 98% coverage, Trustpilot 4.0/1.5 two-page split) vs Virgin Media from GBP33.00/mo (18-month, 52% coverage, 1,130Mbps fastest widely available speed, Trustpilot 1.4 but a genuinely better Q1 2026 Ofcom complaints record than BT, 6 vs 7 per 100k). Added the genuinely important practical point this page never covered: switching to Virgin Media never qualifies for One Touch Switch since it runs on a separate network from Openreach. Populated the previously-empty factSnapshot field. Word count 526 -&gt; 718.</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -10306,7 +10350,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-moving-house), data/guides.ts</t>
+          <t>data/provider-comparisons.ts (bt-vs-virgin-media)</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -10321,7 +10365,7 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10341,19 +10385,19 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Twelfth target from scripts/analyze_content_priority.py's ranked list, and the page whose DATE_RE regex bug was found and fixed earlier this session (58.2 -&gt; 53.2) without ever getting a content rewrite. The old copy was generic to the point of naming no real prices at all -- 'Starlink is the most visible option' with zero named plans, figures or alternatives. Rewritten with real, current Starlink UK pricing (Residential 100/200/Max at GBP40/60/80 per month, Roam at GBP55-100, Standard Kit GBP449 commonly discounted to ~GBP299 or free on Max), and a genuinely current news item: Starlink's Global Roam plan stopped taking new customers 15 July 2026 and was withdrawn entirely for existing customers on 17 August 2026, one week before this rewrite. Named 2 real smaller alternatives (SkyDSL, Bigblu Broadband) and clarified that Eutelsat/OneWeb, despite frequent mention alongside Starlink, sells no UK consumer home-broadband plans at all. Word count 437 -&gt; 1,038.</t>
+          <t>Eleventh target from scripts/analyze_content_priority.py's ranked list: 948 words, structurally sound (evergreen checklist format) but missing a genuinely newsworthy development -- Ofcom closed its One Touch Switch enforcement case on 11 June 2026 after finding more than 2 million customers had already used the process successfully, meaning it is now the industry's permanent standard rather than a monitored pilot, which the old copy still implied. Added this, plus a genuinely missing section on what a house move means for a home phone line given the 31 January 2027 PSTN switch-off (reusing research from the phone-and-broadband and broadband-without-phone-line refreshes earlier this session), Ofcom's Spring 2026 coverage split for the 'check availability' step, and corrected the ETC explanation to reflect Ofcom's actual cap rule (remaining payments, ex-VAT) rather than a flat multiplication. Re-verified the pre-existing GBP183.60/year switching-saving stat against fresh 2026 sources (found independently corroborated) and added the 4.2m/GBP100-240 social tariff stat already used elsewhere on this site. Word count 948 -&gt; 1,446.</t>
         </is>
       </c>
       <c r="F49" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
@@ -10362,7 +10406,7 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>data/priority-pages.ts (satellite)</t>
+          <t>app/guides/[slug]/page.tsx (broadband-moving-house), data/guides.ts</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
@@ -10387,53 +10431,53 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+          <t>Twelfth target from scripts/analyze_content_priority.py's ranked list, and the page whose DATE_RE regex bug was found and fixed earlier this session (58.2 -&gt; 53.2) without ever getting a content rewrite. The old copy was generic to the point of naming no real prices at all -- 'Starlink is the most visible option' with zero named plans, figures or alternatives. Rewritten with real, current Starlink UK pricing (Residential 100/200/Max at GBP40/60/80 per month, Roam at GBP55-100, Standard Kit GBP449 commonly discounted to ~GBP299 or free on Max), and a genuinely current news item: Starlink's Global Roam plan stopped taking new customers 15 July 2026 and was withdrawn entirely for existing customers on 17 August 2026, one week before this rewrite. Named 2 real smaller alternatives (SkyDSL, Bigblu Broadband) and clarified that Eutelsat/OneWeb, despite frequent mention alongside Starlink, sells no UK consumer home-broadband plans at all. Word count 437 -&gt; 1,038.</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>components/</t>
+          <t>data/priority-pages.ts (satellite)</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10443,53 +10487,53 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Thirteenth target from scripts/analyze_content_priority.py's ranked list: 836 words with stale provider prices (EE GBP26.99, Community Fibre GBP21.99, Hyperoptic GBP22, BT GBP30.99, all already corrected on this site's own provider pages) and a wrong Community Fibre top-tier speed claim (920Mbps symmetrical, against the real current 3,000Mbps top tier confirmed in data/providers.ts). Refreshed all 5 existing provider picks against already-vetted current pricing, and added a genuinely new 6th pick, Zen Internet, for a use case the old page didn't cover at all: hosting a private game server, where Zen's free static IP (already documented on its own provider page) is a real, specific advantage over every other provider on the list. Added a short section on how 24-month contracts and scheduled price rises affect the real two-year cost of a gaming-suitable package. Word count 836 -&gt; 1,184; left just under the self-imposed 1,200-word floor rather than pad.</t>
+          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
         </is>
       </c>
       <c r="F51" s="3" t="n">
         <v>38</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-gaming-uk), data/guides.ts</t>
+          <t>components/</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
         </is>
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L51" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Functionality pillar</t>
         </is>
       </c>
     </row>
@@ -10509,16 +10553,16 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Fourteenth target from scripts/analyze_content_priority.py's ranked list: 777 words with a materially wrong 'cheapest tariff' claim -- Vodafone Together Social was listed at GBP12.50/mo for 38Mbps and named the cheapest option, but the real current Vodafone Essentials Broadband tariff is GBP20/mo for 73Mbps (verified directly against Vodafone's own tariff page), meaning Virgin Media Essential Broadband and Community Fibre Essential (both genuinely GBP12.50/mo) are actually jointly cheapest. Also corrected Virgin Media's own tariff, which the old page listed at GBP20/mo. Added a genuinely newsworthy find: a thinkbroadband report published in August 2026 (days before this rewrite) tested how easy major providers make it to find their own social tariffs and scored BT, Sky, Virgin Media and Vodafone poorly, with a pointed BT quote, against smaller altnets scoring better. Corrected the eligibility table (Sky accepts UC/PC only, existing customers only, a real restriction the old page omitted) and added KCOM's Hull-only tariff. Refreshed the awareness stat with the newer, more specific thinkbroadband figures (34% aware, 8.6% UC take-up). Word count 777 -&gt; 1,161.</t>
+          <t>Thirteenth target from scripts/analyze_content_priority.py's ranked list: 836 words with stale provider prices (EE GBP26.99, Community Fibre GBP21.99, Hyperoptic GBP22, BT GBP30.99, all already corrected on this site's own provider pages) and a wrong Community Fibre top-tier speed claim (920Mbps symmetrical, against the real current 3,000Mbps top tier confirmed in data/providers.ts). Refreshed all 5 existing provider picks against already-vetted current pricing, and added a genuinely new 6th pick, Zen Internet, for a use case the old page didn't cover at all: hosting a private game server, where Zen's free static IP (already documented on its own provider page) is a real, specific advantage over every other provider on the list. Added a short section on how 24-month contracts and scheduled price rises affect the real two-year cost of a gaming-suitable package. Word count 836 -&gt; 1,184; left just under the self-imposed 1,200-word floor rather than pad.</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G52" s="2" t="n">
         <v>34</v>
@@ -10530,7 +10574,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-social-tariffs-uk), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-gaming-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -10565,19 +10609,19 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Fifteenth target from scripts/analyze_content_priority.py's ranked list: 565 words, no real prices anywhere, and a stale 'EE is consistently rated the most reliable major UK broadband provider' claim that no longer holds under this session's own Q1 2026 Ofcom complaints research. Rewrote with real current prices for Community Fibre, Hyperoptic, Zen Internet and BT, and added a genuinely new section this page never had: when a business-grade line (static IP, faster fault-fix SLA) is actually worth it for a freelancer or remote worker over a residential package, using real Vodafone Business/Zen Business/Sky Business pricing already researched for this site's business broadband guide. Added concrete video-call upload-bandwidth guidance (3-4 Mbps per HD call) rather than vague 'upload matters' framing. Word count 565 -&gt; 986.</t>
+          <t>Fourteenth target from scripts/analyze_content_priority.py's ranked list: 777 words with a materially wrong 'cheapest tariff' claim -- Vodafone Together Social was listed at GBP12.50/mo for 38Mbps and named the cheapest option, but the real current Vodafone Essentials Broadband tariff is GBP20/mo for 73Mbps (verified directly against Vodafone's own tariff page), meaning Virgin Media Essential Broadband and Community Fibre Essential (both genuinely GBP12.50/mo) are actually jointly cheapest. Also corrected Virgin Media's own tariff, which the old page listed at GBP20/mo. Added a genuinely newsworthy find: a thinkbroadband report published in August 2026 (days before this rewrite) tested how easy major providers make it to find their own social tariffs and scored BT, Sky, Virgin Media and Vodafone poorly, with a pointed BT quote, against smaller altnets scoring better. Corrected the eligibility table (Sky accepts UC/PC only, existing customers only, a real restriction the old page omitted) and added KCOM's Hull-only tariff. Refreshed the awareness stat with the newer, more specific thinkbroadband figures (34% aware, 8.6% UC take-up). Word count 777 -&gt; 1,161.</t>
         </is>
       </c>
       <c r="F53" s="3" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
@@ -10586,7 +10630,7 @@
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-working-from-home), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-social-tariffs-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
@@ -10621,19 +10665,19 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Sixteenth target from scripts/analyze_content_priority.py's ranked list, and the one with the largest factual break of this whole refresh sequence: the page's entire premise named NOW Broadband and TalkTalk as 'the most common names in this price bracket,' but both now start above GBP20/mo (NOW at GBP23, TalkTalk at GBP25, both already corrected on their own provider pages this session). Rebuilt the page around who is actually under GBP20 today by querying data/providers.ts directly for every provider with monthlyPriceFrom &lt; 20: Community Fibre (GBP12.50), Onestream (GBP18.50, 94% Openreach coverage -- the most realistic pick for most addresses), Gigaclear (GBP19.00, rural symmetrical), toob (GBP19.50) and Trooli (GBP19.99). Also caught and excluded Shell Energy (GBP19.99 in the data file) after finding its own provider-page highlights note it closed to new customers and migrated to TalkTalk in 2024 -- an old, non-orderable plan that would have been a real error to list as a current deal. Word count 608 -&gt; 890.</t>
+          <t>Fifteenth target from scripts/analyze_content_priority.py's ranked list: 565 words, no real prices anywhere, and a stale 'EE is consistently rated the most reliable major UK broadband provider' claim that no longer holds under this session's own Q1 2026 Ofcom complaints research. Rewrote with real current prices for Community Fibre, Hyperoptic, Zen Internet and BT, and added a genuinely new section this page never had: when a business-grade line (static IP, faster fault-fix SLA) is actually worth it for a freelancer or remote worker over a residential package, using real Vodafone Business/Zen Business/Sky Business pricing already researched for this site's business broadband guide. Added concrete video-call upload-bandwidth guidance (3-4 Mbps per HD call) rather than vague 'upload matters' framing. Word count 565 -&gt; 986.</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
@@ -10642,7 +10686,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-deals-under-20), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-working-from-home), data/guides.ts</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -10667,7 +10711,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -10677,43 +10721,43 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
+          <t>Sixteenth target from scripts/analyze_content_priority.py's ranked list, and the one with the largest factual break of this whole refresh sequence: the page's entire premise named NOW Broadband and TalkTalk as 'the most common names in this price bracket,' but both now start above GBP20/mo (NOW at GBP23, TalkTalk at GBP25, both already corrected on their own provider pages this session). Rebuilt the page around who is actually under GBP20 today by querying data/providers.ts directly for every provider with monthlyPriceFrom &lt; 20: Community Fibre (GBP12.50), Onestream (GBP18.50, 94% Openreach coverage -- the most realistic pick for most addresses), Gigaclear (GBP19.00, rural symmetrical), toob (GBP19.50) and Trooli (GBP19.99). Also caught and excluded Shell Energy (GBP19.99 in the data file) after finding its own provider-page highlights note it closed to new customers and migrated to TalkTalk in 2024 -- an old, non-orderable plan that would have been a real error to list as a current deal. Word count 608 -&gt; 890.</t>
         </is>
       </c>
       <c r="F55" s="3" t="n">
         <v>35</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-under-20), data/guides.ts</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>None, but easier before the guide count grows further</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L55" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10723,7 +10767,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -10733,43 +10777,43 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
+          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
+          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -10789,19 +10833,19 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
+          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
         </is>
       </c>
       <c r="F57" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
@@ -10810,7 +10854,7 @@
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
+          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
@@ -10845,19 +10889,19 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
+          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -10866,7 +10910,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
+          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -10901,19 +10945,19 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
+          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
         </is>
       </c>
       <c r="F59" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
@@ -10922,7 +10966,7 @@
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
@@ -10937,7 +10981,7 @@
       </c>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10957,48 +11001,104 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
           <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E61" s="3" t="inlineStr">
         <is>
           <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
         </is>
       </c>
-      <c r="F60" s="2" t="n">
+      <c r="F61" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="G60" s="2" t="n">
+      <c r="G61" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="H61" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr">
+      <c r="I61" s="3" t="inlineStr">
         <is>
           <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
         </is>
       </c>
-      <c r="J60" s="2" t="inlineStr">
+      <c r="J61" s="3" t="inlineStr">
         <is>
           <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
-      <c r="K60" s="2" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L60" s="2" t="inlineStr">
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr">
         <is>
           <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L60"/>
+  <autoFilter ref="A1:L61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11039,7 +11139,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>92 total (33 page builds, 59 feature/strategy builds); 78 already marked Done.</t>
+          <t>93 total (33 page builds, 60 feature/strategy builds); 79 already marked Done.</t>
         </is>
       </c>
     </row>
@@ -11275,7 +11375,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -11333,7 +11433,7 @@
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -11391,7 +11491,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -11449,7 +11549,7 @@
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -11507,7 +11607,7 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -11565,7 +11665,7 @@
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -11623,7 +11723,7 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -11681,7 +11781,7 @@
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -11739,7 +11839,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -11797,7 +11897,7 @@
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -11855,7 +11955,7 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -11913,7 +12013,7 @@
       </c>
       <c r="P13" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -11971,7 +12071,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12129,7 @@
       </c>
       <c r="P15" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12087,7 +12187,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12141,7 +12241,7 @@
       </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12199,7 +12299,7 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12257,7 +12357,7 @@
       </c>
       <c r="P19" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12315,7 +12415,7 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12369,7 +12469,7 @@
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12427,7 +12527,7 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12485,7 +12585,7 @@
       </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12543,7 +12643,7 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12601,7 +12701,7 @@
       </c>
       <c r="P25" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12659,7 +12759,7 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12717,7 +12817,7 @@
       </c>
       <c r="P27" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12775,7 +12875,7 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12833,7 +12933,7 @@
       </c>
       <c r="P29" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12891,7 +12991,7 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>
@@ -12949,7 +13049,7 @@
       </c>
       <c r="P31" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25T20:44:19.638288+00:00</t>
+          <t>2026-08-25T21:02:40.387960+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Best Broadband for Streaming guide
Twenty-sixth target from the content-priority-analysis list: 699
words naming providers (Sky, Virgin Media, Community Fibre,
Hyperoptic) with zero real prices attached. Added current prices for
all 4, plus Virgin Media's real 1,130 Mbps top speed.

Added a genuinely new, technically accurate explanation this page
never covered: why evening buffering specifically affects FTTC and
cable connections (shared capacity per street cabinet/node) but not
full fibre (dedicated line per property), with a matching new FAQ.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L94" headerRowCount="1">
-  <autoFilter ref="A1:L94"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L95" headerRowCount="1">
+  <autoFilter ref="A1:L95"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L61" headerRowCount="1">
-  <autoFilter ref="A1:L61"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L62" headerRowCount="1">
+  <autoFilter ref="A1:L62"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L94"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4905,8 +4905,52 @@
       <c r="K94" s="2" t="inlineStr"/>
       <c r="L94" s="2" t="inlineStr"/>
     </row>
+    <row r="95">
+      <c r="A95" s="3" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>content-refresh-best-broadband-for-streaming-guide</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="G95" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J95" s="3" t="inlineStr"/>
+      <c r="K95" s="3" t="inlineStr"/>
+      <c r="L95" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L94"/>
+  <autoFilter ref="A1:L95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7658,7 +7702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11097,8 +11141,64 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L61"/>
+  <autoFilter ref="A1:L62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11139,7 +11239,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>93 total (33 page builds, 60 feature/strategy builds); 79 already marked Done.</t>
+          <t>94 total (33 page builds, 61 feature/strategy builds); 80 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Can I Leave Broadband Early After a Price Rise guide
Twenty-seventh target from the content-priority-analysis list: 783
words of correct but entirely abstract legal explanation with zero
real examples of what "clearly disclosed" vs "vague" price-rise
wording looks like in practice.

Added the concrete contrast this session's own research had already
surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence
rise upfront, while Sky's contract terms for years after the first
only say prices "may rise" without a fixed figure. Added the specific
30-day notice/exit-window rule with a matching new FAQ.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$96</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L95" headerRowCount="1">
-  <autoFilter ref="A1:L95"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L96" headerRowCount="1">
+  <autoFilter ref="A1:L96"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L62" headerRowCount="1">
-  <autoFilter ref="A1:L62"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L63" headerRowCount="1">
+  <autoFilter ref="A1:L63"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4949,8 +4949,52 @@
       <c r="K95" s="3" t="inlineStr"/>
       <c r="L95" s="3" t="inlineStr"/>
     </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>content-refresh-can-i-leave-broadband-early-guide</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G96" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr"/>
+      <c r="K96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L95"/>
+  <autoFilter ref="A1:L96"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7702,7 +7746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11197,8 +11241,64 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="G63" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L63" s="3" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L62"/>
+  <autoFilter ref="A1:L63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11239,7 +11339,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>94 total (33 page builds, 61 feature/strategy builds); 80 already marked Done.</t>
+          <t>95 total (33 page builds, 62 feature/strategy builds); 81 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Best Broadband for Rural Areas guide
Twenty-eighth target from the content-priority-analysis list: 635
words naming only BT and EE, with a real content gap for a
rural-specific guide -- no mention of satellite broadband at all,
despite Starlink being one of the classic genuine rural use cases.

Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93%
urban gigabit-capable), real 5G pricing (National Broadband as the
multi-network specialist genuinely suited to rural addresses, Three,
EE Smart 5G Hub), a full Starlink section with real pricing, and the
Gigabit Broadband Voucher Scheme as a cost-effective alternative to
satellite worth checking first.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$97</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L96" headerRowCount="1">
-  <autoFilter ref="A1:L96"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L97" headerRowCount="1">
+  <autoFilter ref="A1:L97"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L63" headerRowCount="1">
-  <autoFilter ref="A1:L63"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L64" headerRowCount="1">
+  <autoFilter ref="A1:L64"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4993,8 +4993,52 @@
       <c r="K96" s="2" t="inlineStr"/>
       <c r="L96" s="2" t="inlineStr"/>
     </row>
+    <row r="97">
+      <c r="A97" s="3" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G97" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="H97" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I97" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J97" s="3" t="inlineStr"/>
+      <c r="K97" s="3" t="inlineStr"/>
+      <c r="L97" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L96"/>
+  <autoFilter ref="A1:L97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7746,7 +7790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11297,8 +11341,64 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L63"/>
+  <autoFilter ref="A1:L64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11339,7 +11439,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>95 total (33 page builds, 62 feature/strategy builds); 81 already marked Done.</t>
+          <t>96 total (33 page builds, 63 feature/strategy builds); 82 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of 4 thin comparison pages
Final 4 targets in this batch, all comparison pages with the same
problem: entirely generic, number-free copy repeating a "TalkTalk is
usually cheaper" claim that is now factually wrong -- TalkTalk starts
at GBP25/mo, more expensive than both BT (GBP23.99) and Sky (GBP23.00).

Rewrote all 4 with real current prices, Ofcom Q1 2026 complaints
figures and populated factSnapshot fields:
- bt-vs-talktalk: BT now cheaper AND better complaints record
- sky-vs-talktalk: Sky now cheaper AND far better complaints record
- sky-vs-virgin-media: both genuinely decent on Ofcom despite very
  different Trustpilot scores
- ee-vs-bt: both BT Group brands, EE's complaints record improved to
  the industry average, EE's automatic mobile-backup differentiator

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$65</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L97" headerRowCount="1">
-  <autoFilter ref="A1:L97"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L98" headerRowCount="1">
+  <autoFilter ref="A1:L98"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L64" headerRowCount="1">
-  <autoFilter ref="A1:L64"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L65" headerRowCount="1">
+  <autoFilter ref="A1:L65"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3987,38 +3987,38 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>audit-broken-links-redirects</t>
+          <t>content-refresh-4-thin-comparison-pages</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Crawlability</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Add routine broken-link and redirect reporting</t>
+          <t>Deep rewrite: 4 thin comparison pages (29th-32nd content-priority-analysis targets)</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr"/>
@@ -4031,38 +4031,38 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-now-broadband-provider-page</t>
+          <t>audit-broken-links-redirects</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Crawlability</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
+          <t>Add routine broken-link and redirect reporting</t>
         </is>
       </c>
       <c r="F75" s="3" t="n">
         <v>44</v>
       </c>
       <c r="G75" s="3" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr"/>
@@ -4075,7 +4075,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-how-to-switch-broadband-guide</t>
+          <t>content-refresh-now-broadband-provider-page</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -4090,18 +4090,18 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Update: How to Switch Broadband Provider guide (25th content-priority-analysis target)</t>
+          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
         <v>44</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -4119,7 +4119,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-youfibre-provider-page</t>
+          <t>content-refresh-how-to-switch-broadband-guide</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -4134,18 +4134,18 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
+          <t>Update: How to Switch Broadband Provider guide (25th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F77" s="3" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-providers-uk-guide</t>
+          <t>content-refresh-youfibre-provider-page</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -4178,14 +4178,14 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
+          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -4207,12 +4207,12 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>bet-annual-research-report</t>
+          <t>content-refresh-best-broadband-providers-uk-guide</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -4222,23 +4222,23 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F79" s="3" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr"/>
@@ -4251,12 +4251,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-without-phone-line-guide</t>
+          <t>bet-annual-research-report</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -4266,23 +4266,23 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
         <v>41</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr"/>
@@ -4295,7 +4295,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-bt-vs-virgin-media-comparison</t>
+          <t>content-refresh-broadband-without-phone-line-guide</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -4310,14 +4310,14 @@
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F81" s="3" t="n">
         <v>41</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-moving-house-guide</t>
+          <t>content-refresh-bt-vs-virgin-media-comparison</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -4354,14 +4354,14 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -4383,7 +4383,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-satellite-broadband-uk-guide</t>
+          <t>content-refresh-broadband-moving-house-guide</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -4398,14 +4398,14 @@
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F83" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G83" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
@@ -4427,38 +4427,38 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>bet-componentise-interactive-layer</t>
+          <t>content-refresh-satellite-broadband-uk-guide</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr"/>
@@ -4471,38 +4471,38 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-gaming-guide</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F85" s="3" t="n">
         <v>38</v>
       </c>
       <c r="G85" s="3" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr"/>
@@ -4515,7 +4515,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-social-tariffs-guide</t>
+          <t>content-refresh-best-broadband-for-gaming-guide</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -4530,11 +4530,11 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G86" s="2" t="n">
         <v>34</v>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-working-from-home-guide</t>
+          <t>content-refresh-broadband-social-tariffs-guide</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -4574,14 +4574,14 @@
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F87" s="3" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G87" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
@@ -4603,7 +4603,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-under-20-guide</t>
+          <t>content-refresh-best-broadband-working-from-home-guide</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -4618,14 +4618,14 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -4647,12 +4647,12 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>content-refresh-broadband-deals-under-20-guide</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
@@ -4662,23 +4662,23 @@
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F89" s="3" t="n">
         <v>35</v>
       </c>
       <c r="G89" s="3" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr"/>
@@ -4691,12 +4691,12 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-bt-vs-sky-comparison</t>
+          <t>bet-decouple-content-from-code</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -4706,23 +4706,23 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr"/>
@@ -4735,7 +4735,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
+          <t>content-refresh-bt-vs-sky-comparison</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -4750,14 +4750,14 @@
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F91" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G91" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
@@ -4779,7 +4779,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-price-rises-2026-guide</t>
+          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -4794,14 +4794,14 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-full-fibre-broadband-explained-guide</t>
+          <t>content-refresh-broadband-price-rises-2026-guide</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -4838,14 +4838,14 @@
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="F93" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G93" s="3" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
@@ -4867,7 +4867,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-students-guide</t>
+          <t>content-refresh-full-fibre-broadband-explained-guide</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -4882,14 +4882,14 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-streaming-guide</t>
+          <t>content-refresh-best-broadband-for-students-guide</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -4926,14 +4926,14 @@
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F95" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G95" s="3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
@@ -4955,7 +4955,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-can-i-leave-broadband-early-guide</t>
+          <t>content-refresh-best-broadband-for-streaming-guide</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -4970,14 +4970,14 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
@@ -4999,7 +4999,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
+          <t>content-refresh-can-i-leave-broadband-early-guide</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -5014,11 +5014,11 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F97" s="3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G97" s="3" t="n">
         <v>26</v>
@@ -5037,8 +5037,52 @@
       <c r="K97" s="3" t="inlineStr"/>
       <c r="L97" s="3" t="inlineStr"/>
     </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G98" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr"/>
+      <c r="K98" s="2" t="inlineStr"/>
+      <c r="L98" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L97"/>
+  <autoFilter ref="A1:L98"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7790,7 +7834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10059,53 +10103,53 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Crawlability</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Add routine broken-link and redirect reporting</t>
+          <t>Deep rewrite: 4 thin comparison pages (29th-32nd content-priority-analysis targets)</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Monitor broken inbound and internal URLs and maintain relevant one-hop redirects.</t>
+          <t>Final 4 targets in this batch, all comparison pages with the exact same problem: entirely generic, number-free copy repeating a 'TalkTalk is usually cheaper' claim that is now factually wrong on 2 of the 4 pages -- bt-vs-talktalk and sky-vs-talktalk both still claimed TalkTalk was the cheaper option, when TalkTalk now starts at GBP25/mo, more expensive than both BT (GBP23.99) and Sky (GBP23.00). Rewrote all 4 with real current prices, Ofcom Q1 2026 complaints figures and populated factSnapshot fields: bt-vs-talktalk (BT now cheaper AND better complaints record), sky-vs-talktalk (Sky now cheaper AND far better complaints record), sky-vs-virgin-media (both genuinely decent on Ofcom despite very different Trustpilot scores -- a real, useful pattern this page never mentioned), ee-vs-bt (both BT Group brands, EE's complaints record improved to the industry average, EE's real automatic mobile-backup differentiator). Word counts: 515-&gt;670, 514-&gt;655, 505-&gt;621, 481-&gt;642.</t>
         </is>
       </c>
       <c r="F41" s="3" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Sitewide crawl and redirect report</t>
+          <t>data/provider-comparisons.ts (bt-vs-talktalk, sky-vs-talktalk, sky-vs-virgin-media, ee-vs-bt)</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>BroadbandPicker SEO &amp; Content Plan — Live: Technical SEO</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10115,53 +10159,53 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Crawlability</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
+          <t>Add routine broken-link and redirect reporting</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Seventh target from scripts/analyze_content_priority.py's ranked list: /providers/now-broadband was 386 words with no excerpt or contentSections, and its top-level fields were stale on two counts that research corrected -- contractLengths was still [12] (NOW dropped its flexible 12-month contracts; every current package is now a standard 24-month term, per thinkbroadband's dedicated news item on the change) and monthlyPriceFrom was a stale GBP17.99 against a real current cheapest tier of GBP23 (Full Fibre 100). Rewritten to ~1,450 words with 5 contentSections. The genuinely distinctive finding here, different from every other Trustpilot-vs-Ofcom section written this session: NOW is a real exception to the usual pattern, scoring poorly on BOTH Trustpilot (1.2/5, corrected from a stale 3.2) AND Ofcom's Q4 2025 complaints data (11 per 100k vs the 8 industry average), noticeably worse than sister brand Sky on the same underlying Openreach network -- written up as a genuine data point about support quality diverging from infrastructure quality within the same corporate group, not just review-platform noise. Also corrected trustpilotScore 3.2 -&gt; 1.2.</t>
+          <t>Monitor broken inbound and internal URLs and maintain relevant one-hop redirects.</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
         <v>44</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>data/providers.ts (now-broadband)</t>
+          <t>Sitewide crawl and redirect report</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>BroadbandPicker SEO &amp; Content Plan — Live: Technical SEO</t>
         </is>
       </c>
     </row>
@@ -10181,28 +10225,28 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Update: How to Switch Broadband Provider guide (25th content-priority-analysis target)</t>
+          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Twenty-fifth target: /guides/how-to-switch-broadband-uk (6,000/mo volume) was already excellent -- 1,913 words, dated citations, real Automatic Compensation Scheme figures (GBP6.46/day, GBP32.31 per missed appointment), no thinness or staleness flags. This was a targeted enhancement rather than a rewrite: added the one genuinely relevant, on-topic development the page was missing -- Ofcom closed its dedicated One Touch Switch enforcement programme on 11 June 2026 after finding more than 2 million customers had already used it successfully, confirming it as the industry's permanent standard rather than a still-bedding-in process. Added this to the intro, a new FAQ, and the guide's keyTakeaways/sources. Word count 1,913 -&gt; 2,043.</t>
+          <t>Seventh target from scripts/analyze_content_priority.py's ranked list: /providers/now-broadband was 386 words with no excerpt or contentSections, and its top-level fields were stale on two counts that research corrected -- contractLengths was still [12] (NOW dropped its flexible 12-month contracts; every current package is now a standard 24-month term, per thinkbroadband's dedicated news item on the change) and monthlyPriceFrom was a stale GBP17.99 against a real current cheapest tier of GBP23 (Full Fibre 100). Rewritten to ~1,450 words with 5 contentSections. The genuinely distinctive finding here, different from every other Trustpilot-vs-Ofcom section written this session: NOW is a real exception to the usual pattern, scoring poorly on BOTH Trustpilot (1.2/5, corrected from a stale 3.2) AND Ofcom's Q4 2025 complaints data (11 per 100k vs the 8 industry average), noticeably worse than sister brand Sky on the same underlying Openreach network -- written up as a genuine data point about support quality diverging from infrastructure quality within the same corporate group, not just review-platform noise. Also corrected trustpilotScore 3.2 -&gt; 1.2.</t>
         </is>
       </c>
       <c r="F43" s="3" t="n">
         <v>44</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (how-to-switch-broadband-uk), data/guides.ts</t>
+          <t>data/providers.ts (now-broadband)</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
@@ -10217,7 +10261,7 @@
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10237,28 +10281,28 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
+          <t>Update: How to Switch Broadband Provider guide (25th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Eighth target from scripts/analyze_content_priority.py's ranked list: /providers/youfibre was 397 words with no excerpt or contentSections. Rewritten to ~1,575 words with 6 contentSections. The standout finding, verified against a primary Virgin Media O2 press release after a first-pass WebSearch AI summary over-stated it as a done deal: YouFibre's parent company, Substantial Group (Netomnia), is being acquired for GBP2bn by nexfibre (a joint venture of InfraVia, Liberty Global and Telefonica), which then plans to resell the YouFibre/Brsk retail brands to Virgin Media O2 for GBP150m -- announced Feb 2026, referred to the CMA for a Phase 2 investigation on 1 July 2026, and NOT yet completed (expected ~Q3 2026 at the earliest). Also wrote up the real, documented fallout from the March 2026 Brsk-to-YouFibre customer migration (billing errors, login/password-reset failures, reported speed drops, overwhelmed support chat), sourced from ISPreview rather than the vague pre-existing 'Trustpilot sentiment has been mixed' line. Updated the speeds array to the real current tiers (200/1000/2000/8000 Mbps symmetrical, replacing stale 200/900/1800) and contractLengths from [1,12,24] to [1,24] to match the two options confirmed by current pricing research.</t>
+          <t>Twenty-fifth target: /guides/how-to-switch-broadband-uk (6,000/mo volume) was already excellent -- 1,913 words, dated citations, real Automatic Compensation Scheme figures (GBP6.46/day, GBP32.31 per missed appointment), no thinness or staleness flags. This was a targeted enhancement rather than a rewrite: added the one genuinely relevant, on-topic development the page was missing -- Ofcom closed its dedicated One Touch Switch enforcement programme on 11 June 2026 after finding more than 2 million customers had already used it successfully, confirming it as the industry's permanent standard rather than a still-bedding-in process. Added this to the intro, a new FAQ, and the guide's keyTakeaways/sources. Word count 1,913 -&gt; 2,043.</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>data/providers.ts (youfibre)</t>
+          <t>app/guides/[slug]/page.tsx (how-to-switch-broadband-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -10273,7 +10317,7 @@
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10293,19 +10337,19 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
+          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Ninth target from scripts/analyze_content_priority.py's ranked list. This ranking page's data was badly stale: it cited Q4 2025 Ofcom complaints figures and June-2026 Trustpilot scores that had already been superseded by this site's own freshly-researched provider pages (Sky, NOW Broadband, BT, Virgin Media, EE, Plusnet, Vodafone, TalkTalk from earlier this session). Rather than re-researching each provider from scratch, cross-referenced this page's ranking table against data/providers.ts's own already-vetted current fields (price, Trustpilot, reviewedDate) and fetched a fresh single-source Ofcom Q1 2026 complaints table (published 23 July 2026, record-low industry average of 6 per 100k) to replace the mixed-quarter data. Corrected several materially wrong claims: TalkTalk was still framed as 'budget only' at GBP19.99 when it is now GBP25 and no longer the cheapest big-name option; Community Fibre was described as 'London-only' when coverage has expanded into Surrey and Sussex; EE's 'best for reliability' halo no longer holds under Q1 2026 data (6 per 100k, tied with Virgin Media, not uniquely best). Added a new section contrasting sister brands Sky (5 per 100k) and NOW Broadband (11 per 100k, different quarter, footnoted) on the identical Openreach network, a genuine support-quality data point. Word count 872 -&gt; 1,333.</t>
+          <t>Eighth target from scripts/analyze_content_priority.py's ranked list: /providers/youfibre was 397 words with no excerpt or contentSections. Rewritten to ~1,575 words with 6 contentSections. The standout finding, verified against a primary Virgin Media O2 press release after a first-pass WebSearch AI summary over-stated it as a done deal: YouFibre's parent company, Substantial Group (Netomnia), is being acquired for GBP2bn by nexfibre (a joint venture of InfraVia, Liberty Global and Telefonica), which then plans to resell the YouFibre/Brsk retail brands to Virgin Media O2 for GBP150m -- announced Feb 2026, referred to the CMA for a Phase 2 investigation on 1 July 2026, and NOT yet completed (expected ~Q3 2026 at the earliest). Also wrote up the real, documented fallout from the March 2026 Brsk-to-YouFibre customer migration (billing errors, login/password-reset failures, reported speed drops, overwhelmed support chat), sourced from ISPreview rather than the vague pre-existing 'Trustpilot sentiment has been mixed' line. Updated the speeds array to the real current tiers (200/1000/2000/8000 Mbps symmetrical, replacing stale 200/900/1800) and contractLengths from [1,12,24] to [1,24] to match the two options confirmed by current pricing research.</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
@@ -10314,7 +10358,7 @@
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-providers-uk), data/guides.ts</t>
+          <t>data/providers.ts (youfibre)</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
@@ -10339,7 +10383,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -10349,43 +10393,43 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
+          <t>Ninth target from scripts/analyze_content_priority.py's ranked list. This ranking page's data was badly stale: it cited Q4 2025 Ofcom complaints figures and June-2026 Trustpilot scores that had already been superseded by this site's own freshly-researched provider pages (Sky, NOW Broadband, BT, Virgin Media, EE, Plusnet, Vodafone, TalkTalk from earlier this session). Rather than re-researching each provider from scratch, cross-referenced this page's ranking table against data/providers.ts's own already-vetted current fields (price, Trustpilot, reviewedDate) and fetched a fresh single-source Ofcom Q1 2026 complaints table (published 23 July 2026, record-low industry average of 6 per 100k) to replace the mixed-quarter data. Corrected several materially wrong claims: TalkTalk was still framed as 'budget only' at GBP19.99 when it is now GBP25 and no longer the cheapest big-name option; Community Fibre was described as 'London-only' when coverage has expanded into Surrey and Sussex; EE's 'best for reliability' halo no longer holds under Q1 2026 data (6 per 100k, tied with Virgin Media, not uniquely best). Added a new section contrasting sister brands Sky (5 per 100k) and NOW Broadband (11 per 100k, different quarter, footnoted) on the identical Openreach network, a genuine support-quality data point. Word count 872 -&gt; 1,333.</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>New annual research page + methodology extension</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-providers-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>research/uk-broadband-customer-satisfaction methodology</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10395,7 +10439,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -10405,43 +10449,43 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Tenth target from scripts/analyze_content_priority.py's ranked list: 770 words, stale pricing table (every one of 8 providers priced against months-old figures already corrected on this site's own provider pages), and a wrong PSTN switch-off date ('by the end of 2027' -- the real, now-locked-in date is 31 January 2027). Rewrote using the same PSTN research gathered for the best-phone-and-broadband-deals refresh earlier this session (5.2m -&gt; 3.2m migration stat, Ofcom's 1-hour power-cut battery backup minimum, the PSTN Charter's telecare protections), added a genuinely missing section -- 'What happens to a home phone during a power cut?' -- since the old version covered whether a line is needed at all but never addressed the actual practical question once Digital Voice is the default. Refreshed all 8 provider prices against data/providers.ts's own current fields, updated Virgin Media coverage 52% (was 53%) and added Ofcom's Spring 2026 Connected Nations split (89% gigabit-capable, 82% full fibre, 93% urban vs 66% rural). Word count 770 -&gt; 1,196; left just under the self-imposed 1,200-word floor rather than pad.</t>
+          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
         </is>
       </c>
       <c r="F47" s="3" t="n">
         <v>41</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-without-phone-line), data/guides.ts</t>
+          <t>New annual research page + methodology extension</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>research/uk-broadband-customer-satisfaction methodology</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -10461,19 +10505,19 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Twenty-first target from the wider top-30 content-priority-analysis list: 526 words of entirely generic, number-free copy ('BT has no setup fee in the current dataset' -- itself wrong, BT's setup fee is GBP30). Rewrote using already-vetted current data from this session's own BT and Virgin Media provider-page work: BT from GBP23.99/mo (24-month, 98% coverage, Trustpilot 4.0/1.5 two-page split) vs Virgin Media from GBP33.00/mo (18-month, 52% coverage, 1,130Mbps fastest widely available speed, Trustpilot 1.4 but a genuinely better Q1 2026 Ofcom complaints record than BT, 6 vs 7 per 100k). Added the genuinely important practical point this page never covered: switching to Virgin Media never qualifies for One Touch Switch since it runs on a separate network from Openreach. Populated the previously-empty factSnapshot field. Word count 526 -&gt; 718.</t>
+          <t>Tenth target from scripts/analyze_content_priority.py's ranked list: 770 words, stale pricing table (every one of 8 providers priced against months-old figures already corrected on this site's own provider pages), and a wrong PSTN switch-off date ('by the end of 2027' -- the real, now-locked-in date is 31 January 2027). Rewrote using the same PSTN research gathered for the best-phone-and-broadband-deals refresh earlier this session (5.2m -&gt; 3.2m migration stat, Ofcom's 1-hour power-cut battery backup minimum, the PSTN Charter's telecare protections), added a genuinely missing section -- 'What happens to a home phone during a power cut?' -- since the old version covered whether a line is needed at all but never addressed the actual practical question once Digital Voice is the default. Refreshed all 8 provider prices against data/providers.ts's own current fields, updated Virgin Media coverage 52% (was 53%) and added Ofcom's Spring 2026 Connected Nations split (89% gigabit-capable, 82% full fibre, 93% urban vs 66% rural). Word count 770 -&gt; 1,196; left just under the self-imposed 1,200-word floor rather than pad.</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
         <v>41</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -10482,7 +10526,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>data/provider-comparisons.ts (bt-vs-virgin-media)</t>
+          <t>app/guides/[slug]/page.tsx (broadband-without-phone-line), data/guides.ts</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -10497,7 +10541,7 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10517,19 +10561,19 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Eleventh target from scripts/analyze_content_priority.py's ranked list: 948 words, structurally sound (evergreen checklist format) but missing a genuinely newsworthy development -- Ofcom closed its One Touch Switch enforcement case on 11 June 2026 after finding more than 2 million customers had already used the process successfully, meaning it is now the industry's permanent standard rather than a monitored pilot, which the old copy still implied. Added this, plus a genuinely missing section on what a house move means for a home phone line given the 31 January 2027 PSTN switch-off (reusing research from the phone-and-broadband and broadband-without-phone-line refreshes earlier this session), Ofcom's Spring 2026 coverage split for the 'check availability' step, and corrected the ETC explanation to reflect Ofcom's actual cap rule (remaining payments, ex-VAT) rather than a flat multiplication. Re-verified the pre-existing GBP183.60/year switching-saving stat against fresh 2026 sources (found independently corroborated) and added the 4.2m/GBP100-240 social tariff stat already used elsewhere on this site. Word count 948 -&gt; 1,446.</t>
+          <t>Twenty-first target from the wider top-30 content-priority-analysis list: 526 words of entirely generic, number-free copy ('BT has no setup fee in the current dataset' -- itself wrong, BT's setup fee is GBP30). Rewrote using already-vetted current data from this session's own BT and Virgin Media provider-page work: BT from GBP23.99/mo (24-month, 98% coverage, Trustpilot 4.0/1.5 two-page split) vs Virgin Media from GBP33.00/mo (18-month, 52% coverage, 1,130Mbps fastest widely available speed, Trustpilot 1.4 but a genuinely better Q1 2026 Ofcom complaints record than BT, 6 vs 7 per 100k). Added the genuinely important practical point this page never covered: switching to Virgin Media never qualifies for One Touch Switch since it runs on a separate network from Openreach. Populated the previously-empty factSnapshot field. Word count 526 -&gt; 718.</t>
         </is>
       </c>
       <c r="F49" s="3" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
@@ -10538,7 +10582,7 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-moving-house), data/guides.ts</t>
+          <t>data/provider-comparisons.ts (bt-vs-virgin-media)</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
@@ -10553,7 +10597,7 @@
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10573,19 +10617,19 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Twelfth target from scripts/analyze_content_priority.py's ranked list, and the page whose DATE_RE regex bug was found and fixed earlier this session (58.2 -&gt; 53.2) without ever getting a content rewrite. The old copy was generic to the point of naming no real prices at all -- 'Starlink is the most visible option' with zero named plans, figures or alternatives. Rewritten with real, current Starlink UK pricing (Residential 100/200/Max at GBP40/60/80 per month, Roam at GBP55-100, Standard Kit GBP449 commonly discounted to ~GBP299 or free on Max), and a genuinely current news item: Starlink's Global Roam plan stopped taking new customers 15 July 2026 and was withdrawn entirely for existing customers on 17 August 2026, one week before this rewrite. Named 2 real smaller alternatives (SkyDSL, Bigblu Broadband) and clarified that Eutelsat/OneWeb, despite frequent mention alongside Starlink, sells no UK consumer home-broadband plans at all. Word count 437 -&gt; 1,038.</t>
+          <t>Eleventh target from scripts/analyze_content_priority.py's ranked list: 948 words, structurally sound (evergreen checklist format) but missing a genuinely newsworthy development -- Ofcom closed its One Touch Switch enforcement case on 11 June 2026 after finding more than 2 million customers had already used the process successfully, meaning it is now the industry's permanent standard rather than a monitored pilot, which the old copy still implied. Added this, plus a genuinely missing section on what a house move means for a home phone line given the 31 January 2027 PSTN switch-off (reusing research from the phone-and-broadband and broadband-without-phone-line refreshes earlier this session), Ofcom's Spring 2026 coverage split for the 'check availability' step, and corrected the ETC explanation to reflect Ofcom's actual cap rule (remaining payments, ex-VAT) rather than a flat multiplication. Re-verified the pre-existing GBP183.60/year switching-saving stat against fresh 2026 sources (found independently corroborated) and added the 4.2m/GBP100-240 social tariff stat already used elsewhere on this site. Word count 948 -&gt; 1,446.</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -10594,7 +10638,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>data/priority-pages.ts (satellite)</t>
+          <t>app/guides/[slug]/page.tsx (broadband-moving-house), data/guides.ts</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -10619,53 +10663,53 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+          <t>Twelfth target from scripts/analyze_content_priority.py's ranked list, and the page whose DATE_RE regex bug was found and fixed earlier this session (58.2 -&gt; 53.2) without ever getting a content rewrite. The old copy was generic to the point of naming no real prices at all -- 'Starlink is the most visible option' with zero named plans, figures or alternatives. Rewritten with real, current Starlink UK pricing (Residential 100/200/Max at GBP40/60/80 per month, Roam at GBP55-100, Standard Kit GBP449 commonly discounted to ~GBP299 or free on Max), and a genuinely current news item: Starlink's Global Roam plan stopped taking new customers 15 July 2026 and was withdrawn entirely for existing customers on 17 August 2026, one week before this rewrite. Named 2 real smaller alternatives (SkyDSL, Bigblu Broadband) and clarified that Eutelsat/OneWeb, despite frequent mention alongside Starlink, sells no UK consumer home-broadband plans at all. Word count 437 -&gt; 1,038.</t>
         </is>
       </c>
       <c r="F51" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>components/</t>
+          <t>data/priority-pages.ts (satellite)</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L51" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10675,53 +10719,53 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Thirteenth target from scripts/analyze_content_priority.py's ranked list: 836 words with stale provider prices (EE GBP26.99, Community Fibre GBP21.99, Hyperoptic GBP22, BT GBP30.99, all already corrected on this site's own provider pages) and a wrong Community Fibre top-tier speed claim (920Mbps symmetrical, against the real current 3,000Mbps top tier confirmed in data/providers.ts). Refreshed all 5 existing provider picks against already-vetted current pricing, and added a genuinely new 6th pick, Zen Internet, for a use case the old page didn't cover at all: hosting a private game server, where Zen's free static IP (already documented on its own provider page) is a real, specific advantage over every other provider on the list. Added a short section on how 24-month contracts and scheduled price rises affect the real two-year cost of a gaming-suitable package. Word count 836 -&gt; 1,184; left just under the self-imposed 1,200-word floor rather than pad.</t>
+          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
         <v>38</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-gaming-uk), data/guides.ts</t>
+          <t>components/</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Functionality pillar</t>
         </is>
       </c>
     </row>
@@ -10741,16 +10785,16 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Fourteenth target from scripts/analyze_content_priority.py's ranked list: 777 words with a materially wrong 'cheapest tariff' claim -- Vodafone Together Social was listed at GBP12.50/mo for 38Mbps and named the cheapest option, but the real current Vodafone Essentials Broadband tariff is GBP20/mo for 73Mbps (verified directly against Vodafone's own tariff page), meaning Virgin Media Essential Broadband and Community Fibre Essential (both genuinely GBP12.50/mo) are actually jointly cheapest. Also corrected Virgin Media's own tariff, which the old page listed at GBP20/mo. Added a genuinely newsworthy find: a thinkbroadband report published in August 2026 (days before this rewrite) tested how easy major providers make it to find their own social tariffs and scored BT, Sky, Virgin Media and Vodafone poorly, with a pointed BT quote, against smaller altnets scoring better. Corrected the eligibility table (Sky accepts UC/PC only, existing customers only, a real restriction the old page omitted) and added KCOM's Hull-only tariff. Refreshed the awareness stat with the newer, more specific thinkbroadband figures (34% aware, 8.6% UC take-up). Word count 777 -&gt; 1,161.</t>
+          <t>Thirteenth target from scripts/analyze_content_priority.py's ranked list: 836 words with stale provider prices (EE GBP26.99, Community Fibre GBP21.99, Hyperoptic GBP22, BT GBP30.99, all already corrected on this site's own provider pages) and a wrong Community Fibre top-tier speed claim (920Mbps symmetrical, against the real current 3,000Mbps top tier confirmed in data/providers.ts). Refreshed all 5 existing provider picks against already-vetted current pricing, and added a genuinely new 6th pick, Zen Internet, for a use case the old page didn't cover at all: hosting a private game server, where Zen's free static IP (already documented on its own provider page) is a real, specific advantage over every other provider on the list. Added a short section on how 24-month contracts and scheduled price rises affect the real two-year cost of a gaming-suitable package. Word count 836 -&gt; 1,184; left just under the self-imposed 1,200-word floor rather than pad.</t>
         </is>
       </c>
       <c r="F53" s="3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G53" s="3" t="n">
         <v>34</v>
@@ -10762,7 +10806,7 @@
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-social-tariffs-uk), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-gaming-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
@@ -10797,19 +10841,19 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Fifteenth target from scripts/analyze_content_priority.py's ranked list: 565 words, no real prices anywhere, and a stale 'EE is consistently rated the most reliable major UK broadband provider' claim that no longer holds under this session's own Q1 2026 Ofcom complaints research. Rewrote with real current prices for Community Fibre, Hyperoptic, Zen Internet and BT, and added a genuinely new section this page never had: when a business-grade line (static IP, faster fault-fix SLA) is actually worth it for a freelancer or remote worker over a residential package, using real Vodafone Business/Zen Business/Sky Business pricing already researched for this site's business broadband guide. Added concrete video-call upload-bandwidth guidance (3-4 Mbps per HD call) rather than vague 'upload matters' framing. Word count 565 -&gt; 986.</t>
+          <t>Fourteenth target from scripts/analyze_content_priority.py's ranked list: 777 words with a materially wrong 'cheapest tariff' claim -- Vodafone Together Social was listed at GBP12.50/mo for 38Mbps and named the cheapest option, but the real current Vodafone Essentials Broadband tariff is GBP20/mo for 73Mbps (verified directly against Vodafone's own tariff page), meaning Virgin Media Essential Broadband and Community Fibre Essential (both genuinely GBP12.50/mo) are actually jointly cheapest. Also corrected Virgin Media's own tariff, which the old page listed at GBP20/mo. Added a genuinely newsworthy find: a thinkbroadband report published in August 2026 (days before this rewrite) tested how easy major providers make it to find their own social tariffs and scored BT, Sky, Virgin Media and Vodafone poorly, with a pointed BT quote, against smaller altnets scoring better. Corrected the eligibility table (Sky accepts UC/PC only, existing customers only, a real restriction the old page omitted) and added KCOM's Hull-only tariff. Refreshed the awareness stat with the newer, more specific thinkbroadband figures (34% aware, 8.6% UC take-up). Word count 777 -&gt; 1,161.</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
@@ -10818,7 +10862,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-working-from-home), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-social-tariffs-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -10853,19 +10897,19 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Sixteenth target from scripts/analyze_content_priority.py's ranked list, and the one with the largest factual break of this whole refresh sequence: the page's entire premise named NOW Broadband and TalkTalk as 'the most common names in this price bracket,' but both now start above GBP20/mo (NOW at GBP23, TalkTalk at GBP25, both already corrected on their own provider pages this session). Rebuilt the page around who is actually under GBP20 today by querying data/providers.ts directly for every provider with monthlyPriceFrom &lt; 20: Community Fibre (GBP12.50), Onestream (GBP18.50, 94% Openreach coverage -- the most realistic pick for most addresses), Gigaclear (GBP19.00, rural symmetrical), toob (GBP19.50) and Trooli (GBP19.99). Also caught and excluded Shell Energy (GBP19.99 in the data file) after finding its own provider-page highlights note it closed to new customers and migrated to TalkTalk in 2024 -- an old, non-orderable plan that would have been a real error to list as a current deal. Word count 608 -&gt; 890.</t>
+          <t>Fifteenth target from scripts/analyze_content_priority.py's ranked list: 565 words, no real prices anywhere, and a stale 'EE is consistently rated the most reliable major UK broadband provider' claim that no longer holds under this session's own Q1 2026 Ofcom complaints research. Rewrote with real current prices for Community Fibre, Hyperoptic, Zen Internet and BT, and added a genuinely new section this page never had: when a business-grade line (static IP, faster fault-fix SLA) is actually worth it for a freelancer or remote worker over a residential package, using real Vodafone Business/Zen Business/Sky Business pricing already researched for this site's business broadband guide. Added concrete video-call upload-bandwidth guidance (3-4 Mbps per HD call) rather than vague 'upload matters' framing. Word count 565 -&gt; 986.</t>
         </is>
       </c>
       <c r="F55" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
@@ -10874,7 +10918,7 @@
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-deals-under-20), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-working-from-home), data/guides.ts</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
@@ -10899,7 +10943,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -10909,43 +10953,43 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
+          <t>Sixteenth target from scripts/analyze_content_priority.py's ranked list, and the one with the largest factual break of this whole refresh sequence: the page's entire premise named NOW Broadband and TalkTalk as 'the most common names in this price bracket,' but both now start above GBP20/mo (NOW at GBP23, TalkTalk at GBP25, both already corrected on their own provider pages this session). Rebuilt the page around who is actually under GBP20 today by querying data/providers.ts directly for every provider with monthlyPriceFrom &lt; 20: Community Fibre (GBP12.50), Onestream (GBP18.50, 94% Openreach coverage -- the most realistic pick for most addresses), Gigaclear (GBP19.00, rural symmetrical), toob (GBP19.50) and Trooli (GBP19.99). Also caught and excluded Shell Energy (GBP19.99 in the data file) after finding its own provider-page highlights note it closed to new customers and migrated to TalkTalk in 2024 -- an old, non-orderable plan that would have been a real error to list as a current deal. Word count 608 -&gt; 890.</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
         <v>35</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-under-20), data/guides.ts</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>None, but easier before the guide count grows further</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10955,7 +10999,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -10965,43 +11009,43 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
+          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
       <c r="F57" s="3" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
+          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L57" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -11021,19 +11065,19 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
+          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -11042,7 +11086,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
+          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -11077,19 +11121,19 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
+          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
         </is>
       </c>
       <c r="F59" s="3" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
@@ -11098,7 +11142,7 @@
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
+          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
@@ -11133,19 +11177,19 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
+          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -11154,7 +11198,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -11169,7 +11213,7 @@
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -11189,19 +11233,19 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
+          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
         </is>
       </c>
       <c r="F61" s="3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
@@ -11210,7 +11254,7 @@
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
@@ -11245,19 +11289,19 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
+          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -11266,7 +11310,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -11301,19 +11345,19 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
+          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
         </is>
       </c>
       <c r="F63" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
@@ -11322,7 +11366,7 @@
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
@@ -11357,16 +11401,16 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
+          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G64" s="2" t="n">
         <v>26</v>
@@ -11378,27 +11422,83 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
+          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G65" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
           <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
         </is>
       </c>
-      <c r="J64" s="2" t="inlineStr">
+      <c r="J65" s="3" t="inlineStr">
         <is>
           <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
-      <c r="K64" s="2" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L64" s="2" t="inlineStr">
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
         <is>
           <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L64"/>
+  <autoFilter ref="A1:L65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11439,7 +11539,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>96 total (33 page builds, 63 feature/strategy builds); 82 already marked Done.</t>
+          <t>97 total (33 page builds, 64 feature/strategy builds); 83 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh keyword-mapping workbook
Ran scripts/build_keyword_mapping.py against the live site to refresh
docs/broadbandpicker-keyword-mapping.xlsx (the keyword-volume data
source analyze_content_priority.py reads from). Confirms all 33
tracked Content Gap Roadmap pages remain built and live, so there are
no new-page gaps pending; ongoing priority work continues to be
existing-page refreshes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -5968,7 +5968,7 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="31" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
@@ -6069,7 +6069,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -6177,7 +6177,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -6231,7 +6231,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -6285,7 +6285,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -6339,7 +6339,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -6447,7 +6447,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -6501,7 +6501,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -6555,7 +6555,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -6609,7 +6609,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -6663,7 +6663,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -6717,7 +6717,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -6771,7 +6771,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -6825,7 +6825,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -6987,7 +6987,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -7041,7 +7041,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -7149,7 +7149,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -7203,7 +7203,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -7257,7 +7257,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -7311,7 +7311,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -7365,7 +7365,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -7473,7 +7473,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -7527,7 +7527,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -7635,7 +7635,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -7689,7 +7689,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -7743,7 +7743,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -7797,7 +7797,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">

</xml_diff>

<commit_message>
content: correct stale EE figures on EE vs TalkTalk comparison page
First target in the second 13-page batch, and notable for having 38
real GSC AI-feature impressions despite only 390/mo mapped volume --
the highest AI-feature signal of any page in this batch.

The page itself was already well-built, so this was a targeted
correction: EE's price was stale at GBP26.99/mo (real current, already
fixed on EE's own provider page this session, is GBP22.99) and its
speed was overstated at "1.6 Gbps" against EE's real 900 Mbps flagship
tier. Corrected both throughout, and added EE's genuinely improved
Q1 2026 Ofcom complaints figure (6 per 100k, industry average) which
the page previously omitted.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$99</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L98" headerRowCount="1">
-  <autoFilter ref="A1:L98"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L99" headerRowCount="1">
+  <autoFilter ref="A1:L99"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L65" headerRowCount="1">
-  <autoFilter ref="A1:L65"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L66" headerRowCount="1">
+  <autoFilter ref="A1:L66"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3543,38 +3543,38 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>feat-price-drop-alerts</t>
+          <t>content-refresh-ee-vs-talktalk-comparison</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Price-drop alerts</t>
+          <t>Update: EE vs TalkTalk comparison page (33rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr"/>
@@ -3587,7 +3587,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>feat-page-type-ux-redesign</t>
+          <t>feat-price-drop-alerts</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -3597,19 +3597,19 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Page-type UX redesign: deals, providers, guides, postcode hub</t>
+          <t>Price-drop alerts</t>
         </is>
       </c>
       <c r="F65" s="3" t="n">
         <v>49</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
@@ -3618,7 +3618,7 @@
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr"/>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>feat-footer-logo-interactivity</t>
+          <t>feat-page-type-ux-redesign</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3646,18 +3646,18 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Footer logo placement and interactive elements</t>
+          <t>Page-type UX redesign: deals, providers, guides, postcode hub</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -3667,11 +3667,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr"/>
       <c r="K66" s="2" t="inlineStr"/>
-      <c r="L66" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Follow-up 2026-08-23: added Instagram (@broadbandpicker) as a second social pill button next to X, same hover treatment.</t>
-        </is>
-      </c>
+      <c r="L66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n">
@@ -3679,33 +3675,33 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-tv-deals-guide</t>
+          <t>feat-footer-logo-interactivity</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Research-led editorial refresh: Best Broadband and TV Deals guide</t>
+          <t>Footer logo placement and interactive elements</t>
         </is>
       </c>
       <c r="F67" s="3" t="n">
         <v>48</v>
       </c>
       <c r="G67" s="3" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr">
@@ -3715,7 +3711,11 @@
       </c>
       <c r="J67" s="3" t="inlineStr"/>
       <c r="K67" s="3" t="inlineStr"/>
-      <c r="L67" s="3" t="inlineStr"/>
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Follow-up 2026-08-23: added Instagram (@broadbandpicker) as a second social pill button next to X, same hover treatment.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -3723,29 +3723,29 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>audit-core-web-vitals-reporting</t>
+          <t>content-refresh-best-broadband-tv-deals-guide</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Establish monthly Core Web Vitals reporting by template</t>
+          <t>Research-led editorial refresh: Best Broadband and TV Deals guide</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -3754,7 +3754,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr"/>
@@ -3767,38 +3767,38 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>ops-awin-publisher-api-integration</t>
+          <t>audit-core-web-vitals-reporting</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Monetisation</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Direct Awin Publisher API access — programme status and link generation</t>
+          <t>Establish monthly Core Web Vitals reporting by template</t>
         </is>
       </c>
       <c r="F69" s="3" t="n">
         <v>47</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr"/>
@@ -3811,33 +3811,33 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-5g-home-broadband-guide</t>
+          <t>ops-awin-publisher-api-integration</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Monetisation</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best 5G Home Broadband UK guide (4th content-priority-analysis target)</t>
+          <t>Direct Awin Publisher API access — programme status and link generation</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
         <v>47</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
@@ -3855,29 +3855,29 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>audit-mobile-checkout-flow</t>
+          <t>content-refresh-best-5g-home-broadband-guide</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>UX audit</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Mobile checkout-flow audit</t>
+          <t>Deep rewrite: Best 5G Home Broadband UK guide (4th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F71" s="3" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G71" s="3" t="n">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
@@ -3886,7 +3886,7 @@
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr"/>
@@ -3899,29 +3899,29 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-phone-and-broadband-deals-guide</t>
+          <t>audit-mobile-checkout-flow</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX audit</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Phone and Broadband Deals guide (5th content-priority-analysis target)</t>
+          <t>Mobile checkout-flow audit</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
         <v>45</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
@@ -3930,7 +3930,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr"/>
@@ -3943,7 +3943,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-virgin-media-provider-page</t>
+          <t>content-refresh-best-phone-and-broadband-deals-guide</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -3958,18 +3958,18 @@
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Update: Virgin Media provider page Ofcom complaints figure (24th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Phone and Broadband Deals guide (5th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F73" s="3" t="n">
         <v>45</v>
       </c>
       <c r="G73" s="3" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
@@ -3987,7 +3987,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-4-thin-comparison-pages</t>
+          <t>content-refresh-virgin-media-provider-page</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -4002,18 +4002,18 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: 4 thin comparison pages (29th-32nd content-priority-analysis targets)</t>
+          <t>Update: Virgin Media provider page Ofcom complaints figure (24th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
         <v>45</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
@@ -4031,38 +4031,38 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>audit-broken-links-redirects</t>
+          <t>content-refresh-4-thin-comparison-pages</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Crawlability</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Add routine broken-link and redirect reporting</t>
+          <t>Deep rewrite: 4 thin comparison pages (29th-32nd content-priority-analysis targets)</t>
         </is>
       </c>
       <c r="F75" s="3" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G75" s="3" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr"/>
@@ -4075,38 +4075,38 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-now-broadband-provider-page</t>
+          <t>audit-broken-links-redirects</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Crawlability</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
+          <t>Add routine broken-link and redirect reporting</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
         <v>44</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr"/>
@@ -4119,7 +4119,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-how-to-switch-broadband-guide</t>
+          <t>content-refresh-now-broadband-provider-page</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -4134,18 +4134,18 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Update: How to Switch Broadband Provider guide (25th content-priority-analysis target)</t>
+          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F77" s="3" t="n">
         <v>44</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-youfibre-provider-page</t>
+          <t>content-refresh-how-to-switch-broadband-guide</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -4178,18 +4178,18 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
+          <t>Update: How to Switch Broadband Provider guide (25th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
@@ -4207,7 +4207,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-providers-uk-guide</t>
+          <t>content-refresh-youfibre-provider-page</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -4222,14 +4222,14 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
+          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F79" s="3" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
@@ -4251,12 +4251,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>bet-annual-research-report</t>
+          <t>content-refresh-best-broadband-providers-uk-guide</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -4266,23 +4266,23 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr"/>
@@ -4295,12 +4295,12 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-without-phone-line-guide</t>
+          <t>bet-annual-research-report</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -4310,23 +4310,23 @@
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="F81" s="3" t="n">
         <v>41</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr"/>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-bt-vs-virgin-media-comparison</t>
+          <t>content-refresh-broadband-without-phone-line-guide</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -4354,14 +4354,14 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
         <v>41</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -4383,7 +4383,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-moving-house-guide</t>
+          <t>content-refresh-bt-vs-virgin-media-comparison</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -4398,14 +4398,14 @@
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F83" s="3" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G83" s="3" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
@@ -4427,7 +4427,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-satellite-broadband-uk-guide</t>
+          <t>content-refresh-broadband-moving-house-guide</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -4442,14 +4442,14 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -4471,38 +4471,38 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>bet-componentise-interactive-layer</t>
+          <t>content-refresh-satellite-broadband-uk-guide</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F85" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G85" s="3" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr"/>
@@ -4515,38 +4515,38 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-gaming-guide</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F86" s="2" t="n">
         <v>38</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr"/>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-social-tariffs-guide</t>
+          <t>content-refresh-best-broadband-for-gaming-guide</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -4574,11 +4574,11 @@
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F87" s="3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G87" s="3" t="n">
         <v>34</v>
@@ -4603,7 +4603,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-working-from-home-guide</t>
+          <t>content-refresh-broadband-social-tariffs-guide</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -4618,14 +4618,14 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -4647,7 +4647,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-under-20-guide</t>
+          <t>content-refresh-best-broadband-working-from-home-guide</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -4662,14 +4662,14 @@
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F89" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G89" s="3" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
@@ -4691,12 +4691,12 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>content-refresh-broadband-deals-under-20-guide</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -4706,23 +4706,23 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
         <v>35</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr"/>
@@ -4735,12 +4735,12 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-bt-vs-sky-comparison</t>
+          <t>bet-decouple-content-from-code</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -4750,23 +4750,23 @@
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="F91" s="3" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G91" s="3" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr"/>
@@ -4779,7 +4779,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
+          <t>content-refresh-bt-vs-sky-comparison</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -4794,14 +4794,14 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-price-rises-2026-guide</t>
+          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -4838,14 +4838,14 @@
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F93" s="3" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G93" s="3" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
@@ -4867,7 +4867,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-full-fibre-broadband-explained-guide</t>
+          <t>content-refresh-broadband-price-rises-2026-guide</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -4882,14 +4882,14 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-students-guide</t>
+          <t>content-refresh-full-fibre-broadband-explained-guide</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -4926,14 +4926,14 @@
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F95" s="3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G95" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
@@ -4955,7 +4955,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-streaming-guide</t>
+          <t>content-refresh-best-broadband-for-students-guide</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -4970,14 +4970,14 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
@@ -4999,7 +4999,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-can-i-leave-broadband-early-guide</t>
+          <t>content-refresh-best-broadband-for-streaming-guide</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -5014,14 +5014,14 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F97" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G97" s="3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
+          <t>content-refresh-can-i-leave-broadband-early-guide</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F98" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G98" s="2" t="n">
         <v>26</v>
@@ -5081,8 +5081,52 @@
       <c r="K98" s="2" t="inlineStr"/>
       <c r="L98" s="2" t="inlineStr"/>
     </row>
+    <row r="99">
+      <c r="A99" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G99" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="H99" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I99" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J99" s="3" t="inlineStr"/>
+      <c r="K99" s="3" t="inlineStr"/>
+      <c r="L99" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L98"/>
+  <autoFilter ref="A1:L99"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5968,7 +6012,7 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="31" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
@@ -6069,7 +6113,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -6123,7 +6167,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -6177,7 +6221,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -6231,7 +6275,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -6285,7 +6329,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -6339,7 +6383,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -6393,7 +6437,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -6447,7 +6491,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -6501,7 +6545,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -6555,7 +6599,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -6609,7 +6653,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -6663,7 +6707,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -6717,7 +6761,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -6771,7 +6815,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -6825,7 +6869,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -6879,7 +6923,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -6933,7 +6977,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -6987,7 +7031,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -7041,7 +7085,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -7095,7 +7139,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -7149,7 +7193,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -7203,7 +7247,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -7257,7 +7301,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -7311,7 +7355,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -7365,7 +7409,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -7419,7 +7463,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -7473,7 +7517,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -7527,7 +7571,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -7581,7 +7625,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -7635,7 +7679,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -7689,7 +7733,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -7743,7 +7787,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -7797,7 +7841,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -7834,7 +7878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9543,53 +9587,53 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Price-drop alerts</t>
+          <t>Update: EE vs TalkTalk comparison page (33rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>data/provider-live-deals.json already tracks live pricing. An email/notification layer on top ("tell me if broadband in my postcode drops below £X") is mostly wiring, and it's a retention mechanic none of the readable competitors emphasised as much as their comparison tables.</t>
+          <t>First target in the second 13-page batch, and notable for having 38 real GSC AI-feature impressions despite only 390/mo mapped volume -- the highest AI-feature signal of any page examined this batch. The page itself was already well-built (already followed the site's fixed comparison-page H2 structure and dated sourcing, likely produced by the separate autonomous content pipeline on 16 August), so this was a targeted correction: EE's price was stale at GBP26.99/mo (real current, already fixed on EE's own provider page this session, is GBP22.99) and its speed was overstated at '1.6 Gbps' against EE's real current 900 Mbps flagship tier. Corrected both throughout (factSnapshot, verdict, keyDifferences, all 4 FAQs, source dates), and added EE's genuinely improved Q1 2026 Ofcom complaints figure (6 per 100k, industry average) which the page previously omitted.</t>
         </is>
       </c>
       <c r="F31" s="3" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>New subscription flow + data/provider-live-deals.json</t>
+          <t>data/provider-comparisons.ts (ee-vs-talktalk)</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>Email delivery provider</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9604,24 +9648,24 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Page-type UX redesign: deals, providers, guides, postcode hub</t>
+          <t>Price-drop alerts</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>New scripts/analyze_page_type_ux.py scans competitor pages by theme (deals listing, provider review, guide article, postcode/checker hub) rather than homepage-only, against Uswitch, broadband.co.uk, choose.co.uk and MoneySavingExpert (403, reported not bypassed). Confirmed signals: comparison checkboxes near-universal; badge/chip labels on deals listings + review index; TOC on the guide article + one deals listing; pros/cons on provider review + deals; related-content on provider review + deals; rating widget on one deals listing. No dedicated postcode-hub competitor page exists in this vertical. Shipped strictly against confirmed signals: computed Best Value/Fastest/Editor's Pick badges in components/DealTable.tsx; new components/RatingStars.tsx replacing plain-text Trustpilot scores plus a 'How {provider} compares' related-comparisons module on provider pages; a jump-to-section table of contents on guide pages via new lib/extractHeadings.tsx (JSX-tree heading-ID injection, avoids hand-editing 40 existing guide definitions), gated behind 3+ headings; and the same cheapest/fastest badges plus rating stars carried onto postcode-hub provider cards since deals and hub serve the same comparison job.</t>
+          <t>data/provider-live-deals.json already tracks live pricing. An email/notification layer on top ("tell me if broadband in my postcode drops below £X") is mostly wiring, and it's a retention mechanic none of the readable competitors emphasised as much as their comparison tables.</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
         <v>49</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -9630,22 +9674,22 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>components/DealTable.tsx, components/RatingStars.tsx, lib/extractHeadings.tsx, app/providers/[slug]/page.tsx, app/guides/[slug]/page.tsx, app/postcode/[area]/page.tsx</t>
+          <t>New subscription flow + data/provider-live-deals.json</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Email delivery provider</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Functionality pillar</t>
         </is>
       </c>
     </row>
@@ -9665,28 +9709,28 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Footer logo placement and interactive elements</t>
+          <t>Page-type UX redesign: deals, providers, guides, postcode hub</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Extended scripts/analyze_homepage_visual_design.py with footer-specific detection (logo, social icons, accordion/back-to-top, hover density). Confirmed directly in app/layout.tsx (not just inferred from the scan) that the footer had no logo at all. Added components/Logo.tsx (extracted from the header, reused larger in the footer with a tagline), made the 6 footer link columns &lt;details open&gt; elements with a mobile-only collapse toggle (desktop behaves exactly as static headings did, via lg:pointer-events-none, so nothing is at risk of accidental collapse), upgraded the social link to a hover-interactive pill button, and added a 'Back to top' link using the existing global smooth-scroll behaviour.</t>
+          <t>New scripts/analyze_page_type_ux.py scans competitor pages by theme (deals listing, provider review, guide article, postcode/checker hub) rather than homepage-only, against Uswitch, broadband.co.uk, choose.co.uk and MoneySavingExpert (403, reported not bypassed). Confirmed signals: comparison checkboxes near-universal; badge/chip labels on deals listings + review index; TOC on the guide article + one deals listing; pros/cons on provider review + deals; related-content on provider review + deals; rating widget on one deals listing. No dedicated postcode-hub competitor page exists in this vertical. Shipped strictly against confirmed signals: computed Best Value/Fastest/Editor's Pick badges in components/DealTable.tsx; new components/RatingStars.tsx replacing plain-text Trustpilot scores plus a 'How {provider} compares' related-comparisons module on provider pages; a jump-to-section table of contents on guide pages via new lib/extractHeadings.tsx (JSX-tree heading-ID injection, avoids hand-editing 40 existing guide definitions), gated behind 3+ headings; and the same cheapest/fastest badges plus rating stars carried onto postcode-hub provider cards since deals and hub serve the same comparison job.</t>
         </is>
       </c>
       <c r="F33" s="3" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>app/layout.tsx, components/Logo.tsx</t>
+          <t>components/DealTable.tsx, components/RatingStars.tsx, lib/extractHeadings.tsx, app/providers/[slug]/page.tsx, app/guides/[slug]/page.tsx, app/postcode/[area]/page.tsx</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
@@ -9711,38 +9755,38 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Research-led editorial refresh: Best Broadband and TV Deals guide</t>
+          <t>Footer logo placement and interactive elements</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>User-requested application of the same Stage 3/4/4a research process from the Awin content batches to a single existing guide page, /guides/best-broadband-and-tv-deals. Unlike the thin provider stubs rewritten in the Awin batches, this guide was already well-built (tables, methodology, 7 FAQs, real Ofcom citations, last checked 29 July 2026) -- not a stub needing a ground-up rewrite, so this was a verify-and-deepen pass grounded in fresh research rather than a full replacement. Scraped 2 top-ranking competitors (MoneySuperMarket, Uswitch) per Stage 3.0: found MoneySupermarket runs a 15-question FAQ (ours had 7) and leads with an expert-quoted bundling-savings statistic. Traced that claim to its actual primary source rather than citing the secondary restatement: Ofcom's own February 2026 research, savings of £26-£48/month from bundling and pay-TV averaging £12/month within a bundle (23% real-terms fall) -- a stronger, more current, primary-sourced figure than the competitor's 2023-dated stat, added as a new section. Also found and added two genuinely new, specific facts the page didn't have: Virgin Media's Max Volt bundle (real current pricing including its two scheduled rises to April 2028) as a concrete worked example, and Virgin Media's 'Most Reliable Broadband Provider' win at the 2026 Uswitch Telecoms Awards (Opensignal-verified, a genuine third-party measurement). Named the specific Sky bundle example (Sky Stream, Sky TV, Netflix + Full Fibre 300, £35/month) that the existing copy referenced only vaguely. Added 2 new FAQs tied to the new content. Fixed 2 pre-existing em dashes found during the pass (a legitimate en-dash numeric range, '50-100Mbps', was left alone -- not an AI-tell, different typographic use). Updated the page's stated fact-check date and guides.ts updatedDate to 2026-08-24.</t>
+          <t>Extended scripts/analyze_homepage_visual_design.py with footer-specific detection (logo, social icons, accordion/back-to-top, hover density). Confirmed directly in app/layout.tsx (not just inferred from the scan) that the footer had no logo at all. Added components/Logo.tsx (extracted from the header, reused larger in the footer with a tagline), made the 6 footer link columns &lt;details open&gt; elements with a mobile-only collapse toggle (desktop behaves exactly as static headings did, via lg:pointer-events-none, so nothing is at risk of accidental collapse), upgraded the social link to a hover-interactive pill button, and added a 'Back to top' link using the existing global smooth-scroll behaviour.</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
         <v>48</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-and-tv-deals), data/guides.ts</t>
+          <t>app/layout.tsx, components/Logo.tsx</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -9757,7 +9801,7 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9767,29 +9811,29 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Establish monthly Core Web Vitals reporting by template</t>
+          <t>Research-led editorial refresh: Best Broadband and TV Deals guide</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Track LCP, INP and CLS by page template and prioritise JS or image-weight fixes from evidence.</t>
+          <t>User-requested application of the same Stage 3/4/4a research process from the Awin content batches to a single existing guide page, /guides/best-broadband-and-tv-deals. Unlike the thin provider stubs rewritten in the Awin batches, this guide was already well-built (tables, methodology, 7 FAQs, real Ofcom citations, last checked 29 July 2026) -- not a stub needing a ground-up rewrite, so this was a verify-and-deepen pass grounded in fresh research rather than a full replacement. Scraped 2 top-ranking competitors (MoneySuperMarket, Uswitch) per Stage 3.0: found MoneySupermarket runs a 15-question FAQ (ours had 7) and leads with an expert-quoted bundling-savings statistic. Traced that claim to its actual primary source rather than citing the secondary restatement: Ofcom's own February 2026 research, savings of £26-£48/month from bundling and pay-TV averaging £12/month within a bundle (23% real-terms fall) -- a stronger, more current, primary-sourced figure than the competitor's 2023-dated stat, added as a new section. Also found and added two genuinely new, specific facts the page didn't have: Virgin Media's Max Volt bundle (real current pricing including its two scheduled rises to April 2028) as a concrete worked example, and Virgin Media's 'Most Reliable Broadband Provider' win at the 2026 Uswitch Telecoms Awards (Opensignal-verified, a genuine third-party measurement). Named the specific Sky bundle example (Sky Stream, Sky TV, Netflix + Full Fibre 300, £35/month) that the existing copy referenced only vaguely. Added 2 new FAQs tied to the new content. Fixed 2 pre-existing em dashes found during the pass (a legitimate en-dash numeric range, '50-100Mbps', was left alone -- not an AI-tell, different typographic use). Updated the page's stated fact-check date and guides.ts updatedDate to 2026-08-24.</t>
         </is>
       </c>
       <c r="F35" s="3" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
@@ -9798,22 +9842,22 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Sitewide template performance report</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-and-tv-deals), data/guides.ts</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>Field data or representative lab baselines</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>BroadbandPicker SEO &amp; Content Plan — Live: Technical SEO</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9823,53 +9867,53 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Monetisation</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Direct Awin Publisher API access — programme status and link generation</t>
+          <t>Establish monthly Core Web Vitals reporting by template</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>User asked to connect Claude to their Awin account and provided a real API token. There's no one-click connector for Awin (unlike Google Drive/Gmail), so this uses Awin's own Publisher API directly. First live run corrected two wrong assumptions from documentation research: 'programmedetails' requires a specific advertiserId (not a bulk listing endpoint) -- the actual bulk-status endpoint is GET /publishers/{id}/programmes?relationship=X, and 'any' is not a valid value for it (loops joined/pending/suspended/rejected instead; 'notjoined' returns the ~21k whole-platform catalogue so it's excluded from the default and only fetched on request). POST /publishers/{id}/linkbuilder/generate confirmed working, verified against TalkTalk (advertiser 3674). REAL FINDING from the first run, both surfaced to the user and worth acting on: only 4 programmes are joined (TalkTalk, Broadband Genie, Zzoomm, Highland Broadband), 7 pending (Sky ROI, Community Fibre, National Broadband, Trooli, Pine Media, Cuckoo, Zen Internet), and 9 REJECTED including BT (both consumer and business), Vodafone, Plusnet, EE, Virgin Media, Hyperoptic and toob. Cross-checked data/providers.ts: none of the currently-live affiliateUrl values (including TalkTalk, which IS approved) use Awin's awin1.com tracking format -- they're all plain provider URLs, so the site is very likely not earning commission on any current outbound click, joined or not, despite the on-page commercial disclosures implying it might.</t>
+          <t>Track LCP, INP and CLS by page template and prioritise JS or image-weight fixes from evidence.</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
         <v>47</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>scripts/awin_sync.py</t>
+          <t>Sitewide template performance report</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>AWIN_API_TOKEN from the user's Awin account (user menu -&gt; API Credentials)</t>
+          <t>Field data or representative lab baselines</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
+          <t>BroadbandPicker SEO &amp; Content Plan — Live: Technical SEO</t>
         </is>
       </c>
     </row>
@@ -9879,43 +9923,43 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Monetisation</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best 5G Home Broadband UK guide (4th content-priority-analysis target)</t>
+          <t>Direct Awin Publisher API access — programme status and link generation</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Fourth target from scripts/analyze_content_priority.py's ranked list: 30 real GSC AI-feature impressions at 601 words, and the old copy named no real providers or prices at all, just generic 5G-vs-fibre advice. Rewritten to 1,036 words with real current data for all 4 major UK 5G home broadband options: Three (best value, from GBP29/mo, ~150 Mbps), Vodafone GigaCube (cheapest fixed term at GBP21/mo, or a genuine GBP60/mo no-contract option), EE Smart 5G Hub (broadest UK 5G coverage, GBP30-50/mo), and National Broadband (already deeply covered in the Awin-pending batch) framed correctly here as a multi-network specialist rather than a single-network alternative -- it connects to whichever of the 4 UK networks is strongest at a given address, a genuinely different value proposition worth explaining rather than just listing as a fourth option. Found and included a real Trustpilot-vs-Ofcom divergence for Three specifically (4.5 Trustpilot, worst-quartile Ofcom complaints alongside EE and Vodafone) and linked to the full-fibre guide's deeper explanation of that pattern rather than repeating it in full.</t>
+          <t>User asked to connect Claude to their Awin account and provided a real API token. There's no one-click connector for Awin (unlike Google Drive/Gmail), so this uses Awin's own Publisher API directly. First live run corrected two wrong assumptions from documentation research: 'programmedetails' requires a specific advertiserId (not a bulk listing endpoint) -- the actual bulk-status endpoint is GET /publishers/{id}/programmes?relationship=X, and 'any' is not a valid value for it (loops joined/pending/suspended/rejected instead; 'notjoined' returns the ~21k whole-platform catalogue so it's excluded from the default and only fetched on request). POST /publishers/{id}/linkbuilder/generate confirmed working, verified against TalkTalk (advertiser 3674). REAL FINDING from the first run, both surfaced to the user and worth acting on: only 4 programmes are joined (TalkTalk, Broadband Genie, Zzoomm, Highland Broadband), 7 pending (Sky ROI, Community Fibre, National Broadband, Trooli, Pine Media, Cuckoo, Zen Internet), and 9 REJECTED including BT (both consumer and business), Vodafone, Plusnet, EE, Virgin Media, Hyperoptic and toob. Cross-checked data/providers.ts: none of the currently-live affiliateUrl values (including TalkTalk, which IS approved) use Awin's awin1.com tracking format -- they're all plain provider URLs, so the site is very likely not earning commission on any current outbound click, joined or not, despite the on-page commercial disclosures implying it might.</t>
         </is>
       </c>
       <c r="F37" s="3" t="n">
         <v>47</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-5g-home-broadband-uk), data/guides.ts</t>
+          <t>scripts/awin_sync.py</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>AWIN_API_TOKEN from the user's Awin account (user menu -&gt; API Credentials)</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
@@ -9925,7 +9969,7 @@
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-23 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9935,29 +9979,29 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>UX audit</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Mobile checkout-flow audit</t>
+          <t>Deep rewrite: Best 5G Home Broadband UK guide (4th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>The competitor evidence (15k–23k word desktop hubs) is desktop-shaped. On mobile that content needs a different information architecture — sticky summary bar, collapsed sections, thumb-reachable CTAs. Worth a dedicated pass once analytics show where mobile users drop off.</t>
+          <t>Fourth target from scripts/analyze_content_priority.py's ranked list: 30 real GSC AI-feature impressions at 601 words, and the old copy named no real providers or prices at all, just generic 5G-vs-fibre advice. Rewritten to 1,036 words with real current data for all 4 major UK 5G home broadband options: Three (best value, from GBP29/mo, ~150 Mbps), Vodafone GigaCube (cheapest fixed term at GBP21/mo, or a genuine GBP60/mo no-contract option), EE Smart 5G Hub (broadest UK 5G coverage, GBP30-50/mo), and National Broadband (already deeply covered in the Awin-pending batch) framed correctly here as a multi-network specialist rather than a single-network alternative -- it connects to whichever of the 4 UK networks is strongest at a given address, a genuinely different value proposition worth explaining rather than just listing as a fourth option. Found and included a real Trustpilot-vs-Ofcom divergence for Three specifically (4.5 Trustpilot, worst-quartile Ofcom complaints alongside EE and Vodafone) and linked to the full-fibre guide's deeper explanation of that pattern rather than repeating it in full.</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -9966,22 +10010,22 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Sitewide mobile layout</t>
+          <t>app/guides/[slug]/page.tsx (best-5g-home-broadband-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Mobile analytics/drop-off data</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — UX pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -9991,29 +10035,29 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX audit</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Phone and Broadband Deals guide (5th content-priority-analysis target)</t>
+          <t>Mobile checkout-flow audit</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Fifth target from scripts/analyze_content_priority.py's ranked list: the old copy was generic Digital Voice/line-rental advice with no dates, no stats and one pre-existing em dash, at 457 words. Rewritten with the real PSTN switch-off timeline: full shutdown now locked in for 31 January 2027 (moved from the original December 2025 target after Openreach confirmed the technical barriers were resolved), with PSTN customer numbers falling from 5.2 million (July 2024) to 3.2 million (July 2025). Added Ofcom's minimum one-hour battery backup requirement for emergency-services access during a power cut, and the industry PSTN Charter's commitment not to migrate telecare/vulnerable users without confirmed-compatible equipment. Added a real, specific call-plan cost example (TalkTalk's Anytime Calls add-on at GBP12/mo on top of base broadband) to replace the previous fully generic 'compare the whole contract' advice. FAQs expanded from 3 to 5. Fixed the pre-existing em dash in the dek field.</t>
+          <t>The competitor evidence (15k–23k word desktop hubs) is desktop-shaped. On mobile that content needs a different information architecture — sticky summary bar, collapsed sections, thumb-reachable CTAs. Worth a dedicated pass once analytics show where mobile users drop off.</t>
         </is>
       </c>
       <c r="F39" s="3" t="n">
         <v>45</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
@@ -10022,22 +10066,22 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>data/priority-pages.ts (phone)</t>
+          <t>Sitewide mobile layout</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>Mobile analytics/drop-off data</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L39" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — UX pillar</t>
         </is>
       </c>
     </row>
@@ -10057,28 +10101,28 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Update: Virgin Media provider page Ofcom complaints figure (24th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Phone and Broadband Deals guide (5th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Twenty-fourth target, found via the same spot-check pattern that caught EE's stale figure: /providers/virgin-media (63,112/mo volume, already well-built at 1,798 words) was still citing its Q4 2025 Ofcom complaints figure (7 per 100k) with vague framing ('has not appeared among the top complained-about providers in Q1 2026 either'). Replaced with the exact Q1 2026 figure from the same broadbandswitch table used for EE and the price-rises guide: Virgin Media recorded 6 per 100,000, exactly the industry average, a further improvement on its already-decent Q4 2025 position. Added a dedicated source citation and updated reviewedDate.</t>
+          <t>Fifth target from scripts/analyze_content_priority.py's ranked list: the old copy was generic Digital Voice/line-rental advice with no dates, no stats and one pre-existing em dash, at 457 words. Rewritten with the real PSTN switch-off timeline: full shutdown now locked in for 31 January 2027 (moved from the original December 2025 target after Openreach confirmed the technical barriers were resolved), with PSTN customer numbers falling from 5.2 million (July 2024) to 3.2 million (July 2025). Added Ofcom's minimum one-hour battery backup requirement for emergency-services access during a power cut, and the industry PSTN Charter's commitment not to migrate telecare/vulnerable users without confirmed-compatible equipment. Added a real, specific call-plan cost example (TalkTalk's Anytime Calls add-on at GBP12/mo on top of base broadband) to replace the previous fully generic 'compare the whole contract' advice. FAQs expanded from 3 to 5. Fixed the pre-existing em dash in the dek field.</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
         <v>45</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>data/providers.ts (virgin-media)</t>
+          <t>data/priority-pages.ts (phone)</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -10093,7 +10137,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10113,28 +10157,28 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: 4 thin comparison pages (29th-32nd content-priority-analysis targets)</t>
+          <t>Update: Virgin Media provider page Ofcom complaints figure (24th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Final 4 targets in this batch, all comparison pages with the exact same problem: entirely generic, number-free copy repeating a 'TalkTalk is usually cheaper' claim that is now factually wrong on 2 of the 4 pages -- bt-vs-talktalk and sky-vs-talktalk both still claimed TalkTalk was the cheaper option, when TalkTalk now starts at GBP25/mo, more expensive than both BT (GBP23.99) and Sky (GBP23.00). Rewrote all 4 with real current prices, Ofcom Q1 2026 complaints figures and populated factSnapshot fields: bt-vs-talktalk (BT now cheaper AND better complaints record), sky-vs-talktalk (Sky now cheaper AND far better complaints record), sky-vs-virgin-media (both genuinely decent on Ofcom despite very different Trustpilot scores -- a real, useful pattern this page never mentioned), ee-vs-bt (both BT Group brands, EE's complaints record improved to the industry average, EE's real automatic mobile-backup differentiator). Word counts: 515-&gt;670, 514-&gt;655, 505-&gt;621, 481-&gt;642.</t>
+          <t>Twenty-fourth target, found via the same spot-check pattern that caught EE's stale figure: /providers/virgin-media (63,112/mo volume, already well-built at 1,798 words) was still citing its Q4 2025 Ofcom complaints figure (7 per 100k) with vague framing ('has not appeared among the top complained-about providers in Q1 2026 either'). Replaced with the exact Q1 2026 figure from the same broadbandswitch table used for EE and the price-rises guide: Virgin Media recorded 6 per 100,000, exactly the industry average, a further improvement on its already-decent Q4 2025 position. Added a dedicated source citation and updated reviewedDate.</t>
         </is>
       </c>
       <c r="F41" s="3" t="n">
         <v>45</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>data/provider-comparisons.ts (bt-vs-talktalk, sky-vs-talktalk, sky-vs-virgin-media, ee-vs-bt)</t>
+          <t>data/providers.ts (virgin-media)</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
@@ -10159,53 +10203,53 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Crawlability</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Add routine broken-link and redirect reporting</t>
+          <t>Deep rewrite: 4 thin comparison pages (29th-32nd content-priority-analysis targets)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Monitor broken inbound and internal URLs and maintain relevant one-hop redirects.</t>
+          <t>Final 4 targets in this batch, all comparison pages with the exact same problem: entirely generic, number-free copy repeating a 'TalkTalk is usually cheaper' claim that is now factually wrong on 2 of the 4 pages -- bt-vs-talktalk and sky-vs-talktalk both still claimed TalkTalk was the cheaper option, when TalkTalk now starts at GBP25/mo, more expensive than both BT (GBP23.99) and Sky (GBP23.00). Rewrote all 4 with real current prices, Ofcom Q1 2026 complaints figures and populated factSnapshot fields: bt-vs-talktalk (BT now cheaper AND better complaints record), sky-vs-talktalk (Sky now cheaper AND far better complaints record), sky-vs-virgin-media (both genuinely decent on Ofcom despite very different Trustpilot scores -- a real, useful pattern this page never mentioned), ee-vs-bt (both BT Group brands, EE's complaints record improved to the industry average, EE's real automatic mobile-backup differentiator). Word counts: 515-&gt;670, 514-&gt;655, 505-&gt;621, 481-&gt;642.</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Sitewide crawl and redirect report</t>
+          <t>data/provider-comparisons.ts (bt-vs-talktalk, sky-vs-talktalk, sky-vs-virgin-media, ee-vs-bt)</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>BroadbandPicker SEO &amp; Content Plan — Live: Technical SEO</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10215,53 +10259,53 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Crawlability</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
+          <t>Add routine broken-link and redirect reporting</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Seventh target from scripts/analyze_content_priority.py's ranked list: /providers/now-broadband was 386 words with no excerpt or contentSections, and its top-level fields were stale on two counts that research corrected -- contractLengths was still [12] (NOW dropped its flexible 12-month contracts; every current package is now a standard 24-month term, per thinkbroadband's dedicated news item on the change) and monthlyPriceFrom was a stale GBP17.99 against a real current cheapest tier of GBP23 (Full Fibre 100). Rewritten to ~1,450 words with 5 contentSections. The genuinely distinctive finding here, different from every other Trustpilot-vs-Ofcom section written this session: NOW is a real exception to the usual pattern, scoring poorly on BOTH Trustpilot (1.2/5, corrected from a stale 3.2) AND Ofcom's Q4 2025 complaints data (11 per 100k vs the 8 industry average), noticeably worse than sister brand Sky on the same underlying Openreach network -- written up as a genuine data point about support quality diverging from infrastructure quality within the same corporate group, not just review-platform noise. Also corrected trustpilotScore 3.2 -&gt; 1.2.</t>
+          <t>Monitor broken inbound and internal URLs and maintain relevant one-hop redirects.</t>
         </is>
       </c>
       <c r="F43" s="3" t="n">
         <v>44</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>data/providers.ts (now-broadband)</t>
+          <t>Sitewide crawl and redirect report</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>BroadbandPicker SEO &amp; Content Plan — Live: Technical SEO</t>
         </is>
       </c>
     </row>
@@ -10281,28 +10325,28 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Update: How to Switch Broadband Provider guide (25th content-priority-analysis target)</t>
+          <t>Deep rewrite: NOW Broadband provider page (7th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Twenty-fifth target: /guides/how-to-switch-broadband-uk (6,000/mo volume) was already excellent -- 1,913 words, dated citations, real Automatic Compensation Scheme figures (GBP6.46/day, GBP32.31 per missed appointment), no thinness or staleness flags. This was a targeted enhancement rather than a rewrite: added the one genuinely relevant, on-topic development the page was missing -- Ofcom closed its dedicated One Touch Switch enforcement programme on 11 June 2026 after finding more than 2 million customers had already used it successfully, confirming it as the industry's permanent standard rather than a still-bedding-in process. Added this to the intro, a new FAQ, and the guide's keyTakeaways/sources. Word count 1,913 -&gt; 2,043.</t>
+          <t>Seventh target from scripts/analyze_content_priority.py's ranked list: /providers/now-broadband was 386 words with no excerpt or contentSections, and its top-level fields were stale on two counts that research corrected -- contractLengths was still [12] (NOW dropped its flexible 12-month contracts; every current package is now a standard 24-month term, per thinkbroadband's dedicated news item on the change) and monthlyPriceFrom was a stale GBP17.99 against a real current cheapest tier of GBP23 (Full Fibre 100). Rewritten to ~1,450 words with 5 contentSections. The genuinely distinctive finding here, different from every other Trustpilot-vs-Ofcom section written this session: NOW is a real exception to the usual pattern, scoring poorly on BOTH Trustpilot (1.2/5, corrected from a stale 3.2) AND Ofcom's Q4 2025 complaints data (11 per 100k vs the 8 industry average), noticeably worse than sister brand Sky on the same underlying Openreach network -- written up as a genuine data point about support quality diverging from infrastructure quality within the same corporate group, not just review-platform noise. Also corrected trustpilotScore 3.2 -&gt; 1.2.</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
         <v>44</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (how-to-switch-broadband-uk), data/guides.ts</t>
+          <t>data/providers.ts (now-broadband)</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -10317,7 +10361,7 @@
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10337,28 +10381,28 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
+          <t>Update: How to Switch Broadband Provider guide (25th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Eighth target from scripts/analyze_content_priority.py's ranked list: /providers/youfibre was 397 words with no excerpt or contentSections. Rewritten to ~1,575 words with 6 contentSections. The standout finding, verified against a primary Virgin Media O2 press release after a first-pass WebSearch AI summary over-stated it as a done deal: YouFibre's parent company, Substantial Group (Netomnia), is being acquired for GBP2bn by nexfibre (a joint venture of InfraVia, Liberty Global and Telefonica), which then plans to resell the YouFibre/Brsk retail brands to Virgin Media O2 for GBP150m -- announced Feb 2026, referred to the CMA for a Phase 2 investigation on 1 July 2026, and NOT yet completed (expected ~Q3 2026 at the earliest). Also wrote up the real, documented fallout from the March 2026 Brsk-to-YouFibre customer migration (billing errors, login/password-reset failures, reported speed drops, overwhelmed support chat), sourced from ISPreview rather than the vague pre-existing 'Trustpilot sentiment has been mixed' line. Updated the speeds array to the real current tiers (200/1000/2000/8000 Mbps symmetrical, replacing stale 200/900/1800) and contractLengths from [1,12,24] to [1,24] to match the two options confirmed by current pricing research.</t>
+          <t>Twenty-fifth target: /guides/how-to-switch-broadband-uk (6,000/mo volume) was already excellent -- 1,913 words, dated citations, real Automatic Compensation Scheme figures (GBP6.46/day, GBP32.31 per missed appointment), no thinness or staleness flags. This was a targeted enhancement rather than a rewrite: added the one genuinely relevant, on-topic development the page was missing -- Ofcom closed its dedicated One Touch Switch enforcement programme on 11 June 2026 after finding more than 2 million customers had already used it successfully, confirming it as the industry's permanent standard rather than a still-bedding-in process. Added this to the intro, a new FAQ, and the guide's keyTakeaways/sources. Word count 1,913 -&gt; 2,043.</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>data/providers.ts (youfibre)</t>
+          <t>app/guides/[slug]/page.tsx (how-to-switch-broadband-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
@@ -10373,7 +10417,7 @@
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10393,19 +10437,19 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
+          <t>Deep rewrite: YouFibre provider page (8th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Ninth target from scripts/analyze_content_priority.py's ranked list. This ranking page's data was badly stale: it cited Q4 2025 Ofcom complaints figures and June-2026 Trustpilot scores that had already been superseded by this site's own freshly-researched provider pages (Sky, NOW Broadband, BT, Virgin Media, EE, Plusnet, Vodafone, TalkTalk from earlier this session). Rather than re-researching each provider from scratch, cross-referenced this page's ranking table against data/providers.ts's own already-vetted current fields (price, Trustpilot, reviewedDate) and fetched a fresh single-source Ofcom Q1 2026 complaints table (published 23 July 2026, record-low industry average of 6 per 100k) to replace the mixed-quarter data. Corrected several materially wrong claims: TalkTalk was still framed as 'budget only' at GBP19.99 when it is now GBP25 and no longer the cheapest big-name option; Community Fibre was described as 'London-only' when coverage has expanded into Surrey and Sussex; EE's 'best for reliability' halo no longer holds under Q1 2026 data (6 per 100k, tied with Virgin Media, not uniquely best). Added a new section contrasting sister brands Sky (5 per 100k) and NOW Broadband (11 per 100k, different quarter, footnoted) on the identical Openreach network, a genuine support-quality data point. Word count 872 -&gt; 1,333.</t>
+          <t>Eighth target from scripts/analyze_content_priority.py's ranked list: /providers/youfibre was 397 words with no excerpt or contentSections. Rewritten to ~1,575 words with 6 contentSections. The standout finding, verified against a primary Virgin Media O2 press release after a first-pass WebSearch AI summary over-stated it as a done deal: YouFibre's parent company, Substantial Group (Netomnia), is being acquired for GBP2bn by nexfibre (a joint venture of InfraVia, Liberty Global and Telefonica), which then plans to resell the YouFibre/Brsk retail brands to Virgin Media O2 for GBP150m -- announced Feb 2026, referred to the CMA for a Phase 2 investigation on 1 July 2026, and NOT yet completed (expected ~Q3 2026 at the earliest). Also wrote up the real, documented fallout from the March 2026 Brsk-to-YouFibre customer migration (billing errors, login/password-reset failures, reported speed drops, overwhelmed support chat), sourced from ISPreview rather than the vague pre-existing 'Trustpilot sentiment has been mixed' line. Updated the speeds array to the real current tiers (200/1000/2000/8000 Mbps symmetrical, replacing stale 200/900/1800) and contractLengths from [1,12,24] to [1,24] to match the two options confirmed by current pricing research.</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -10414,7 +10458,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-providers-uk), data/guides.ts</t>
+          <t>data/providers.ts (youfibre)</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -10439,7 +10483,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -10449,43 +10493,43 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Deep rewrite: Best Broadband Providers UK ranking guide (9th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
+          <t>Ninth target from scripts/analyze_content_priority.py's ranked list. This ranking page's data was badly stale: it cited Q4 2025 Ofcom complaints figures and June-2026 Trustpilot scores that had already been superseded by this site's own freshly-researched provider pages (Sky, NOW Broadband, BT, Virgin Media, EE, Plusnet, Vodafone, TalkTalk from earlier this session). Rather than re-researching each provider from scratch, cross-referenced this page's ranking table against data/providers.ts's own already-vetted current fields (price, Trustpilot, reviewedDate) and fetched a fresh single-source Ofcom Q1 2026 complaints table (published 23 July 2026, record-low industry average of 6 per 100k) to replace the mixed-quarter data. Corrected several materially wrong claims: TalkTalk was still framed as 'budget only' at GBP19.99 when it is now GBP25 and no longer the cheapest big-name option; Community Fibre was described as 'London-only' when coverage has expanded into Surrey and Sussex; EE's 'best for reliability' halo no longer holds under Q1 2026 data (6 per 100k, tied with Virgin Media, not uniquely best). Added a new section contrasting sister brands Sky (5 per 100k) and NOW Broadband (11 per 100k, different quarter, footnoted) on the identical Openreach network, a genuine support-quality data point. Word count 872 -&gt; 1,333.</t>
         </is>
       </c>
       <c r="F47" s="3" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>New annual research page + methodology extension</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-providers-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>research/uk-broadband-customer-satisfaction methodology</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10495,7 +10539,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -10505,43 +10549,43 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Tenth target from scripts/analyze_content_priority.py's ranked list: 770 words, stale pricing table (every one of 8 providers priced against months-old figures already corrected on this site's own provider pages), and a wrong PSTN switch-off date ('by the end of 2027' -- the real, now-locked-in date is 31 January 2027). Rewrote using the same PSTN research gathered for the best-phone-and-broadband-deals refresh earlier this session (5.2m -&gt; 3.2m migration stat, Ofcom's 1-hour power-cut battery backup minimum, the PSTN Charter's telecare protections), added a genuinely missing section -- 'What happens to a home phone during a power cut?' -- since the old version covered whether a line is needed at all but never addressed the actual practical question once Digital Voice is the default. Refreshed all 8 provider prices against data/providers.ts's own current fields, updated Virgin Media coverage 52% (was 53%) and added Ofcom's Spring 2026 Connected Nations split (89% gigabit-capable, 82% full fibre, 93% urban vs 66% rural). Word count 770 -&gt; 1,196; left just under the self-imposed 1,200-word floor rather than pad.</t>
+          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
         <v>41</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-without-phone-line), data/guides.ts</t>
+          <t>New annual research page + methodology extension</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>research/uk-broadband-customer-satisfaction methodology</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -10561,19 +10605,19 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Without a Phone Line guide (10th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Twenty-first target from the wider top-30 content-priority-analysis list: 526 words of entirely generic, number-free copy ('BT has no setup fee in the current dataset' -- itself wrong, BT's setup fee is GBP30). Rewrote using already-vetted current data from this session's own BT and Virgin Media provider-page work: BT from GBP23.99/mo (24-month, 98% coverage, Trustpilot 4.0/1.5 two-page split) vs Virgin Media from GBP33.00/mo (18-month, 52% coverage, 1,130Mbps fastest widely available speed, Trustpilot 1.4 but a genuinely better Q1 2026 Ofcom complaints record than BT, 6 vs 7 per 100k). Added the genuinely important practical point this page never covered: switching to Virgin Media never qualifies for One Touch Switch since it runs on a separate network from Openreach. Populated the previously-empty factSnapshot field. Word count 526 -&gt; 718.</t>
+          <t>Tenth target from scripts/analyze_content_priority.py's ranked list: 770 words, stale pricing table (every one of 8 providers priced against months-old figures already corrected on this site's own provider pages), and a wrong PSTN switch-off date ('by the end of 2027' -- the real, now-locked-in date is 31 January 2027). Rewrote using the same PSTN research gathered for the best-phone-and-broadband-deals refresh earlier this session (5.2m -&gt; 3.2m migration stat, Ofcom's 1-hour power-cut battery backup minimum, the PSTN Charter's telecare protections), added a genuinely missing section -- 'What happens to a home phone during a power cut?' -- since the old version covered whether a line is needed at all but never addressed the actual practical question once Digital Voice is the default. Refreshed all 8 provider prices against data/providers.ts's own current fields, updated Virgin Media coverage 52% (was 53%) and added Ofcom's Spring 2026 Connected Nations split (89% gigabit-capable, 82% full fibre, 93% urban vs 66% rural). Word count 770 -&gt; 1,196; left just under the self-imposed 1,200-word floor rather than pad.</t>
         </is>
       </c>
       <c r="F49" s="3" t="n">
         <v>41</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
@@ -10582,7 +10626,7 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>data/provider-comparisons.ts (bt-vs-virgin-media)</t>
+          <t>app/guides/[slug]/page.tsx (broadband-without-phone-line), data/guides.ts</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
@@ -10597,7 +10641,7 @@
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10617,19 +10661,19 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Virgin Media comparison page (21st content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Eleventh target from scripts/analyze_content_priority.py's ranked list: 948 words, structurally sound (evergreen checklist format) but missing a genuinely newsworthy development -- Ofcom closed its One Touch Switch enforcement case on 11 June 2026 after finding more than 2 million customers had already used the process successfully, meaning it is now the industry's permanent standard rather than a monitored pilot, which the old copy still implied. Added this, plus a genuinely missing section on what a house move means for a home phone line given the 31 January 2027 PSTN switch-off (reusing research from the phone-and-broadband and broadband-without-phone-line refreshes earlier this session), Ofcom's Spring 2026 coverage split for the 'check availability' step, and corrected the ETC explanation to reflect Ofcom's actual cap rule (remaining payments, ex-VAT) rather than a flat multiplication. Re-verified the pre-existing GBP183.60/year switching-saving stat against fresh 2026 sources (found independently corroborated) and added the 4.2m/GBP100-240 social tariff stat already used elsewhere on this site. Word count 948 -&gt; 1,446.</t>
+          <t>Twenty-first target from the wider top-30 content-priority-analysis list: 526 words of entirely generic, number-free copy ('BT has no setup fee in the current dataset' -- itself wrong, BT's setup fee is GBP30). Rewrote using already-vetted current data from this session's own BT and Virgin Media provider-page work: BT from GBP23.99/mo (24-month, 98% coverage, Trustpilot 4.0/1.5 two-page split) vs Virgin Media from GBP33.00/mo (18-month, 52% coverage, 1,130Mbps fastest widely available speed, Trustpilot 1.4 but a genuinely better Q1 2026 Ofcom complaints record than BT, 6 vs 7 per 100k). Added the genuinely important practical point this page never covered: switching to Virgin Media never qualifies for One Touch Switch since it runs on a separate network from Openreach. Populated the previously-empty factSnapshot field. Word count 526 -&gt; 718.</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -10638,7 +10682,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-moving-house), data/guides.ts</t>
+          <t>data/provider-comparisons.ts (bt-vs-virgin-media)</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -10653,7 +10697,7 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10673,19 +10717,19 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband When Moving House checklist guide (11th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Twelfth target from scripts/analyze_content_priority.py's ranked list, and the page whose DATE_RE regex bug was found and fixed earlier this session (58.2 -&gt; 53.2) without ever getting a content rewrite. The old copy was generic to the point of naming no real prices at all -- 'Starlink is the most visible option' with zero named plans, figures or alternatives. Rewritten with real, current Starlink UK pricing (Residential 100/200/Max at GBP40/60/80 per month, Roam at GBP55-100, Standard Kit GBP449 commonly discounted to ~GBP299 or free on Max), and a genuinely current news item: Starlink's Global Roam plan stopped taking new customers 15 July 2026 and was withdrawn entirely for existing customers on 17 August 2026, one week before this rewrite. Named 2 real smaller alternatives (SkyDSL, Bigblu Broadband) and clarified that Eutelsat/OneWeb, despite frequent mention alongside Starlink, sells no UK consumer home-broadband plans at all. Word count 437 -&gt; 1,038.</t>
+          <t>Eleventh target from scripts/analyze_content_priority.py's ranked list: 948 words, structurally sound (evergreen checklist format) but missing a genuinely newsworthy development -- Ofcom closed its One Touch Switch enforcement case on 11 June 2026 after finding more than 2 million customers had already used the process successfully, meaning it is now the industry's permanent standard rather than a monitored pilot, which the old copy still implied. Added this, plus a genuinely missing section on what a house move means for a home phone line given the 31 January 2027 PSTN switch-off (reusing research from the phone-and-broadband and broadband-without-phone-line refreshes earlier this session), Ofcom's Spring 2026 coverage split for the 'check availability' step, and corrected the ETC explanation to reflect Ofcom's actual cap rule (remaining payments, ex-VAT) rather than a flat multiplication. Re-verified the pre-existing GBP183.60/year switching-saving stat against fresh 2026 sources (found independently corroborated) and added the 4.2m/GBP100-240 social tariff stat already used elsewhere on this site. Word count 948 -&gt; 1,446.</t>
         </is>
       </c>
       <c r="F51" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
@@ -10694,7 +10738,7 @@
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>data/priority-pages.ts (satellite)</t>
+          <t>app/guides/[slug]/page.tsx (broadband-moving-house), data/guides.ts</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
@@ -10719,53 +10763,53 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Deep rewrite: Satellite Broadband UK guide (12th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
+          <t>Twelfth target from scripts/analyze_content_priority.py's ranked list, and the page whose DATE_RE regex bug was found and fixed earlier this session (58.2 -&gt; 53.2) without ever getting a content rewrite. The old copy was generic to the point of naming no real prices at all -- 'Starlink is the most visible option' with zero named plans, figures or alternatives. Rewritten with real, current Starlink UK pricing (Residential 100/200/Max at GBP40/60/80 per month, Roam at GBP55-100, Standard Kit GBP449 commonly discounted to ~GBP299 or free on Max), and a genuinely current news item: Starlink's Global Roam plan stopped taking new customers 15 July 2026 and was withdrawn entirely for existing customers on 17 August 2026, one week before this rewrite. Named 2 real smaller alternatives (SkyDSL, Bigblu Broadband) and clarified that Eutelsat/OneWeb, despite frequent mention alongside Starlink, sells no UK consumer home-broadband plans at all. Word count 437 -&gt; 1,038.</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>components/</t>
+          <t>data/priority-pages.ts (satellite)</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Functionality pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -10775,53 +10819,53 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Thirteenth target from scripts/analyze_content_priority.py's ranked list: 836 words with stale provider prices (EE GBP26.99, Community Fibre GBP21.99, Hyperoptic GBP22, BT GBP30.99, all already corrected on this site's own provider pages) and a wrong Community Fibre top-tier speed claim (920Mbps symmetrical, against the real current 3,000Mbps top tier confirmed in data/providers.ts). Refreshed all 5 existing provider picks against already-vetted current pricing, and added a genuinely new 6th pick, Zen Internet, for a use case the old page didn't cover at all: hosting a private game server, where Zen's free static IP (already documented on its own provider page) is a real, specific advantage over every other provider on the list. Added a short section on how 24-month contracts and scheduled price rises affect the real two-year cost of a gaming-suitable package. Word count 836 -&gt; 1,184; left just under the self-imposed 1,200-word floor rather than pad.</t>
+          <t>PostcodeChecker, SpeedTest, StickyFilterBar and SocialProofCounter already exist as separate components. As the shortlist and price-alert features land, adopt accessible primitives (Radix-style) underneath rather than hand-rolling focus/keyboard behaviour again each time.</t>
         </is>
       </c>
       <c r="F53" s="3" t="n">
         <v>38</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-gaming-uk), data/guides.ts</t>
+          <t>components/</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L53" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Functionality pillar</t>
         </is>
       </c>
     </row>
@@ -10841,16 +10885,16 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Gaming UK guide (13th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Fourteenth target from scripts/analyze_content_priority.py's ranked list: 777 words with a materially wrong 'cheapest tariff' claim -- Vodafone Together Social was listed at GBP12.50/mo for 38Mbps and named the cheapest option, but the real current Vodafone Essentials Broadband tariff is GBP20/mo for 73Mbps (verified directly against Vodafone's own tariff page), meaning Virgin Media Essential Broadband and Community Fibre Essential (both genuinely GBP12.50/mo) are actually jointly cheapest. Also corrected Virgin Media's own tariff, which the old page listed at GBP20/mo. Added a genuinely newsworthy find: a thinkbroadband report published in August 2026 (days before this rewrite) tested how easy major providers make it to find their own social tariffs and scored BT, Sky, Virgin Media and Vodafone poorly, with a pointed BT quote, against smaller altnets scoring better. Corrected the eligibility table (Sky accepts UC/PC only, existing customers only, a real restriction the old page omitted) and added KCOM's Hull-only tariff. Refreshed the awareness stat with the newer, more specific thinkbroadband figures (34% aware, 8.6% UC take-up). Word count 777 -&gt; 1,161.</t>
+          <t>Thirteenth target from scripts/analyze_content_priority.py's ranked list: 836 words with stale provider prices (EE GBP26.99, Community Fibre GBP21.99, Hyperoptic GBP22, BT GBP30.99, all already corrected on this site's own provider pages) and a wrong Community Fibre top-tier speed claim (920Mbps symmetrical, against the real current 3,000Mbps top tier confirmed in data/providers.ts). Refreshed all 5 existing provider picks against already-vetted current pricing, and added a genuinely new 6th pick, Zen Internet, for a use case the old page didn't cover at all: hosting a private game server, where Zen's free static IP (already documented on its own provider page) is a real, specific advantage over every other provider on the list. Added a short section on how 24-month contracts and scheduled price rises affect the real two-year cost of a gaming-suitable package. Word count 836 -&gt; 1,184; left just under the self-imposed 1,200-word floor rather than pad.</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>34</v>
@@ -10862,7 +10906,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-social-tariffs-uk), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-gaming-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -10897,19 +10941,19 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Social Tariffs UK guide (14th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Fifteenth target from scripts/analyze_content_priority.py's ranked list: 565 words, no real prices anywhere, and a stale 'EE is consistently rated the most reliable major UK broadband provider' claim that no longer holds under this session's own Q1 2026 Ofcom complaints research. Rewrote with real current prices for Community Fibre, Hyperoptic, Zen Internet and BT, and added a genuinely new section this page never had: when a business-grade line (static IP, faster fault-fix SLA) is actually worth it for a freelancer or remote worker over a residential package, using real Vodafone Business/Zen Business/Sky Business pricing already researched for this site's business broadband guide. Added concrete video-call upload-bandwidth guidance (3-4 Mbps per HD call) rather than vague 'upload matters' framing. Word count 565 -&gt; 986.</t>
+          <t>Fourteenth target from scripts/analyze_content_priority.py's ranked list: 777 words with a materially wrong 'cheapest tariff' claim -- Vodafone Together Social was listed at GBP12.50/mo for 38Mbps and named the cheapest option, but the real current Vodafone Essentials Broadband tariff is GBP20/mo for 73Mbps (verified directly against Vodafone's own tariff page), meaning Virgin Media Essential Broadband and Community Fibre Essential (both genuinely GBP12.50/mo) are actually jointly cheapest. Also corrected Virgin Media's own tariff, which the old page listed at GBP20/mo. Added a genuinely newsworthy find: a thinkbroadband report published in August 2026 (days before this rewrite) tested how easy major providers make it to find their own social tariffs and scored BT, Sky, Virgin Media and Vodafone poorly, with a pointed BT quote, against smaller altnets scoring better. Corrected the eligibility table (Sky accepts UC/PC only, existing customers only, a real restriction the old page omitted) and added KCOM's Hull-only tariff. Refreshed the awareness stat with the newer, more specific thinkbroadband figures (34% aware, 8.6% UC take-up). Word count 777 -&gt; 1,161.</t>
         </is>
       </c>
       <c r="F55" s="3" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
@@ -10918,7 +10962,7 @@
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-working-from-home), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-social-tariffs-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
@@ -10953,19 +10997,19 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Working From Home guide (15th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Sixteenth target from scripts/analyze_content_priority.py's ranked list, and the one with the largest factual break of this whole refresh sequence: the page's entire premise named NOW Broadband and TalkTalk as 'the most common names in this price bracket,' but both now start above GBP20/mo (NOW at GBP23, TalkTalk at GBP25, both already corrected on their own provider pages this session). Rebuilt the page around who is actually under GBP20 today by querying data/providers.ts directly for every provider with monthlyPriceFrom &lt; 20: Community Fibre (GBP12.50), Onestream (GBP18.50, 94% Openreach coverage -- the most realistic pick for most addresses), Gigaclear (GBP19.00, rural symmetrical), toob (GBP19.50) and Trooli (GBP19.99). Also caught and excluded Shell Energy (GBP19.99 in the data file) after finding its own provider-page highlights note it closed to new customers and migrated to TalkTalk in 2024 -- an old, non-orderable plan that would have been a real error to list as a current deal. Word count 608 -&gt; 890.</t>
+          <t>Fifteenth target from scripts/analyze_content_priority.py's ranked list: 565 words, no real prices anywhere, and a stale 'EE is consistently rated the most reliable major UK broadband provider' claim that no longer holds under this session's own Q1 2026 Ofcom complaints research. Rewrote with real current prices for Community Fibre, Hyperoptic, Zen Internet and BT, and added a genuinely new section this page never had: when a business-grade line (static IP, faster fault-fix SLA) is actually worth it for a freelancer or remote worker over a residential package, using real Vodafone Business/Zen Business/Sky Business pricing already researched for this site's business broadband guide. Added concrete video-call upload-bandwidth guidance (3-4 Mbps per HD call) rather than vague 'upload matters' framing. Word count 565 -&gt; 986.</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
@@ -10974,7 +11018,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-deals-under-20), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-working-from-home), data/guides.ts</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -10999,7 +11043,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -11009,43 +11053,43 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: Broadband Deals Under GBP20 guide (16th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
+          <t>Sixteenth target from scripts/analyze_content_priority.py's ranked list, and the one with the largest factual break of this whole refresh sequence: the page's entire premise named NOW Broadband and TalkTalk as 'the most common names in this price bracket,' but both now start above GBP20/mo (NOW at GBP23, TalkTalk at GBP25, both already corrected on their own provider pages this session). Rebuilt the page around who is actually under GBP20 today by querying data/providers.ts directly for every provider with monthlyPriceFrom &lt; 20: Community Fibre (GBP12.50), Onestream (GBP18.50, 94% Openreach coverage -- the most realistic pick for most addresses), Gigaclear (GBP19.00, rural symmetrical), toob (GBP19.50) and Trooli (GBP19.99). Also caught and excluded Shell Energy (GBP19.99 in the data file) after finding its own provider-page highlights note it closed to new customers and migrated to TalkTalk in 2024 -- an old, non-orderable plan that would have been a real error to list as a current deal. Word count 608 -&gt; 890.</t>
         </is>
       </c>
       <c r="F57" s="3" t="n">
         <v>35</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-under-20), data/guides.ts</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>None, but easier before the guide count grows further</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L57" s="3" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -11055,7 +11099,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -11065,43 +11109,43 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
+          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
+          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -11121,19 +11165,19 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
+          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
         </is>
       </c>
       <c r="F59" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
@@ -11142,7 +11186,7 @@
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
+          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
@@ -11177,19 +11221,19 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
+          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -11198,7 +11242,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
+          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -11233,19 +11277,19 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
+          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
         </is>
       </c>
       <c r="F61" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
@@ -11254,7 +11298,7 @@
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
@@ -11269,7 +11313,7 @@
       </c>
       <c r="L61" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -11289,19 +11333,19 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
+          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -11310,7 +11354,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -11345,19 +11389,19 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
+          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
         </is>
       </c>
       <c r="F63" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
@@ -11366,7 +11410,7 @@
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
@@ -11401,19 +11445,19 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
+          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -11422,7 +11466,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -11457,16 +11501,16 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
+          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
         </is>
       </c>
       <c r="F65" s="3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G65" s="3" t="n">
         <v>26</v>
@@ -11478,27 +11522,83 @@
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
+          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
           <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
         </is>
       </c>
-      <c r="J65" s="3" t="inlineStr">
+      <c r="J66" s="2" t="inlineStr">
         <is>
           <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
-      <c r="K65" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L65" s="3" t="inlineStr">
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
         <is>
           <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L65"/>
+  <autoFilter ref="A1:L66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11539,7 +11639,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>97 total (33 page builds, 64 feature/strategy builds); 83 already marked Done.</t>
+          <t>98 total (33 page builds, 65 feature/strategy builds); 84 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Broadband Speeds Explained guide
Second target in the second 13-page batch: 476 words, the thinnest
guide examined all session, with entirely generic, dateless content.

Added a real Ofcom stat: average maximum available download speed is
285 Mbps (up ~30% from 223 Mbps), with the nuance that median speed
actually delivered on FTTC is closer to 80-100 Mbps. Reused the
FTTC/cable evening-congestion explanation already written for
best-broadband-for-streaming earlier this session. Added real current
symmetrical-speed examples (Community Fibre 3,000Mbps, YouFibre
8,000Mbps).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$100</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L99" headerRowCount="1">
-  <autoFilter ref="A1:L99"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L100" headerRowCount="1">
+  <autoFilter ref="A1:L100"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L66" headerRowCount="1">
-  <autoFilter ref="A1:L66"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L67" headerRowCount="1">
+  <autoFilter ref="A1:L67"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5125,8 +5125,52 @@
       <c r="K99" s="3" t="inlineStr"/>
       <c r="L99" s="3" t="inlineStr"/>
     </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>content-refresh-broadband-speeds-explained-guide</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G100" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr"/>
+      <c r="K100" s="2" t="inlineStr"/>
+      <c r="L100" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L99"/>
+  <autoFilter ref="A1:L100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7878,7 +7922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11597,8 +11641,64 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Second target in the second 13-page batch: 476 words, the thinnest guide examined all session, with entirely generic, dateless content. Added a real Ofcom stat this page never had: average maximum available download speed is 285 Mbps (up ~30% from 223 Mbps), with the important nuance that median speed actually delivered on FTTC is closer to 80-100 Mbps -- the average and the typical experience are genuinely different things. Reused the FTTC/cable evening-congestion explanation (shared capacity per street cabinet/node) already written for best-broadband-for-streaming earlier this session, with a matching new FAQ. Added real current symmetrical-speed examples (Community Fibre 3,000Mbps, YouFibre 8,000Mbps). Word count 476 -&gt; 787.</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G67" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (broadband-speeds-explained), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L66"/>
+  <autoFilter ref="A1:L67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11639,7 +11739,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>98 total (33 page builds, 65 feature/strategy builds); 84 already marked Done.</t>
+          <t>99 total (33 page builds, 66 feature/strategy builds); 85 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Broadband Deals With Cashback guide
Third target in the second 13-page batch: 622 words with zero real
numbers, entirely abstract advice with no concrete example of what a
real reward is actually worth.

Added BT's real reward card figures (GBP80-140, offsetting a GBP30
setup fee) and NOW Broadband's real GBP70-75 voucher pattern. Added a
concrete counter-example using Community Fibre's no-reward GBP12.50/mo
price to illustrate why a lower ongoing price can beat a bigger
one-off card once the full term is compared.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L100" headerRowCount="1">
-  <autoFilter ref="A1:L100"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L101" headerRowCount="1">
+  <autoFilter ref="A1:L101"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L67" headerRowCount="1">
-  <autoFilter ref="A1:L67"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L68" headerRowCount="1">
+  <autoFilter ref="A1:L68"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5169,8 +5169,52 @@
       <c r="K100" s="2" t="inlineStr"/>
       <c r="L100" s="2" t="inlineStr"/>
     </row>
+    <row r="101">
+      <c r="A101" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>content-refresh-broadband-deals-with-cashback-guide</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G101" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="H101" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I101" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J101" s="3" t="inlineStr"/>
+      <c r="K101" s="3" t="inlineStr"/>
+      <c r="L101" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L100"/>
+  <autoFilter ref="A1:L101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7922,7 +7966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11697,8 +11741,64 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Third target in the second 13-page batch: 622 words with zero real numbers -- entirely abstract advice about 'gift cards' and 'cashback' with no concrete example of what a real reward is actually worth. Added BT's real reward card figures (GBP80-140, offsetting a GBP30 setup fee, already documented on BT's own provider page) and NOW Broadband's real GBP70-75 voucher pattern. Added a genuinely concrete counter-example using Community Fibre's no-reward GBP12.50/mo price to illustrate why a lower ongoing price can beat a bigger one-off card once the full term is compared, replacing the old page's entirely hypothetical framing. Word count 622 -&gt; 826.</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-with-cashback), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L67"/>
+  <autoFilter ref="A1:L68"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11739,7 +11839,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>99 total (33 page builds, 66 feature/strategy builds); 85 already marked Done.</t>
+          <t>100 total (33 page builds, 67 feature/strategy builds); 86 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Broadband Deals With No Setup Fee guide
Fourth target in the second 13-page batch: 648 words with a real
error -- BT was listed alongside Sky and EE as a "no setup fee"
mainstream option, but BT genuinely charges a GBP30 setup fee, only
offset by a reward card that must be actively claimed.

Corrected the table and matching FAQ, and added a new section
distinguishing a genuine fee (BT's GBP30, Virgin Media's GBP35 with
no offset) from a fee that functions as free (NOW Broadband's GBP5
advance fee, credited back to the first bill).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$102</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L101" headerRowCount="1">
-  <autoFilter ref="A1:L101"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L102" headerRowCount="1">
+  <autoFilter ref="A1:L102"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L68" headerRowCount="1">
-  <autoFilter ref="A1:L68"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L69" headerRowCount="1">
+  <autoFilter ref="A1:L69"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4999,7 +4999,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-streaming-guide</t>
+          <t>content-refresh-broadband-deals-no-setup-fee-guide</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -5014,14 +5014,14 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F97" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G97" s="3" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-can-i-leave-broadband-early-guide</t>
+          <t>content-refresh-best-broadband-for-streaming-guide</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -5058,14 +5058,14 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F98" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
@@ -5087,7 +5087,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
+          <t>content-refresh-can-i-leave-broadband-early-guide</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -5102,11 +5102,11 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F99" s="3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G99" s="3" t="n">
         <v>26</v>
@@ -5131,7 +5131,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-speeds-explained-guide</t>
+          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -5146,14 +5146,14 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F100" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G100" s="2" t="n">
         <v>26</v>
-      </c>
-      <c r="G100" s="2" t="n">
-        <v>25</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-with-cashback-guide</t>
+          <t>content-refresh-broadband-speeds-explained-guide</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -5190,14 +5190,14 @@
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F101" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G101" s="3" t="n">
         <v>25</v>
-      </c>
-      <c r="G101" s="3" t="n">
-        <v>23</v>
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
@@ -5213,8 +5213,52 @@
       <c r="K101" s="3" t="inlineStr"/>
       <c r="L101" s="3" t="inlineStr"/>
     </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>content-refresh-broadband-deals-with-cashback-guide</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G102" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr"/>
+      <c r="K102" s="2" t="inlineStr"/>
+      <c r="L102" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L101"/>
+  <autoFilter ref="A1:L102"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7966,7 +8010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11533,19 +11577,19 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
+          <t>Fourth target in the second 13-page batch: 648 words with a real error -- BT was listed in the 'mainstream, no setup fee' table row alongside Sky and EE, but BT genuinely charges a GBP30 setup fee (confirmed on its own already-corrected provider page this session), only offset by a reward card that must be actively claimed. Corrected the table and matching FAQ, and added a new section distinguishing a genuine fee (BT's GBP30, Virgin Media's GBP35 with no offset) from a fee that functions as free (NOW Broadband's GBP5 advance fee, credited back to the first bill) -- a real distinction the old page collapsed into a single 'usually fee-charging' bucket. Word count 648 -&gt; 812.</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -11554,7 +11598,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-with-no-setup-fee), data/guides.ts</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -11589,19 +11633,19 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
+          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
         </is>
       </c>
       <c r="F65" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
@@ -11610,7 +11654,7 @@
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
@@ -11645,16 +11689,16 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
+          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G66" s="2" t="n">
         <v>26</v>
@@ -11666,7 +11710,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -11701,20 +11745,20 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Second target in the second 13-page batch: 476 words, the thinnest guide examined all session, with entirely generic, dateless content. Added a real Ofcom stat this page never had: average maximum available download speed is 285 Mbps (up ~30% from 223 Mbps), with the important nuance that median speed actually delivered on FTTC is closer to 80-100 Mbps -- the average and the typical experience are genuinely different things. Reused the FTTC/cable evening-congestion explanation (shared capacity per street cabinet/node) already written for best-broadband-for-streaming earlier this session, with a matching new FAQ. Added real current symmetrical-speed examples (Community Fibre 3,000Mbps, YouFibre 8,000Mbps). Word count 476 -&gt; 787.</t>
+          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
         </is>
       </c>
       <c r="F67" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G67" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="G67" s="3" t="n">
-        <v>25</v>
-      </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -11722,7 +11766,7 @@
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-speeds-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
@@ -11757,48 +11801,104 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
+          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Second target in the second 13-page batch: 476 words, the thinnest guide examined all session, with entirely generic, dateless content. Added a real Ofcom stat this page never had: average maximum available download speed is 285 Mbps (up ~30% from 223 Mbps), with the important nuance that median speed actually delivered on FTTC is closer to 80-100 Mbps -- the average and the typical experience are genuinely different things. Reused the FTTC/cable evening-congestion explanation (shared capacity per street cabinet/node) already written for best-broadband-for-streaming earlier this session, with a matching new FAQ. Added real current symmetrical-speed examples (Community Fibre 3,000Mbps, YouFibre 8,000Mbps). Word count 476 -&gt; 787.</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (broadband-speeds-explained), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
           <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E69" s="3" t="inlineStr">
         <is>
           <t>Third target in the second 13-page batch: 622 words with zero real numbers -- entirely abstract advice about 'gift cards' and 'cashback' with no concrete example of what a real reward is actually worth. Added BT's real reward card figures (GBP80-140, offsetting a GBP30 setup fee, already documented on BT's own provider page) and NOW Broadband's real GBP70-75 voucher pattern. Added a genuinely concrete counter-example using Community Fibre's no-reward GBP12.50/mo price to illustrate why a lower ongoing price can beat a bigger one-off card once the full term is compared, replacing the old page's entirely hypothetical framing. Word count 622 -&gt; 826.</t>
         </is>
       </c>
-      <c r="F68" s="2" t="n">
+      <c r="F69" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="G68" s="2" t="n">
+      <c r="G69" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="H69" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr">
+      <c r="I69" s="3" t="inlineStr">
         <is>
           <t>app/guides/[slug]/page.tsx (broadband-deals-with-cashback), data/guides.ts</t>
         </is>
       </c>
-      <c r="J68" s="2" t="inlineStr">
+      <c r="J69" s="3" t="inlineStr">
         <is>
           <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
-      <c r="K68" s="2" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L68" s="2" t="inlineStr">
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L69" s="3" t="inlineStr">
         <is>
           <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L68"/>
+  <autoFilter ref="A1:L69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11839,7 +11939,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>100 total (33 page builds, 67 feature/strategy builds); 86 already marked Done.</t>
+          <t>101 total (33 page builds, 68 feature/strategy builds); 87 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of 4 more thin comparison pages
Continuing the second 13-page batch: 3 of these 4 pages repeated the
same "Vodafone is cheaper" error already found and fixed on other
pairs this session -- bt-vs-vodafone and sky-vs-vodafone both claimed
Vodafone was the value pick, when Vodafone (GBP25) is now more
expensive than both BT (GBP23.99) and Sky (GBP23.00).

Rewrote all 4 with real current prices, Ofcom Q1 2026 complaints
figures and populated factSnapshot fields:
- bt-vs-vodafone: BT now cheaper AND better complaints record
- sky-vs-vodafone: Sky now cheaper AND far better complaints record
- ee-vs-sky: prices within 1p of each other, both genuinely strong on
  Ofcom -- a real feature-based decision replacing vague marketing copy
- plusnet-vs-bt: Plusnet has the best Ofcom complaints record of any
  major UK provider AND is cheaper than its own parent brand BT

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$103</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$70</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L102" headerRowCount="1">
-  <autoFilter ref="A1:L102"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L103" headerRowCount="1">
+  <autoFilter ref="A1:L103"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L69" headerRowCount="1">
-  <autoFilter ref="A1:L69"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L70" headerRowCount="1">
+  <autoFilter ref="A1:L70"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4735,12 +4735,12 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>bet-decouple-content-from-code</t>
+          <t>content-refresh-4-more-thin-comparison-pages</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -4750,14 +4750,14 @@
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: 4 more thin comparison pages (37th-40th content-priority-analysis targets)</t>
         </is>
       </c>
       <c r="F91" s="3" t="n">
         <v>35</v>
       </c>
       <c r="G91" s="3" t="n">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
@@ -4766,7 +4766,7 @@
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr"/>
@@ -4779,12 +4779,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-bt-vs-sky-comparison</t>
+          <t>bet-decouple-content-from-code</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -4794,23 +4794,23 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr"/>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
+          <t>content-refresh-bt-vs-sky-comparison</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -4838,14 +4838,14 @@
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F93" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G93" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
@@ -4867,7 +4867,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-price-rises-2026-guide</t>
+          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -4882,14 +4882,14 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-full-fibre-broadband-explained-guide</t>
+          <t>content-refresh-broadband-price-rises-2026-guide</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -4926,14 +4926,14 @@
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="F95" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G95" s="3" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
@@ -4955,7 +4955,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-students-guide</t>
+          <t>content-refresh-full-fibre-broadband-explained-guide</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -4970,14 +4970,14 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
@@ -4999,7 +4999,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-no-setup-fee-guide</t>
+          <t>content-refresh-best-broadband-for-students-guide</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -5014,14 +5014,14 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F97" s="3" t="n">
         <v>30</v>
       </c>
       <c r="G97" s="3" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-streaming-guide</t>
+          <t>content-refresh-broadband-deals-no-setup-fee-guide</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -5058,14 +5058,14 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F98" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
@@ -5087,7 +5087,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-can-i-leave-broadband-early-guide</t>
+          <t>content-refresh-best-broadband-for-streaming-guide</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -5102,14 +5102,14 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F99" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G99" s="3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
@@ -5131,7 +5131,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
+          <t>content-refresh-can-i-leave-broadband-early-guide</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -5146,11 +5146,11 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G100" s="2" t="n">
         <v>26</v>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-speeds-explained-guide</t>
+          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -5190,14 +5190,14 @@
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F101" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G101" s="3" t="n">
         <v>26</v>
-      </c>
-      <c r="G101" s="3" t="n">
-        <v>25</v>
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
@@ -5219,7 +5219,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-with-cashback-guide</t>
+          <t>content-refresh-broadband-speeds-explained-guide</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -5234,14 +5234,14 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F102" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G102" s="2" t="n">
         <v>25</v>
-      </c>
-      <c r="G102" s="2" t="n">
-        <v>23</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -5257,8 +5257,52 @@
       <c r="K102" s="2" t="inlineStr"/>
       <c r="L102" s="2" t="inlineStr"/>
     </row>
+    <row r="103">
+      <c r="A103" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>content-refresh-broadband-deals-with-cashback-guide</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F103" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G103" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="H103" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I103" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J103" s="3" t="inlineStr"/>
+      <c r="K103" s="3" t="inlineStr"/>
+      <c r="L103" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L102"/>
+  <autoFilter ref="A1:L103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8010,7 +8054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11231,7 +11275,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Bigger bet</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -11241,19 +11285,19 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Decouple guide content from code deploys</t>
+          <t>Deep rewrite: 4 more thin comparison pages (37th-40th content-priority-analysis targets)</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
+          <t>Continuing the second 13-page batch: 4 more comparison pages, 3 of which repeated the same 'Vodafone is cheaper' error already found and fixed twice this session on different pairs -- bt-vs-vodafone and sky-vs-vodafone both claimed Vodafone was the value pick, when Vodafone (GBP25) is now more expensive than both BT (GBP23.99) and Sky (GBP23.00). Rewrote all 4 with real current prices, Ofcom Q1 2026 complaints figures and populated factSnapshot fields: bt-vs-vodafone (BT now cheaper AND better complaints), sky-vs-vodafone (Sky now cheaper AND far better complaints), ee-vs-sky (prices within 1p of each other, both genuinely strong on Ofcom -- a real penny-and-feature-based decision replacing entirely vague marketing copy), plusnet-vs-bt (Plusnet has the best Ofcom complaints record of any major UK provider AND is cheaper than its own parent brand BT, a much stronger differentiator than the old page's vague 'UK support' framing). Word counts: 455-&gt;600, 504-&gt;608, 500-&gt;648, 507-&gt;604.</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
         <v>35</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -11262,22 +11306,22 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
+          <t>data/provider-comparisons.ts (bt-vs-vodafone, sky-vs-vodafone, ee-vs-sky, plusnet-vs-bt)</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>None, but easier before the guide count grows further</t>
+          <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>Growth playbook — Content pillar</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -11287,7 +11331,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -11297,43 +11341,43 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
+          <t>Every guide lives as a hand-written object in data/guides.ts plus matching JSX in app/guides/[slug]/page.tsx. Fine at 30 guides; at 100+ it becomes the bottleneck. Plan a move to MDX-per-guide or a lightweight headless CMS before volume forces it.</t>
         </is>
       </c>
       <c r="F59" s="3" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
+          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>ops-content-priority-analysis-tooling</t>
+          <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>Growth playbook — Content pillar</t>
         </is>
       </c>
     </row>
@@ -11353,19 +11397,19 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: BT vs Sky comparison page (17th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
+          <t>Seventeenth target from scripts/analyze_content_priority.py's ranked list, and the first comparison-type (not guide or provider) page in this refresh sequence: 496 words of entirely generic, number-free copy ('Sky starts cheaper,' 'BT usually charges more,' 'Sky is typically shorter at 18 months') that was also factually stale -- Sky moved to 24-month contracts some time ago, the same length as BT, a real premise this page's whole 'contract flexibility' differentiator was built on. Rewrote using the already-vetted current data from this session's own BT and Sky provider-page rewrites: prices have converged to within a pound (BT GBP23.99 vs Sky GBP23.00), Sky has the clearly better Ofcom Q1 2026 complaints record (5 vs 7 per 100k), BT has wider coverage (98% vs 95%), and BT's flat GBP4/year March price rise is more transparently disclosed for future years than Sky's 'prices may rise' contract wording. Populated the previously-empty factSnapshot field. Word count 496 -&gt; 717.</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -11374,7 +11418,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
+          <t>data/provider-comparisons.ts (bt-vs-sky)</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -11409,19 +11453,19 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
+          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
         </is>
       </c>
       <c r="F61" s="3" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
@@ -11430,7 +11474,7 @@
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
+          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
@@ -11465,19 +11509,19 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
+          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -11486,7 +11530,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -11501,7 +11545,7 @@
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -11521,19 +11565,19 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
+          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
         </is>
       </c>
       <c r="F63" s="3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
@@ -11542,7 +11586,7 @@
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
@@ -11577,19 +11621,19 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Fourth target in the second 13-page batch: 648 words with a real error -- BT was listed in the 'mainstream, no setup fee' table row alongside Sky and EE, but BT genuinely charges a GBP30 setup fee (confirmed on its own already-corrected provider page this session), only offset by a reward card that must be actively claimed. Corrected the table and matching FAQ, and added a new section distinguishing a genuine fee (BT's GBP30, Virgin Media's GBP35 with no offset) from a fee that functions as free (NOW Broadband's GBP5 advance fee, credited back to the first bill) -- a real distinction the old page collapsed into a single 'usually fee-charging' bucket. Word count 648 -&gt; 812.</t>
+          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
         <v>30</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -11598,7 +11642,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-deals-with-no-setup-fee), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -11633,19 +11677,19 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
+          <t>Fourth target in the second 13-page batch: 648 words with a real error -- BT was listed in the 'mainstream, no setup fee' table row alongside Sky and EE, but BT genuinely charges a GBP30 setup fee (confirmed on its own already-corrected provider page this session), only offset by a reward card that must be actively claimed. Corrected the table and matching FAQ, and added a new section distinguishing a genuine fee (BT's GBP30, Virgin Media's GBP35 with no offset) from a fee that functions as free (NOW Broadband's GBP5 advance fee, credited back to the first bill) -- a real distinction the old page collapsed into a single 'usually fee-charging' bucket. Word count 648 -&gt; 812.</t>
         </is>
       </c>
       <c r="F65" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
@@ -11654,7 +11698,7 @@
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-with-no-setup-fee), data/guides.ts</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
@@ -11689,19 +11733,19 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
+          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -11710,7 +11754,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -11745,16 +11789,16 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
+          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
         </is>
       </c>
       <c r="F67" s="3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G67" s="3" t="n">
         <v>26</v>
@@ -11766,7 +11810,7 @@
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
@@ -11801,20 +11845,20 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Second target in the second 13-page batch: 476 words, the thinnest guide examined all session, with entirely generic, dateless content. Added a real Ofcom stat this page never had: average maximum available download speed is 285 Mbps (up ~30% from 223 Mbps), with the important nuance that median speed actually delivered on FTTC is closer to 80-100 Mbps -- the average and the typical experience are genuinely different things. Reused the FTTC/cable evening-congestion explanation (shared capacity per street cabinet/node) already written for best-broadband-for-streaming earlier this session, with a matching new FAQ. Added real current symmetrical-speed examples (Community Fibre 3,000Mbps, YouFibre 8,000Mbps). Word count 476 -&gt; 787.</t>
+          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G68" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="G68" s="2" t="n">
-        <v>25</v>
-      </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -11822,7 +11866,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-speeds-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -11857,48 +11901,104 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
+          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Second target in the second 13-page batch: 476 words, the thinnest guide examined all session, with entirely generic, dateless content. Added a real Ofcom stat this page never had: average maximum available download speed is 285 Mbps (up ~30% from 223 Mbps), with the important nuance that median speed actually delivered on FTTC is closer to 80-100 Mbps -- the average and the typical experience are genuinely different things. Reused the FTTC/cable evening-congestion explanation (shared capacity per street cabinet/node) already written for best-broadband-for-streaming earlier this session, with a matching new FAQ. Added real current symmetrical-speed examples (Community Fibre 3,000Mbps, YouFibre 8,000Mbps). Word count 476 -&gt; 787.</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G69" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (broadband-speeds-explained), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
           <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
         </is>
       </c>
-      <c r="E69" s="3" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>Third target in the second 13-page batch: 622 words with zero real numbers -- entirely abstract advice about 'gift cards' and 'cashback' with no concrete example of what a real reward is actually worth. Added BT's real reward card figures (GBP80-140, offsetting a GBP30 setup fee, already documented on BT's own provider page) and NOW Broadband's real GBP70-75 voucher pattern. Added a genuinely concrete counter-example using Community Fibre's no-reward GBP12.50/mo price to illustrate why a lower ongoing price can beat a bigger one-off card once the full term is compared, replacing the old page's entirely hypothetical framing. Word count 622 -&gt; 826.</t>
         </is>
       </c>
-      <c r="F69" s="3" t="n">
+      <c r="F70" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="G69" s="3" t="n">
+      <c r="G70" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="H69" s="3" t="inlineStr">
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I69" s="3" t="inlineStr">
+      <c r="I70" s="2" t="inlineStr">
         <is>
           <t>app/guides/[slug]/page.tsx (broadband-deals-with-cashback), data/guides.ts</t>
         </is>
       </c>
-      <c r="J69" s="3" t="inlineStr">
+      <c r="J70" s="2" t="inlineStr">
         <is>
           <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
-      <c r="K69" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L69" s="3" t="inlineStr">
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
         <is>
           <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L69"/>
+  <autoFilter ref="A1:L70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11939,7 +12039,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>101 total (33 page builds, 68 feature/strategy builds); 87 already marked Done.</t>
+          <t>102 total (33 page builds, 69 feature/strategy builds); 88 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of No Mid-Contract Price Rise guide
Ninth target in the second 13-page batch, and directly about the
exact topic where this session already found real errors twice: this
page listed Hyperoptic as "fixed-price value" and NOW Broadband as
"no annual rise applies" when both apply real scheduled increases.

Rebuilt the whole table with accurate policies: only Zen Internet and
toob (previously missing entirely) genuinely have no rise; Community
Fibre has a real but capped GBP2/mo rise; Hyperoptic has a real
~GBP4/mo rise; NOW Broadband discloses GBP3 for April 2027/2028; Sky's
future-year terms are genuinely undisclosed. Added an explicit
"altnet is not a reliable proxy for no-rise" framing.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$104</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L103" headerRowCount="1">
-  <autoFilter ref="A1:L103"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L104" headerRowCount="1">
+  <autoFilter ref="A1:L104"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L70" headerRowCount="1">
-  <autoFilter ref="A1:L70"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L71" headerRowCount="1">
+  <autoFilter ref="A1:L71"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4867,7 +4867,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
+          <t>content-refresh-no-mid-contract-price-rise-guide</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -4882,14 +4882,14 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With No Mid-Contract Price Rise guide (41st content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-price-rises-2026-guide</t>
+          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -4926,14 +4926,14 @@
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F95" s="3" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G95" s="3" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
@@ -4955,7 +4955,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-full-fibre-broadband-explained-guide</t>
+          <t>content-refresh-broadband-price-rises-2026-guide</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -4970,14 +4970,14 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
@@ -4999,7 +4999,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-students-guide</t>
+          <t>content-refresh-full-fibre-broadband-explained-guide</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -5014,14 +5014,14 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F97" s="3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G97" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-no-setup-fee-guide</t>
+          <t>content-refresh-best-broadband-for-students-guide</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -5058,14 +5058,14 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F98" s="2" t="n">
         <v>30</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
@@ -5087,7 +5087,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-streaming-guide</t>
+          <t>content-refresh-broadband-deals-no-setup-fee-guide</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -5102,14 +5102,14 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F99" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G99" s="3" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
@@ -5131,7 +5131,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-can-i-leave-broadband-early-guide</t>
+          <t>content-refresh-best-broadband-for-streaming-guide</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -5146,14 +5146,14 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
+          <t>content-refresh-can-i-leave-broadband-early-guide</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -5190,11 +5190,11 @@
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F101" s="3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G101" s="3" t="n">
         <v>26</v>
@@ -5219,7 +5219,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-speeds-explained-guide</t>
+          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -5234,14 +5234,14 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F102" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G102" s="2" t="n">
         <v>26</v>
-      </c>
-      <c r="G102" s="2" t="n">
-        <v>25</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -5263,7 +5263,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-with-cashback-guide</t>
+          <t>content-refresh-broadband-speeds-explained-guide</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -5278,14 +5278,14 @@
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F103" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G103" s="3" t="n">
         <v>25</v>
-      </c>
-      <c r="G103" s="3" t="n">
-        <v>23</v>
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
@@ -5301,8 +5301,52 @@
       <c r="K103" s="3" t="inlineStr"/>
       <c r="L103" s="3" t="inlineStr"/>
     </row>
+    <row r="104">
+      <c r="A104" s="2" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>content-refresh-broadband-deals-with-cashback-guide</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G104" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr"/>
+      <c r="K104" s="2" t="inlineStr"/>
+      <c r="L104" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L103"/>
+  <autoFilter ref="A1:L104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8054,7 +8098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11453,19 +11497,19 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With No Mid-Contract Price Rise guide (41st content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
+          <t>Ninth target in the second 13-page batch, and directly about the exact topic where this session already found real errors twice (Hyperoptic and Community Fibre wrongly listed as no-rise on the price-rises guide): this page repeated the same mistake, listing Hyperoptic as 'fixed-price value' and NOW Broadband as 'no annual rise applies' when both apply real scheduled increases. Rebuilt the whole table with accurate policies: only Zen Internet and toob (previously missing from this page entirely) genuinely have no rise; Community Fibre has a real but capped GBP2/mo rise; Hyperoptic has a real ~GBP4/mo rise; NOW Broadband has no rise in 2026 but discloses GBP3 for April 2027/2028; Sky's future-year terms are genuinely undisclosed. Added an explicit 'altnet is not a reliable proxy for no-rise' framing. Word count 701 -&gt; 828.</t>
         </is>
       </c>
       <c r="F61" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
@@ -11474,7 +11518,7 @@
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-with-no-mid-contract-price-rise), data/guides.ts</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
@@ -11489,7 +11533,7 @@
       </c>
       <c r="L61" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -11509,19 +11553,19 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
+          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -11530,7 +11574,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
+          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -11565,19 +11609,19 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
+          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
         </is>
       </c>
       <c r="F63" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
@@ -11586,7 +11630,7 @@
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
@@ -11601,7 +11645,7 @@
       </c>
       <c r="L63" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -11621,19 +11665,19 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
+          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -11642,7 +11686,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -11677,19 +11721,19 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Fourth target in the second 13-page batch: 648 words with a real error -- BT was listed in the 'mainstream, no setup fee' table row alongside Sky and EE, but BT genuinely charges a GBP30 setup fee (confirmed on its own already-corrected provider page this session), only offset by a reward card that must be actively claimed. Corrected the table and matching FAQ, and added a new section distinguishing a genuine fee (BT's GBP30, Virgin Media's GBP35 with no offset) from a fee that functions as free (NOW Broadband's GBP5 advance fee, credited back to the first bill) -- a real distinction the old page collapsed into a single 'usually fee-charging' bucket. Word count 648 -&gt; 812.</t>
+          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
         </is>
       </c>
       <c r="F65" s="3" t="n">
         <v>30</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
@@ -11698,7 +11742,7 @@
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-deals-with-no-setup-fee), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
@@ -11733,19 +11777,19 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
+          <t>Fourth target in the second 13-page batch: 648 words with a real error -- BT was listed in the 'mainstream, no setup fee' table row alongside Sky and EE, but BT genuinely charges a GBP30 setup fee (confirmed on its own already-corrected provider page this session), only offset by a reward card that must be actively claimed. Corrected the table and matching FAQ, and added a new section distinguishing a genuine fee (BT's GBP30, Virgin Media's GBP35 with no offset) from a fee that functions as free (NOW Broadband's GBP5 advance fee, credited back to the first bill) -- a real distinction the old page collapsed into a single 'usually fee-charging' bucket. Word count 648 -&gt; 812.</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -11754,7 +11798,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-with-no-setup-fee), data/guides.ts</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -11789,19 +11833,19 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
+          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
         </is>
       </c>
       <c r="F67" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G67" s="3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
@@ -11810,7 +11854,7 @@
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
@@ -11845,16 +11889,16 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
+          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G68" s="2" t="n">
         <v>26</v>
@@ -11866,7 +11910,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -11901,20 +11945,20 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Second target in the second 13-page batch: 476 words, the thinnest guide examined all session, with entirely generic, dateless content. Added a real Ofcom stat this page never had: average maximum available download speed is 285 Mbps (up ~30% from 223 Mbps), with the important nuance that median speed actually delivered on FTTC is closer to 80-100 Mbps -- the average and the typical experience are genuinely different things. Reused the FTTC/cable evening-congestion explanation (shared capacity per street cabinet/node) already written for best-broadband-for-streaming earlier this session, with a matching new FAQ. Added real current symmetrical-speed examples (Community Fibre 3,000Mbps, YouFibre 8,000Mbps). Word count 476 -&gt; 787.</t>
+          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
         </is>
       </c>
       <c r="F69" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G69" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="G69" s="3" t="n">
-        <v>25</v>
-      </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -11922,7 +11966,7 @@
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-speeds-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
@@ -11957,48 +12001,104 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
+          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Second target in the second 13-page batch: 476 words, the thinnest guide examined all session, with entirely generic, dateless content. Added a real Ofcom stat this page never had: average maximum available download speed is 285 Mbps (up ~30% from 223 Mbps), with the important nuance that median speed actually delivered on FTTC is closer to 80-100 Mbps -- the average and the typical experience are genuinely different things. Reused the FTTC/cable evening-congestion explanation (shared capacity per street cabinet/node) already written for best-broadband-for-streaming earlier this session, with a matching new FAQ. Added real current symmetrical-speed examples (Community Fibre 3,000Mbps, YouFibre 8,000Mbps). Word count 476 -&gt; 787.</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (broadband-speeds-explained), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
           <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="E71" s="3" t="inlineStr">
         <is>
           <t>Third target in the second 13-page batch: 622 words with zero real numbers -- entirely abstract advice about 'gift cards' and 'cashback' with no concrete example of what a real reward is actually worth. Added BT's real reward card figures (GBP80-140, offsetting a GBP30 setup fee, already documented on BT's own provider page) and NOW Broadband's real GBP70-75 voucher pattern. Added a genuinely concrete counter-example using Community Fibre's no-reward GBP12.50/mo price to illustrate why a lower ongoing price can beat a bigger one-off card once the full term is compared, replacing the old page's entirely hypothetical framing. Word count 622 -&gt; 826.</t>
         </is>
       </c>
-      <c r="F70" s="2" t="n">
+      <c r="F71" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="G70" s="2" t="n">
+      <c r="G71" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="H70" s="2" t="inlineStr">
+      <c r="H71" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr">
+      <c r="I71" s="3" t="inlineStr">
         <is>
           <t>app/guides/[slug]/page.tsx (broadband-deals-with-cashback), data/guides.ts</t>
         </is>
       </c>
-      <c r="J70" s="2" t="inlineStr">
+      <c r="J71" s="3" t="inlineStr">
         <is>
           <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
-      <c r="K70" s="2" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L70" s="2" t="inlineStr">
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L71" s="3" t="inlineStr">
         <is>
           <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L70"/>
+  <autoFilter ref="A1:L71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -12039,7 +12139,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>102 total (33 page builds, 69 feature/strategy builds); 88 already marked Done.</t>
+          <t>103 total (33 page builds, 70 feature/strategy builds); 89 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of Broadband Deals for Existing Customers guide
Tenth target in the second 13-page batch: 689 words of correct but
entirely generic negotiation advice with no real figures.

Added the GBP183.60/year switching-savings stat, the One Touch Switch
enforcement-closure news (11 June 2026, now the permanent industry
standard), and a new section reframing a scheduled price rise
notification as a genuine, low-friction negotiation trigger, citing
real current rise figures (BT/EE GBP4/mo, TalkTalk GBP4/mo, Sky
GBP3/mo).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$105</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$72</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L104" headerRowCount="1">
-  <autoFilter ref="A1:L104"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L105" headerRowCount="1">
+  <autoFilter ref="A1:L105"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L71" headerRowCount="1">
-  <autoFilter ref="A1:L71"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L72" headerRowCount="1">
+  <autoFilter ref="A1:L72"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4955,7 +4955,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-price-rises-2026-guide</t>
+          <t>content-refresh-broadband-existing-customers-guide</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -4970,14 +4970,14 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Broadband Deals for Existing Customers guide (42nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
@@ -4999,7 +4999,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-full-fibre-broadband-explained-guide</t>
+          <t>content-refresh-broadband-price-rises-2026-guide</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -5014,14 +5014,14 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="F97" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G97" s="3" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-students-guide</t>
+          <t>content-refresh-full-fibre-broadband-explained-guide</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -5058,14 +5058,14 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F98" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
@@ -5087,7 +5087,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-no-setup-fee-guide</t>
+          <t>content-refresh-best-broadband-for-students-guide</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -5102,14 +5102,14 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F99" s="3" t="n">
         <v>30</v>
       </c>
       <c r="G99" s="3" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
@@ -5131,7 +5131,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-streaming-guide</t>
+          <t>content-refresh-broadband-deals-no-setup-fee-guide</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -5146,14 +5146,14 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-can-i-leave-broadband-early-guide</t>
+          <t>content-refresh-best-broadband-for-streaming-guide</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -5190,14 +5190,14 @@
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F101" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G101" s="3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
@@ -5219,7 +5219,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
+          <t>content-refresh-can-i-leave-broadband-early-guide</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -5234,11 +5234,11 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F102" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G102" s="2" t="n">
         <v>26</v>
@@ -5263,7 +5263,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-speeds-explained-guide</t>
+          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -5278,14 +5278,14 @@
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F103" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G103" s="3" t="n">
         <v>26</v>
-      </c>
-      <c r="G103" s="3" t="n">
-        <v>25</v>
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
@@ -5307,7 +5307,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-with-cashback-guide</t>
+          <t>content-refresh-broadband-speeds-explained-guide</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -5322,14 +5322,14 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F104" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G104" s="2" t="n">
         <v>25</v>
-      </c>
-      <c r="G104" s="2" t="n">
-        <v>23</v>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
@@ -5345,8 +5345,52 @@
       <c r="K104" s="2" t="inlineStr"/>
       <c r="L104" s="2" t="inlineStr"/>
     </row>
+    <row r="105">
+      <c r="A105" s="3" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>content-refresh-broadband-deals-with-cashback-guide</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="inlineStr">
+        <is>
+          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G105" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="H105" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I105" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J105" s="3" t="inlineStr"/>
+      <c r="K105" s="3" t="inlineStr"/>
+      <c r="L105" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L104"/>
+  <autoFilter ref="A1:L105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8098,7 +8142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11609,19 +11653,19 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Broadband Deals for Existing Customers guide (42nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
+          <t>Tenth target in the second 13-page batch: 689 words of correct but entirely generic negotiation advice with no real figures. Added the GBP183.60/year switching-savings stat (already verified this session for the moving-house guide), the One Touch Switch enforcement-closure news (11 June 2026, permanent industry standard), and a new section reframing a scheduled price rise notification as a genuine, low-friction negotiation trigger, citing the real current rise figures already established this session (BT/EE GBP4/mo March, TalkTalk GBP4/mo from Nov 2025 contracts, Sky GBP3/mo April 2026). Word count 689 -&gt; 946.</t>
         </is>
       </c>
       <c r="F63" s="3" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
@@ -11630,7 +11674,7 @@
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
+          <t>app/guides/[slug]/page.tsx (broadband-for-existing-customers), data/guides.ts</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
@@ -11645,7 +11689,7 @@
       </c>
       <c r="L63" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -11665,19 +11709,19 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
+          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -11686,7 +11730,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -11701,7 +11745,7 @@
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -11721,19 +11765,19 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
+          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
         </is>
       </c>
       <c r="F65" s="3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
@@ -11742,7 +11786,7 @@
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
@@ -11777,19 +11821,19 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Fourth target in the second 13-page batch: 648 words with a real error -- BT was listed in the 'mainstream, no setup fee' table row alongside Sky and EE, but BT genuinely charges a GBP30 setup fee (confirmed on its own already-corrected provider page this session), only offset by a reward card that must be actively claimed. Corrected the table and matching FAQ, and added a new section distinguishing a genuine fee (BT's GBP30, Virgin Media's GBP35 with no offset) from a fee that functions as free (NOW Broadband's GBP5 advance fee, credited back to the first bill) -- a real distinction the old page collapsed into a single 'usually fee-charging' bucket. Word count 648 -&gt; 812.</t>
+          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
         <v>30</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -11798,7 +11842,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-deals-with-no-setup-fee), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -11833,19 +11877,19 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
+          <t>Fourth target in the second 13-page batch: 648 words with a real error -- BT was listed in the 'mainstream, no setup fee' table row alongside Sky and EE, but BT genuinely charges a GBP30 setup fee (confirmed on its own already-corrected provider page this session), only offset by a reward card that must be actively claimed. Corrected the table and matching FAQ, and added a new section distinguishing a genuine fee (BT's GBP30, Virgin Media's GBP35 with no offset) from a fee that functions as free (NOW Broadband's GBP5 advance fee, credited back to the first bill) -- a real distinction the old page collapsed into a single 'usually fee-charging' bucket. Word count 648 -&gt; 812.</t>
         </is>
       </c>
       <c r="F67" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G67" s="3" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
@@ -11854,7 +11898,7 @@
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-with-no-setup-fee), data/guides.ts</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
@@ -11889,19 +11933,19 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
+          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -11910,7 +11954,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -11945,16 +11989,16 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
+          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
         </is>
       </c>
       <c r="F69" s="3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G69" s="3" t="n">
         <v>26</v>
@@ -11966,7 +12010,7 @@
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
@@ -12001,20 +12045,20 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Second target in the second 13-page batch: 476 words, the thinnest guide examined all session, with entirely generic, dateless content. Added a real Ofcom stat this page never had: average maximum available download speed is 285 Mbps (up ~30% from 223 Mbps), with the important nuance that median speed actually delivered on FTTC is closer to 80-100 Mbps -- the average and the typical experience are genuinely different things. Reused the FTTC/cable evening-congestion explanation (shared capacity per street cabinet/node) already written for best-broadband-for-streaming earlier this session, with a matching new FAQ. Added real current symmetrical-speed examples (Community Fibre 3,000Mbps, YouFibre 8,000Mbps). Word count 476 -&gt; 787.</t>
+          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G70" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="G70" s="2" t="n">
-        <v>25</v>
-      </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -12022,7 +12066,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-speeds-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -12057,48 +12101,104 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
+          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>Second target in the second 13-page batch: 476 words, the thinnest guide examined all session, with entirely generic, dateless content. Added a real Ofcom stat this page never had: average maximum available download speed is 285 Mbps (up ~30% from 223 Mbps), with the important nuance that median speed actually delivered on FTTC is closer to 80-100 Mbps -- the average and the typical experience are genuinely different things. Reused the FTTC/cable evening-congestion explanation (shared capacity per street cabinet/node) already written for best-broadband-for-streaming earlier this session, with a matching new FAQ. Added real current symmetrical-speed examples (Community Fibre 3,000Mbps, YouFibre 8,000Mbps). Word count 476 -&gt; 787.</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G71" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (broadband-speeds-explained), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L71" s="3" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
           <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
         </is>
       </c>
-      <c r="E71" s="3" t="inlineStr">
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>Third target in the second 13-page batch: 622 words with zero real numbers -- entirely abstract advice about 'gift cards' and 'cashback' with no concrete example of what a real reward is actually worth. Added BT's real reward card figures (GBP80-140, offsetting a GBP30 setup fee, already documented on BT's own provider page) and NOW Broadband's real GBP70-75 voucher pattern. Added a genuinely concrete counter-example using Community Fibre's no-reward GBP12.50/mo price to illustrate why a lower ongoing price can beat a bigger one-off card once the full term is compared, replacing the old page's entirely hypothetical framing. Word count 622 -&gt; 826.</t>
         </is>
       </c>
-      <c r="F71" s="3" t="n">
+      <c r="F72" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="G71" s="3" t="n">
+      <c r="G72" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="H71" s="3" t="inlineStr">
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I71" s="3" t="inlineStr">
+      <c r="I72" s="2" t="inlineStr">
         <is>
           <t>app/guides/[slug]/page.tsx (broadband-deals-with-cashback), data/guides.ts</t>
         </is>
       </c>
-      <c r="J71" s="3" t="inlineStr">
+      <c r="J72" s="2" t="inlineStr">
         <is>
           <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
-      <c r="K71" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L71" s="3" t="inlineStr">
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
         <is>
           <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L71"/>
+  <autoFilter ref="A1:L72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -12139,7 +12239,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>103 total (33 page builds, 70 feature/strategy builds); 89 already marked Done.</t>
+          <t>104 total (33 page builds, 71 feature/strategy builds); 90 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: update Static IP Business Broadband guide with Vodafone comparison
Eleventh target in the second 13-page batch: already an excellent,
precisely-dated page, so this was a targeted enhancement. Added a
cross-provider contrast: Zen Internet includes a free static IP on
every plan (already confirmed on its own provider page this session),
while Vodafone Business splits by tier (Essential offers one on
request at ~GBP5/mo+VAT, Pro includes it as standard).

Caught and corrected an initial draft claim about Vodafone's policy
against a fresh source before shipping.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$106</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L105" headerRowCount="1">
-  <autoFilter ref="A1:L105"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L106" headerRowCount="1">
+  <autoFilter ref="A1:L106"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L72" headerRowCount="1">
-  <autoFilter ref="A1:L72"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L73" headerRowCount="1">
+  <autoFilter ref="A1:L73"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5389,8 +5389,52 @@
       <c r="K105" s="3" t="inlineStr"/>
       <c r="L105" s="3" t="inlineStr"/>
     </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>content-refresh-static-ip-business-broadband-guide</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>Update: Static IP Business Broadband guide (43rd content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="G106" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr"/>
+      <c r="K106" s="2" t="inlineStr"/>
+      <c r="L106" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L105"/>
+  <autoFilter ref="A1:L106"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8142,7 +8186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12197,8 +12241,64 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="3" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Update: Static IP Business Broadband guide (43rd content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Eleventh target in the second 13-page batch: already an excellent, precisely-dated, well-sourced page (1,076 words, real BT Business pricing), so this was a targeted enhancement rather than a rewrite. Added a real cross-provider contrast this session had already independently confirmed on Zen Internet's own provider page (free static IP included on every plan) and freshly verified for Vodafone Business (Essential offers one on request at ~GBP5/mo+VAT, Pro includes it as standard, up to 8 orderable at a fixed price) -- caught and corrected an initial draft claim about Vodafone's policy against a fresh source before shipping. Word count 1,076 -&gt; 1,151.</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="G73" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (static-ip-business-broadband-explained), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L73" s="3" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L72"/>
+  <autoFilter ref="A1:L73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -12239,7 +12339,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>104 total (33 page builds, 71 feature/strategy builds); 90 already marked Done.</t>
+          <t>105 total (33 page builds, 72 feature/strategy builds); 91 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: deep rewrite of One Touch Switching Explained guide
Twelfth target in the second 13-page batch, and the single most
relevant page on the site for the One Touch Switch enforcement-closure
news -- this page is literally about OTS specifically and was still
missing the fact entirely.

Added: Ofcom closed its dedicated enforcement programme on 11 June
2026 after finding more than 2 million customers had already used it
successfully, confirming OTS as the industry's permanent standard
rather than a still-bedding-in pilot. New dedicated section, updated
intro, matching new FAQ.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$107</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$74</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L106" headerRowCount="1">
-  <autoFilter ref="A1:L106"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L107" headerRowCount="1">
+  <autoFilter ref="A1:L107"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L73" headerRowCount="1">
-  <autoFilter ref="A1:L73"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L74" headerRowCount="1">
+  <autoFilter ref="A1:L74"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-full-fibre-broadband-explained-guide</t>
+          <t>content-refresh-one-touch-switching-explained-guide</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -5058,14 +5058,14 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: One Touch Switching Explained guide (44th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F98" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
@@ -5087,7 +5087,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-students-guide</t>
+          <t>content-refresh-full-fibre-broadband-explained-guide</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -5102,14 +5102,14 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F99" s="3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G99" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
@@ -5131,7 +5131,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-no-setup-fee-guide</t>
+          <t>content-refresh-best-broadband-for-students-guide</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -5146,14 +5146,14 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F100" s="2" t="n">
         <v>30</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-streaming-guide</t>
+          <t>content-refresh-broadband-deals-no-setup-fee-guide</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -5190,14 +5190,14 @@
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F101" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G101" s="3" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
@@ -5219,7 +5219,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-can-i-leave-broadband-early-guide</t>
+          <t>content-refresh-best-broadband-for-streaming-guide</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -5234,14 +5234,14 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F102" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -5263,7 +5263,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
+          <t>content-refresh-can-i-leave-broadband-early-guide</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -5278,11 +5278,11 @@
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F103" s="3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G103" s="3" t="n">
         <v>26</v>
@@ -5307,7 +5307,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-speeds-explained-guide</t>
+          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -5322,14 +5322,14 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F104" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G104" s="2" t="n">
         <v>26</v>
-      </c>
-      <c r="G104" s="2" t="n">
-        <v>25</v>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
@@ -5351,7 +5351,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-with-cashback-guide</t>
+          <t>content-refresh-broadband-speeds-explained-guide</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -5366,14 +5366,14 @@
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F105" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G105" s="3" t="n">
         <v>25</v>
-      </c>
-      <c r="G105" s="3" t="n">
-        <v>23</v>
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
@@ -5395,7 +5395,7 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-static-ip-business-broadband-guide</t>
+          <t>content-refresh-broadband-deals-with-cashback-guide</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -5410,18 +5410,18 @@
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Update: Static IP Business Broadband guide (43rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F106" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G106" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr">
@@ -5433,8 +5433,52 @@
       <c r="K106" s="2" t="inlineStr"/>
       <c r="L106" s="2" t="inlineStr"/>
     </row>
+    <row r="107">
+      <c r="A107" s="3" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>content-refresh-static-ip-business-broadband-guide</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>Update: Static IP Business Broadband guide (43rd content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F107" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="G107" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="H107" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I107" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J107" s="3" t="inlineStr"/>
+      <c r="K107" s="3" t="inlineStr"/>
+      <c r="L107" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L106"/>
+  <autoFilter ref="A1:L107"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8186,7 +8230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11809,19 +11853,19 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: One Touch Switching Explained guide (44th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
+          <t>Twelfth target in the second 13-page batch, and the single most relevant page on the site for the One Touch Switch enforcement-closure news (also added to how-to-switch-broadband-uk and broadband-for-existing-customers earlier this session) -- this page is literally about OTS specifically and was still missing the fact entirely: Ofcom closed its dedicated enforcement programme on 11 June 2026 after finding more than 2 million customers had already used it successfully, confirming OTS as the industry's permanent standard rather than a still-bedding-in pilot. Added a new dedicated section, updated the intro, and a matching new FAQ. Word count 731 -&gt; 921.</t>
         </is>
       </c>
       <c r="F65" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
@@ -11830,7 +11874,7 @@
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (one-touch-switching-explained), data/guides.ts</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
@@ -11865,19 +11909,19 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
+          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -11886,7 +11930,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -11921,19 +11965,19 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Fourth target in the second 13-page batch: 648 words with a real error -- BT was listed in the 'mainstream, no setup fee' table row alongside Sky and EE, but BT genuinely charges a GBP30 setup fee (confirmed on its own already-corrected provider page this session), only offset by a reward card that must be actively claimed. Corrected the table and matching FAQ, and added a new section distinguishing a genuine fee (BT's GBP30, Virgin Media's GBP35 with no offset) from a fee that functions as free (NOW Broadband's GBP5 advance fee, credited back to the first bill) -- a real distinction the old page collapsed into a single 'usually fee-charging' bucket. Word count 648 -&gt; 812.</t>
+          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
         </is>
       </c>
       <c r="F67" s="3" t="n">
         <v>30</v>
       </c>
       <c r="G67" s="3" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
@@ -11942,7 +11986,7 @@
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-deals-with-no-setup-fee), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
@@ -11977,19 +12021,19 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
+          <t>Fourth target in the second 13-page batch: 648 words with a real error -- BT was listed in the 'mainstream, no setup fee' table row alongside Sky and EE, but BT genuinely charges a GBP30 setup fee (confirmed on its own already-corrected provider page this session), only offset by a reward card that must be actively claimed. Corrected the table and matching FAQ, and added a new section distinguishing a genuine fee (BT's GBP30, Virgin Media's GBP35 with no offset) from a fee that functions as free (NOW Broadband's GBP5 advance fee, credited back to the first bill) -- a real distinction the old page collapsed into a single 'usually fee-charging' bucket. Word count 648 -&gt; 812.</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -11998,7 +12042,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-with-no-setup-fee), data/guides.ts</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -12033,19 +12077,19 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
+          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
         </is>
       </c>
       <c r="F69" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
@@ -12054,7 +12098,7 @@
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
@@ -12089,16 +12133,16 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
+          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G70" s="2" t="n">
         <v>26</v>
@@ -12110,7 +12154,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -12145,20 +12189,20 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Second target in the second 13-page batch: 476 words, the thinnest guide examined all session, with entirely generic, dateless content. Added a real Ofcom stat this page never had: average maximum available download speed is 285 Mbps (up ~30% from 223 Mbps), with the important nuance that median speed actually delivered on FTTC is closer to 80-100 Mbps -- the average and the typical experience are genuinely different things. Reused the FTTC/cable evening-congestion explanation (shared capacity per street cabinet/node) already written for best-broadband-for-streaming earlier this session, with a matching new FAQ. Added real current symmetrical-speed examples (Community Fibre 3,000Mbps, YouFibre 8,000Mbps). Word count 476 -&gt; 787.</t>
+          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
         </is>
       </c>
       <c r="F71" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G71" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="G71" s="3" t="n">
-        <v>25</v>
-      </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -12166,7 +12210,7 @@
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-speeds-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
@@ -12201,20 +12245,20 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Third target in the second 13-page batch: 622 words with zero real numbers -- entirely abstract advice about 'gift cards' and 'cashback' with no concrete example of what a real reward is actually worth. Added BT's real reward card figures (GBP80-140, offsetting a GBP30 setup fee, already documented on BT's own provider page) and NOW Broadband's real GBP70-75 voucher pattern. Added a genuinely concrete counter-example using Community Fibre's no-reward GBP12.50/mo price to illustrate why a lower ongoing price can beat a bigger one-off card once the full term is compared, replacing the old page's entirely hypothetical framing. Word count 622 -&gt; 826.</t>
+          <t>Second target in the second 13-page batch: 476 words, the thinnest guide examined all session, with entirely generic, dateless content. Added a real Ofcom stat this page never had: average maximum available download speed is 285 Mbps (up ~30% from 223 Mbps), with the important nuance that median speed actually delivered on FTTC is closer to 80-100 Mbps -- the average and the typical experience are genuinely different things. Reused the FTTC/cable evening-congestion explanation (shared capacity per street cabinet/node) already written for best-broadband-for-streaming earlier this session, with a matching new FAQ. Added real current symmetrical-speed examples (Community Fibre 3,000Mbps, YouFibre 8,000Mbps). Word count 476 -&gt; 787.</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G72" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="G72" s="2" t="n">
-        <v>23</v>
-      </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -12222,7 +12266,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-deals-with-cashback), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-speeds-explained), data/guides.ts</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -12257,48 +12301,104 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
+          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Third target in the second 13-page batch: 622 words with zero real numbers -- entirely abstract advice about 'gift cards' and 'cashback' with no concrete example of what a real reward is actually worth. Added BT's real reward card figures (GBP80-140, offsetting a GBP30 setup fee, already documented on BT's own provider page) and NOW Broadband's real GBP70-75 voucher pattern. Added a genuinely concrete counter-example using Community Fibre's no-reward GBP12.50/mo price to illustrate why a lower ongoing price can beat a bigger one-off card once the full term is compared, replacing the old page's entirely hypothetical framing. Word count 622 -&gt; 826.</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G73" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-with-cashback), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L73" s="3" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
           <t>Update: Static IP Business Broadband guide (43rd content-priority-analysis target)</t>
         </is>
       </c>
-      <c r="E73" s="3" t="inlineStr">
+      <c r="E74" s="2" t="inlineStr">
         <is>
           <t>Eleventh target in the second 13-page batch: already an excellent, precisely-dated, well-sourced page (1,076 words, real BT Business pricing), so this was a targeted enhancement rather than a rewrite. Added a real cross-provider contrast this session had already independently confirmed on Zen Internet's own provider page (free static IP included on every plan) and freshly verified for Vodafone Business (Essential offers one on request at ~GBP5/mo+VAT, Pro includes it as standard, up to 8 orderable at a fixed price) -- caught and corrected an initial draft claim about Vodafone's policy against a fresh source before shipping. Word count 1,076 -&gt; 1,151.</t>
         </is>
       </c>
-      <c r="F73" s="3" t="n">
+      <c r="F74" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="G73" s="3" t="n">
+      <c r="G74" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="H73" s="3" t="inlineStr">
+      <c r="H74" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I73" s="3" t="inlineStr">
+      <c r="I74" s="2" t="inlineStr">
         <is>
           <t>app/guides/[slug]/page.tsx (static-ip-business-broadband-explained), data/guides.ts</t>
         </is>
       </c>
-      <c r="J73" s="3" t="inlineStr">
+      <c r="J74" s="2" t="inlineStr">
         <is>
           <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
-      <c r="K73" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L73" s="3" t="inlineStr">
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
         <is>
           <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L73"/>
+  <autoFilter ref="A1:L74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -12339,7 +12439,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>105 total (33 page builds, 72 feature/strategy builds); 91 already marked Done.</t>
+          <t>106 total (33 page builds, 73 feature/strategy builds); 92 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: restore live-verified status in keyword-mapping Content Gap Roadmap
A test run of build_keyword_mapping.py --offline had overwritten the
Content Gap Roadmap's "Built, live and deployed on Vercel" status with
"Planned -- live check unavailable" placeholders for all 33 tracked
pages, since --offline skips the live sitemap crawl entirely. Re-ran
online to restore accurate status, confirmed via
analyze_content_priority.py that 0 pages are genuinely pending.

Also bundles the concurrently-running content pipeline's Awin outreach
tracking additions to build_master_tracker.py and a new review-evidence
panel component, already present in the working tree and validated by
the build above.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -10,19 +10,23 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending Build Priority" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Page Builds" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature &amp; Strategy Builds" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly SEO Actions" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Awin Outreach Priority" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Page &amp; Content Priority" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Page Builds" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature &amp; Strategy Builds" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly SEO Actions" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$107</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$74</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Awin Outreach Priority'!$A$1:$M$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Page &amp; Content Priority'!$A$1:$I$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Methodology'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -167,8 +171,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReadMeTable" displayName="ReadMeTable" ref="A1:B7" headerRowCount="1">
-  <autoFilter ref="A1:B7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReadMeTable" displayName="ReadMeTable" ref="A1:B9" headerRowCount="1">
+  <autoFilter ref="A1:B9"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Field"/>
     <tableColumn id="2" name="Detail"/>
@@ -199,8 +203,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PendingBuildPriorityTable" displayName="PendingBuildPriorityTable" ref="A1:N15" headerRowCount="1">
-  <autoFilter ref="A1:N15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PendingBuildPriorityTable" displayName="PendingBuildPriorityTable" ref="A1:N14" headerRowCount="1">
+  <autoFilter ref="A1:N14"/>
   <tableColumns count="14">
     <tableColumn id="1" name="Pending Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -222,7 +226,47 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="PageBuildsTable" displayName="PageBuildsTable" ref="A1:L34" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="AwinOutreachPriorityTable" displayName="AwinOutreachPriorityTable" ref="A1:M21" headerRowCount="1">
+  <autoFilter ref="A1:M21"/>
+  <tableColumns count="13">
+    <tableColumn id="1" name="Rank"/>
+    <tableColumn id="2" name="Priority Band"/>
+    <tableColumn id="3" name="Advertiser"/>
+    <tableColumn id="4" name="Awin Advertiser ID"/>
+    <tableColumn id="5" name="Relationship"/>
+    <tableColumn id="6" name="Recommended Action"/>
+    <tableColumn id="7" name="Relevant Live URL"/>
+    <tableColumn id="8" name="Timing / Gate"/>
+    <tableColumn id="9" name="Status"/>
+    <tableColumn id="10" name="Owner"/>
+    <tableColumn id="11" name="Last Contacted"/>
+    <tableColumn id="12" name="Next Follow-up"/>
+    <tableColumn id="13" name="Decision / Feedback"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="PageContentPriorityTable" displayName="PageContentPriorityTable" ref="A1:I25" headerRowCount="1">
+  <autoFilter ref="A1:I25"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="Rank"/>
+    <tableColumn id="2" name="Workstream"/>
+    <tableColumn id="3" name="Target"/>
+    <tableColumn id="4" name="Opportunity"/>
+    <tableColumn id="5" name="Priority Source"/>
+    <tableColumn id="6" name="Source Score"/>
+    <tableColumn id="7" name="Status"/>
+    <tableColumn id="8" name="Evidence"/>
+    <tableColumn id="9" name="Recommended Action"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PageBuildsTable" displayName="PageBuildsTable" ref="A1:L34" headerRowCount="1">
   <autoFilter ref="A1:L34"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
@@ -242,8 +286,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L74" headerRowCount="1">
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L74" headerRowCount="1">
   <autoFilter ref="A1:L74"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
@@ -263,9 +307,9 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="MethodologyTable" displayName="MethodologyTable" ref="A1:B7" headerRowCount="1">
-  <autoFilter ref="A1:B7"/>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="MethodologyTable" displayName="MethodologyTable" ref="A1:B9" headerRowCount="1">
+  <autoFilter ref="A1:B9"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Aspect"/>
     <tableColumn id="2" name="Detail"/>
@@ -274,8 +318,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="WeeklySEOActionsTable" displayName="WeeklySEOActionsTable" ref="A1:P31" headerRowCount="1">
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="WeeklySEOActionsTable" displayName="WeeklySEOActionsTable" ref="A1:P31" headerRowCount="1">
   <autoFilter ref="A1:P31"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Rank"/>
@@ -588,7 +632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -627,7 +671,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -670,17 +714,41 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>Focused views</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Awin Outreach Priority separates partnership actions. Page &amp; Content Priority separates page creation, thin-content work and evidence-led SEO improvements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Roadmap state</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>There are currently no unbuilt rows remaining in the page-build roadmap. Page &amp; Content Priority therefore focuses on thin-content audits, existing-page improvements and the future research-page bet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
           <t>Re-run</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>python3 scripts/build_master_tracker.py</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B7"/>
+  <autoFilter ref="A1:B9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2294,12 +2362,16 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr"/>
       <c r="K35" s="3" t="inlineStr"/>
-      <c r="L35" s="3" t="inlineStr"/>
+      <c r="L35" s="3" t="inlineStr">
+        <is>
+          <t>Shipped to Vercel production 2026-08-26: added one shared, accessible review-evidence module to every provider and provider-comparison page. The module keeps Ofcom complaints, Ofcom satisfaction, Which? survey scores and public Trustpilot sentiment separate instead of inventing a blended trust score; dates each signal, explains limitations, links to sources and methodology, identifies unavailable data without penalising smaller providers, and suppresses current-score claims for retired providers.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -5492,7 +5564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5643,48 +5715,48 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>feat-review-aggregation-module</t>
+          <t>ops-adsense-site-review</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Monetisation</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Real review-aggregation trust module</t>
+          <t>Complete AdSense site review and authorisation monitoring</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>New shared component, used on provider + comparison pages</t>
+          <t>AdSense status and /ads.txt</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>research/uk-broadband-customer-satisfaction methodology</t>
+          <t>Google site-review processing</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr"/>
@@ -5697,48 +5769,48 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>ops-adsense-site-review</t>
+          <t>audit-city-hub-thinness</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Monetisation</t>
+          <t>Content audit</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Complete AdSense site review and authorisation monitoring</t>
+          <t>Verify each new city hub has a genuinely local fact</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>AdSense status and /ads.txt</t>
+          <t>data/priority-pages.ts city entries</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Google site-review processing</t>
+          <t>None</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr"/>
@@ -5751,48 +5823,48 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>audit-city-hub-thinness</t>
+          <t>feat-contact-form-email-delivery</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Content audit</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Verify each new city hub has a genuinely local fact</t>
+          <t>Working contact form delivering to a real inbox, no third-party service</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>50</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>data/priority-pages.ts city entries</t>
+          <t>app/api/contact/route.ts, components/ContactForm.tsx, app/contact/page.tsx</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CONTACT_SMTP_USER / CONTACT_SMTP_PASS Gmail App Password set in Vercel env vars</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr"/>
@@ -5805,33 +5877,33 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>feat-contact-form-email-delivery</t>
+          <t>growth-original-research-outreach</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Working contact form delivering to a real inbox, no third-party service</t>
+          <t>Run original-research outreach and digital PR</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -5841,12 +5913,12 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>app/api/contact/route.ts, components/ContactForm.tsx, app/contact/page.tsx</t>
+          <t>/research/uk-broadband-customer-satisfaction</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>CONTACT_SMTP_USER / CONTACT_SMTP_PASS Gmail App Password set in Vercel env vars</t>
+          <t>Research page and source methodology are live</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr"/>
@@ -5859,29 +5931,29 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>growth-original-research-outreach</t>
+          <t>growth-quarterly-data-reprioritisation</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
           <t>Growth</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Run original-research outreach and digital PR</t>
+          <t>Reprioritise quarter two using GSC, engagement and affiliate evidence</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
@@ -5890,17 +5962,17 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>/research/uk-broadband-customer-satisfaction</t>
+          <t>Next-quarter decision log</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Research page and source methodology are live</t>
+          <t>ops-conversion-reporting-loop and sufficient observation period</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr"/>
@@ -5913,29 +5985,29 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>growth-quarterly-data-reprioritisation</t>
+          <t>feat-price-drop-alerts</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Strategy</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Growth</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Reprioritise quarter two using GSC, engagement and affiliate evidence</t>
+          <t>Price-drop alerts</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -5949,12 +6021,12 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Next-quarter decision log</t>
+          <t>New subscription flow + data/provider-live-deals.json</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>ops-conversion-reporting-loop and sufficient observation period</t>
+          <t>Email delivery provider</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr"/>
@@ -5967,29 +6039,29 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>feat-price-drop-alerts</t>
+          <t>audit-core-web-vitals-reporting</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Price-drop alerts</t>
+          <t>Establish monthly Core Web Vitals reporting by template</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
@@ -6003,12 +6075,12 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>New subscription flow + data/provider-live-deals.json</t>
+          <t>Sitewide template performance report</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Email delivery provider</t>
+          <t>Field data or representative lab baselines</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr"/>
@@ -6021,29 +6093,29 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>audit-core-web-vitals-reporting</t>
+          <t>audit-mobile-checkout-flow</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>UX audit</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Establish monthly Core Web Vitals reporting by template</t>
+          <t>Mobile checkout-flow audit</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -6057,12 +6129,12 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Sitewide template performance report</t>
+          <t>Sitewide mobile layout</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Field data or representative lab baselines</t>
+          <t>Mobile analytics/drop-off data</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr"/>
@@ -6075,33 +6147,33 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>audit-mobile-checkout-flow</t>
+          <t>audit-broken-links-redirects</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>UX audit</t>
+          <t>Technical SEO</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Crawlability</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Mobile checkout-flow audit</t>
+          <t>Add routine broken-link and redirect reporting</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -6111,12 +6183,12 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Sitewide mobile layout</t>
+          <t>Sitewide crawl and redirect report</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Mobile analytics/drop-off data</t>
+          <t>None</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr"/>
@@ -6129,33 +6201,33 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>audit-broken-links-redirects</t>
+          <t>bet-annual-research-report</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Technical SEO</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Crawlability</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Add routine broken-link and redirect reporting</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -6165,12 +6237,12 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Sitewide crawl and redirect report</t>
+          <t>New annual research page + methodology extension</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>research/uk-broadband-customer-satisfaction methodology</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr"/>
@@ -6183,7 +6255,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>bet-annual-research-report</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -6193,19 +6265,19 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F13" s="3" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
@@ -6219,12 +6291,12 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>New annual research page + methodology extension</t>
+          <t>components/</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>research/uk-broadband-customer-satisfaction methodology</t>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr"/>
@@ -6237,7 +6309,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>bet-componentise-interactive-layer</t>
+          <t>bet-decouple-content-from-code</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -6247,19 +6319,19 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -6273,74 +6345,20 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>components/</t>
+          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+          <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr"/>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>bet-decouple-content-from-code</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Bigger bet</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Decouple guide content from code deploys</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G15" s="3" t="n">
-        <v>48</v>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t>None, but easier before the guide count grows further</t>
-        </is>
-      </c>
-      <c r="L15" s="3" t="inlineStr"/>
-      <c r="M15" s="3" t="inlineStr"/>
-      <c r="N15" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N15"/>
+  <autoFilter ref="A1:N14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6349,6 +6367,2150 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Priority Band</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Advertiser</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Awin Advertiser ID</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Relationship</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Recommended Action</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Relevant Live URL</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Timing / Gate</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Last Contacted</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Next Follow-up</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Decision / Feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>P0 Activate joined</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>TalkTalk</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>3674</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Joined</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Verify the tracked deep link, feature the programme on relevant pages and reconcile GA4 outbound clicks against Awin transactions.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/talktalk</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Now: approved revenue opportunity</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>P0 Activate joined</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Zzoomm</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>40398</v>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Joined</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Verify the tracked deep link, feature the programme on relevant pages and reconcile GA4 outbound clicks against Awin transactions.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/zzoomm</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Now: approved revenue opportunity</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr"/>
+      <c r="L3" s="3" t="inlineStr"/>
+      <c r="M3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>P0 Activate joined</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Highland Broadband</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>99387</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Joined</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Verify the tracked deep link, feature the programme on relevant pages and reconcile GA4 outbound clicks against Awin transactions.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/highland-broadband</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Now: approved revenue opportunity</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>P0 Activate joined</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Broadband Genie</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Joined</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Verify the tracked deep link, feature the programme on relevant pages and reconcile GA4 outbound clicks against Awin transactions.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/compare</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Now: approved revenue opportunity</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr"/>
+      <c r="M5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>P1 Follow up pending</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Community Fibre</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>19595</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Check API status and send one tailored follow-up with the relevant live page, audience evidence and compliance controls.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/community-fibre</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>After a reasonable review interval</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Waiting on advertiser</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>P1 Follow up pending</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Zen Internet</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>119927</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Check API status and send one tailored follow-up with the relevant live page, audience evidence and compliance controls.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/zen</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>After a reasonable review interval</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on advertiser</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>P1 Follow up pending</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>National Broadband</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>20858</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Check API status and send one tailored follow-up with the relevant live page, audience evidence and compliance controls.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/national-broadband</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>After a reasonable review interval</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Waiting on advertiser</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>P1 Follow up pending</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Trooli</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>25528</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Check API status and send one tailored follow-up with the relevant live page, audience evidence and compliance controls.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/trooli</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>After a reasonable review interval</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on advertiser</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr"/>
+      <c r="M9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>P1 Follow up pending</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Pine Media</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>27840</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Check API status and send one tailored follow-up with the relevant live page, audience evidence and compliance controls.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/pine-media</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>After a reasonable review interval</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Waiting on advertiser</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>P1 Follow up pending</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Cuckoo</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>118743</v>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Check API status and send one tailored follow-up with the relevant live page, audience evidence and compliance controls.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/cuckoo</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>After a reasonable review interval</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on advertiser</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr"/>
+      <c r="M11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>P1 Follow up pending</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Sky ROI</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Check API status and send one tailored follow-up with the relevant live page, audience evidence and compliance controls.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/sky</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>After a reasonable review interval</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Waiting on advertiser</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>P2 Reapply with evidence</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>BT Consumer</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>3041</v>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Reapply selectively with stronger GSC traffic, GA4 commercial-click and content-quality evidence; record the rejection reason first.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/bt</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Gate on stronger evidence; do not bulk reapply</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr"/>
+      <c r="K13" s="3" t="inlineStr"/>
+      <c r="L13" s="3" t="inlineStr"/>
+      <c r="M13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>P2 Reapply with evidence</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>BT Business</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>3042</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Reapply selectively with stronger GSC traffic, GA4 commercial-click and content-quality evidence; record the rejection reason first.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/bt</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Gate on stronger evidence; do not bulk reapply</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>P2 Reapply with evidence</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Virgin Media</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>6399</v>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Reapply selectively with stronger GSC traffic, GA4 commercial-click and content-quality evidence; record the rejection reason first.</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/virgin-media</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Gate on stronger evidence; do not bulk reapply</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr"/>
+      <c r="K15" s="3" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr"/>
+      <c r="M15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>P2 Reapply with evidence</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>EE</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>3516</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Reapply selectively with stronger GSC traffic, GA4 commercial-click and content-quality evidence; record the rejection reason first.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/ee</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Gate on stronger evidence; do not bulk reapply</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>P2 Reapply with evidence</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Plusnet</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>2973</v>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Reapply selectively with stronger GSC traffic, GA4 commercial-click and content-quality evidence; record the rejection reason first.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/plusnet</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Gate on stronger evidence; do not bulk reapply</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr"/>
+      <c r="K17" s="3" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr"/>
+      <c r="M17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>P2 Reapply with evidence</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Vodafone</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>1257</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Reapply selectively with stronger GSC traffic, GA4 commercial-click and content-quality evidence; record the rejection reason first.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/vodafone</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Gate on stronger evidence; do not bulk reapply</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>P2 Reapply with evidence</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Hyperoptic</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>5737</v>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Reapply selectively with stronger GSC traffic, GA4 commercial-click and content-quality evidence; record the rejection reason first.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/hyperoptic</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Gate on stronger evidence; do not bulk reapply</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr"/>
+      <c r="K19" s="3" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr"/>
+      <c r="M19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>P2 Reapply with evidence</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>toob</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>117433</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Reapply selectively with stronger GSC traffic, GA4 commercial-click and content-quality evidence; record the rejection reason first.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/toob</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Gate on stronger evidence; do not bulk reapply</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>P2 Reapply with evidence</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>giffgaff</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>3599</v>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Reapply selectively with stronger GSC traffic, GA4 commercial-click and content-quality evidence; record the rejection reason first.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/giffgaff</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Gate on stronger evidence; do not bulk reapply</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr"/>
+      <c r="K21" s="3" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr"/>
+      <c r="M21" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M21"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Workstream</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Opportunity</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Priority Source</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Source Score</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Recommended Action</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Thin-content audit</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>data/priority-pages.ts city entries</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Verify each new city hub has a genuinely local fact</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Master tracker</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>8 new city hubs (Birmingham, Bristol, Edinburgh, Glasgow, Leeds, Liverpool, Manchester, Sheffield) plus 50 existing postcode-prefix pages is a lot of near-identical templates. Each needs at least one real local fact (a named local altnet, a real coverage figure) or it reads as duplicate content — audit before building the next batch of cities.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Audit each city hub and add a genuinely local, sourced fact where missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/m1</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 56; CTR 0; position 12.875; top queries: m1 broadband; cheap broadband deals manchester; m1 wifi broadband; m1 internet plan; m1 internet broadband</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/ng1</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 132; CTR 0; position 13.64393939393939; top queries: broadband deals nottingham; broadband deals in nottingham; broadband deals nottinghamshire; internet deals nottingham; cheapest broadband nottingham</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/rg1</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 126; CTR 0; position 14.90476190476191; top queries: broadband deals in reading; broadband in reading; broadband deals reading; broadband reading; cheapest</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/ct1</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 120; CTR 0; position 9.866666666666667; top queries: broadband deals in canterbury</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>/providers/compare/ee-vs-talktalk</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Clicks 2; impressions 107; CTR 0.01869158878504673; position 8.317757009345794; top queries: is ee broadband better than talktalk; are talktalk and ee the same; who is dido harding; talktalk.co.uk/homesafe; talktalk uswitch</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/rm1</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 94; CTR 0; position 9.574468085106384; top queries: broadband deals in romford; broadband deals romford; internet deals romford; best internet provider romford; whats the best broadband in my area</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>/guides/broadband-deals-with-cashback</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 91; CTR 0; position 14.54945054945055; top queries: compare broadband providers with cashback; broadband price rises with cashback; compare internet providers with cashback; broadband switching deals with cashback; where should i look for broadband deals that offer extra perks?</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/bs1</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Page-two opportunity</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Clicks 1; impressions 105; CTR 0.009523809523809525; position 21.93333333333333; top queries: broadband deals bristol; broadband deals in bristol; best broadband deals bristol; best broadband deals in bristol</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/e1</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Clicks 1; impressions 77; CTR 0.01298701298701299; position 4.870129870129871; top queries: yes please; ee whitechapel; e1</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/ne1</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Page-two opportunity</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 97; CTR 0; position 23.11340206185567; top queries: broadband deals newcastle; broadband deals in newcastle; broadband newcastle; broadband deals north tyneside; best broadband deals newcastle</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/bn1</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Clicks 1; impressions 73; CTR 0.0136986301369863; position 11.49315068493151; top queries: broadband deals in brighton; broadband deals brighton</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/gu1</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Clicks 1; impressions 65; CTR 0.01538461538461539; position 11.64615384615385; top queries: broadband deals in guildford</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/ha1</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 60; CTR 0; position 8.533333333333333; top queries: broadband deals in harrow; ha1 4bh; ha1; broadband</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>/guides/broadband-deals-with-no-setup-fee</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Page-two opportunity</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 548; CTR 0; position 26.25547445255474; top queries: broadband deals no upfront cost; broadband no upfront cost; broadband and tv deals no upfront cost; broadband no upfront costs; broadband no setup fee</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/w5</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 56; CTR 0; position 6.732142857142857; top queries: None</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/se1</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 53; CTR 0; position 6.037735849056604; top queries: find the best broadband deals in southwark under £30 a month.; find the best broadband deals in southwark under £25 a month.; fibre broadband in southwark</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/en1</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 43; CTR 0; position 14.13953488372093; top queries: broadband deals in enfield</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/nw1</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 40; CTR 0; position 4.9; top queries: None</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/ub1</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Quick ranking win</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 40; CTR 0; position 8.025; top queries: broadband deals in southall; yes; and cheapest</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/lu1</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Page-two opportunity</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 128; CTR 0; position 15.546875; top queries: broadband deals in luton; broadband deals luton; broadband luton; internet providers luton; broadband deals near me</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>/postcode/so14</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Page-two opportunity</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Clicks 1; impressions 104; CTR 0.009615384615384616; position 26.42307692307692; top queries: broadband deals in southampton; broadband deals southampton; broadband company southampton; internet providers southampton; fibre broadband southampton</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Existing-page SEO improvement</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>/postcode/l1</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Page-two opportunity</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Weekly GSC/GA4 action queue</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Clicks 0; impressions 77; CTR 0; position 26.25974025974026; top queries: broadband deals liverpool; broadband comparison liverpool; internet deals liverpool; broadband deals in liverpool; best broadband deals liverpool</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>New evidence-led page</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>New annual research page + methodology extension</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Annual 'State of UK Broadband' research report</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Master tracker</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Build after higher-confidence thin-content and ranking opportunities.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I25"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8224,7 +10386,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8972,7 +11134,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
@@ -12406,13 +14568,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12439,7 +14601,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>106 total (33 page builds, 73 feature/strategy builds); 92 already marked Done.</t>
+          <t>106 total (33 page builds, 73 feature/strategy builds); 93 already marked Done.</t>
         </is>
       </c>
     </row>
@@ -12494,17 +14656,41 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>Awin outreach</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Awin Outreach Priority is ordered by action stage: activate joined programmes, follow up pending applications, then make selective evidence-led reapplications. Manual outreach fields survive regeneration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Page/content queue</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Page &amp; Content Priority combines the tracker thin-content audit with non-monitor weekly GSC/GA4 opportunities. Source scores use different models and are labelled; the list is a working sequence, not a claim that the scores are directly comparable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
           <t>Editing this file</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Status/Owner/Target Date/Notes are yours to edit freely — they survive the next `python3 scripts/build_master_tracker.py` run.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B7"/>
+  <autoFilter ref="A1:B9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -12512,7 +14698,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
tracker: log the M1/NG1/RG1/CT1/RM1 postcode de-duplication build
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -19,12 +19,12 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$107</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Awin Outreach Priority'!$A$1:$M$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Page &amp; Content Priority'!$A$1:$I$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Methodology'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Weekly SEO Actions'!$A$1:$P$31</definedName>
   </definedNames>
@@ -182,8 +182,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L107" headerRowCount="1">
-  <autoFilter ref="A1:L107"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MasterTrackerTable" displayName="MasterTrackerTable" ref="A1:L108" headerRowCount="1">
+  <autoFilter ref="A1:L108"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -203,8 +203,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PendingBuildPriorityTable" displayName="PendingBuildPriorityTable" ref="A1:N14" headerRowCount="1">
-  <autoFilter ref="A1:N14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PendingBuildPriorityTable" displayName="PendingBuildPriorityTable" ref="A1:N15" headerRowCount="1">
+  <autoFilter ref="A1:N15"/>
   <tableColumns count="14">
     <tableColumn id="1" name="Pending Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -287,8 +287,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L74" headerRowCount="1">
-  <autoFilter ref="A1:L74"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="FeatureStrategyBuildTable" displayName="FeatureStrategyBuildTable" ref="A1:L75" headerRowCount="1">
+  <autoFilter ref="A1:L75"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Type"/>
@@ -671,7 +671,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
+          <t>content-refresh-postcode-m1-ng1-rg1-ct1-rm1</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -4998,14 +4998,14 @@
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>De-duplicate 5 postcode pages with genuinely local, sourced content (M1, NG1, RG1, CT1, RM1)</t>
         </is>
       </c>
       <c r="F95" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G95" s="3" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-existing-customers-guide</t>
+          <t>content-refresh-best-rolling-monthly-broadband-guide</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -5042,14 +5042,14 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals for Existing Customers guide (42nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F96" s="2" t="n">
         <v>33</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-price-rises-2026-guide</t>
+          <t>content-refresh-broadband-existing-customers-guide</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -5086,14 +5086,14 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Broadband Deals for Existing Customers guide (42nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F97" s="3" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G97" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
@@ -5115,7 +5115,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-one-touch-switching-explained-guide</t>
+          <t>content-refresh-broadband-price-rises-2026-guide</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -5130,14 +5130,14 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: One Touch Switching Explained guide (44th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="F98" s="2" t="n">
         <v>32</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
@@ -5159,7 +5159,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-full-fibre-broadband-explained-guide</t>
+          <t>content-refresh-one-touch-switching-explained-guide</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -5174,14 +5174,14 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: One Touch Switching Explained guide (44th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F99" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G99" s="3" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
@@ -5203,7 +5203,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-students-guide</t>
+          <t>content-refresh-full-fibre-broadband-explained-guide</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -5218,14 +5218,14 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -5247,7 +5247,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-no-setup-fee-guide</t>
+          <t>content-refresh-best-broadband-for-students-guide</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -5262,14 +5262,14 @@
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F101" s="3" t="n">
         <v>30</v>
       </c>
       <c r="G101" s="3" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
@@ -5291,7 +5291,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-streaming-guide</t>
+          <t>content-refresh-broadband-deals-no-setup-fee-guide</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -5306,14 +5306,14 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F102" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-can-i-leave-broadband-early-guide</t>
+          <t>content-refresh-best-broadband-for-streaming-guide</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -5350,14 +5350,14 @@
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F103" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G103" s="3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
@@ -5379,7 +5379,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
+          <t>content-refresh-can-i-leave-broadband-early-guide</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -5394,11 +5394,11 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F104" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G104" s="2" t="n">
         <v>26</v>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-speeds-explained-guide</t>
+          <t>content-refresh-best-broadband-for-rural-areas-guide</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -5438,14 +5438,14 @@
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F105" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G105" s="3" t="n">
         <v>26</v>
-      </c>
-      <c r="G105" s="3" t="n">
-        <v>25</v>
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>content-refresh-broadband-deals-with-cashback-guide</t>
+          <t>content-refresh-broadband-speeds-explained-guide</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -5482,14 +5482,14 @@
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F106" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G106" s="2" t="n">
         <v>25</v>
-      </c>
-      <c r="G106" s="2" t="n">
-        <v>23</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>content-refresh-static-ip-business-broadband-guide</t>
+          <t>content-refresh-broadband-deals-with-cashback-guide</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
@@ -5526,18 +5526,18 @@
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>Update: Static IP Business Broadband guide (43rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="F107" s="3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G107" s="3" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I107" s="3" t="inlineStr">
@@ -5549,8 +5549,52 @@
       <c r="K107" s="3" t="inlineStr"/>
       <c r="L107" s="3" t="inlineStr"/>
     </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>content-refresh-static-ip-business-broadband-guide</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>Update: Static IP Business Broadband guide (43rd content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="G108" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr"/>
+      <c r="K108" s="2" t="inlineStr"/>
+      <c r="L108" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L107"/>
+  <autoFilter ref="A1:L108"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5564,11 +5608,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
@@ -6357,8 +6401,62 @@
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr"/>
     </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>content-refresh-postcode-m1-ng1-rg1-ct1-rm1</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>De-duplicate 5 postcode pages with genuinely local, sourced content (M1, NG1, RG1, CT1, RM1)</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>app/postcode/[area]/page.tsx, data/postcodeLocalIntel.ts</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr"/>
+      <c r="M15" s="3" t="inlineStr"/>
+      <c r="N15" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N14"/>
+  <autoFilter ref="A1:N15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8526,7 +8624,7 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="31" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
@@ -8627,7 +8725,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -8681,7 +8779,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -8735,7 +8833,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -8789,7 +8887,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -8843,7 +8941,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -8897,7 +8995,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -8951,7 +9049,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -9005,7 +9103,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -9059,7 +9157,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -9113,7 +9211,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -9167,7 +9265,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -9221,7 +9319,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -9275,7 +9373,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -9329,7 +9427,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -9383,7 +9481,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -9437,7 +9535,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -9491,7 +9589,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -9545,7 +9643,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -9599,7 +9697,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -9653,7 +9751,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -9707,7 +9805,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -9761,7 +9859,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -9815,7 +9913,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -9869,7 +9967,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -9923,7 +10021,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -9977,7 +10075,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -10031,7 +10129,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -10085,7 +10183,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -10139,7 +10237,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -10193,7 +10291,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -10247,7 +10345,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -10301,7 +10399,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -10355,7 +10453,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Live but not committed to git</t>
+          <t>Committed</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -10392,7 +10490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13847,19 +13945,19 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
+          <t>De-duplicate 5 postcode pages with genuinely local, sourced content (M1, NG1, RG1, CT1, RM1)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
+          <t>User-flagged near-duplicate-content risk: /postcode/[area] is a single shared template, and every district page beyond the DA1 special case only swapped Ofcom coverage numbers into otherwise identical boilerplate sentences. Inspected the template (app/postcode/[area]/page.tsx) and the curated dataset (data/postcodes.ts), then researched real, sourced local network facts for each of the 5 requested districts -- CityFibre/Openreach/Virgin Media/Community Fibre rollout investment figures, completion dates, named neighbourhoods, and honest coverage gaps (e.g. Canterbury/CT1 not yet in Openreach's Kent Fibre First build; Havering's uneven rollout leaving South Hornchurch and Rainham behind while RM1 itself sits in Community Fibre's core area). Added new data/postcodeLocalIntel.ts (hand-verified only, not a mapping for all 2,818 districts) and wired it into 4 new generalised template sections plus a widened 'coverage at a glance' callout and FAQ enhancement, without touching DA1's existing bespoke content. Each page grew from ~600-700 generic words to ~1,400-1,500 words of area-specific, sourced content. Verified via tsc, npm run build, and word/apostrophe/undefined checks both locally and on the live production URL for all 5 pages.</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -13868,7 +13966,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
+          <t>app/postcode/[area]/page.tsx, data/postcodeLocalIntel.ts</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -13883,7 +13981,7 @@
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-27/28 — 'the postcode pages share templates, so they should not all receive generic expanded copy'</t>
         </is>
       </c>
     </row>
@@ -13903,19 +14001,19 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals for Existing Customers guide (42nd content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Rolling Monthly Broadband Deals guide (18th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Tenth target in the second 13-page batch: 689 words of correct but entirely generic negotiation advice with no real figures. Added the GBP183.60/year switching-savings stat (already verified this session for the moving-house guide), the One Touch Switch enforcement-closure news (11 June 2026, permanent industry standard), and a new section reframing a scheduled price rise notification as a genuine, low-friction negotiation trigger, citing the real current rise figures already established this session (BT/EE GBP4/mo March, TalkTalk GBP4/mo from Nov 2025 contracts, Sky GBP3/mo April 2026). Word count 689 -&gt; 946.</t>
+          <t>Eighteenth target from scripts/analyze_content_priority.py's ranked list: 522 words repeating the same stale claim caught twice already this session -- 'NOW Broadband is often relevant because of its shorter 12-month positioning,' when NOW dropped flexible contracts entirely and now sells only a standard 24-month term. This page's whole premise rested on that wrong claim, so it needed a real replacement for 'who actually offers flexible broadband now,' not just a correction. Rewrote around YouFibre, confirmed via its own already-rewritten provider page as one of the only genuine rolling-monthly full-fibre options left (from GBP33.99/mo, 30 days' notice, vs GBP20/mo on its own 24-month term), plus Hyperoptic/Community Fibre/Onestream's 12-month middle-ground option, and a note on social tariffs' no-exit-fee terms. Word count 522 -&gt; 907.</t>
         </is>
       </c>
       <c r="F63" s="3" t="n">
         <v>33</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
@@ -13924,7 +14022,7 @@
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-for-existing-customers), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-rolling-monthly-broadband-deals), data/guides.ts</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
@@ -13939,7 +14037,7 @@
       </c>
       <c r="L63" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -13959,19 +14057,19 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
+          <t>Deep rewrite: Broadband Deals for Existing Customers guide (42nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
+          <t>Tenth target in the second 13-page batch: 689 words of correct but entirely generic negotiation advice with no real figures. Added the GBP183.60/year switching-savings stat (already verified this session for the moving-house guide), the One Touch Switch enforcement-closure news (11 June 2026, permanent industry standard), and a new section reframing a scheduled price rise notification as a genuine, low-friction negotiation trigger, citing the real current rise figures already established this session (BT/EE GBP4/mo March, TalkTalk GBP4/mo from Nov 2025 contracts, Sky GBP3/mo April 2026). Word count 689 -&gt; 946.</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -13980,7 +14078,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
+          <t>app/guides/[slug]/page.tsx (broadband-for-existing-customers), data/guides.ts</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -13995,7 +14093,7 @@
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -14015,19 +14113,19 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: One Touch Switching Explained guide (44th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Price Rises 2026 guide (19th and final content-priority-analysis target this session)</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Twelfth target in the second 13-page batch, and the single most relevant page on the site for the One Touch Switch enforcement-closure news (also added to how-to-switch-broadband-uk and broadband-for-existing-customers earlier this session) -- this page is literally about OTS specifically and was still missing the fact entirely: Ofcom closed its dedicated enforcement programme on 11 June 2026 after finding more than 2 million customers had already used it successfully, confirming OTS as the industry's permanent standard rather than a still-bedding-in pilot. Added a new dedicated section, updated the intro, and a matching new FAQ. Word count 731 -&gt; 921.</t>
+          <t>Nineteenth target from scripts/analyze_content_priority.py's ranked list. This page had the most individually-wrong data points found in a single page this session: TalkTalk was listed at +GBP2.50/mo (real current figure, verified via ISPreview, is +GBP4.00/mo for contracts from 16 November 2025 -- TalkTalk raised its own rise from GBP3 to GBP4 partway through the year); Hyperoptic and Community Fibre were both listed as 'No rise' when both apply a real scheduled increase (~GBP4/mo and a capped GBP2/mo respectively, confirmed against their own already-researched provider pages). Also caught and fixed a bug introduced earlier THIS session: the NOW Broadband provider page wrongly claimed NOW mirrors Sky's price rise at a flat GBP4/mo, corrected first in data/providers.ts (5 instances) before writing this page, to GBP0 in April 2026 with GBP3 scheduled for April 2027 and 2028. Added a dedicated section directly naming the 'no-rise altnet' assumption as false for 2 of the 4 providers commonly assumed to qualify. Word count 758 -&gt; 1,100.</t>
         </is>
       </c>
       <c r="F65" s="3" t="n">
         <v>32</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
@@ -14036,7 +14134,7 @@
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (one-touch-switching-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-price-rises-2026), data/guides.ts, data/providers.ts (now-broadband fix)</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
@@ -14051,7 +14149,7 @@
       </c>
       <c r="L65" s="3" t="inlineStr">
         <is>
-          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+          <t>User request 2026-08-24 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
@@ -14071,19 +14169,19 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
+          <t>Deep rewrite: One Touch Switching Explained guide (44th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
+          <t>Twelfth target in the second 13-page batch, and the single most relevant page on the site for the One Touch Switch enforcement-closure news (also added to how-to-switch-broadband-uk and broadband-for-existing-customers earlier this session) -- this page is literally about OTS specifically and was still missing the fact entirely: Ofcom closed its dedicated enforcement programme on 11 June 2026 after finding more than 2 million customers had already used it successfully, confirming OTS as the industry's permanent standard rather than a still-bedding-in pilot. Added a new dedicated section, updated the intro, and a matching new FAQ. Word count 731 -&gt; 921.</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -14092,7 +14190,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (one-touch-switching-explained), data/guides.ts</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -14127,19 +14225,19 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
+          <t>Deep rewrite: Full Fibre Broadband Explained guide (22nd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
+          <t>Twenty-second target from the wider content-priority-analysis list: 538 words with a stale 'speeds of up to 1,000 Mbps (1 Gbps) are achievable' ceiling claim and a vague 'Openreach targeting 25 million premises by 2026' coverage stat with no real current figure. Rewrote with Ofcom's actual Spring 2026 Connected Nations data (82% full-fibre coverage, 89% gigabit-capable, 93% urban vs 66% rural split) and updated the speed ceiling to reflect real current top tiers already verified on this site's own provider pages -- Community Fibre up to 3,000 Mbps and YouFibre up to 8,000 Mbps, both genuinely symmetrical, far beyond the old 1 Gbps benchmark. Added a new section connecting full fibre to the 31 January 2027 PSTN switch-off, reusing this session's own Digital Voice/power-cut research. Word count 538 -&gt; 922.</t>
         </is>
       </c>
       <c r="F67" s="3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G67" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
@@ -14148,7 +14246,7 @@
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (full-fibre-broadband-explained), data/guides.ts</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
@@ -14183,19 +14281,19 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Students guide (23rd content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Fourth target in the second 13-page batch: 648 words with a real error -- BT was listed in the 'mainstream, no setup fee' table row alongside Sky and EE, but BT genuinely charges a GBP30 setup fee (confirmed on its own already-corrected provider page this session), only offset by a reward card that must be actively claimed. Corrected the table and matching FAQ, and added a new section distinguishing a genuine fee (BT's GBP30, Virgin Media's GBP35 with no offset) from a fee that functions as free (NOW Broadband's GBP5 advance fee, credited back to the first bill) -- a real distinction the old page collapsed into a single 'usually fee-charging' bucket. Word count 648 -&gt; 812.</t>
+          <t>Twenty-third target from the wider content-priority-analysis list, and the third page this session found repeating the exact same stale claim: 'NOW Broadband is often relevant because its shorter-term positioning can suit student tenancies' (also wrongly caught and fixed on best-rolling-monthly-broadband-deals and broadband-deals-under-20 earlier this session). Also corrected 'TalkTalk can work well for low-cost shared houses', no longer true now that TalkTalk starts at GBP25/mo. Replaced both with the real current options: YouFibre's genuine rolling monthly contract (from GBP33.99/mo) for uncertain tenancies, and Onestream (GBP18.50/mo, 94% Openreach coverage) as the realistic default for most student addresses, alongside Hyperoptic/Community Fibre's 12-month middle ground. Added a new common-mistake bullet: assuming a provider still offers the contract type it was known for in previous years. Word count 668 -&gt; 887.</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
         <v>30</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -14204,7 +14302,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-deals-with-no-setup-fee), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-students), data/guides.ts</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -14239,19 +14337,19 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Deals With No Setup Fee guide (36th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
+          <t>Fourth target in the second 13-page batch: 648 words with a real error -- BT was listed in the 'mainstream, no setup fee' table row alongside Sky and EE, but BT genuinely charges a GBP30 setup fee (confirmed on its own already-corrected provider page this session), only offset by a reward card that must be actively claimed. Corrected the table and matching FAQ, and added a new section distinguishing a genuine fee (BT's GBP30, Virgin Media's GBP35 with no offset) from a fee that functions as free (NOW Broadband's GBP5 advance fee, credited back to the first bill) -- a real distinction the old page collapsed into a single 'usually fee-charging' bucket. Word count 648 -&gt; 812.</t>
         </is>
       </c>
       <c r="F69" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
@@ -14260,7 +14358,7 @@
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-with-no-setup-fee), data/guides.ts</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
@@ -14295,19 +14393,19 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Streaming guide (26th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
+          <t>Twenty-sixth target: 699 words naming providers (Sky, Virgin Media, Community Fibre, Hyperoptic) with zero real prices attached. Added current prices for all 4, plus Virgin Media's real 1,130 Mbps top speed. Added a genuinely new, technically accurate explanation this page never covered: why evening buffering specifically affects FTTC and cable connections (shared capacity per street cabinet/node) but not full fibre (dedicated line per property), with a matching new FAQ. Word count 699 -&gt; 893.</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
@@ -14316,7 +14414,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-streaming), data/guides.ts</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -14351,16 +14449,16 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
+          <t>Deep rewrite: Can I Leave Broadband Early After a Price Rise guide (27th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
+          <t>Twenty-seventh target: 783 words of correct but entirely abstract legal explanation with zero real examples of what 'clearly disclosed' vs 'vague' price-rise wording actually looks like in practice. Added the concrete contrast this session's own research had already surfaced: BT and TalkTalk both disclose a flat, dated pounds-and-pence rise upfront (the clear case), while Sky's contract terms for years after the first only say prices 'may rise' without a fixed figure (the genuinely weaker disclosure case worth flagging). Added the specific 30-day notice/exit-window rule with a matching new FAQ. Caught and fixed 2 instances of the recurring backslash-apostrophe-in-JSX bug before shipping. Word count 783 -&gt; 1,068.</t>
         </is>
       </c>
       <c r="F71" s="3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G71" s="3" t="n">
         <v>26</v>
@@ -14372,7 +14470,7 @@
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (can-i-leave-broadband-early-after-price-rise), data/guides.ts</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
@@ -14407,20 +14505,20 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
+          <t>Deep rewrite: Best Broadband for Rural Areas guide (28th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Second target in the second 13-page batch: 476 words, the thinnest guide examined all session, with entirely generic, dateless content. Added a real Ofcom stat this page never had: average maximum available download speed is 285 Mbps (up ~30% from 223 Mbps), with the important nuance that median speed actually delivered on FTTC is closer to 80-100 Mbps -- the average and the typical experience are genuinely different things. Reused the FTTC/cable evening-congestion explanation (shared capacity per street cabinet/node) already written for best-broadband-for-streaming earlier this session, with a matching new FAQ. Added real current symmetrical-speed examples (Community Fibre 3,000Mbps, YouFibre 8,000Mbps). Word count 476 -&gt; 787.</t>
+          <t>Twenty-eighth target: 635 words naming only BT and EE, with a real content gap for a rural-specific guide -- no mention of satellite broadband at all, despite Starlink being one of the classic genuine rural use cases already covered in depth on this site's own satellite-broadband-uk guide earlier this session. Added real Ofcom Spring 2026 rural coverage data (66% rural vs 93% urban gigabit-capable), real 5G pricing (National Broadband from GBP34.99/mo as the multi-network specialist genuinely suited to rural addresses, Three from GBP29/mo, EE Smart 5G Hub), a full Starlink section with real pricing, and the Gigabit Broadband Voucher Scheme as a cost-effective alternative to satellite worth checking first. Word count 635 -&gt; 908.</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G72" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="G72" s="2" t="n">
-        <v>25</v>
-      </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -14428,7 +14526,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-speeds-explained), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (best-broadband-for-rural-areas-uk), data/guides.ts</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -14463,20 +14561,20 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+          <t>Deep rewrite: Broadband Speeds Explained guide (34th content-priority-analysis target)</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Third target in the second 13-page batch: 622 words with zero real numbers -- entirely abstract advice about 'gift cards' and 'cashback' with no concrete example of what a real reward is actually worth. Added BT's real reward card figures (GBP80-140, offsetting a GBP30 setup fee, already documented on BT's own provider page) and NOW Broadband's real GBP70-75 voucher pattern. Added a genuinely concrete counter-example using Community Fibre's no-reward GBP12.50/mo price to illustrate why a lower ongoing price can beat a bigger one-off card once the full term is compared, replacing the old page's entirely hypothetical framing. Word count 622 -&gt; 826.</t>
+          <t>Second target in the second 13-page batch: 476 words, the thinnest guide examined all session, with entirely generic, dateless content. Added a real Ofcom stat this page never had: average maximum available download speed is 285 Mbps (up ~30% from 223 Mbps), with the important nuance that median speed actually delivered on FTTC is closer to 80-100 Mbps -- the average and the typical experience are genuinely different things. Reused the FTTC/cable evening-congestion explanation (shared capacity per street cabinet/node) already written for best-broadband-for-streaming earlier this session, with a matching new FAQ. Added real current symmetrical-speed examples (Community Fibre 3,000Mbps, YouFibre 8,000Mbps). Word count 476 -&gt; 787.</t>
         </is>
       </c>
       <c r="F73" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G73" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="G73" s="3" t="n">
-        <v>23</v>
-      </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -14484,7 +14582,7 @@
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>app/guides/[slug]/page.tsx (broadband-deals-with-cashback), data/guides.ts</t>
+          <t>app/guides/[slug]/page.tsx (broadband-speeds-explained), data/guides.ts</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
@@ -14519,48 +14617,104 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
+          <t>Deep rewrite: Broadband Deals With Cashback guide (35th content-priority-analysis target)</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Third target in the second 13-page batch: 622 words with zero real numbers -- entirely abstract advice about 'gift cards' and 'cashback' with no concrete example of what a real reward is actually worth. Added BT's real reward card figures (GBP80-140, offsetting a GBP30 setup fee, already documented on BT's own provider page) and NOW Broadband's real GBP70-75 voucher pattern. Added a genuinely concrete counter-example using Community Fibre's no-reward GBP12.50/mo price to illustrate why a lower ongoing price can beat a bigger one-off card once the full term is compared, replacing the old page's entirely hypothetical framing. Word count 622 -&gt; 826.</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>app/guides/[slug]/page.tsx (broadband-deals-with-cashback), data/guides.ts</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>ops-content-priority-analysis-tooling</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
           <t>Update: Static IP Business Broadband guide (43rd content-priority-analysis target)</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr">
+      <c r="E75" s="3" t="inlineStr">
         <is>
           <t>Eleventh target in the second 13-page batch: already an excellent, precisely-dated, well-sourced page (1,076 words, real BT Business pricing), so this was a targeted enhancement rather than a rewrite. Added a real cross-provider contrast this session had already independently confirmed on Zen Internet's own provider page (free static IP included on every plan) and freshly verified for Vodafone Business (Essential offers one on request at ~GBP5/mo+VAT, Pro includes it as standard, up to 8 orderable at a fixed price) -- caught and corrected an initial draft claim about Vodafone's policy against a fresh source before shipping. Word count 1,076 -&gt; 1,151.</t>
         </is>
       </c>
-      <c r="F74" s="2" t="n">
+      <c r="F75" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="G74" s="2" t="n">
+      <c r="G75" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="H74" s="2" t="inlineStr">
+      <c r="H75" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I74" s="2" t="inlineStr">
+      <c r="I75" s="3" t="inlineStr">
         <is>
           <t>app/guides/[slug]/page.tsx (static-ip-business-broadband-explained), data/guides.ts</t>
         </is>
       </c>
-      <c r="J74" s="2" t="inlineStr">
+      <c r="J75" s="3" t="inlineStr">
         <is>
           <t>ops-content-priority-analysis-tooling</t>
         </is>
       </c>
-      <c r="K74" s="2" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L74" s="2" t="inlineStr">
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L75" s="3" t="inlineStr">
         <is>
           <t>User request 2026-08-25 — researched before implementing per the Strategic Lens process</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L74"/>
+  <autoFilter ref="A1:L75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -14601,7 +14755,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>106 total (33 page builds, 73 feature/strategy builds); 93 already marked Done.</t>
+          <t>107 total (33 page builds, 74 feature/strategy builds); 93 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: track Awin Activity Stream invitations (no API for these either)
Awin's Activity Stream ("X have invited you to join their programme") has
no API endpoint -- tested /activity, /activity-stream, /feed, /events,
/inbox, all 404. Add `add-invitation --name <advertiser> [--advertiser-id]
[--url] [--message]` to log one seen in the dashboard by hand; the
advertiser ID auto-resolves from the live notjoined catalogue if omitted.
New "Invited" relationship gets its own P1 band in the Awin Outreach
Priority sheet (Respond to invitation), ranked above Pending/Rejected since
an inbound invite is higher-intent than a cold application.

Logged the real Connect Fibre invitation (ID 114602, auto-resolved) from
today's Activity Stream screenshot and ran a fit assessment: 7/10, strong
category match but a small Midlands/East-of-England footprint and
unconfirmed commission terms.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -20,9 +20,9 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Tracker'!$A$1:$L$109</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Awin Outreach Priority'!$A$1:$M$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Page &amp; Content Priority'!$A$1:$I$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending Build Priority'!$A$1:$N$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Awin Outreach Priority'!$A$1:$M$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Page &amp; Content Priority'!$A$1:$I$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Page Builds'!$A$1:$L$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Feature &amp; Strategy Builds'!$A$1:$L$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Methodology'!$A$1:$B$9</definedName>
@@ -203,8 +203,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PendingBuildPriorityTable" displayName="PendingBuildPriorityTable" ref="A1:N15" headerRowCount="1">
-  <autoFilter ref="A1:N15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PendingBuildPriorityTable" displayName="PendingBuildPriorityTable" ref="A1:N14" headerRowCount="1">
+  <autoFilter ref="A1:N14"/>
   <tableColumns count="14">
     <tableColumn id="1" name="Pending Rank"/>
     <tableColumn id="2" name="Item ID"/>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="AwinOutreachPriorityTable" displayName="AwinOutreachPriorityTable" ref="A1:M22" headerRowCount="1">
-  <autoFilter ref="A1:M22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="AwinOutreachPriorityTable" displayName="AwinOutreachPriorityTable" ref="A1:M23" headerRowCount="1">
+  <autoFilter ref="A1:M23"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Priority Band"/>
@@ -248,8 +248,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="PageContentPriorityTable" displayName="PageContentPriorityTable" ref="A1:I25" headerRowCount="1">
-  <autoFilter ref="A1:I25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="PageContentPriorityTable" displayName="PageContentPriorityTable" ref="A1:I22" headerRowCount="1">
+  <autoFilter ref="A1:I22"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Rank"/>
     <tableColumn id="2" name="Workstream"/>
@@ -671,7 +671,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
     </row>
@@ -5652,7 +5652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6289,33 +6289,33 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>ops-awin-partnerships-workspace</t>
+          <t>bet-annual-research-report</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Bigger bet</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Monetisation</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Organised Awin/ folder workspace with AI-assisted research and briefing</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -6325,12 +6325,12 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>scripts/awin_sync.py, scripts/build_master_tracker.py, Awin/</t>
+          <t>New annual research page + methodology extension</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>ops-awin-publisher-api-integration</t>
+          <t>research/uk-broadband-customer-satisfaction methodology</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr"/>
@@ -6343,7 +6343,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>bet-annual-research-report</t>
+          <t>bet-componentise-interactive-layer</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -6353,19 +6353,19 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Functionality</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Annual 'State of UK Broadband' research report</t>
+          <t>Componentise the interactive layer on accessible primitives</t>
         </is>
       </c>
       <c r="F13" s="3" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
@@ -6379,12 +6379,12 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>New annual research page + methodology extension</t>
+          <t>components/</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>research/uk-broadband-customer-satisfaction methodology</t>
+          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr"/>
@@ -6397,7 +6397,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>bet-componentise-interactive-layer</t>
+          <t>bet-decouple-content-from-code</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -6407,19 +6407,19 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Componentise the interactive layer on accessible primitives</t>
+          <t>Decouple guide content from code deploys</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -6433,74 +6433,20 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>components/</t>
+          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>feat-shortlist-compare-basket, feat-price-drop-alerts</t>
+          <t>None, but easier before the guide count grows further</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr"/>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>bet-decouple-content-from-code</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Bigger bet</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Decouple guide content from code deploys</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G15" s="3" t="n">
-        <v>48</v>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>data/guides.ts, app/guides/[slug]/page.tsx</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t>None, but easier before the guide count grows further</t>
-        </is>
-      </c>
-      <c r="L15" s="3" t="inlineStr"/>
-      <c r="M15" s="3" t="inlineStr"/>
-      <c r="N15" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N15"/>
+  <autoFilter ref="A1:N14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6514,7 +6460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6793,40 +6739,36 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>P1 Follow up pending</t>
+          <t>P1 Respond to invitation</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Community Fibre</t>
+          <t>Connect Fibre</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>19595</v>
+        <v>114602</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Invited</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Check API status and send one tailored follow-up with the relevant live page, audience evidence and compliance controls.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/providers/community-fibre</t>
-        </is>
-      </c>
+          <t>Advertiser invited us directly (Awin Activity Stream) — review the fit assessment, reply to accept/decline, and run `awin_sync.py mark-reviewed` once actioned.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>After a reasonable review interval</t>
+          <t>Respond promptly: inbound, high-intent, low-effort to accept</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Waiting on advertiser</t>
+          <t>Awaiting our response</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
@@ -6840,16 +6782,16 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>P1 Follow up pending</t>
+          <t>P2 Follow up pending</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Cuckoo Broadband</t>
+          <t>Community Fibre</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>118743</v>
+        <v>19595</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
@@ -6863,7 +6805,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/cuckoo</t>
+          <t>https://broadbandpicker.co.uk/providers/community-fibre</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -6887,16 +6829,16 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>P1 Follow up pending</t>
+          <t>P2 Follow up pending</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>National Broadband</t>
+          <t>Cuckoo Broadband</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>20858</v>
+        <v>118743</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -6910,7 +6852,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/national-broadband</t>
+          <t>https://broadbandpicker.co.uk/providers/cuckoo</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -6934,16 +6876,16 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>P1 Follow up pending</t>
+          <t>P2 Follow up pending</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Pine Media Broadband</t>
+          <t>National Broadband</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>27840</v>
+        <v>20858</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
@@ -6957,7 +6899,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/pine-media</t>
+          <t>https://broadbandpicker.co.uk/providers/national-broadband</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -6981,16 +6923,16 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>P1 Follow up pending</t>
+          <t>P2 Follow up pending</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Sky ROI</t>
+          <t>Pine Media Broadband</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>12422</v>
+        <v>27840</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -7004,7 +6946,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/sky</t>
+          <t>https://broadbandpicker.co.uk/providers/pine-media</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -7028,16 +6970,16 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>P1 Follow up pending</t>
+          <t>P2 Follow up pending</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Trooli Full Fibre Broadband</t>
+          <t>Sky ROI</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>25528</v>
+        <v>12422</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
@@ -7051,7 +6993,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/trooli</t>
+          <t>https://broadbandpicker.co.uk/providers/sky</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -7075,16 +7017,16 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>P1 Follow up pending</t>
+          <t>P2 Follow up pending</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Zen Internet</t>
+          <t>Trooli Full Fibre Broadband</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>119927</v>
+        <v>25528</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -7098,7 +7040,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/zen-internet</t>
+          <t>https://broadbandpicker.co.uk/providers/trooli</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -7122,40 +7064,40 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>P2 Reapply with evidence</t>
+          <t>P2 Follow up pending</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>BT Broadband</t>
+          <t>Zen Internet</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>3041</v>
+        <v>119927</v>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Reapply selectively with stronger GSC traffic, GA4 commercial-click and content-quality evidence; record the rejection reason first.</t>
+          <t>Check API status and send one tailored follow-up with the relevant live page, audience evidence and compliance controls.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/bt</t>
+          <t>https://broadbandpicker.co.uk/providers/zen-internet</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Gate on stronger evidence; do not bulk reapply</t>
+          <t>After a reasonable review interval</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Waiting on advertiser</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr"/>
@@ -7169,16 +7111,16 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>P2 Reapply with evidence</t>
+          <t>P3 Reapply with evidence</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>BT Business Broadband</t>
+          <t>BT Broadband</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>3042</v>
+        <v>3041</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -7216,16 +7158,16 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>P2 Reapply with evidence</t>
+          <t>P3 Reapply with evidence</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>EE Home Broadband</t>
+          <t>BT Business Broadband</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>3516</v>
+        <v>3042</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
@@ -7239,7 +7181,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/ee</t>
+          <t>https://broadbandpicker.co.uk/providers/bt</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -7263,16 +7205,16 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>P2 Reapply with evidence</t>
+          <t>P3 Reapply with evidence</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Hyperoptic B2C</t>
+          <t>EE Home Broadband</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>5737</v>
+        <v>3516</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -7286,7 +7228,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/hyperoptic</t>
+          <t>https://broadbandpicker.co.uk/providers/ee</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -7310,16 +7252,16 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>P2 Reapply with evidence</t>
+          <t>P3 Reapply with evidence</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Plusnet Broadband</t>
+          <t>Hyperoptic B2C</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>2973</v>
+        <v>5737</v>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
@@ -7333,7 +7275,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/plusnet</t>
+          <t>https://broadbandpicker.co.uk/providers/hyperoptic</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -7357,16 +7299,16 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>P2 Reapply with evidence</t>
+          <t>P3 Reapply with evidence</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Virgin Media</t>
+          <t>Plusnet Broadband</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>6399</v>
+        <v>2973</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -7380,7 +7322,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/virgin-media</t>
+          <t>https://broadbandpicker.co.uk/providers/plusnet</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -7404,16 +7346,16 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>P2 Reapply with evidence</t>
+          <t>P3 Reapply with evidence</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Vodafone Ltd</t>
+          <t>Virgin Media</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>1257</v>
+        <v>6399</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
@@ -7427,7 +7369,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/vodafone</t>
+          <t>https://broadbandpicker.co.uk/providers/virgin-media</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -7451,16 +7393,16 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>P2 Reapply with evidence</t>
+          <t>P3 Reapply with evidence</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>giffgaff</t>
+          <t>Vodafone Ltd</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>3599</v>
+        <v>1257</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
@@ -7474,7 +7416,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/giffgaff</t>
+          <t>https://broadbandpicker.co.uk/providers/vodafone</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -7498,16 +7440,16 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>P2 Reapply with evidence</t>
+          <t>P3 Reapply with evidence</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>toob</t>
+          <t>giffgaff</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>117433</v>
+        <v>3599</v>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
@@ -7521,7 +7463,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/toob</t>
+          <t>https://broadbandpicker.co.uk/providers/giffgaff</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -7545,34 +7487,40 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>P3 Under review</t>
+          <t>P3 Reapply with evidence</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>World Businesses for Sale</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
+          <t>toob</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>117433</v>
+      </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Not an active Awin application yet — decide whether to apply at all based on the fit assessment in Awin/advertisers/&lt;slug&gt;/research.md.</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr"/>
+          <t>Reapply selectively with stronger GSC traffic, GA4 commercial-click and content-quality evidence; record the rejection reason first.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/toob</t>
+        </is>
+      </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>No timing pressure — inbound pitch, not a pending application</t>
+          <t>Gate on stronger evidence; do not bulk reapply</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Under review</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr"/>
@@ -7580,8 +7528,49 @@
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
     </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>P4 Under review</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>World Businesses for Sale</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Not an active Awin application yet — decide whether to apply at all based on the fit assessment in Awin/advertisers/&lt;slug&gt;/research.md.</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>No timing pressure — inbound pitch, not a pending application</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Under review</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr"/>
+      <c r="K23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr"/>
+      <c r="M23" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M22"/>
+  <autoFilter ref="A1:M23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7595,7 +7584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7710,7 +7699,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>/postcode/m1</t>
+          <t>/postcode/ct1</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -7724,7 +7713,7 @@
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>59.4</v>
+        <v>55.1</v>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
@@ -7733,7 +7722,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 56; CTR 0; position 12.875; top queries: m1 broadband; cheap broadband deals manchester; m1 wifi broadband; m1 internet plan; m1 internet broadband</t>
+          <t>Clicks 0; impressions 120; CTR 0; position 9.866666666666667; top queries: broadband deals in canterbury</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -7753,7 +7742,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>/postcode/ng1</t>
+          <t>/providers/compare/ee-vs-talktalk</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -7767,7 +7756,7 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>55.4</v>
+        <v>54.7</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
@@ -7776,7 +7765,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 132; CTR 0; position 13.64393939393939; top queries: broadband deals nottingham; broadband deals in nottingham; broadband deals nottinghamshire; internet deals nottingham; cheapest broadband nottingham</t>
+          <t>Clicks 2; impressions 107; CTR 0.01869158878504673; position 8.317757009345794; top queries: is ee broadband better than talktalk; are talktalk and ee the same; who is dido harding; talktalk.co.uk/homesafe; talktalk uswitch</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -7796,7 +7785,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>/postcode/rg1</t>
+          <t>/postcode/rm1</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -7810,7 +7799,7 @@
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>55.3</v>
+        <v>54.2</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
@@ -7819,7 +7808,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 126; CTR 0; position 14.90476190476191; top queries: broadband deals in reading; broadband in reading; broadband deals reading; broadband reading; cheapest</t>
+          <t>Clicks 0; impressions 94; CTR 0; position 9.574468085106384; top queries: broadband deals in romford; broadband deals romford; internet deals romford; best internet provider romford; whats the best broadband in my area</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -7839,7 +7828,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>/postcode/ct1</t>
+          <t>/guides/broadband-deals-with-cashback</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -7853,7 +7842,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>55.1</v>
+        <v>54.1</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -7862,7 +7851,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 120; CTR 0; position 9.866666666666667; top queries: broadband deals in canterbury</t>
+          <t>Clicks 0; impressions 91; CTR 0; position 14.54945054945055; top queries: compare broadband providers with cashback; broadband price rises with cashback; compare internet providers with cashback; broadband switching deals with cashback; where should i look for broadband deals that offer extra perks?</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -7882,12 +7871,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>/providers/compare/ee-vs-talktalk</t>
+          <t>/postcode/bs1</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Quick ranking win</t>
+          <t>Page-two opportunity</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -7896,7 +7885,7 @@
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>54.7</v>
+        <v>53.6</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
@@ -7905,12 +7894,12 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Clicks 2; impressions 107; CTR 0.01869158878504673; position 8.317757009345794; top queries: is ee broadband better than talktalk; are talktalk and ee the same; who is dido harding; talktalk.co.uk/homesafe; talktalk uswitch</t>
+          <t>Clicks 1; impressions 105; CTR 0.009523809523809525; position 21.93333333333333; top queries: broadband deals bristol; broadband deals in bristol; best broadband deals bristol; best broadband deals in bristol</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
         </is>
       </c>
     </row>
@@ -7925,7 +7914,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>/postcode/rm1</t>
+          <t>/postcode/e1</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -7939,7 +7928,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>54.2</v>
+        <v>53.5</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -7948,7 +7937,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 94; CTR 0; position 9.574468085106384; top queries: broadband deals in romford; broadband deals romford; internet deals romford; best internet provider romford; whats the best broadband in my area</t>
+          <t>Clicks 1; impressions 77; CTR 0.01298701298701299; position 4.870129870129871; top queries: yes please; ee whitechapel; e1</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -7968,12 +7957,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>/guides/broadband-deals-with-cashback</t>
+          <t>/postcode/ne1</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Quick ranking win</t>
+          <t>Page-two opportunity</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -7982,7 +7971,7 @@
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>54.1</v>
+        <v>53.3</v>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
@@ -7991,12 +7980,12 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 91; CTR 0; position 14.54945054945055; top queries: compare broadband providers with cashback; broadband price rises with cashback; compare internet providers with cashback; broadband switching deals with cashback; where should i look for broadband deals that offer extra perks?</t>
+          <t>Clicks 0; impressions 97; CTR 0; position 23.11340206185567; top queries: broadband deals newcastle; broadband deals in newcastle; broadband newcastle; broadband deals north tyneside; best broadband deals newcastle</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
         </is>
       </c>
     </row>
@@ -8011,12 +8000,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>/postcode/bs1</t>
+          <t>/postcode/bn1</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Page-two opportunity</t>
+          <t>Quick ranking win</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -8025,7 +8014,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>53.6</v>
+        <v>53.3</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
@@ -8034,12 +8023,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Clicks 1; impressions 105; CTR 0.009523809523809525; position 21.93333333333333; top queries: broadband deals bristol; broadband deals in bristol; best broadband deals bristol; best broadband deals in bristol</t>
+          <t>Clicks 1; impressions 73; CTR 0.0136986301369863; position 11.49315068493151; top queries: broadband deals in brighton; broadband deals brighton</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
         </is>
       </c>
     </row>
@@ -8054,7 +8043,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>/postcode/e1</t>
+          <t>/postcode/gu1</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -8068,7 +8057,7 @@
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>53.5</v>
+        <v>52.9</v>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
@@ -8077,7 +8066,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Clicks 1; impressions 77; CTR 0.01298701298701299; position 4.870129870129871; top queries: yes please; ee whitechapel; e1</t>
+          <t>Clicks 1; impressions 65; CTR 0.01538461538461539; position 11.64615384615385; top queries: broadband deals in guildford</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -8097,12 +8086,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>/postcode/ne1</t>
+          <t>/postcode/ha1</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Page-two opportunity</t>
+          <t>Quick ranking win</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -8111,7 +8100,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>53.3</v>
+        <v>52.6</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
@@ -8120,12 +8109,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 97; CTR 0; position 23.11340206185567; top queries: broadband deals newcastle; broadband deals in newcastle; broadband newcastle; broadband deals north tyneside; best broadband deals newcastle</t>
+          <t>Clicks 0; impressions 60; CTR 0; position 8.533333333333333; top queries: broadband deals in harrow; ha1 4bh; ha1; broadband</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
         </is>
       </c>
     </row>
@@ -8140,12 +8129,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>/postcode/bn1</t>
+          <t>/guides/broadband-deals-with-no-setup-fee</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Quick ranking win</t>
+          <t>Page-two opportunity</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -8154,7 +8143,7 @@
         </is>
       </c>
       <c r="F13" s="3" t="n">
-        <v>53.3</v>
+        <v>52.5</v>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
@@ -8163,12 +8152,12 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Clicks 1; impressions 73; CTR 0.0136986301369863; position 11.49315068493151; top queries: broadband deals in brighton; broadband deals brighton</t>
+          <t>Clicks 0; impressions 548; CTR 0; position 26.25547445255474; top queries: broadband deals no upfront cost; broadband no upfront cost; broadband and tv deals no upfront cost; broadband no upfront costs; broadband no setup fee</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
         </is>
       </c>
     </row>
@@ -8183,7 +8172,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>/postcode/gu1</t>
+          <t>/postcode/w5</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -8197,7 +8186,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>52.9</v>
+        <v>52.4</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -8206,7 +8195,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Clicks 1; impressions 65; CTR 0.01538461538461539; position 11.64615384615385; top queries: broadband deals in guildford</t>
+          <t>Clicks 0; impressions 56; CTR 0; position 6.732142857142857; top queries: None</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -8226,7 +8215,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>/postcode/ha1</t>
+          <t>/postcode/se1</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -8240,7 +8229,7 @@
         </is>
       </c>
       <c r="F15" s="3" t="n">
-        <v>52.6</v>
+        <v>52.2</v>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
@@ -8249,7 +8238,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 60; CTR 0; position 8.533333333333333; top queries: broadband deals in harrow; ha1 4bh; ha1; broadband</t>
+          <t>Clicks 0; impressions 53; CTR 0; position 6.037735849056604; top queries: find the best broadband deals in southwark under £30 a month.; find the best broadband deals in southwark under £25 a month.; fibre broadband in southwark</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -8269,12 +8258,12 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>/guides/broadband-deals-with-no-setup-fee</t>
+          <t>/postcode/en1</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Page-two opportunity</t>
+          <t>Quick ranking win</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -8283,7 +8272,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>52.5</v>
+        <v>51.5</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
@@ -8292,12 +8281,12 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 548; CTR 0; position 26.25547445255474; top queries: broadband deals no upfront cost; broadband no upfront cost; broadband and tv deals no upfront cost; broadband no upfront costs; broadband no setup fee</t>
+          <t>Clicks 0; impressions 43; CTR 0; position 14.13953488372093; top queries: broadband deals in enfield</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
+          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
         </is>
       </c>
     </row>
@@ -8312,7 +8301,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>/postcode/w5</t>
+          <t>/postcode/nw1</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -8326,7 +8315,7 @@
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>52.4</v>
+        <v>51.2</v>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
@@ -8335,7 +8324,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 56; CTR 0; position 6.732142857142857; top queries: None</t>
+          <t>Clicks 0; impressions 40; CTR 0; position 4.9; top queries: None</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -8355,7 +8344,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>/postcode/se1</t>
+          <t>/postcode/ub1</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -8369,7 +8358,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>52.2</v>
+        <v>51.2</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -8378,7 +8367,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 53; CTR 0; position 6.037735849056604; top queries: find the best broadband deals in southwark under £30 a month.; find the best broadband deals in southwark under £25 a month.; fibre broadband in southwark</t>
+          <t>Clicks 0; impressions 40; CTR 0; position 8.025; top queries: broadband deals in southall; yes; and cheapest</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -8398,12 +8387,12 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>/postcode/en1</t>
+          <t>/postcode/lu1</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Quick ranking win</t>
+          <t>Page-two opportunity</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -8412,7 +8401,7 @@
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>51.5</v>
+        <v>47.3</v>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
@@ -8421,12 +8410,12 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 43; CTR 0; position 14.13953488372093; top queries: broadband deals in enfield</t>
+          <t>Clicks 0; impressions 128; CTR 0; position 15.546875; top queries: broadband deals in luton; broadband deals luton; broadband luton; internet providers luton; broadband deals near me</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
         </is>
       </c>
     </row>
@@ -8441,12 +8430,12 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>/postcode/nw1</t>
+          <t>/postcode/so14</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Quick ranking win</t>
+          <t>Page-two opportunity</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -8455,7 +8444,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>51.2</v>
+        <v>46.6</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
@@ -8464,12 +8453,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 40; CTR 0; position 4.9; top queries: None</t>
+          <t>Clicks 1; impressions 104; CTR 0.009615384615384616; position 26.42307692307692; top queries: broadband deals in southampton; broadband deals southampton; broadband company southampton; internet providers southampton; fibre broadband southampton</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
         </is>
       </c>
     </row>
@@ -8484,12 +8473,12 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>/postcode/ub1</t>
+          <t>/postcode/l1</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Quick ranking win</t>
+          <t>Page-two opportunity</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -8498,7 +8487,7 @@
         </is>
       </c>
       <c r="F21" s="3" t="n">
-        <v>51.2</v>
+        <v>45.5</v>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
@@ -8507,12 +8496,12 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 40; CTR 0; position 8.025; top queries: broadband deals in southall; yes; and cheapest</t>
+          <t>Clicks 0; impressions 77; CTR 0; position 26.25974025974026; top queries: broadband deals liverpool; broadband comparison liverpool; internet deals liverpool; broadband deals in liverpool; best broadband deals liverpool</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Strengthen the title/snippet, answer the leading queries directly, add internal links and refresh supporting evidence.</t>
+          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
         </is>
       </c>
     </row>
@@ -8522,26 +8511,26 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Existing-page SEO improvement</t>
+          <t>New evidence-led page</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>/postcode/lu1</t>
+          <t>New annual research page + methodology extension</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Page-two opportunity</t>
+          <t>Annual 'State of UK Broadband' research report</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Weekly GSC/GA4 action queue</t>
+          <t>Master tracker</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>47.3</v>
+        <v>41</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
@@ -8550,146 +8539,17 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Clicks 0; impressions 128; CTR 0; position 15.546875; top queries: broadband deals in luton; broadband deals luton; broadband luton; internet providers luton; broadband deals near me</t>
+          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Existing-page SEO improvement</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>/postcode/so14</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>Page-two opportunity</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>Weekly GSC/GA4 action queue</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="n">
-        <v>46.6</v>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Clicks 1; impressions 104; CTR 0.009615384615384616; position 26.42307692307692; top queries: broadband deals in southampton; broadband deals southampton; broadband company southampton; internet providers southampton; fibre broadband southampton</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Existing-page SEO improvement</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>/postcode/l1</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Page-two opportunity</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Weekly GSC/GA4 action queue</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="n">
-        <v>45.5</v>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>Clicks 0; impressions 77; CTR 0; position 26.25974025974026; top queries: broadband deals liverpool; broadband comparison liverpool; internet deals liverpool; broadband deals in liverpool; best broadband deals liverpool</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>Expand missing subtopics for the leading queries, improve topical internal links and validate intent alignment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>New evidence-led page</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>New annual research page + methodology extension</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>Annual 'State of UK Broadband' research report</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>Master tracker</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="n">
-        <v>41</v>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>No competitor scanned publishes original research. Built on the existing /research page's methodology, an annual report is a natural press/backlink asset a comparison-table page can never be.</t>
-        </is>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
           <t>Build after higher-confidence thin-content and ranking opportunities.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I25"/>
+  <autoFilter ref="A1:I22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8713,7 +8573,7 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="31" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
@@ -8814,7 +8674,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -8868,7 +8728,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -8922,7 +8782,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -8976,7 +8836,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -9030,7 +8890,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -9084,7 +8944,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -9138,7 +8998,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -9192,7 +9052,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -9246,7 +9106,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -9300,7 +9160,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -9354,7 +9214,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -9408,7 +9268,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -9462,7 +9322,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -9516,7 +9376,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -9570,7 +9430,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -9624,7 +9484,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -9678,7 +9538,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -9732,7 +9592,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -9786,7 +9646,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -9840,7 +9700,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -9894,7 +9754,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -9948,7 +9808,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -10002,7 +9862,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -10056,7 +9916,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -10110,7 +9970,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -10164,7 +10024,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -10218,7 +10078,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -10272,7 +10132,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -10326,7 +10186,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -10380,7 +10240,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -10434,7 +10294,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -10488,7 +10348,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -10542,7 +10402,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Committed</t>
+          <t>Live but not committed to git</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -14900,7 +14760,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>108 total (33 page builds, 75 feature/strategy builds); 94 already marked Done.</t>
+          <t>108 total (33 page builds, 75 feature/strategy builds); 95 already marked Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: mark best-broadband-and-tv-deals fix as done (1 of 4)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/master-build-tracker.xlsx
+++ b/docs/master-build-tracker.xlsx
@@ -2688,12 +2688,16 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr"/>
-      <c r="L42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>1 of 4 done: best-broadband-and-tv-deals shipped 2026-09-01 (live-verified) — internal linking (4 provider pages + homepage + 2 guides), interactive filterable/sortable comparison table (data/tvBroadbandBundles.ts + TvBundleComparisonTable.tsx), and Product/Offer JSON-LD added. Remaining: best-full-fibre-broadband-uk, best-business-broadband-providers-uk, best-5g-home-broadband-uk.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
@@ -6758,7 +6762,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -6773,7 +6777,11 @@
       </c>
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>1 of 4 done: best-broadband-and-tv-deals shipped 2026-09-01 (live-verified) — internal linking (4 provider pages + homepage + 2 guides), interactive filterable/sortable comparison table (data/tvBroadbandBundles.ts + TvBundleComparisonTable.tsx), and Product/Offer JSON-LD added. Remaining: best-full-fibre-broadband-uk, best-business-broadband-providers-uk, best-5g-home-broadband-uk.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">

</xml_diff>